<commit_message>
Daily workbook: 2026-08-28 05:21 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 28 Aug 2026, 04:22 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 28 Aug 2026, 05:21 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 28 Aug 2026, 04:22 AM · Yahoo Finance data</t>
+          <t>Built 28 Aug 2026, 05:21 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>YouTube Faces Potential Lawsuit from FTC As Regulator Probes Whether It Broke Its Own Policies on Suspended...</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>FTC Probes YouTube Over Suspended Social Media Accounts, Says Report — GOOGL Stock In Focus</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
+      <c r="AZ34" s="79" t="inlineStr">
         <is>
           <t>Market Chatter: Alphabet's YouTube Investigated by FTC on Consumer Protection</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Should SpaceX Join the "Magnificent Seven"? Here's 1 Stock I'd Kick Out to Make Room.</t>
         </is>
       </c>
     </row>
@@ -9592,17 +9592,17 @@
       </c>
       <c r="AX40" s="79" t="inlineStr">
         <is>
+          <t>Is Nebius Group (NasdaqGS:NBIS) Priced For Perfection On AI Growth?</t>
+        </is>
+      </c>
+      <c r="AY40" s="79" t="inlineStr">
+        <is>
           <t>What's Going On With Nebius Stock Thursday</t>
         </is>
       </c>
-      <c r="AY40" s="79" t="inlineStr">
+      <c r="AZ40" s="79" t="inlineStr">
         <is>
           <t>George Soros Is Betting Big on Utility Stocks as AI Power Demand Surges</t>
-        </is>
-      </c>
-      <c r="AZ40" s="79" t="inlineStr">
-        <is>
-          <t>Nebius Group stock surges as funding concerns ease</t>
         </is>
       </c>
     </row>
@@ -9780,17 +9780,17 @@
       </c>
       <c r="AX41" s="90" t="inlineStr">
         <is>
+          <t>The GTA 6 Leak Saga May Be Over — the Money Trail Shows Where It Went</t>
+        </is>
+      </c>
+      <c r="AY41" s="90" t="inlineStr">
+        <is>
           <t>Netflix (NFLX) Stock Falls Amid Market Uptick: What Investors Need to Know</t>
         </is>
       </c>
-      <c r="AY41" s="90" t="inlineStr">
+      <c r="AZ41" s="90" t="inlineStr">
         <is>
           <t>NFLX Has Bounced From This Price Before. Now What?</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>Unusual Options Activity: NFLX, HONA, and MSFT Lead the Way With These 3 Options Strategies</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures Rise With Fed Chief Warsh Due; Nvidia, These 7 Stocks Are In Buy Zones</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
+          <t>Bill Ackman Just Made His Biggest Portfolio Overhaul in Years, Adding Netflix, Visa, and Mastercard to Pers...</t>
+        </is>
+      </c>
+      <c r="AZ43" s="90" t="inlineStr">
+        <is>
           <t>Amkor, FormFactor, Vishay Intertechnology, Allegro MicroSystems, and Intel Shares Skyrocket, What You Need ...</t>
-        </is>
-      </c>
-      <c r="AY43" s="90" t="inlineStr">
-        <is>
-          <t>Nasdaq Futures Sink While S&amp;P 500, Dow Futures Gain Ahead Of Fed Chief Warsh’s Jackson Hole Speech: PYPL, M...</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Asian shares mostly gain after upbeat results for Nvidia and others lift US stocks</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 28 Aug 2026, 04:22 AM · Yahoo Finance data</t>
+          <t>Built 28 Aug 2026, 05:21 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 28 Aug 2026, 04:22 AM · Yahoo Finance data</t>
+          <t>Built 28 Aug 2026, 05:21 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 28 Aug 2026, 04:22 AM · Yahoo Finance data</t>
+          <t>Built 28 Aug 2026, 05:21 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 28 Aug 2026, 04:22 AM · Yahoo Finance data</t>
+          <t>Built 28 Aug 2026, 05:21 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-08-29 02:50 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'08-25'!$5:$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'08-24'!$A$6:$AZ$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'08-24'!$5:$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 29 Aug 2026, 01:05 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 29 Aug 2026, 02:50 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1376,35 +1376,35 @@
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="F8" s="8" t="n"/>
       <c r="G8" s="8" t="n"/>
       <c r="H8" s="14" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="I8" s="8" t="n"/>
       <c r="J8" s="8" t="n"/>
       <c r="K8" s="15" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="L8" s="10" t="n"/>
       <c r="M8" s="10" t="n"/>
       <c r="N8" s="15" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="O8" s="10" t="n"/>
       <c r="P8" s="10" t="n"/>
       <c r="Q8" s="16" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>45</t>
         </is>
       </c>
       <c r="R8" s="12" t="n"/>
@@ -1413,14 +1413,14 @@
     <row r="9" ht="15" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>of 39 names</t>
+          <t>of 40 names</t>
         </is>
       </c>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>of 39 names</t>
+          <t>of 40 names</t>
         </is>
       </c>
       <c r="F9" s="8" t="n"/>
@@ -1441,7 +1441,7 @@
       <c r="M9" s="10" t="n"/>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>of 39 names</t>
+          <t>of 40 names</t>
         </is>
       </c>
       <c r="O9" s="10" t="n"/>
@@ -2197,11 +2197,11 @@
       </c>
       <c r="H35" s="24" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="I35" s="26" t="n">
-        <v>-0.02845037703741871</v>
+        <v>-0.04256684013924827</v>
       </c>
       <c r="J35" s="27" t="n">
         <v>1</v>
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="L35" s="28" t="n">
-        <v>41.50443800949344</v>
+        <v>47.15991440223318</v>
       </c>
     </row>
     <row r="36">
@@ -2237,11 +2237,11 @@
       </c>
       <c r="H36" s="31" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="I36" s="33" t="n">
-        <v>-0.02326562725379</v>
+        <v>-0.02845037703741871</v>
       </c>
       <c r="J36" s="34" t="n">
         <v>1</v>
@@ -2252,7 +2252,7 @@
         </is>
       </c>
       <c r="L36" s="35" t="n">
-        <v>44.83215501734773</v>
+        <v>41.50443800949344</v>
       </c>
     </row>
     <row r="37">
@@ -2277,11 +2277,11 @@
       </c>
       <c r="H37" s="24" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="I37" s="26" t="n">
-        <v>-0.01042150902637939</v>
+        <v>-0.02326562725379</v>
       </c>
       <c r="J37" s="27" t="n">
         <v>1</v>
@@ -2292,7 +2292,7 @@
         </is>
       </c>
       <c r="L37" s="28" t="n">
-        <v>35.78398855531299</v>
+        <v>44.83215501734773</v>
       </c>
     </row>
     <row r="38">
@@ -2317,11 +2317,11 @@
       </c>
       <c r="H38" s="31" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="I38" s="33" t="n">
-        <v>-0.004030459153398613</v>
+        <v>-0.01042150902637939</v>
       </c>
       <c r="J38" s="34" t="n">
         <v>1</v>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="L38" s="35" t="n">
-        <v>43.30756864961271</v>
+        <v>35.78398855531299</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
@@ -2741,22 +2741,22 @@
       </c>
       <c r="H51" s="24" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="I51" s="26" t="n">
-        <v>-0.03588291869363736</v>
+        <v>-0.04256684013924827</v>
       </c>
       <c r="J51" s="27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K51" s="23" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Very Weak</t>
         </is>
       </c>
       <c r="L51" s="28" t="n">
-        <v>48.37686691688126</v>
+        <v>47.15991440223318</v>
       </c>
     </row>
     <row r="52">
@@ -2781,22 +2781,22 @@
       </c>
       <c r="H52" s="31" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="I52" s="33" t="n">
-        <v>-0.03392203277851213</v>
+        <v>-0.03588291869363736</v>
       </c>
       <c r="J52" s="34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K52" s="30" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="L52" s="35" t="n">
-        <v>52.59366691435373</v>
+        <v>48.37686691688126</v>
       </c>
     </row>
   </sheetData>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Aug 2026, 01:05 AM · Yahoo Finance data</t>
+          <t>Built 29 Aug 2026, 02:50 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3132,22 +3132,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>12 of 39</t>
+          <t>12 of 40</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>27 of 39</t>
+          <t>28 of 40</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>4.3 / 9</t>
+          <t>4.2 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>16 of 39</t>
+          <t>16 of 40</t>
         </is>
       </c>
     </row>
@@ -7173,7 +7173,7 @@
         <v>-0.06332041548914424</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
@@ -7361,7 +7361,7 @@
         <v>-0.05517577254916717</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E29" s="30" t="inlineStr">
         <is>
@@ -7737,7 +7737,7 @@
         <v>-0.05943759603113641</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E31" s="30" t="inlineStr">
         <is>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>AppLovin vs. Alphabet: Which High-Growth Digital Media Stock Is the Better Investment in 2026?</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
+          <t>Alphabet (GOOGL) Faces FTC Heat, AI Turmoil And UK Play Store Settlement</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>Stock Market Today, Aug. 28: Marvell Slides 10% on Softer Fiscal 2028 Guidance and Google Deal Timing</t>
-        </is>
-      </c>
-      <c r="AY34" s="79" t="inlineStr">
-        <is>
-          <t>Sector Update: Tech Stocks Fall Late Afternoon</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>$353M Settlement Barely Dents Alphabet’s (GOOGL) Bigger Bet</t>
         </is>
       </c>
     </row>
@@ -8489,7 +8489,7 @@
         <v>-0.1253392097053883</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -9053,7 +9053,7 @@
         <v>-0.07343520222782773</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -9425,57 +9425,171 @@
           <t>NBIS</t>
         </is>
       </c>
-      <c r="C40" s="26" t="n"/>
-      <c r="D40" s="27" t="n"/>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="23" t="n"/>
-      <c r="I40" s="23" t="n"/>
-      <c r="J40" s="23" t="n"/>
-      <c r="K40" s="23" t="n"/>
-      <c r="L40" s="23" t="n"/>
-      <c r="M40" s="23" t="n"/>
-      <c r="N40" s="69" t="n"/>
-      <c r="O40" s="23" t="n"/>
-      <c r="P40" s="25" t="n"/>
+      <c r="C40" s="26" t="n">
+        <v>-0.04256684013924827</v>
+      </c>
+      <c r="D40" s="27" t="n">
+        <v>18</v>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L40" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N40" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="O40" s="23" t="inlineStr">
+        <is>
+          <t>Very Weak</t>
+        </is>
+      </c>
+      <c r="P40" s="25" t="inlineStr">
+        <is>
+          <t>Long-term up, short-term mixed</t>
+        </is>
+      </c>
       <c r="Q40" s="25" t="inlineStr">
         <is>
           <t>Nebius Group N.V.</t>
         </is>
       </c>
-      <c r="R40" s="70" t="n"/>
-      <c r="S40" s="71" t="n"/>
-      <c r="T40" s="72" t="n"/>
-      <c r="U40" s="72" t="n"/>
-      <c r="V40" s="72" t="n"/>
-      <c r="W40" s="73" t="n"/>
-      <c r="X40" s="74" t="n"/>
-      <c r="Y40" s="28" t="n"/>
-      <c r="Z40" s="28" t="n"/>
-      <c r="AA40" s="28" t="n"/>
-      <c r="AB40" s="75" t="n"/>
-      <c r="AC40" s="75" t="n"/>
-      <c r="AD40" s="75" t="n"/>
-      <c r="AE40" s="72" t="n"/>
-      <c r="AF40" s="72" t="n"/>
-      <c r="AG40" s="72" t="n"/>
-      <c r="AH40" s="72" t="n"/>
-      <c r="AI40" s="72" t="n"/>
-      <c r="AJ40" s="72" t="n"/>
-      <c r="AK40" s="72" t="n"/>
-      <c r="AL40" s="72" t="n"/>
-      <c r="AM40" s="76" t="n"/>
-      <c r="AN40" s="29" t="n"/>
-      <c r="AO40" s="77" t="n"/>
-      <c r="AP40" s="72" t="n"/>
-      <c r="AQ40" s="72" t="n"/>
-      <c r="AR40" s="29" t="n"/>
-      <c r="AS40" s="78" t="n"/>
-      <c r="AT40" s="26" t="n"/>
-      <c r="AU40" s="26" t="n"/>
-      <c r="AV40" s="26" t="n"/>
-      <c r="AW40" s="26" t="n"/>
+      <c r="R40" s="70" t="n">
+        <v>209.1799926757812</v>
+      </c>
+      <c r="S40" s="71" t="n">
+        <v>-9.300003051757812</v>
+      </c>
+      <c r="T40" s="72" t="n">
+        <v>211.9700012207031</v>
+      </c>
+      <c r="U40" s="72" t="n">
+        <v>214.2799987792969</v>
+      </c>
+      <c r="V40" s="72" t="n">
+        <v>205.4799957275391</v>
+      </c>
+      <c r="W40" s="73" t="n">
+        <v>13064528</v>
+      </c>
+      <c r="X40" s="74" t="n">
+        <v>0.5282577481795031</v>
+      </c>
+      <c r="Y40" s="28" t="n">
+        <v>47.15991440223318</v>
+      </c>
+      <c r="Z40" s="28" t="n">
+        <v>23.38536963898732</v>
+      </c>
+      <c r="AA40" s="28" t="n">
+        <v>10.26259211559968</v>
+      </c>
+      <c r="AB40" s="75" t="n">
+        <v>1.618478299991892</v>
+      </c>
+      <c r="AC40" s="75" t="n">
+        <v>4.122908923924964</v>
+      </c>
+      <c r="AD40" s="75" t="n">
+        <v>-2.504430623933072</v>
+      </c>
+      <c r="AE40" s="72" t="n">
+        <v>219.0393337059973</v>
+      </c>
+      <c r="AF40" s="72" t="n">
+        <v>219.4930636158715</v>
+      </c>
+      <c r="AG40" s="72" t="n">
+        <v>219.3753997802734</v>
+      </c>
+      <c r="AH40" s="72" t="n">
+        <v>206.6682002258301</v>
+      </c>
+      <c r="AI40" s="72" t="n">
+        <v>151.8271253585816</v>
+      </c>
+      <c r="AJ40" s="72" t="n">
+        <v>274.7259626096215</v>
+      </c>
+      <c r="AK40" s="72" t="n">
+        <v>222.9654998779297</v>
+      </c>
+      <c r="AL40" s="72" t="n">
+        <v>171.2050371462378</v>
+      </c>
+      <c r="AM40" s="76" t="n">
+        <v>0.3668336170639773</v>
+      </c>
+      <c r="AN40" s="29" t="n">
+        <v>46.42912267595656</v>
+      </c>
+      <c r="AO40" s="77" t="n">
+        <v>10.08548385902063</v>
+      </c>
+      <c r="AP40" s="72" t="n">
+        <v>299.8599853515625</v>
+      </c>
+      <c r="AQ40" s="72" t="n">
+        <v>63.2599983215332</v>
+      </c>
+      <c r="AR40" s="29" t="n">
+        <v>-30.24077806495789</v>
+      </c>
+      <c r="AS40" s="78" t="n">
+        <v>61.67371189911682</v>
+      </c>
+      <c r="AT40" s="26" t="n">
+        <v>-0.04540689081968652</v>
+      </c>
+      <c r="AU40" s="26" t="n">
+        <v>0.110120473420084</v>
+      </c>
+      <c r="AV40" s="26" t="n">
+        <v>-0.09481156263498935</v>
+      </c>
+      <c r="AW40" s="26" t="n">
+        <v>1.499014253628212</v>
+      </c>
       <c r="AX40" s="79" t="inlineStr">
         <is>
           <t>Zacks Investment Ideas feature highlights: QQQ, NVIDIA, CoreWeave, Nebius, TeraWulf, Cipher and IREN</t>
@@ -9671,12 +9785,12 @@
       </c>
       <c r="AY41" s="90" t="inlineStr">
         <is>
+          <t>Netflix Stock Is Up 25% From Its 2026 Lows. More Gains for NFLX Could Be in Store.</t>
+        </is>
+      </c>
+      <c r="AZ41" s="90" t="inlineStr">
+        <is>
           <t>Netflix Stock Price Prediction: The Road Back to $100</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>Where Will Netflix Stock Be in 5 Years?</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9993,7 @@
         <v>-0.04574959589106331</v>
       </c>
       <c r="D43" s="34" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E43" s="30" t="inlineStr">
         <is>
@@ -9957,7 +10071,7 @@
         <v>229.2599945068359</v>
       </c>
       <c r="V43" s="83" t="n">
-        <v>216.8099975585938</v>
+        <v>216.8200073242188</v>
       </c>
       <c r="W43" s="84" t="n">
         <v>194036188</v>
@@ -9972,7 +10086,7 @@
         <v>44.35832261100078</v>
       </c>
       <c r="AA43" s="35" t="n">
-        <v>16.84031568016377</v>
+        <v>16.84184550764452</v>
       </c>
       <c r="AB43" s="86" t="n">
         <v>2.348894281795168</v>
@@ -10014,7 +10128,7 @@
         <v>10.81203662259366</v>
       </c>
       <c r="AO43" s="88" t="n">
-        <v>3.522423226324357</v>
+        <v>3.5220945739461</v>
       </c>
       <c r="AP43" s="83" t="n">
         <v>236.5399932861328</v>
@@ -10042,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Why Elastic Stock Snapped Back Today</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>This AI Energy Stock Is Up Nearly 2,000% in the Last Two Years. Could It Be Nvidia's Next Big Investment?</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>Nvidia Drops 3.3% as $315 Target Meets a $108 Billion Test</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Nvidia Quietly Became Its Own Market Category</t>
         </is>
       </c>
     </row>
@@ -10230,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Expert ranks top 5 U.S. tech companies to recruit from</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>Can PLTR Stock Live Up To Its Multiple?</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>Palantir’s Pentagon AI surge comes with a question investors can’t ignore</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>NVIDIA (NVDA), Palantir Technologies (PLTR), and the AI Achilles’ Heel: Steve Eisman’s Concentration Warnin...</t>
         </is>
       </c>
     </row>
@@ -10443,7 +10557,7 @@
         <v>-0.04649784460844808</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
@@ -11529,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Aug 2026, 01:05 AM · Yahoo Finance data</t>
+          <t>Built 29 Aug 2026, 02:50 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -11554,22 +11668,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>21 of 39</t>
+          <t>22 of 40</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>18 of 39</t>
+          <t>18 of 40</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>5.3 / 9</t>
+          <t>5.2 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>22 of 39</t>
+          <t>22 of 40</t>
         </is>
       </c>
     </row>
@@ -14663,7 +14777,7 @@
         <v>0.003604958753321119</v>
       </c>
       <c r="D24" s="27" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
@@ -14839,7 +14953,7 @@
         <v>-0.008857794924257756</v>
       </c>
       <c r="D25" s="34" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E25" s="30" t="inlineStr">
         <is>
@@ -15015,7 +15129,7 @@
         <v>-0.01544486334918349</v>
       </c>
       <c r="D26" s="27" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
@@ -15191,7 +15305,7 @@
         <v>0.01865234899615387</v>
       </c>
       <c r="D27" s="34" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E27" s="30" t="inlineStr">
         <is>
@@ -15367,7 +15481,7 @@
         <v>0.01652994979538658</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
@@ -15895,7 +16009,7 @@
         <v>-0.00959387829211289</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E31" s="30" t="inlineStr">
         <is>
@@ -16071,7 +16185,7 @@
         <v>-0.01374842694128908</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
@@ -16247,7 +16361,7 @@
         <v>0.01819671921894161</v>
       </c>
       <c r="D33" s="34" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E33" s="30" t="inlineStr">
         <is>
@@ -16423,7 +16537,7 @@
         <v>-0.004099128939600072</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
@@ -16951,7 +17065,7 @@
         <v>0.01750710664804522</v>
       </c>
       <c r="D37" s="34" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E37" s="30" t="inlineStr">
         <is>
@@ -17303,7 +17417,7 @@
         <v>-0.003207597706004428</v>
       </c>
       <c r="D39" s="34" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E39" s="30" t="inlineStr">
         <is>
@@ -17475,57 +17589,171 @@
           <t>NBIS</t>
         </is>
       </c>
-      <c r="C40" s="26" t="n"/>
-      <c r="D40" s="27" t="n"/>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="23" t="n"/>
-      <c r="I40" s="23" t="n"/>
-      <c r="J40" s="23" t="n"/>
-      <c r="K40" s="23" t="n"/>
-      <c r="L40" s="23" t="n"/>
-      <c r="M40" s="23" t="n"/>
-      <c r="N40" s="69" t="n"/>
-      <c r="O40" s="23" t="n"/>
-      <c r="P40" s="25" t="n"/>
+      <c r="C40" s="26" t="n">
+        <v>0.02126865426791058</v>
+      </c>
+      <c r="D40" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L40" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N40" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="O40" s="23" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="P40" s="25" t="inlineStr">
+        <is>
+          <t>Long-term up, short-term mixed</t>
+        </is>
+      </c>
       <c r="Q40" s="25" t="inlineStr">
         <is>
           <t>Nebius Group N.V.</t>
         </is>
       </c>
-      <c r="R40" s="70" t="n"/>
-      <c r="S40" s="71" t="n"/>
-      <c r="T40" s="72" t="n"/>
-      <c r="U40" s="72" t="n"/>
-      <c r="V40" s="72" t="n"/>
-      <c r="W40" s="73" t="n"/>
-      <c r="X40" s="74" t="n"/>
-      <c r="Y40" s="28" t="n"/>
-      <c r="Z40" s="28" t="n"/>
-      <c r="AA40" s="28" t="n"/>
-      <c r="AB40" s="75" t="n"/>
-      <c r="AC40" s="75" t="n"/>
-      <c r="AD40" s="75" t="n"/>
-      <c r="AE40" s="72" t="n"/>
-      <c r="AF40" s="72" t="n"/>
-      <c r="AG40" s="72" t="n"/>
-      <c r="AH40" s="72" t="n"/>
-      <c r="AI40" s="72" t="n"/>
-      <c r="AJ40" s="72" t="n"/>
-      <c r="AK40" s="72" t="n"/>
-      <c r="AL40" s="72" t="n"/>
-      <c r="AM40" s="76" t="n"/>
-      <c r="AN40" s="29" t="n"/>
-      <c r="AO40" s="77" t="n"/>
-      <c r="AP40" s="72" t="n"/>
-      <c r="AQ40" s="72" t="n"/>
-      <c r="AR40" s="29" t="n"/>
-      <c r="AS40" s="78" t="n"/>
-      <c r="AT40" s="26" t="n"/>
-      <c r="AU40" s="26" t="n"/>
-      <c r="AV40" s="26" t="n"/>
-      <c r="AW40" s="26" t="n"/>
+      <c r="R40" s="70" t="n">
+        <v>218.4799957275391</v>
+      </c>
+      <c r="S40" s="71" t="n">
+        <v>4.550003051757812</v>
+      </c>
+      <c r="T40" s="72" t="n">
+        <v>223.3699951171875</v>
+      </c>
+      <c r="U40" s="72" t="n">
+        <v>228.5</v>
+      </c>
+      <c r="V40" s="72" t="n">
+        <v>215.4100036621094</v>
+      </c>
+      <c r="W40" s="73" t="n">
+        <v>16068200</v>
+      </c>
+      <c r="X40" s="74" t="n">
+        <v>0.6335217880799794</v>
+      </c>
+      <c r="Y40" s="28" t="n">
+        <v>49.72579556929819</v>
+      </c>
+      <c r="Z40" s="28" t="n">
+        <v>36.19525194259934</v>
+      </c>
+      <c r="AA40" s="28" t="n">
+        <v>10.83636146691733</v>
+      </c>
+      <c r="AB40" s="75" t="n">
+        <v>2.893221850498094</v>
+      </c>
+      <c r="AC40" s="75" t="n">
+        <v>4.749016579908232</v>
+      </c>
+      <c r="AD40" s="75" t="n">
+        <v>-1.855794729410138</v>
+      </c>
+      <c r="AE40" s="72" t="n">
+        <v>221.8562882860591</v>
+      </c>
+      <c r="AF40" s="72" t="n">
+        <v>220.5243707098805</v>
+      </c>
+      <c r="AG40" s="72" t="n">
+        <v>220.81</v>
+      </c>
+      <c r="AH40" s="72" t="n">
+        <v>205.750400314331</v>
+      </c>
+      <c r="AI40" s="72" t="n">
+        <v>151.3309753799439</v>
+      </c>
+      <c r="AJ40" s="72" t="n">
+        <v>275.408517849765</v>
+      </c>
+      <c r="AK40" s="72" t="n">
+        <v>222.0270004272461</v>
+      </c>
+      <c r="AL40" s="72" t="n">
+        <v>168.6454830047272</v>
+      </c>
+      <c r="AM40" s="76" t="n">
+        <v>0.4667768464538746</v>
+      </c>
+      <c r="AN40" s="29" t="n">
+        <v>48.08560879514382</v>
+      </c>
+      <c r="AO40" s="77" t="n">
+        <v>9.941251693103386</v>
+      </c>
+      <c r="AP40" s="72" t="n">
+        <v>299.8599853515625</v>
+      </c>
+      <c r="AQ40" s="72" t="n">
+        <v>63.2599983215332</v>
+      </c>
+      <c r="AR40" s="29" t="n">
+        <v>-27.13932955362874</v>
+      </c>
+      <c r="AS40" s="78" t="n">
+        <v>65.60439810434366</v>
+      </c>
+      <c r="AT40" s="26" t="n">
+        <v>-0.007405410377959165</v>
+      </c>
+      <c r="AU40" s="26" t="n">
+        <v>0.474025056862718</v>
+      </c>
+      <c r="AV40" s="26" t="n">
+        <v>-0.0347265208868246</v>
+      </c>
+      <c r="AW40" s="26" t="n">
+        <v>1.610118761702035</v>
+      </c>
       <c r="AX40" s="25" t="n"/>
       <c r="AY40" s="25" t="n"/>
       <c r="AZ40" s="25" t="n"/>
@@ -17541,7 +17769,7 @@
         <v>-0.01988709507475095</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -17717,7 +17945,7 @@
         <v>0.01729109585150757</v>
       </c>
       <c r="D42" s="27" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
@@ -18245,7 +18473,7 @@
         <v>0.006474453644578437</v>
       </c>
       <c r="D45" s="34" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
@@ -18421,7 +18649,7 @@
         <v>0.02039888890746222</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
@@ -18597,7 +18825,7 @@
         <v>-0.009617401970342554</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -19351,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Aug 2026, 01:05 AM · Yahoo Finance data</t>
+          <t>Built 29 Aug 2026, 02:50 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19376,22 +19604,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>20 of 39</t>
+          <t>20 of 40</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>19 of 39</t>
+          <t>20 of 40</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>4.7 / 9</t>
+          <t>4.6 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>18 of 39</t>
+          <t>18 of 40</t>
         </is>
       </c>
     </row>
@@ -24421,7 +24649,7 @@
         <v>-0.06230744635067853</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -25297,57 +25525,171 @@
           <t>NBIS</t>
         </is>
       </c>
-      <c r="C40" s="26" t="n"/>
-      <c r="D40" s="27" t="n"/>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="23" t="n"/>
-      <c r="I40" s="23" t="n"/>
-      <c r="J40" s="23" t="n"/>
-      <c r="K40" s="23" t="n"/>
-      <c r="L40" s="23" t="n"/>
-      <c r="M40" s="23" t="n"/>
-      <c r="N40" s="69" t="n"/>
-      <c r="O40" s="23" t="n"/>
-      <c r="P40" s="25" t="n"/>
+      <c r="C40" s="26" t="n">
+        <v>-0.03622114925758713</v>
+      </c>
+      <c r="D40" s="27" t="n">
+        <v>24</v>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L40" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N40" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="O40" s="23" t="inlineStr">
+        <is>
+          <t>Very Weak</t>
+        </is>
+      </c>
+      <c r="P40" s="25" t="inlineStr">
+        <is>
+          <t>Long-term up, short-term mixed</t>
+        </is>
+      </c>
       <c r="Q40" s="25" t="inlineStr">
         <is>
           <t>Nebius Group N.V.</t>
         </is>
       </c>
-      <c r="R40" s="70" t="n"/>
-      <c r="S40" s="71" t="n"/>
-      <c r="T40" s="72" t="n"/>
-      <c r="U40" s="72" t="n"/>
-      <c r="V40" s="72" t="n"/>
-      <c r="W40" s="73" t="n"/>
-      <c r="X40" s="74" t="n"/>
-      <c r="Y40" s="28" t="n"/>
-      <c r="Z40" s="28" t="n"/>
-      <c r="AA40" s="28" t="n"/>
-      <c r="AB40" s="75" t="n"/>
-      <c r="AC40" s="75" t="n"/>
-      <c r="AD40" s="75" t="n"/>
-      <c r="AE40" s="72" t="n"/>
-      <c r="AF40" s="72" t="n"/>
-      <c r="AG40" s="72" t="n"/>
-      <c r="AH40" s="72" t="n"/>
-      <c r="AI40" s="72" t="n"/>
-      <c r="AJ40" s="72" t="n"/>
-      <c r="AK40" s="72" t="n"/>
-      <c r="AL40" s="72" t="n"/>
-      <c r="AM40" s="76" t="n"/>
-      <c r="AN40" s="29" t="n"/>
-      <c r="AO40" s="77" t="n"/>
-      <c r="AP40" s="72" t="n"/>
-      <c r="AQ40" s="72" t="n"/>
-      <c r="AR40" s="29" t="n"/>
-      <c r="AS40" s="78" t="n"/>
-      <c r="AT40" s="26" t="n"/>
-      <c r="AU40" s="26" t="n"/>
-      <c r="AV40" s="26" t="n"/>
-      <c r="AW40" s="26" t="n"/>
+      <c r="R40" s="70" t="n">
+        <v>213.9299926757812</v>
+      </c>
+      <c r="S40" s="71" t="n">
+        <v>-8.040008544921875</v>
+      </c>
+      <c r="T40" s="72" t="n">
+        <v>215.5</v>
+      </c>
+      <c r="U40" s="72" t="n">
+        <v>221.4700012207031</v>
+      </c>
+      <c r="V40" s="72" t="n">
+        <v>213.6000061035156</v>
+      </c>
+      <c r="W40" s="73" t="n">
+        <v>10562800</v>
+      </c>
+      <c r="X40" s="74" t="n">
+        <v>0.3959811816342677</v>
+      </c>
+      <c r="Y40" s="28" t="n">
+        <v>48.45164047982113</v>
+      </c>
+      <c r="Z40" s="28" t="n">
+        <v>33.23286593556736</v>
+      </c>
+      <c r="AA40" s="28" t="n">
+        <v>11.40910369743057</v>
+      </c>
+      <c r="AB40" s="75" t="n">
+        <v>3.531265535503451</v>
+      </c>
+      <c r="AC40" s="75" t="n">
+        <v>5.212965262260766</v>
+      </c>
+      <c r="AD40" s="75" t="n">
+        <v>-1.681699726757315</v>
+      </c>
+      <c r="AE40" s="72" t="n">
+        <v>222.820943302779</v>
+      </c>
+      <c r="AF40" s="72" t="n">
+        <v>220.7288082081147</v>
+      </c>
+      <c r="AG40" s="72" t="n">
+        <v>221.7424002075195</v>
+      </c>
+      <c r="AH40" s="72" t="n">
+        <v>204.6910003662109</v>
+      </c>
+      <c r="AI40" s="72" t="n">
+        <v>150.7949753952026</v>
+      </c>
+      <c r="AJ40" s="72" t="n">
+        <v>275.876030632897</v>
+      </c>
+      <c r="AK40" s="72" t="n">
+        <v>220.5245002746582</v>
+      </c>
+      <c r="AL40" s="72" t="n">
+        <v>165.1729699164194</v>
+      </c>
+      <c r="AM40" s="76" t="n">
+        <v>0.4404306659978788</v>
+      </c>
+      <c r="AN40" s="29" t="n">
+        <v>50.19989188439358</v>
+      </c>
+      <c r="AO40" s="77" t="n">
+        <v>10.4097692066209</v>
+      </c>
+      <c r="AP40" s="72" t="n">
+        <v>299.8599853515625</v>
+      </c>
+      <c r="AQ40" s="72" t="n">
+        <v>63.2599983215332</v>
+      </c>
+      <c r="AR40" s="29" t="n">
+        <v>-28.65670542037645</v>
+      </c>
+      <c r="AS40" s="78" t="n">
+        <v>63.68131978600869</v>
+      </c>
+      <c r="AT40" s="26" t="n">
+        <v>-0.04452881416920695</v>
+      </c>
+      <c r="AU40" s="26" t="n">
+        <v>0.2607106464604538</v>
+      </c>
+      <c r="AV40" s="26" t="n">
+        <v>0.02668329264713387</v>
+      </c>
+      <c r="AW40" s="26" t="n">
+        <v>1.555761161173679</v>
+      </c>
       <c r="AX40" s="25" t="n"/>
       <c r="AY40" s="25" t="n"/>
       <c r="AZ40" s="25" t="n"/>
@@ -27173,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Aug 2026, 01:05 AM · Yahoo Finance data</t>
+          <t>Built 29 Aug 2026, 02:50 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27198,22 +27540,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>26 of 39</t>
+          <t>27 of 40</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>12 of 39</t>
+          <t>12 of 40</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>4.7 / 9</t>
+          <t>4.8 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>20 of 39</t>
+          <t>20 of 40</t>
         </is>
       </c>
     </row>
@@ -30307,7 +30649,7 @@
         <v>-0.001417807716048269</v>
       </c>
       <c r="D24" s="27" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
@@ -30483,7 +30825,7 @@
         <v>0.04910781100335249</v>
       </c>
       <c r="D25" s="34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E25" s="30" t="inlineStr">
         <is>
@@ -30659,7 +31001,7 @@
         <v>-0.003853969311243932</v>
       </c>
       <c r="D26" s="27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
@@ -30835,7 +31177,7 @@
         <v>0.02919452610931228</v>
       </c>
       <c r="D27" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E27" s="30" t="inlineStr">
         <is>
@@ -31011,7 +31353,7 @@
         <v>0.01164251107089753</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
@@ -31187,7 +31529,7 @@
         <v>-0.005453089990515525</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E29" s="30" t="inlineStr">
         <is>
@@ -31363,7 +31705,7 @@
         <v>-0.005630559360753851</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
@@ -31539,7 +31881,7 @@
         <v>0.04585902606191405</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31" s="30" t="inlineStr">
         <is>
@@ -31715,7 +32057,7 @@
         <v>0.02075363380321549</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
@@ -31891,7 +32233,7 @@
         <v>0.04226782117639094</v>
       </c>
       <c r="D33" s="34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E33" s="30" t="inlineStr">
         <is>
@@ -32067,7 +32409,7 @@
         <v>-0.003627499385601141</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
@@ -32419,7 +32761,7 @@
         <v>0.002521214936021421</v>
       </c>
       <c r="D36" s="27" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
@@ -32595,7 +32937,7 @@
         <v>0.009029147603226262</v>
       </c>
       <c r="D37" s="34" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E37" s="30" t="inlineStr">
         <is>
@@ -32771,7 +33113,7 @@
         <v>0.0342494061135572</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -32947,7 +33289,7 @@
         <v>0.0247575082199325</v>
       </c>
       <c r="D39" s="34" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E39" s="30" t="inlineStr">
         <is>
@@ -33119,57 +33461,171 @@
           <t>NBIS</t>
         </is>
       </c>
-      <c r="C40" s="26" t="n"/>
-      <c r="D40" s="27" t="n"/>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="23" t="n"/>
-      <c r="I40" s="23" t="n"/>
-      <c r="J40" s="23" t="n"/>
-      <c r="K40" s="23" t="n"/>
-      <c r="L40" s="23" t="n"/>
-      <c r="M40" s="23" t="n"/>
-      <c r="N40" s="69" t="n"/>
-      <c r="O40" s="23" t="n"/>
-      <c r="P40" s="25" t="n"/>
+      <c r="C40" s="26" t="n">
+        <v>0.0524394166542832</v>
+      </c>
+      <c r="D40" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I40" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L40" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M40" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N40" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="O40" s="23" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P40" s="25" t="inlineStr">
+        <is>
+          <t>Long-term up, short-term mixed</t>
+        </is>
+      </c>
       <c r="Q40" s="25" t="inlineStr">
         <is>
           <t>Nebius Group N.V.</t>
         </is>
       </c>
-      <c r="R40" s="70" t="n"/>
-      <c r="S40" s="71" t="n"/>
-      <c r="T40" s="72" t="n"/>
-      <c r="U40" s="72" t="n"/>
-      <c r="V40" s="72" t="n"/>
-      <c r="W40" s="73" t="n"/>
-      <c r="X40" s="74" t="n"/>
-      <c r="Y40" s="28" t="n"/>
-      <c r="Z40" s="28" t="n"/>
-      <c r="AA40" s="28" t="n"/>
-      <c r="AB40" s="75" t="n"/>
-      <c r="AC40" s="75" t="n"/>
-      <c r="AD40" s="75" t="n"/>
-      <c r="AE40" s="72" t="n"/>
-      <c r="AF40" s="72" t="n"/>
-      <c r="AG40" s="72" t="n"/>
-      <c r="AH40" s="72" t="n"/>
-      <c r="AI40" s="72" t="n"/>
-      <c r="AJ40" s="72" t="n"/>
-      <c r="AK40" s="72" t="n"/>
-      <c r="AL40" s="72" t="n"/>
-      <c r="AM40" s="76" t="n"/>
-      <c r="AN40" s="29" t="n"/>
-      <c r="AO40" s="77" t="n"/>
-      <c r="AP40" s="72" t="n"/>
-      <c r="AQ40" s="72" t="n"/>
-      <c r="AR40" s="29" t="n"/>
-      <c r="AS40" s="78" t="n"/>
-      <c r="AT40" s="26" t="n"/>
-      <c r="AU40" s="26" t="n"/>
-      <c r="AV40" s="26" t="n"/>
-      <c r="AW40" s="26" t="n"/>
+      <c r="R40" s="70" t="n">
+        <v>221.9700012207031</v>
+      </c>
+      <c r="S40" s="71" t="n">
+        <v>11.05999755859375</v>
+      </c>
+      <c r="T40" s="72" t="n">
+        <v>217.9600067138672</v>
+      </c>
+      <c r="U40" s="72" t="n">
+        <v>223.4400024414062</v>
+      </c>
+      <c r="V40" s="72" t="n">
+        <v>213.5500030517578</v>
+      </c>
+      <c r="W40" s="73" t="n">
+        <v>13547900</v>
+      </c>
+      <c r="X40" s="74" t="n">
+        <v>0.4815206041016987</v>
+      </c>
+      <c r="Y40" s="28" t="n">
+        <v>50.5539280953977</v>
+      </c>
+      <c r="Z40" s="28" t="n">
+        <v>41.25690745085653</v>
+      </c>
+      <c r="AA40" s="28" t="n">
+        <v>12.2225942722081</v>
+      </c>
+      <c r="AB40" s="75" t="n">
+        <v>4.757550469118314</v>
+      </c>
+      <c r="AC40" s="75" t="n">
+        <v>5.633390193950094</v>
+      </c>
+      <c r="AD40" s="75" t="n">
+        <v>-0.8758397248317795</v>
+      </c>
+      <c r="AE40" s="72" t="n">
+        <v>225.3612149104927</v>
+      </c>
+      <c r="AF40" s="72" t="n">
+        <v>221.408689761348</v>
+      </c>
+      <c r="AG40" s="72" t="n">
+        <v>222.6652005004883</v>
+      </c>
+      <c r="AH40" s="72" t="n">
+        <v>203.6399004364014</v>
+      </c>
+      <c r="AI40" s="72" t="n">
+        <v>150.2725254440307</v>
+      </c>
+      <c r="AJ40" s="72" t="n">
+        <v>280.9375445928216</v>
+      </c>
+      <c r="AK40" s="72" t="n">
+        <v>217.2390007019043</v>
+      </c>
+      <c r="AL40" s="72" t="n">
+        <v>153.540456810987</v>
+      </c>
+      <c r="AM40" s="76" t="n">
+        <v>0.5371358608047665</v>
+      </c>
+      <c r="AN40" s="29" t="n">
+        <v>58.64374599874407</v>
+      </c>
+      <c r="AO40" s="77" t="n">
+        <v>10.51440292459219</v>
+      </c>
+      <c r="AP40" s="72" t="n">
+        <v>299.8599853515625</v>
+      </c>
+      <c r="AQ40" s="72" t="n">
+        <v>63.2599983215332</v>
+      </c>
+      <c r="AR40" s="29" t="n">
+        <v>-25.97545118917398</v>
+      </c>
+      <c r="AS40" s="78" t="n">
+        <v>67.07946390505357</v>
+      </c>
+      <c r="AT40" s="26" t="n">
+        <v>-0.1065088444840486</v>
+      </c>
+      <c r="AU40" s="26" t="n">
+        <v>0.1814455793694161</v>
+      </c>
+      <c r="AV40" s="26" t="n">
+        <v>0.0668557330833961</v>
+      </c>
+      <c r="AW40" s="26" t="n">
+        <v>1.65181287097651</v>
+      </c>
       <c r="AX40" s="25" t="n"/>
       <c r="AY40" s="25" t="n"/>
       <c r="AZ40" s="25" t="n"/>
@@ -33185,7 +33641,7 @@
         <v>0.02774654619960137</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -33361,7 +33817,7 @@
         <v>0.0391566608262095</v>
       </c>
       <c r="D42" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
@@ -33537,7 +33993,7 @@
         <v>0.02192060350092895</v>
       </c>
       <c r="D43" s="34" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E43" s="30" t="inlineStr">
         <is>
@@ -33713,7 +34169,7 @@
         <v>-0.01796579494613015</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
@@ -33889,7 +34345,7 @@
         <v>0.0128051396891955</v>
       </c>
       <c r="D45" s="34" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
@@ -34065,7 +34521,7 @@
         <v>-0.02006436938605949</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
@@ -34241,7 +34697,7 @@
         <v>-0.008271254571852515</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -34417,7 +34873,7 @@
         <v>0.003725426988085312</v>
       </c>
       <c r="D48" s="27" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
@@ -34995,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Aug 2026, 01:05 AM · Yahoo Finance data</t>
+          <t>Built 29 Aug 2026, 02:50 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35020,22 +35476,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>14 of 39</t>
+          <t>14 of 40</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>25 of 39</t>
+          <t>26 of 40</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>4.2 / 9</t>
+          <t>4.1 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>14 of 39</t>
+          <t>14 of 40</t>
         </is>
       </c>
     </row>
@@ -39009,7 +39465,7 @@
         <v>-0.09176988946435649</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E29" s="30" t="inlineStr">
         <is>
@@ -40065,7 +40521,7 @@
         <v>-0.04942692554991801</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -40769,7 +41225,7 @@
         <v>-0.05828630599876616</v>
       </c>
       <c r="D39" s="34" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E39" s="30" t="inlineStr">
         <is>
@@ -40941,57 +41397,171 @@
           <t>NBIS</t>
         </is>
       </c>
-      <c r="C40" s="26" t="n"/>
-      <c r="D40" s="27" t="n"/>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="23" t="n"/>
-      <c r="I40" s="23" t="n"/>
-      <c r="J40" s="23" t="n"/>
-      <c r="K40" s="23" t="n"/>
-      <c r="L40" s="23" t="n"/>
-      <c r="M40" s="23" t="n"/>
-      <c r="N40" s="69" t="n"/>
-      <c r="O40" s="23" t="n"/>
-      <c r="P40" s="25" t="n"/>
+      <c r="C40" s="26" t="n">
+        <v>-0.03751198392524591</v>
+      </c>
+      <c r="D40" s="27" t="n">
+        <v>19</v>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L40" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N40" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="O40" s="23" t="inlineStr">
+        <is>
+          <t>Very Weak</t>
+        </is>
+      </c>
+      <c r="P40" s="25" t="inlineStr">
+        <is>
+          <t>Long-term up, short-term mixed</t>
+        </is>
+      </c>
       <c r="Q40" s="25" t="inlineStr">
         <is>
           <t>Nebius Group N.V.</t>
         </is>
       </c>
-      <c r="R40" s="70" t="n"/>
-      <c r="S40" s="71" t="n"/>
-      <c r="T40" s="72" t="n"/>
-      <c r="U40" s="72" t="n"/>
-      <c r="V40" s="72" t="n"/>
-      <c r="W40" s="73" t="n"/>
-      <c r="X40" s="74" t="n"/>
-      <c r="Y40" s="28" t="n"/>
-      <c r="Z40" s="28" t="n"/>
-      <c r="AA40" s="28" t="n"/>
-      <c r="AB40" s="75" t="n"/>
-      <c r="AC40" s="75" t="n"/>
-      <c r="AD40" s="75" t="n"/>
-      <c r="AE40" s="72" t="n"/>
-      <c r="AF40" s="72" t="n"/>
-      <c r="AG40" s="72" t="n"/>
-      <c r="AH40" s="72" t="n"/>
-      <c r="AI40" s="72" t="n"/>
-      <c r="AJ40" s="72" t="n"/>
-      <c r="AK40" s="72" t="n"/>
-      <c r="AL40" s="72" t="n"/>
-      <c r="AM40" s="76" t="n"/>
-      <c r="AN40" s="29" t="n"/>
-      <c r="AO40" s="77" t="n"/>
-      <c r="AP40" s="72" t="n"/>
-      <c r="AQ40" s="72" t="n"/>
-      <c r="AR40" s="29" t="n"/>
-      <c r="AS40" s="78" t="n"/>
-      <c r="AT40" s="26" t="n"/>
-      <c r="AU40" s="26" t="n"/>
-      <c r="AV40" s="26" t="n"/>
-      <c r="AW40" s="26" t="n"/>
+      <c r="R40" s="70" t="n">
+        <v>210.9100036621094</v>
+      </c>
+      <c r="S40" s="71" t="n">
+        <v>-8.220001220703125</v>
+      </c>
+      <c r="T40" s="72" t="n">
+        <v>211.2019958496094</v>
+      </c>
+      <c r="U40" s="72" t="n">
+        <v>213.75</v>
+      </c>
+      <c r="V40" s="72" t="n">
+        <v>201.8910064697266</v>
+      </c>
+      <c r="W40" s="73" t="n">
+        <v>16882300</v>
+      </c>
+      <c r="X40" s="74" t="n">
+        <v>0.5840942159542905</v>
+      </c>
+      <c r="Y40" s="28" t="n">
+        <v>47.65263001805049</v>
+      </c>
+      <c r="Z40" s="28" t="n">
+        <v>30.21887445956007</v>
+      </c>
+      <c r="AA40" s="28" t="n">
+        <v>13.09866104504544</v>
+      </c>
+      <c r="AB40" s="75" t="n">
+        <v>5.434916180262093</v>
+      </c>
+      <c r="AC40" s="75" t="n">
+        <v>5.852350125158037</v>
+      </c>
+      <c r="AD40" s="75" t="n">
+        <v>-0.4174339448959445</v>
+      </c>
+      <c r="AE40" s="72" t="n">
+        <v>226.3301331075754</v>
+      </c>
+      <c r="AF40" s="72" t="n">
+        <v>221.3525586154125</v>
+      </c>
+      <c r="AG40" s="72" t="n">
+        <v>222.8730004882813</v>
+      </c>
+      <c r="AH40" s="72" t="n">
+        <v>202.4397003936768</v>
+      </c>
+      <c r="AI40" s="72" t="n">
+        <v>149.7476754379273</v>
+      </c>
+      <c r="AJ40" s="72" t="n">
+        <v>281.5419454408989</v>
+      </c>
+      <c r="AK40" s="72" t="n">
+        <v>214.6250007629395</v>
+      </c>
+      <c r="AL40" s="72" t="n">
+        <v>147.7080560849801</v>
+      </c>
+      <c r="AM40" s="76" t="n">
+        <v>0.4722417310091736</v>
+      </c>
+      <c r="AN40" s="29" t="n">
+        <v>62.3570827630388</v>
+      </c>
+      <c r="AO40" s="77" t="n">
+        <v>11.45999131841995</v>
+      </c>
+      <c r="AP40" s="72" t="n">
+        <v>299.8599853515625</v>
+      </c>
+      <c r="AQ40" s="72" t="n">
+        <v>63.2599983215332</v>
+      </c>
+      <c r="AR40" s="29" t="n">
+        <v>-29.6638384695331</v>
+      </c>
+      <c r="AS40" s="78" t="n">
+        <v>62.40490846765617</v>
+      </c>
+      <c r="AT40" s="26" t="n">
+        <v>-0.2155105119063957</v>
+      </c>
+      <c r="AU40" s="26" t="n">
+        <v>0.1232358676206422</v>
+      </c>
+      <c r="AV40" s="26" t="n">
+        <v>-0.01797271748178908</v>
+      </c>
+      <c r="AW40" s="26" t="n">
+        <v>1.519682205942697</v>
+      </c>
       <c r="AX40" s="25" t="n"/>
       <c r="AY40" s="25" t="n"/>
       <c r="AZ40" s="25" t="n"/>
@@ -41887,7 +42457,7 @@
         <v>-0.05911534978045907</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
@@ -42063,7 +42633,7 @@
         <v>-0.06450802201163175</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -42239,7 +42809,7 @@
         <v>-0.03833427136104406</v>
       </c>
       <c r="D48" s="27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
@@ -43294,7 +43864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G48"/>
+  <dimension ref="B2:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -44284,21 +44854,21 @@
     <row r="39">
       <c r="B39" s="31" t="inlineStr">
         <is>
-          <t>ASTS</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="C39" s="102" t="inlineStr">
         <is>
-          <t>AST SpaceMobile, Inc.</t>
+          <t>Nebius Group N.V.</t>
         </is>
       </c>
       <c r="D39" s="107" t="inlineStr">
         <is>
-          <t>Closed below lower band</t>
+          <t>8 EMA crossed below 21</t>
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>-0.05517577254916717</v>
+        <v>-0.04256684013924827</v>
       </c>
       <c r="F39" s="34" t="n">
         <v>1</v>
@@ -44312,21 +44882,21 @@
     <row r="40">
       <c r="B40" s="24" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="C40" s="101" t="inlineStr">
         <is>
-          <t>Arm Holdings plc</t>
+          <t>Nebius Group N.V.</t>
         </is>
       </c>
       <c r="D40" s="106" t="inlineStr">
         <is>
-          <t>MACD crossed down</t>
+          <t>Gapped down 3.0% at the open</t>
         </is>
       </c>
       <c r="E40" s="26" t="n">
-        <v>-0.06332041548914424</v>
+        <v>-0.04256684013924827</v>
       </c>
       <c r="F40" s="27" t="n">
         <v>1</v>
@@ -44340,21 +44910,21 @@
     <row r="41">
       <c r="B41" s="31" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ASTS</t>
         </is>
       </c>
       <c r="C41" s="102" t="inlineStr">
         <is>
-          <t>Arm Holdings plc</t>
+          <t>AST SpaceMobile, Inc.</t>
         </is>
       </c>
       <c r="D41" s="107" t="inlineStr">
         <is>
-          <t>Gapped down 1.7% at the open</t>
+          <t>Closed below lower band</t>
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>-0.06332041548914424</v>
+        <v>-0.05517577254916717</v>
       </c>
       <c r="F41" s="34" t="n">
         <v>1</v>
@@ -44368,12 +44938,12 @@
     <row r="42">
       <c r="B42" s="24" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="C42" s="101" t="inlineStr">
         <is>
-          <t>IREN Limited</t>
+          <t>Arm Holdings plc</t>
         </is>
       </c>
       <c r="D42" s="106" t="inlineStr">
@@ -44382,7 +44952,7 @@
         </is>
       </c>
       <c r="E42" s="26" t="n">
-        <v>-0.1253392097053883</v>
+        <v>-0.06332041548914424</v>
       </c>
       <c r="F42" s="27" t="n">
         <v>1</v>
@@ -44396,21 +44966,21 @@
     <row r="43">
       <c r="B43" s="31" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="C43" s="102" t="inlineStr">
         <is>
-          <t>IREN Limited</t>
+          <t>Arm Holdings plc</t>
         </is>
       </c>
       <c r="D43" s="107" t="inlineStr">
         <is>
-          <t>8 EMA crossed below 21</t>
+          <t>Gapped down 1.7% at the open</t>
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>-0.1253392097053883</v>
+        <v>-0.06332041548914424</v>
       </c>
       <c r="F43" s="34" t="n">
         <v>1</v>
@@ -44434,7 +45004,7 @@
       </c>
       <c r="D44" s="106" t="inlineStr">
         <is>
-          <t>Closed below lower band</t>
+          <t>MACD crossed down</t>
         </is>
       </c>
       <c r="E44" s="26" t="n">
@@ -44462,7 +45032,7 @@
       </c>
       <c r="D45" s="107" t="inlineStr">
         <is>
-          <t>Volume 2.0x its 20-day average</t>
+          <t>8 EMA crossed below 21</t>
         </is>
       </c>
       <c r="E45" s="33" t="n">
@@ -44490,7 +45060,7 @@
       </c>
       <c r="D46" s="106" t="inlineStr">
         <is>
-          <t>Gapped down 7.3% at the open</t>
+          <t>Closed below lower band</t>
         </is>
       </c>
       <c r="E46" s="26" t="n">
@@ -44508,24 +45078,24 @@
     <row r="47">
       <c r="B47" s="31" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="C47" s="102" t="inlineStr">
         <is>
-          <t>Broadcom Inc.</t>
+          <t>IREN Limited</t>
         </is>
       </c>
       <c r="D47" s="107" t="inlineStr">
         <is>
-          <t>Lost the 200 DMA</t>
+          <t>Volume 2.0x its 20-day average</t>
         </is>
       </c>
       <c r="E47" s="33" t="n">
-        <v>-0.007401625495918829</v>
+        <v>-0.1253392097053883</v>
       </c>
       <c r="F47" s="34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" s="30" t="inlineStr">
         <is>
@@ -44536,37 +45106,93 @@
     <row r="48">
       <c r="B48" s="24" t="inlineStr">
         <is>
+          <t>IREN</t>
+        </is>
+      </c>
+      <c r="C48" s="101" t="inlineStr">
+        <is>
+          <t>IREN Limited</t>
+        </is>
+      </c>
+      <c r="D48" s="106" t="inlineStr">
+        <is>
+          <t>Gapped down 7.3% at the open</t>
+        </is>
+      </c>
+      <c r="E48" s="26" t="n">
+        <v>-0.1253392097053883</v>
+      </c>
+      <c r="F48" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="23" t="inlineStr">
+        <is>
+          <t>Very Weak</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="31" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C49" s="102" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="D49" s="107" t="inlineStr">
+        <is>
+          <t>Lost the 200 DMA</t>
+        </is>
+      </c>
+      <c r="E49" s="33" t="n">
+        <v>-0.007401625495918829</v>
+      </c>
+      <c r="F49" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="30" t="inlineStr">
+        <is>
+          <t>Very Weak</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="24" t="inlineStr">
+        <is>
           <t>CRWV</t>
         </is>
       </c>
-      <c r="C48" s="101" t="inlineStr">
+      <c r="C50" s="101" t="inlineStr">
         <is>
           <t>CoreWeave, Inc.</t>
         </is>
       </c>
-      <c r="D48" s="106" t="inlineStr">
+      <c r="D50" s="106" t="inlineStr">
         <is>
           <t>Gapped down 2.0% at the open</t>
         </is>
       </c>
-      <c r="E48" s="26" t="n">
+      <c r="E50" s="26" t="n">
         <v>-0.02960829037404245</v>
       </c>
-      <c r="F48" s="27" t="n">
+      <c r="F50" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G48" s="23" t="inlineStr">
+      <c r="G50" s="23" t="inlineStr">
         <is>
           <t>Very Weak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B5:G48"/>
+  <autoFilter ref="B5:G50"/>
   <mergeCells count="1">
     <mergeCell ref="B2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E48">
+  <conditionalFormatting sqref="E6:E50">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>

</xml_diff>

<commit_message>
Daily workbook: 2026-08-29 03:09 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 29 Aug 2026, 02:50 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 29 Aug 2026, 03:09 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Aug 2026, 02:50 AM · Yahoo Finance data</t>
+          <t>Built 29 Aug 2026, 03:09 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -8088,17 +8088,17 @@
       </c>
       <c r="AX32" s="79" t="inlineStr">
         <is>
+          <t>Wall Street Sees CoreWeave Anywhere From $74 to $250. Somebody Is Very Wrong</t>
+        </is>
+      </c>
+      <c r="AY32" s="79" t="inlineStr">
+        <is>
           <t>Could CoreWeave (CRWV) Stock Win as AI Demand Continues to Outpace GPU Supply?</t>
         </is>
       </c>
-      <c r="AY32" s="79" t="inlineStr">
+      <c r="AZ32" s="79" t="inlineStr">
         <is>
           <t>CoreWeave (CRWV) Enters Next Generation Engineering AI Workloads</t>
-        </is>
-      </c>
-      <c r="AZ32" s="79" t="inlineStr">
-        <is>
-          <t>Nvidia’s GPU Price Hikes Look Bad for CoreWeave. Truist Says the Opposite May Be True</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Aug 2026, 02:50 AM · Yahoo Finance data</t>
+          <t>Built 29 Aug 2026, 03:09 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Aug 2026, 02:50 AM · Yahoo Finance data</t>
+          <t>Built 29 Aug 2026, 03:09 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Aug 2026, 02:50 AM · Yahoo Finance data</t>
+          <t>Built 29 Aug 2026, 03:09 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Aug 2026, 02:50 AM · Yahoo Finance data</t>
+          <t>Built 29 Aug 2026, 03:09 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-08-31 23:53 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 31 Aug 2026, 09:59 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 31 Aug 2026, 11:53 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 31 Aug 2026, 09:59 PM · Yahoo Finance data</t>
+          <t>Built 31 Aug 2026, 11:53 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>What Tim Cook told employees on his last day at Apple</t>
+          <t>Apple To Begin New Chapter With CEO John Ternus</t>
         </is>
       </c>
     </row>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
+          <t>AMD Expands Global AI Footprint With New Saudi Platform</t>
+        </is>
+      </c>
+      <c r="AY25" s="90" t="inlineStr">
+        <is>
           <t>Not Nvidia, Not AMD. Micron Could Be September's Biggest AI Winner or Loser.</t>
         </is>
       </c>
-      <c r="AY25" s="90" t="inlineStr">
+      <c r="AZ25" s="90" t="inlineStr">
         <is>
           <t>Wall Street Is Looking Here. I’m Looking Somewhere Else</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>AMD Enters a Sovereign AI Showcase, Not a Revenue Windfall</t>
         </is>
       </c>
     </row>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>US regulator, 22 states accuse Amazon of 'manipulating' ad auctions: lawsuit</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
           <t>FTC, 22 states sue Amazon over deceptive advertising practices</t>
         </is>
       </c>
-      <c r="AY26" s="79" t="inlineStr">
-        <is>
-          <t>FTC sues Amazon for manipulating ad auction prices</t>
-        </is>
-      </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>FTC sues Amazon, alleging it overcharged advertisers</t>
+          <t>FTC, 22 States File Suit Against Amazon Alleging It Secretly Upcharged Companies for Ads</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Broadcom's Next Earnings Report on September 2 Could Send the Stock Soaring. Here's Why.</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Is Broadcom (AVGO) Stock a Buy Before Its Q3 Earnings?</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>VGT’s $58 Billion AI Chip Concentration Could Derail Your 2027 Returns</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Broadcom Has Trailed the S&amp;P 500 This Year. That Shouldn't Last Much Longer.</t>
         </is>
       </c>
     </row>
@@ -8276,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
+          <t>Dell Earnings Could Swing the Stock 11% This Week, a $52 Straddle Shows</t>
+        </is>
+      </c>
+      <c r="AY33" s="90" t="inlineStr">
+        <is>
           <t>Buy Dell Technologies Stock Before Q2 Earnings as AI Server Demand Soars?</t>
         </is>
       </c>
-      <c r="AY33" s="90" t="inlineStr">
+      <c r="AZ33" s="90" t="inlineStr">
         <is>
           <t>Back-to-School Success with Dell and Waterdrop Filter: The Simple Habits Helping Kids Learn, Focus and Thri...</t>
-        </is>
-      </c>
-      <c r="AZ33" s="90" t="inlineStr">
-        <is>
-          <t>Dell Stock Flashes Major Last-Minute Signal Before Earnings</t>
         </is>
       </c>
     </row>
@@ -8662,7 +8662,7 @@
       </c>
       <c r="AZ35" s="90" t="inlineStr">
         <is>
-          <t>Investors Freaked Out Over IREN’s $30 Billion Capex — CEO Explains Why They’re Dead Wrong</t>
+          <t>A $4 Billion Reason to Buy the Recent Dip in IREN Stock Today</t>
         </is>
       </c>
     </row>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Strategy Just Bought Bitcoin for the First Time in Over Two Months. Here's Why the Timing Matters.</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Stock Market Today, Aug. 31: Stocks Edge Lower as Oil Prices Surge Again</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>Bitcoin is back—and so is Michael Saylor’s Strategy, which made its first buy in two months</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>Bitcoin Bulls Rejoice as Strategy Buys $370 Million Worth of Coins</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>JPMorgan Built a Version of JEPI Designed to Keep the IRS Waiting</t>
+          <t>Nvidia (NVDA) Invests $3.5 Billion in MediaTek. Is This the Next Leg of Its AI Growth?</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>S&amp;P500, Dow End Lower On US-Iran Flare-Up, While Dow Records Fifth Straight Month Of Gains — NVDA, META, AO...</t>
+          <t>Nvidia stock flashes unusual signal for investors</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>You Could Buy Nvidia for Its 106% Revenue Growth and 75% Gross Margin. But There's an Even Better Reason th...</t>
+          <t>Jensen Huang Told Investors in June to 'Buy at a Discount' During Nvidia's Sell-Off. Nearly Three Months La...</t>
         </is>
       </c>
     </row>
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>The Ceiling SanDisk Wrote Into Its Own Contracts</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
           <t>Qualcomm vs. Sandisk: Comparing Gradual Revenue Contraction Against Rapid Revenue Acceleration</t>
         </is>
       </c>
-      <c r="AY47" s="90" t="inlineStr">
+      <c r="AZ47" s="90" t="inlineStr">
         <is>
           <t>Can SanDisk Avoid the Memory Trap That’s Burned Investors Before?</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>Sandisk (SNDK) Backs $31 Billion Japan Flash Memory Expansion Through 2032</t>
         </is>
       </c>
     </row>
@@ -11101,12 +11101,12 @@
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>Elon Musk’s SpaceX Blade Plan Knocks Howmet As HWM Suffers Steepest Slide In 16 Months</t>
+          <t>Dow Jones Futures: Trump's Iran Warning Sparks Stock Market Losses; Elon Musk-Led SpaceX, Tesla Rally</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Stock Market Today, Aug. 31: Tesla Stock Surges on Cybercab Event Anticipation</t>
+          <t>Why Tesla (TSLA) Stock Is Up Today</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 31 Aug 2026, 09:59 PM · Yahoo Finance data</t>
+          <t>Built 31 Aug 2026, 11:53 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 31 Aug 2026, 09:59 PM · Yahoo Finance data</t>
+          <t>Built 31 Aug 2026, 11:53 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 31 Aug 2026, 09:59 PM · Yahoo Finance data</t>
+          <t>Built 31 Aug 2026, 11:53 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 31 Aug 2026, 09:59 PM · Yahoo Finance data</t>
+          <t>Built 31 Aug 2026, 11:53 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-01 00:36 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 31 Aug 2026, 11:53 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 1 Sep 2026, 12:36 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 31 Aug 2026, 11:53 PM · Yahoo Finance data</t>
+          <t>Built 1 Sep 2026, 12:36 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Apple To Begin New Chapter With CEO John Ternus</t>
+          <t>Apple shares ‘shocking evidence’ against former employee accused of stealing company data for OpenAI</t>
         </is>
       </c>
     </row>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
+          <t>Here's What September Has Done to AMD Stock Over the Past 10 Years</t>
+        </is>
+      </c>
+      <c r="AY25" s="90" t="inlineStr">
+        <is>
           <t>AMD Expands Global AI Footprint With New Saudi Platform</t>
         </is>
       </c>
-      <c r="AY25" s="90" t="inlineStr">
+      <c r="AZ25" s="90" t="inlineStr">
         <is>
           <t>Not Nvidia, Not AMD. Micron Could Be September's Biggest AI Winner or Loser.</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>Wall Street Is Looking Here. I’m Looking Somewhere Else</t>
         </is>
       </c>
     </row>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>FTC Lawsuit Puts Amazon’s (AMZN) High-Margin Advertising Business in Focus</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
           <t>US regulator, 22 states accuse Amazon of 'manipulating' ad auctions: lawsuit</t>
         </is>
       </c>
-      <c r="AY26" s="79" t="inlineStr">
+      <c r="AZ26" s="79" t="inlineStr">
         <is>
           <t>FTC, 22 states sue Amazon over deceptive advertising practices</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>FTC, 22 States File Suit Against Amazon Alleging It Secretly Upcharged Companies for Ads</t>
         </is>
       </c>
     </row>
@@ -8474,7 +8474,7 @@
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Marvell and Google: Misplaced Fear Should Drive Your Purchase Decision</t>
+          <t>Meta just turned teen safety into a competitive advantage</t>
         </is>
       </c>
     </row>
@@ -9780,17 +9780,17 @@
       </c>
       <c r="AX41" s="90" t="inlineStr">
         <is>
+          <t>Duolingo Stock Gets an Upgrade. This Analyst Sees a Netflix-Like Comeback.</t>
+        </is>
+      </c>
+      <c r="AY41" s="90" t="inlineStr">
+        <is>
           <t>Netflix vs. Meta: The Better Media Stock May Surprise You</t>
         </is>
       </c>
-      <c r="AY41" s="90" t="inlineStr">
+      <c r="AZ41" s="90" t="inlineStr">
         <is>
           <t>Jim Cramer Calls Netflix “A Buy, Not a Huge Buy” After Shares Fall 35% in a Year</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>The Bull Case for Netflix Stock Is Stronger Than You Think</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Nvidia (NVDA) Invests $3.5 Billion in MediaTek. Is This the Next Leg of Its AI Growth?</t>
+          <t>Dow Jones Futures: Trump's Iran Warning Sparks Stock Market Losses; Elon Musk-Led SpaceX, Tesla Rally</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Nvidia stock flashes unusual signal for investors</t>
+          <t>Anthropic Seals $35 Billion Cloud Deal With Nvidia-Backed Lambda</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Jensen Huang Told Investors in June to 'Buy at a Discount' During Nvidia's Sell-Off. Nearly Three Months La...</t>
+          <t>Why Deere Stock Rallied Today</t>
         </is>
       </c>
     </row>
@@ -10913,12 +10913,12 @@
       </c>
       <c r="AY47" s="90" t="inlineStr">
         <is>
-          <t>Qualcomm vs. Sandisk: Comparing Gradual Revenue Contraction Against Rapid Revenue Acceleration</t>
+          <t>Dear Sandisk Stock Fans, Mark Your Calendars for August 31</t>
         </is>
       </c>
       <c r="AZ47" s="90" t="inlineStr">
         <is>
-          <t>Can SanDisk Avoid the Memory Trap That’s Burned Investors Before?</t>
+          <t>A $31 Billion Reason to Buy Sandisk Stock Now</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 31 Aug 2026, 11:53 PM · Yahoo Finance data</t>
+          <t>Built 1 Sep 2026, 12:36 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 31 Aug 2026, 11:53 PM · Yahoo Finance data</t>
+          <t>Built 1 Sep 2026, 12:36 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 31 Aug 2026, 11:53 PM · Yahoo Finance data</t>
+          <t>Built 1 Sep 2026, 12:36 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 31 Aug 2026, 11:53 PM · Yahoo Finance data</t>
+          <t>Built 1 Sep 2026, 12:36 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-01 23:17 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 1 Sep 2026, 10:38 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 1 Sep 2026, 11:17 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1628,16 +1628,16 @@
         <v>4</v>
       </c>
       <c r="G17" s="35" t="n">
-        <v>48.9318172316673</v>
+        <v>48.94633859203591</v>
       </c>
       <c r="H17" s="36" t="n">
-        <v>0.4105939432430761</v>
+        <v>0.3333067427351732</v>
       </c>
       <c r="I17" s="33" t="n">
-        <v>-0.02515719868514421</v>
+        <v>-0.01467864877879865</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v>0.002351521940810342</v>
+        <v>0.004595797629547427</v>
       </c>
     </row>
     <row r="18">
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="F47" s="28" t="n">
-        <v>48.9318172316673</v>
+        <v>48.94633859203591</v>
       </c>
       <c r="H47" s="24" t="inlineStr">
         <is>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 1 Sep 2026, 10:38 PM · Yahoo Finance data</t>
+          <t>Built 1 Sep 2026, 11:17 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -4383,58 +4383,58 @@
         <v>9238776</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.048007388931834</v>
+        <v>1.087833876780699</v>
       </c>
       <c r="Y11" s="28" t="n">
-        <v>48.9318172316673</v>
+        <v>48.94633859203591</v>
       </c>
       <c r="Z11" s="28" t="n">
-        <v>35.83809803113058</v>
+        <v>22.9167549696944</v>
       </c>
       <c r="AA11" s="28" t="n">
-        <v>15.76101063524304</v>
+        <v>14.9702235353203</v>
       </c>
       <c r="AB11" s="75" t="n">
-        <v>0.1865988883489678</v>
+        <v>0.1464442725417143</v>
       </c>
       <c r="AC11" s="75" t="n">
-        <v>0.3005447210037976</v>
+        <v>0.2757090788078762</v>
       </c>
       <c r="AD11" s="75" t="n">
-        <v>-0.1139458326548298</v>
+        <v>-0.1292648062661618</v>
       </c>
       <c r="AE11" s="72" t="n">
-        <v>85.61741899815361</v>
+        <v>85.55228582561726</v>
       </c>
       <c r="AF11" s="72" t="n">
-        <v>85.5429222476041</v>
+        <v>85.52929049436101</v>
       </c>
       <c r="AG11" s="72" t="n">
-        <v>84.90139999389649</v>
+        <v>84.96679992675782</v>
       </c>
       <c r="AH11" s="72" t="n">
-        <v>84.26700012207031</v>
+        <v>84.28700012207031</v>
       </c>
       <c r="AI11" s="72" t="n">
-        <v>83.16500022888184</v>
+        <v>83.20565021514892</v>
       </c>
       <c r="AJ11" s="72" t="n">
-        <v>86.98105359710452</v>
+        <v>86.98321531696089</v>
       </c>
       <c r="AK11" s="72" t="n">
-        <v>85.57000007629395</v>
+        <v>85.57399978637696</v>
       </c>
       <c r="AL11" s="72" t="n">
-        <v>84.15894655548338</v>
+        <v>84.16478425579302</v>
       </c>
       <c r="AM11" s="76" t="n">
-        <v>0.3866095185000036</v>
+        <v>0.3850425008292723</v>
       </c>
       <c r="AN11" s="29" t="n">
-        <v>3.298009862223858</v>
+        <v>3.293560039502272</v>
       </c>
       <c r="AO11" s="77" t="n">
-        <v>1.395424253334772</v>
+        <v>1.351383848292627</v>
       </c>
       <c r="AP11" s="72" t="n">
         <v>90.13999938964844</v>
@@ -4449,13 +4449,13 @@
         <v>67.35647006454938</v>
       </c>
       <c r="AT11" s="26" t="n">
-        <v>-0.02515719868514421</v>
+        <v>-0.01467864877879865</v>
       </c>
       <c r="AU11" s="26" t="n">
-        <v>0.002351521940810342</v>
+        <v>0.004595797629547427</v>
       </c>
       <c r="AV11" s="26" t="n">
-        <v>0.03925394695380402</v>
+        <v>0.04179393978269985</v>
       </c>
       <c r="AW11" s="26" t="n">
         <v>0.09745107704794687</v>
@@ -5222,17 +5222,17 @@
       </c>
       <c r="AX15" s="79" t="inlineStr">
         <is>
+          <t>Better Tech ETF for Artificial Intelligence: Vanguard's VGT with Broad Exposure or State Street XLK's Conce...</t>
+        </is>
+      </c>
+      <c r="AY15" s="79" t="inlineStr">
+        <is>
           <t>Stock Market News for Sep 1, 2026</t>
         </is>
       </c>
-      <c r="AY15" s="79" t="inlineStr">
+      <c r="AZ15" s="79" t="inlineStr">
         <is>
           <t>Sector Update: Tech Stocks Gain Late Afternoon</t>
-        </is>
-      </c>
-      <c r="AZ15" s="79" t="inlineStr">
-        <is>
-          <t>Sector Update: Tech Stocks Gain Thursday Afternoon</t>
         </is>
       </c>
     </row>
@@ -6965,12 +6965,12 @@
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>FTC alleges Amazon overcharged advertisers for years</t>
+          <t>Suzelle Snowden Started With One Class on the Beach 30 years ago, Now She's Running the World's Largest Fit...</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Amazon's $69 Billion Ad Machine Just Ran Into a $20 Billion Problem</t>
+          <t>Whirlpool (WHR) Dips More Than Broader Market: What You Should Know</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Broadcom's earnings loom, but this reveal came first</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>28 Analysts Share Their Broadcom Stock Forecast Before Q3 Earnings</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>Two Stocks That Will Benefit From OpenAI Announcement</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Broadcom Faces Crucial Earnings Test After AI Chip Sales Surge 143%</t>
         </is>
       </c>
     </row>
@@ -8286,7 +8286,7 @@
       </c>
       <c r="AZ33" s="90" t="inlineStr">
         <is>
-          <t>CEO Michael Dell Just Delivered Fantastic News for Dell Shareholders</t>
+          <t>Dow Jones Futures: Market Breaks Key Levels As Oil Prices Jump; Dell, Credo, Palo Alto Are Earnings Movers</t>
         </is>
       </c>
     </row>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Google prepares Gemini 3.8 Flash to narrow AI coding gap, WSJ reports</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>Stock Market Today, Sept. 1: Fervo Energy Surges 28% on 396-Megawatt Google Power Deal</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
+      <c r="AZ34" s="79" t="inlineStr">
         <is>
           <t>FRVO Stock Clocks Best Day In A Month After Google Deal: Analyst Says Agreement Arrived Earlier Than Expected</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Google Just Locked In Nearly 1 Gigawatt of Geothermal Power</t>
         </is>
       </c>
     </row>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
-          <t>MDB Stock Dives After-Hours Despite Raised Full-Year Forecast — What’s Driving The Selloff?</t>
+          <t>Dow Jones Futures: Market Breaks Key Levels As Oil Prices Jump; Dell, Credo, Palo Alto Are Earnings Movers</t>
         </is>
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
-          <t>MongoDB Inc. Q2 2027 Earnings: Recap of $MDB Earnings, Forecast</t>
+          <t>Market Chatter: Dropbox Accounts Breached In Hack Affecting About 5,000 Users</t>
         </is>
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>Box (BOX) Q2 2027 Earnings Call Transcript</t>
+          <t>MongoDB Q2 Earnings Call Highlights</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Not Nvidia. Not OpenAI. This Artificial Intelligence (AI) Stock Will Be the Ultimate Winner.</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
+          <t>Nvidia was just the beginning — Here are AI’s next big winners</t>
+        </is>
+      </c>
+      <c r="AZ43" s="90" t="inlineStr">
+        <is>
           <t>Nvidia Shareholders Should Brace Themselves for 1 Particular Thing in the Months to Come. Here’s What It Me...</t>
-        </is>
-      </c>
-      <c r="AY43" s="90" t="inlineStr">
-        <is>
-          <t>CEO Michael Dell Just Delivered Fantastic News for Dell Shareholders</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>28 Analysts Share Their Broadcom Stock Forecast Before Q3 Earnings</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 1 Sep 2026, 10:38 PM · Yahoo Finance data</t>
+          <t>Built 1 Sep 2026, 11:17 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -12253,7 +12253,7 @@
         <v>-0.003622402212613562</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
@@ -12784,10 +12784,10 @@
         </is>
       </c>
       <c r="C11" s="26" t="n">
-        <v>-0.001175346403020305</v>
+        <v>-0.005500217765873949</v>
       </c>
       <c r="D11" s="27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
@@ -12796,7 +12796,7 @@
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G11" s="23" t="inlineStr">
@@ -12816,7 +12816,7 @@
       </c>
       <c r="J11" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Same</t>
         </is>
       </c>
       <c r="K11" s="23" t="inlineStr">
@@ -12835,7 +12835,7 @@
         </is>
       </c>
       <c r="N11" s="69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O11" s="23" t="inlineStr">
         <is>
@@ -12856,7 +12856,7 @@
         <v>84.98000335693359</v>
       </c>
       <c r="S11" s="71" t="n">
-        <v>-0.09999847412109375</v>
+        <v>-0.4699935913085938</v>
       </c>
       <c r="T11" s="72" t="n">
         <v>85.34999847412109</v>
@@ -12871,58 +12871,58 @@
         <v>7012600</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>0.7806306180947875</v>
+        <v>0.8066036460840454</v>
       </c>
       <c r="Y11" s="28" t="n">
-        <v>47.47290145839173</v>
+        <v>47.48693481569663</v>
       </c>
       <c r="Z11" s="28" t="n">
         <v>28.03472477944208</v>
       </c>
       <c r="AA11" s="28" t="n">
-        <v>15.92319707054252</v>
+        <v>15.16847015679679</v>
       </c>
       <c r="AB11" s="75" t="n">
-        <v>0.2418924086119318</v>
+        <v>0.1940077921954639</v>
       </c>
       <c r="AC11" s="75" t="n">
-        <v>0.329031179167505</v>
+        <v>0.3080252803744166</v>
       </c>
       <c r="AD11" s="75" t="n">
-        <v>-0.08713877055557318</v>
+        <v>-0.1140174881789527</v>
       </c>
       <c r="AE11" s="72" t="n">
-        <v>85.72239585476893</v>
+        <v>85.63865320436504</v>
       </c>
       <c r="AF11" s="72" t="n">
-        <v>85.57221447236451</v>
+        <v>85.55721954379712</v>
       </c>
       <c r="AG11" s="72" t="n">
-        <v>84.86240005493164</v>
+        <v>84.90539993286133</v>
       </c>
       <c r="AH11" s="72" t="n">
-        <v>84.24230010986328</v>
+        <v>84.26900009155274</v>
       </c>
       <c r="AI11" s="72" t="n">
-        <v>83.12590023040771</v>
+        <v>83.16600021362305</v>
       </c>
       <c r="AJ11" s="72" t="n">
-        <v>86.98921164214956</v>
+        <v>86.98466080490893</v>
       </c>
       <c r="AK11" s="72" t="n">
-        <v>85.55050010681153</v>
+        <v>85.57999992370605</v>
       </c>
       <c r="AL11" s="72" t="n">
-        <v>84.1117885714735</v>
+        <v>84.17533904250318</v>
       </c>
       <c r="AM11" s="76" t="n">
-        <v>0.3017334483441489</v>
+        <v>0.286426540810812</v>
       </c>
       <c r="AN11" s="29" t="n">
-        <v>3.363420514296864</v>
+        <v>3.282684932122265</v>
       </c>
       <c r="AO11" s="77" t="n">
-        <v>1.400726645825778</v>
+        <v>1.353147829686729</v>
       </c>
       <c r="AP11" s="72" t="n">
         <v>90.13999938964844</v>
@@ -12937,13 +12937,13 @@
         <v>65.55408875565456</v>
       </c>
       <c r="AT11" s="26" t="n">
-        <v>-0.01174548821871158</v>
+        <v>-0.02824463896517315</v>
       </c>
       <c r="AU11" s="26" t="n">
-        <v>-0.005732980657204401</v>
+        <v>-0.0008230416497647663</v>
       </c>
       <c r="AV11" s="26" t="n">
-        <v>0.02496682672045547</v>
+        <v>0.03596250910077115</v>
       </c>
       <c r="AW11" s="26" t="n">
         <v>0.09397532213026283</v>
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 1 Sep 2026, 10:38 PM · Yahoo Finance data</t>
+          <t>Built 1 Sep 2026, 11:17 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19604,12 +19604,12 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>14 of 40</t>
+          <t>15 of 40</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>26 of 40</t>
+          <t>25 of 40</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
@@ -20011,7 +20011,7 @@
         <v>-0.008539388474021248</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" s="23" t="inlineStr">
         <is>
@@ -20189,7 +20189,7 @@
         <v>-0.002447827045478523</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
@@ -20367,7 +20367,7 @@
         <v>0.003800922632101411</v>
       </c>
       <c r="D9" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
@@ -20720,19 +20720,19 @@
         </is>
       </c>
       <c r="C11" s="26" t="n">
-        <v>-0.01379384326320543</v>
+        <v>0.004348790658493584</v>
       </c>
       <c r="D11" s="27" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G11" s="23" t="inlineStr">
@@ -20789,76 +20789,76 @@
         </is>
       </c>
       <c r="R11" s="70" t="n">
-        <v>85.08000183105469</v>
+        <v>85.44999694824219</v>
       </c>
       <c r="S11" s="71" t="n">
-        <v>-1.189994812011719</v>
+        <v>0.3699951171875</v>
       </c>
       <c r="T11" s="72" t="n">
-        <v>85.30999755859375</v>
+        <v>85.5</v>
       </c>
       <c r="U11" s="72" t="n">
-        <v>85.86000061035156</v>
+        <v>85.61000061035156</v>
       </c>
       <c r="V11" s="72" t="n">
-        <v>85.06999969482422</v>
+        <v>85.20999908447266</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>8492100</v>
+        <v>6807200</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>0.9228772958231383</v>
+        <v>0.758633140829468</v>
       </c>
       <c r="Y11" s="28" t="n">
-        <v>47.94394812605087</v>
+        <v>49.78740689917412</v>
       </c>
       <c r="Z11" s="28" t="n">
-        <v>30.92485485403817</v>
+        <v>41.61835818032277</v>
       </c>
       <c r="AA11" s="28" t="n">
-        <v>16.73591344057998</v>
+        <v>16.06676903557024</v>
       </c>
       <c r="AB11" s="75" t="n">
-        <v>0.3364391794618058</v>
+        <v>0.2793847748701808</v>
       </c>
       <c r="AC11" s="75" t="n">
-        <v>0.3508158718063983</v>
+        <v>0.3365296524191548</v>
       </c>
       <c r="AD11" s="75" t="n">
-        <v>-0.01437669234459249</v>
+        <v>-0.05714487754897402</v>
       </c>
       <c r="AE11" s="72" t="n">
-        <v>85.9345079970076</v>
+        <v>85.82683887505974</v>
       </c>
       <c r="AF11" s="72" t="n">
-        <v>85.6314355839076</v>
+        <v>85.61494116248348</v>
       </c>
       <c r="AG11" s="72" t="n">
-        <v>84.83639999389648</v>
+        <v>84.87179992675782</v>
       </c>
       <c r="AH11" s="72" t="n">
-        <v>84.20510009765626</v>
+        <v>84.24700004577636</v>
       </c>
       <c r="AI11" s="72" t="n">
-        <v>83.08315021514892</v>
+        <v>83.12825019836426</v>
       </c>
       <c r="AJ11" s="72" t="n">
-        <v>86.9874742051806</v>
+        <v>86.98984187178345</v>
       </c>
       <c r="AK11" s="72" t="n">
-        <v>85.55400009155274</v>
+        <v>85.57399978637696</v>
       </c>
       <c r="AL11" s="72" t="n">
-        <v>84.12052597792487</v>
+        <v>84.15815770097046</v>
       </c>
       <c r="AM11" s="76" t="n">
-        <v>0.3346680083052058</v>
+        <v>0.4562088034347526</v>
       </c>
       <c r="AN11" s="29" t="n">
-        <v>3.351039371844408</v>
+        <v>3.309047348355667</v>
       </c>
       <c r="AO11" s="77" t="n">
-        <v>1.466016456168893</v>
+        <v>1.399709783339811</v>
       </c>
       <c r="AP11" s="72" t="n">
         <v>90.13999938964844</v>
@@ -20867,22 +20867,22 @@
         <v>75.16000366210938</v>
       </c>
       <c r="AR11" s="29" t="n">
-        <v>-5.613487456019262</v>
+        <v>-5.203020271980218</v>
       </c>
       <c r="AS11" s="78" t="n">
-        <v>66.22163550226182</v>
+        <v>68.6915635577639</v>
       </c>
       <c r="AT11" s="26" t="n">
-        <v>-0.002812914493998675</v>
+        <v>-0.006279810779654227</v>
       </c>
       <c r="AU11" s="26" t="n">
-        <v>-0.02609888694330786</v>
+        <v>-0.0002340502185004256</v>
       </c>
       <c r="AV11" s="26" t="n">
-        <v>0.007698703346315838</v>
+        <v>0.03063554666435997</v>
       </c>
       <c r="AW11" s="26" t="n">
-        <v>0.09526263512882416</v>
+        <v>0.1000257030450693</v>
       </c>
       <c r="AX11" s="25" t="n"/>
       <c r="AY11" s="25" t="n"/>
@@ -20901,7 +20901,7 @@
         <v>-0.01092528481292099</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
@@ -21079,7 +21079,7 @@
         <v>-0.01065622006694034</v>
       </c>
       <c r="D13" s="27" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E13" s="23" t="inlineStr">
         <is>
@@ -21257,7 +21257,7 @@
         <v>-0.008198223248004122</v>
       </c>
       <c r="D14" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E14" s="30" t="inlineStr">
         <is>
@@ -21613,7 +21613,7 @@
         <v>-0.004030459153398613</v>
       </c>
       <c r="D16" s="34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
@@ -21791,7 +21791,7 @@
         <v>-0.007584418043843133</v>
       </c>
       <c r="D17" s="27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 1 Sep 2026, 10:38 PM · Yahoo Finance data</t>
+          <t>Built 1 Sep 2026, 11:17 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 1 Sep 2026, 10:38 PM · Yahoo Finance data</t>
+          <t>Built 1 Sep 2026, 11:17 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -43548,16 +43548,16 @@
         <v>0.003177178540842984</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>-0.02515719868514421</v>
+        <v>-0.01467864877879865</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>0.002351521940810342</v>
+        <v>0.004595797629547427</v>
       </c>
       <c r="G11" s="33" t="n">
-        <v>0.03925394695380402</v>
+        <v>0.04179393978269985</v>
       </c>
       <c r="H11" s="33" t="n">
-        <v>-0.03900348461482828</v>
+        <v>-0.0283792788282905</v>
       </c>
       <c r="I11" s="33" t="n">
         <v>0.09745107704794687</v>

</xml_diff>

<commit_message>
Daily workbook: 2026-09-03 22:37 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 3 Sep 2026, 08:01 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 3 Sep 2026, 10:37 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1523,22 +1523,22 @@
         </is>
       </c>
       <c r="E14" s="26" t="n">
-        <v>0.01543529989600545</v>
+        <v>0.01560876739959438</v>
       </c>
       <c r="F14" s="27" t="n">
         <v>8</v>
       </c>
       <c r="G14" s="28" t="n">
-        <v>60.4423848474622</v>
+        <v>60.51478853366662</v>
       </c>
       <c r="H14" s="29" t="n">
-        <v>3.144178463200342</v>
+        <v>3.161435108605559</v>
       </c>
       <c r="I14" s="26" t="n">
-        <v>0.01157564195890104</v>
+        <v>0.01174845011449688</v>
       </c>
       <c r="J14" s="26" t="n">
-        <v>0.009482745466561138</v>
+        <v>0.009655196091224338</v>
       </c>
     </row>
     <row r="15">
@@ -1589,22 +1589,22 @@
         </is>
       </c>
       <c r="E16" s="26" t="n">
-        <v>0.01296290601799632</v>
+        <v>0.01290846970806347</v>
       </c>
       <c r="F16" s="27" t="n">
         <v>8</v>
       </c>
       <c r="G16" s="28" t="n">
-        <v>53.30975797119432</v>
+        <v>53.29494491643694</v>
       </c>
       <c r="H16" s="29" t="n">
-        <v>1.877148705754395</v>
+        <v>1.871785406098092</v>
       </c>
       <c r="I16" s="26" t="n">
-        <v>-0.01394414333440253</v>
+        <v>-0.013997133667914</v>
       </c>
       <c r="J16" s="26" t="n">
-        <v>0.000376483589107357</v>
+        <v>0.0003227236695815261</v>
       </c>
     </row>
     <row r="17">
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="E18" s="26" t="n">
-        <v>0.01018633244166245</v>
+        <v>0.0103021113084425</v>
       </c>
       <c r="F18" s="27" t="n">
         <v>2</v>
       </c>
       <c r="G18" s="28" t="n">
-        <v>36.44308780900172</v>
+        <v>36.50808171075061</v>
       </c>
       <c r="H18" s="29" t="n">
-        <v>-3.763345273529972</v>
+        <v>-3.75252777449977</v>
       </c>
       <c r="I18" s="26" t="n">
-        <v>-0.02382555756663962</v>
+        <v>-0.02371367685008763</v>
       </c>
       <c r="J18" s="26" t="n">
-        <v>-0.06337543563493342</v>
+        <v>-0.06326808778515758</v>
       </c>
     </row>
     <row r="19">
@@ -1688,22 +1688,22 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
-        <v>0.008717340089801739</v>
+        <v>0.008539397794954384</v>
       </c>
       <c r="F19" s="34" t="n">
         <v>7</v>
       </c>
       <c r="G19" s="35" t="n">
-        <v>56.81104466027816</v>
+        <v>56.75377954276501</v>
       </c>
       <c r="H19" s="36" t="n">
-        <v>2.662342166136944</v>
+        <v>2.64460384611116</v>
       </c>
       <c r="I19" s="33" t="n">
-        <v>0.01786193158923965</v>
+        <v>0.01768237614714829</v>
       </c>
       <c r="J19" s="33" t="n">
-        <v>0.02281950677930222</v>
+        <v>0.02263907679855559</v>
       </c>
     </row>
     <row r="20">
@@ -1721,22 +1721,22 @@
         </is>
       </c>
       <c r="E20" s="26" t="n">
-        <v>0.007968131407967594</v>
+        <v>0.008436855537846455</v>
       </c>
       <c r="F20" s="27" t="n">
         <v>2</v>
       </c>
       <c r="G20" s="28" t="n">
-        <v>43.00853421006479</v>
+        <v>43.26204319173591</v>
       </c>
       <c r="H20" s="29" t="n">
-        <v>-3.337457584480208</v>
+        <v>-3.293377075693615</v>
       </c>
       <c r="I20" s="26" t="n">
-        <v>-0.003937053785110778</v>
+        <v>-0.003473865790152075</v>
       </c>
       <c r="J20" s="26" t="n">
-        <v>-0.01488780412621638</v>
+        <v>-0.0144297084360292</v>
       </c>
     </row>
     <row r="21">
@@ -1754,22 +1754,22 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
-        <v>0.001965864954553087</v>
+        <v>0.00179241147189213</v>
       </c>
       <c r="F21" s="34" t="n">
         <v>7</v>
       </c>
       <c r="G21" s="35" t="n">
-        <v>61.30211948766858</v>
+        <v>61.24050752750126</v>
       </c>
       <c r="H21" s="36" t="n">
-        <v>4.762522905060274</v>
+        <v>4.744767058530708</v>
       </c>
       <c r="I21" s="33" t="n">
-        <v>0.009966146618659355</v>
+        <v>0.009791308181914093</v>
       </c>
       <c r="J21" s="33" t="n">
-        <v>0.05561640728770745</v>
+        <v>0.05543366618982959</v>
       </c>
     </row>
     <row r="22">
@@ -1787,22 +1787,22 @@
         </is>
       </c>
       <c r="E22" s="26" t="n">
-        <v>-0.003273690907203086</v>
+        <v>-0.003156747888692357</v>
       </c>
       <c r="F22" s="27" t="n">
         <v>3</v>
       </c>
       <c r="G22" s="28" t="n">
-        <v>48.89800079075733</v>
+        <v>48.95291184688658</v>
       </c>
       <c r="H22" s="29" t="n">
-        <v>0.2714682934706225</v>
+        <v>0.2829968980809339</v>
       </c>
       <c r="I22" s="26" t="n">
-        <v>0.001998097852452752</v>
+        <v>0.00211565939470959</v>
       </c>
       <c r="J22" s="26" t="n">
-        <v>-0.0009375580609161105</v>
+        <v>-0.0008203409506870596</v>
       </c>
     </row>
     <row r="23">
@@ -1820,22 +1820,22 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
-        <v>-0.005854605643518473</v>
+        <v>-0.006232329108589174</v>
       </c>
       <c r="F23" s="34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G23" s="35" t="n">
-        <v>51.18485252513628</v>
+        <v>51.01920682289664</v>
       </c>
       <c r="H23" s="36" t="n">
-        <v>1.599653196166129</v>
+        <v>1.561834729939116</v>
       </c>
       <c r="I23" s="33" t="n">
-        <v>-0.01108397816384998</v>
+        <v>-0.0114597147397596</v>
       </c>
       <c r="J23" s="33" t="n">
-        <v>0</v>
+        <v>-0.0003799479102503112</v>
       </c>
     </row>
     <row r="24">
@@ -1853,22 +1853,22 @@
         </is>
       </c>
       <c r="E24" s="26" t="n">
-        <v>-0.006913919215374764</v>
+        <v>-0.007373206433021195</v>
       </c>
       <c r="F24" s="27" t="n">
         <v>7</v>
       </c>
       <c r="G24" s="28" t="n">
-        <v>67.85891849823807</v>
+        <v>67.62030622942083</v>
       </c>
       <c r="H24" s="29" t="n">
-        <v>9.568309040509382</v>
+        <v>9.518745306511555</v>
       </c>
       <c r="I24" s="26" t="n">
-        <v>0.037885718310118</v>
+        <v>0.03740571194106179</v>
       </c>
       <c r="J24" s="26" t="n">
-        <v>0.1280736484832767</v>
+        <v>0.1275519315673546</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -2077,11 +2077,11 @@
       </c>
       <c r="H32" s="31" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>SOXL</t>
         </is>
       </c>
       <c r="I32" s="33" t="n">
-        <v>0.003979398222152097</v>
+        <v>0.003667131125943079</v>
       </c>
       <c r="J32" s="34" t="n">
         <v>2</v>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="L32" s="35" t="n">
-        <v>46.65428964450938</v>
+        <v>39.31394302464612</v>
       </c>
     </row>
     <row r="33">
@@ -2117,11 +2117,11 @@
       </c>
       <c r="H33" s="24" t="inlineStr">
         <is>
-          <t>SOXL</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="I33" s="26" t="n">
-        <v>0.004043256336109913</v>
+        <v>0.004013443884859136</v>
       </c>
       <c r="J33" s="27" t="n">
         <v>2</v>
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="L33" s="28" t="n">
-        <v>39.33796822889906</v>
+        <v>46.67148684589938</v>
       </c>
     </row>
     <row r="34">
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="C34" s="33" t="n">
-        <v>0.04823240480617752</v>
+        <v>0.04914669207938038</v>
       </c>
       <c r="D34" s="34" t="n">
         <v>8</v>
@@ -2153,7 +2153,7 @@
         </is>
       </c>
       <c r="F34" s="35" t="n">
-        <v>62.47909653795556</v>
+        <v>62.5415624260926</v>
       </c>
       <c r="H34" s="31" t="inlineStr">
         <is>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="I34" s="33" t="n">
-        <v>0.007968131407967594</v>
+        <v>0.008436855537846455</v>
       </c>
       <c r="J34" s="34" t="n">
         <v>2</v>
@@ -2172,7 +2172,7 @@
         </is>
       </c>
       <c r="L34" s="35" t="n">
-        <v>43.00853421006479</v>
+        <v>43.26204319173591</v>
       </c>
     </row>
     <row r="35">
@@ -2201,7 +2201,7 @@
         </is>
       </c>
       <c r="I35" s="26" t="n">
-        <v>0.01018633244166245</v>
+        <v>0.0103021113084425</v>
       </c>
       <c r="J35" s="27" t="n">
         <v>2</v>
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="L35" s="28" t="n">
-        <v>36.44308780900172</v>
+        <v>36.50808171075061</v>
       </c>
     </row>
     <row r="36">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="C37" s="26" t="n">
-        <v>0.01543529989600545</v>
+        <v>0.01560876739959438</v>
       </c>
       <c r="D37" s="27" t="n">
         <v>8</v>
@@ -2273,7 +2273,7 @@
         </is>
       </c>
       <c r="F37" s="28" t="n">
-        <v>60.4423848474622</v>
+        <v>60.51478853366662</v>
       </c>
       <c r="H37" s="24" t="inlineStr">
         <is>
@@ -2302,7 +2302,7 @@
         </is>
       </c>
       <c r="C38" s="33" t="n">
-        <v>0.01296290601799632</v>
+        <v>0.01290846970806347</v>
       </c>
       <c r="D38" s="34" t="n">
         <v>8</v>
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="F38" s="35" t="n">
-        <v>53.30975797119432</v>
+        <v>53.29494491643694</v>
       </c>
       <c r="H38" s="31" t="inlineStr">
         <is>
@@ -2501,22 +2501,22 @@
       </c>
       <c r="H45" s="24" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="I45" s="26" t="n">
-        <v>-0.007621931717695318</v>
+        <v>-0.007373206433021195</v>
       </c>
       <c r="J45" s="27" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K45" s="23" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="L45" s="28" t="n">
-        <v>42.78947923002418</v>
+        <v>67.62030622942083</v>
       </c>
     </row>
     <row r="46">
@@ -2541,22 +2541,22 @@
       </c>
       <c r="H46" s="31" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="I46" s="33" t="n">
-        <v>-0.006913919215374764</v>
+        <v>-0.007113790014099619</v>
       </c>
       <c r="J46" s="34" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K46" s="30" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="L46" s="35" t="n">
-        <v>67.85891849823807</v>
+        <v>42.85202081378689</v>
       </c>
     </row>
     <row r="47">
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="C47" s="26" t="n">
-        <v>0.04823240480617752</v>
+        <v>0.04914669207938038</v>
       </c>
       <c r="D47" s="27" t="n">
         <v>8</v>
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="F47" s="28" t="n">
-        <v>62.47909653795556</v>
+        <v>62.5415624260926</v>
       </c>
       <c r="H47" s="24" t="inlineStr">
         <is>
@@ -2585,10 +2585,10 @@
         </is>
       </c>
       <c r="I47" s="26" t="n">
-        <v>-0.005854605643518473</v>
+        <v>-0.006232329108589174</v>
       </c>
       <c r="J47" s="27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K47" s="23" t="inlineStr">
         <is>
@@ -2596,7 +2596,7 @@
         </is>
       </c>
       <c r="L47" s="28" t="n">
-        <v>51.18485252513628</v>
+        <v>51.01920682289664</v>
       </c>
     </row>
     <row r="48">
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="I49" s="26" t="n">
-        <v>-0.003273690907203086</v>
+        <v>-0.003156747888692357</v>
       </c>
       <c r="J49" s="27" t="n">
         <v>3</v>
@@ -2676,7 +2676,7 @@
         </is>
       </c>
       <c r="L49" s="28" t="n">
-        <v>48.89800079075733</v>
+        <v>48.95291184688658</v>
       </c>
     </row>
     <row r="50">
@@ -2686,10 +2686,10 @@
         </is>
       </c>
       <c r="C50" s="33" t="n">
-        <v>0.04394065917242362</v>
+        <v>0.04399258781898019</v>
       </c>
       <c r="D50" s="34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
@@ -2697,7 +2697,7 @@
         </is>
       </c>
       <c r="F50" s="35" t="n">
-        <v>53.85734515399562</v>
+        <v>53.86463558689864</v>
       </c>
       <c r="H50" s="31" t="inlineStr">
         <is>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 3 Sep 2026, 08:01 PM · Yahoo Finance data</t>
+          <t>Built 3 Sep 2026, 10:37 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3536,7 +3536,7 @@
         </is>
       </c>
       <c r="C7" s="26" t="n">
-        <v>0.01018633244166245</v>
+        <v>0.0103021113084425</v>
       </c>
       <c r="D7" s="27" t="n">
         <v>5</v>
@@ -3605,76 +3605,76 @@
         </is>
       </c>
       <c r="R7" s="70" t="n">
-        <v>174.5399932861328</v>
+        <v>174.5599975585938</v>
       </c>
       <c r="S7" s="71" t="n">
-        <v>1.759994506835938</v>
+        <v>1.779998779296875</v>
       </c>
       <c r="T7" s="72" t="n">
         <v>173.7599945068359</v>
       </c>
       <c r="U7" s="72" t="n">
-        <v>174.5500030517578</v>
+        <v>174.5599975585938</v>
       </c>
       <c r="V7" s="72" t="n">
         <v>172.0200042724609</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>7835876</v>
+        <v>8340536</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>1.241891757562664</v>
+        <v>1.31660899058603</v>
       </c>
       <c r="Y7" s="28" t="n">
-        <v>36.44308780900172</v>
+        <v>36.50808171075061</v>
       </c>
       <c r="Z7" s="28" t="n">
-        <v>18.51615331547175</v>
+        <v>18.64300345523912</v>
       </c>
       <c r="AA7" s="28" t="n">
-        <v>25.31380752301438</v>
+        <v>25.30789385702951</v>
       </c>
       <c r="AB7" s="75" t="n">
-        <v>-2.153873731340553</v>
+        <v>-2.152277948922034</v>
       </c>
       <c r="AC7" s="75" t="n">
-        <v>-1.113390433685862</v>
+        <v>-1.113071277202158</v>
       </c>
       <c r="AD7" s="75" t="n">
-        <v>-1.040483297654691</v>
+        <v>-1.039206671719876</v>
       </c>
       <c r="AE7" s="72" t="n">
-        <v>175.9471690671849</v>
+        <v>175.9516144610652</v>
       </c>
       <c r="AF7" s="72" t="n">
-        <v>178.9338963206002</v>
+        <v>178.9357148908239</v>
       </c>
       <c r="AG7" s="72" t="n">
-        <v>181.3653994750977</v>
+        <v>181.3657995605469</v>
       </c>
       <c r="AH7" s="72" t="n">
-        <v>177.6534996032715</v>
+        <v>177.6536996459961</v>
       </c>
       <c r="AI7" s="72" t="n">
-        <v>170.6227997589111</v>
+        <v>170.6228997802734</v>
       </c>
       <c r="AJ7" s="72" t="n">
-        <v>189.763689617162</v>
+        <v>189.7619603825642</v>
       </c>
       <c r="AK7" s="72" t="n">
-        <v>180.7189994812012</v>
+        <v>180.7199996948242</v>
       </c>
       <c r="AL7" s="72" t="n">
-        <v>171.6743093452403</v>
+        <v>171.6780390070842</v>
       </c>
       <c r="AM7" s="76" t="n">
-        <v>0.1584180274733118</v>
+        <v>0.1593657974767113</v>
       </c>
       <c r="AN7" s="29" t="n">
-        <v>10.0096726541491</v>
+        <v>10.00659661687565</v>
       </c>
       <c r="AO7" s="77" t="n">
-        <v>1.439149376148468</v>
+        <v>1.43939341945109</v>
       </c>
       <c r="AP7" s="72" t="n">
         <v>188.1900024414062</v>
@@ -3683,22 +3683,22 @@
         <v>147.1399993896484</v>
       </c>
       <c r="AR7" s="29" t="n">
-        <v>-7.253312598007655</v>
+        <v>-7.24268277059843</v>
       </c>
       <c r="AS7" s="78" t="n">
-        <v>66.7478486224158</v>
+        <v>66.79658009860039</v>
       </c>
       <c r="AT7" s="26" t="n">
-        <v>-0.02382555756663962</v>
+        <v>-0.02371367685008763</v>
       </c>
       <c r="AU7" s="26" t="n">
-        <v>-0.06337543563493342</v>
+        <v>-0.06326808778515758</v>
       </c>
       <c r="AV7" s="26" t="n">
-        <v>-0.009196243995793107</v>
+        <v>-0.009082686593175682</v>
       </c>
       <c r="AW7" s="26" t="n">
-        <v>0.1251933907957785</v>
+        <v>0.1253223507821801</v>
       </c>
       <c r="AX7" s="79" t="inlineStr">
         <is>
@@ -3726,7 +3726,7 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>0.001965864954553087</v>
+        <v>0.00179241147189213</v>
       </c>
       <c r="D8" s="34" t="n">
         <v>8</v>
@@ -3795,10 +3795,10 @@
         </is>
       </c>
       <c r="R8" s="81" t="n">
-        <v>173.2899932861328</v>
+        <v>173.2599945068359</v>
       </c>
       <c r="S8" s="82" t="n">
-        <v>0.339996337890625</v>
+        <v>0.30999755859375</v>
       </c>
       <c r="T8" s="83" t="n">
         <v>174.0700073242188</v>
@@ -3810,61 +3810,61 @@
         <v>171.3899993896484</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>5571056</v>
+        <v>5933824</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.746844129311832</v>
+        <v>0.7935464651417891</v>
       </c>
       <c r="Y8" s="35" t="n">
-        <v>61.30211948766858</v>
+        <v>61.24050752750126</v>
       </c>
       <c r="Z8" s="35" t="n">
-        <v>69.18052956779573</v>
+        <v>68.90121146767028</v>
       </c>
       <c r="AA8" s="35" t="n">
         <v>27.67604920258904</v>
       </c>
       <c r="AB8" s="86" t="n">
-        <v>2.385782238825414</v>
+        <v>2.383389173810258</v>
       </c>
       <c r="AC8" s="86" t="n">
-        <v>2.721020654964855</v>
+        <v>2.720542041961823</v>
       </c>
       <c r="AD8" s="86" t="n">
-        <v>-0.3352384161394411</v>
+        <v>-0.3371528681515654</v>
       </c>
       <c r="AE8" s="83" t="n">
-        <v>172.3412267109</v>
+        <v>172.3345603155007</v>
       </c>
       <c r="AF8" s="83" t="n">
-        <v>170.4057594910344</v>
+        <v>170.4030323292801</v>
       </c>
       <c r="AG8" s="83" t="n">
-        <v>165.4121994018555</v>
+        <v>165.4115994262695</v>
       </c>
       <c r="AH8" s="83" t="n">
-        <v>156.7725999450684</v>
+        <v>156.7722999572754</v>
       </c>
       <c r="AI8" s="83" t="n">
-        <v>155.2762998962402</v>
+        <v>155.2761499023437</v>
       </c>
       <c r="AJ8" s="83" t="n">
-        <v>176.9101711652937</v>
+        <v>176.9063765261217</v>
       </c>
       <c r="AK8" s="83" t="n">
-        <v>171.0254974365234</v>
+        <v>171.0239974975586</v>
       </c>
       <c r="AL8" s="83" t="n">
-        <v>165.1408237077531</v>
+        <v>165.1416184689955</v>
       </c>
       <c r="AM8" s="87" t="n">
-        <v>0.6924062364356923</v>
+        <v>0.6900589029047605</v>
       </c>
       <c r="AN8" s="36" t="n">
-        <v>6.881633226594673</v>
+        <v>6.879010097570775</v>
       </c>
       <c r="AO8" s="88" t="n">
-        <v>1.532508124251243</v>
+        <v>1.532773467518285</v>
       </c>
       <c r="AP8" s="83" t="n">
         <v>176.6000061035156</v>
@@ -3873,22 +3873,22 @@
         <v>133.7299957275391</v>
       </c>
       <c r="AR8" s="36" t="n">
-        <v>-1.874299378813504</v>
+        <v>-1.891286229470401</v>
       </c>
       <c r="AS8" s="89" t="n">
-        <v>92.27895494226969</v>
+        <v>92.20897880036119</v>
       </c>
       <c r="AT8" s="33" t="n">
-        <v>0.009966146618659355</v>
+        <v>0.009791308181914093</v>
       </c>
       <c r="AU8" s="33" t="n">
-        <v>0.05561640728770745</v>
+        <v>0.05543366618982959</v>
       </c>
       <c r="AV8" s="33" t="n">
-        <v>0.1394660126230156</v>
+        <v>0.1392687560545276</v>
       </c>
       <c r="AW8" s="33" t="n">
-        <v>0.1194443790042614</v>
+        <v>0.1192505884441486</v>
       </c>
       <c r="AX8" s="90" t="inlineStr">
         <is>
@@ -3897,12 +3897,12 @@
       </c>
       <c r="AY8" s="90" t="inlineStr">
         <is>
+          <t>Bristol-Myers Squibb Stock: Is BMY Outperforming the Healthcare Sector?</t>
+        </is>
+      </c>
+      <c r="AZ8" s="90" t="inlineStr">
+        <is>
           <t>Abbott Laboratories Stock: Is ABT Underperforming the Healthcare Sector?</t>
-        </is>
-      </c>
-      <c r="AZ8" s="90" t="inlineStr">
-        <is>
-          <t>How Is AbbVie’s Stock Performance Compared to Other Healthcare Stocks</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3916,7 @@
         </is>
       </c>
       <c r="C9" s="26" t="n">
-        <v>0.01543529989600545</v>
+        <v>0.01560876739959438</v>
       </c>
       <c r="D9" s="27" t="n">
         <v>1</v>
@@ -3928,7 +3928,7 @@
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G9" s="23" t="inlineStr">
@@ -3985,10 +3985,10 @@
         </is>
       </c>
       <c r="R9" s="70" t="n">
-        <v>58.54999923706055</v>
+        <v>58.56000137329102</v>
       </c>
       <c r="S9" s="71" t="n">
-        <v>0.8899993896484375</v>
+        <v>0.9000015258789062</v>
       </c>
       <c r="T9" s="72" t="n">
         <v>58</v>
@@ -4000,61 +4000,61 @@
         <v>57.99900054931641</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>31745401</v>
+        <v>32643053</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>1.15796305916888</v>
+        <v>1.188760123219851</v>
       </c>
       <c r="Y9" s="28" t="n">
-        <v>60.4423848474622</v>
+        <v>60.51478853366662</v>
       </c>
       <c r="Z9" s="28" t="n">
-        <v>97.04146285858748</v>
+        <v>97.63330572001905</v>
       </c>
       <c r="AA9" s="28" t="n">
         <v>20.01864967579689</v>
       </c>
       <c r="AB9" s="75" t="n">
-        <v>0.3353941092978303</v>
+        <v>0.3361920005070971</v>
       </c>
       <c r="AC9" s="75" t="n">
-        <v>0.4113443820370709</v>
+        <v>0.4115039602789242</v>
       </c>
       <c r="AD9" s="75" t="n">
-        <v>-0.0759502727392406</v>
+        <v>-0.07531195977182714</v>
       </c>
       <c r="AE9" s="72" t="n">
-        <v>57.91020396099223</v>
+        <v>57.91242665793233</v>
       </c>
       <c r="AF9" s="72" t="n">
-        <v>57.67634644961277</v>
+        <v>57.67725573472463</v>
       </c>
       <c r="AG9" s="72" t="n">
-        <v>56.76520004272461</v>
+        <v>56.76540008544922</v>
       </c>
       <c r="AH9" s="72" t="n">
-        <v>54.42589992523193</v>
+        <v>54.42599994659424</v>
       </c>
       <c r="AI9" s="72" t="n">
-        <v>53.45440002441406</v>
+        <v>53.45445003509521</v>
       </c>
       <c r="AJ9" s="72" t="n">
-        <v>58.61799333221823</v>
+        <v>58.62032940234909</v>
       </c>
       <c r="AK9" s="72" t="n">
-        <v>57.83849983215332</v>
+        <v>57.83899993896485</v>
       </c>
       <c r="AL9" s="72" t="n">
-        <v>57.0590063320884</v>
+        <v>57.0576704755806</v>
       </c>
       <c r="AM9" s="76" t="n">
-        <v>0.9563857202452463</v>
+        <v>0.9613939881412046</v>
       </c>
       <c r="AN9" s="29" t="n">
-        <v>2.695413962419487</v>
+        <v>2.701739187083979</v>
       </c>
       <c r="AO9" s="77" t="n">
-        <v>1.130793263502062</v>
+        <v>1.130600122313456</v>
       </c>
       <c r="AP9" s="72" t="n">
         <v>58.59999847412109</v>
@@ -4063,36 +4063,36 @@
         <v>47.66999816894531</v>
       </c>
       <c r="AR9" s="29" t="n">
-        <v>-0.08532293235916644</v>
+        <v>-0.06825444005384984</v>
       </c>
       <c r="AS9" s="78" t="n">
-        <v>99.54255045137674</v>
+        <v>99.63406130179943</v>
       </c>
       <c r="AT9" s="26" t="n">
-        <v>0.01157564195890104</v>
+        <v>0.01174845011449688</v>
       </c>
       <c r="AU9" s="26" t="n">
-        <v>0.009482745466561138</v>
+        <v>0.009655196091224338</v>
       </c>
       <c r="AV9" s="26" t="n">
-        <v>0.1218624406534616</v>
+        <v>0.1220540891779616</v>
       </c>
       <c r="AW9" s="26" t="n">
-        <v>0.06901586174372687</v>
+        <v>0.06919848245117377</v>
       </c>
       <c r="AX9" s="79" t="inlineStr">
         <is>
+          <t>Sector Update: Financial Stocks Gain Late Afternoon</t>
+        </is>
+      </c>
+      <c r="AY9" s="79" t="inlineStr">
+        <is>
           <t>Sector Update: Financial Stocks Higher Thursday Afternoon</t>
         </is>
       </c>
-      <c r="AY9" s="79" t="inlineStr">
+      <c r="AZ9" s="79" t="inlineStr">
         <is>
           <t>Exchange-Traded Funds Rise as US Equities Advance After Midday</t>
-        </is>
-      </c>
-      <c r="AZ9" s="79" t="inlineStr">
-        <is>
-          <t>Sector Update: Financial Stocks Higher Late Afternoon</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>-0.006913919215374764</v>
+        <v>-0.007373206433021195</v>
       </c>
       <c r="D10" s="34" t="n">
         <v>11</v>
@@ -4175,10 +4175,10 @@
         </is>
       </c>
       <c r="R10" s="81" t="n">
-        <v>64.64990234375</v>
+        <v>64.62000274658203</v>
       </c>
       <c r="S10" s="82" t="n">
-        <v>-0.4500961303710938</v>
+        <v>-0.4799957275390625</v>
       </c>
       <c r="T10" s="83" t="n">
         <v>65.12000274658203</v>
@@ -4190,61 +4190,61 @@
         <v>64.58249664306641</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>23356482</v>
+        <v>24069781</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>0.919676734864996</v>
+        <v>0.9464342422426696</v>
       </c>
       <c r="Y10" s="35" t="n">
-        <v>67.85891849823807</v>
+        <v>67.62030622942083</v>
       </c>
       <c r="Z10" s="35" t="n">
-        <v>79.33265375467209</v>
+        <v>78.62244874844264</v>
       </c>
       <c r="AA10" s="35" t="n">
         <v>28.38186567925541</v>
       </c>
       <c r="AB10" s="86" t="n">
-        <v>1.493461536769338</v>
+        <v>1.491076383718905</v>
       </c>
       <c r="AC10" s="86" t="n">
-        <v>1.423253159474421</v>
+        <v>1.422776128864334</v>
       </c>
       <c r="AD10" s="86" t="n">
-        <v>0.07020837729491736</v>
+        <v>0.06830025485457081</v>
       </c>
       <c r="AE10" s="83" t="n">
-        <v>63.89730620972787</v>
+        <v>63.89066185480165</v>
       </c>
       <c r="AF10" s="83" t="n">
-        <v>62.42400394485963</v>
+        <v>62.42128579966254</v>
       </c>
       <c r="AG10" s="83" t="n">
-        <v>59.00419830322266</v>
+        <v>59.0036003112793</v>
       </c>
       <c r="AH10" s="83" t="n">
-        <v>58.13069911956787</v>
+        <v>58.13040012359619</v>
       </c>
       <c r="AI10" s="83" t="n">
-        <v>54.73654941558838</v>
+        <v>54.73639991760254</v>
       </c>
       <c r="AJ10" s="83" t="n">
-        <v>66.06958407987308</v>
+        <v>66.06453981783808</v>
       </c>
       <c r="AK10" s="83" t="n">
-        <v>62.54449520111084</v>
+        <v>62.54300022125244</v>
       </c>
       <c r="AL10" s="83" t="n">
-        <v>59.01940632234859</v>
+        <v>59.0214606246668</v>
       </c>
       <c r="AM10" s="87" t="n">
-        <v>0.7986317813607056</v>
+        <v>0.7948997829448485</v>
       </c>
       <c r="AN10" s="36" t="n">
-        <v>11.27225942883503</v>
+        <v>11.26117897807212</v>
       </c>
       <c r="AO10" s="88" t="n">
-        <v>1.805156816068809</v>
+        <v>1.805992059945803</v>
       </c>
       <c r="AP10" s="83" t="n">
         <v>65.51999664306641</v>
@@ -4253,22 +4253,22 @@
         <v>42.34999847412109</v>
       </c>
       <c r="AR10" s="36" t="n">
-        <v>-1.327982820353946</v>
+        <v>-1.373617128503957</v>
       </c>
       <c r="AS10" s="89" t="n">
-        <v>96.24473729789676</v>
+        <v>96.11569284588622</v>
       </c>
       <c r="AT10" s="33" t="n">
-        <v>0.037885718310118</v>
+        <v>0.03740571194106179</v>
       </c>
       <c r="AU10" s="33" t="n">
-        <v>0.1280736484832767</v>
+        <v>0.1275519315673546</v>
       </c>
       <c r="AV10" s="33" t="n">
-        <v>0.100423869680851</v>
+        <v>0.09991494036735382</v>
       </c>
       <c r="AW10" s="33" t="n">
-        <v>0.4459830835962213</v>
+        <v>0.4453143383987213</v>
       </c>
       <c r="AX10" s="90" t="inlineStr">
         <is>
@@ -4296,7 +4296,7 @@
         </is>
       </c>
       <c r="C11" s="26" t="n">
-        <v>-0.003273690907203086</v>
+        <v>-0.003156747888692357</v>
       </c>
       <c r="D11" s="27" t="n">
         <v>9</v>
@@ -4365,10 +4365,10 @@
         </is>
       </c>
       <c r="R11" s="70" t="n">
-        <v>85.25</v>
+        <v>85.26000213623047</v>
       </c>
       <c r="S11" s="71" t="n">
-        <v>-0.279998779296875</v>
+        <v>-0.2699966430664062</v>
       </c>
       <c r="T11" s="72" t="n">
         <v>85.37000274658203</v>
@@ -4380,61 +4380,61 @@
         <v>84.78500366210938</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>9952632</v>
+        <v>10264950</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.15490762915421</v>
+        <v>1.188994593899611</v>
       </c>
       <c r="Y11" s="28" t="n">
-        <v>48.89800079075733</v>
+        <v>48.95291184688658</v>
       </c>
       <c r="Z11" s="28" t="n">
-        <v>22.9167549696944</v>
+        <v>23.26405077777307</v>
       </c>
       <c r="AA11" s="28" t="n">
         <v>14.15434989105051</v>
       </c>
       <c r="AB11" s="75" t="n">
-        <v>0.0930269268367141</v>
+        <v>0.09382481804597376</v>
       </c>
       <c r="AC11" s="75" t="n">
-        <v>0.215834653576467</v>
+        <v>0.2159942318183189</v>
       </c>
       <c r="AD11" s="75" t="n">
-        <v>-0.1228077267397529</v>
+        <v>-0.1221694137723452</v>
       </c>
       <c r="AE11" s="72" t="n">
-        <v>85.48125911562225</v>
+        <v>85.48348181256236</v>
       </c>
       <c r="AF11" s="72" t="n">
-        <v>85.50395898536421</v>
+        <v>85.50486827047607</v>
       </c>
       <c r="AG11" s="72" t="n">
-        <v>85.01919982910157</v>
+        <v>85.01939987182617</v>
       </c>
       <c r="AH11" s="72" t="n">
-        <v>84.35560005187989</v>
+        <v>84.35570007324219</v>
       </c>
       <c r="AI11" s="72" t="n">
-        <v>83.28665019989013</v>
+        <v>83.28670021057128</v>
       </c>
       <c r="AJ11" s="72" t="n">
-        <v>86.98783487597555</v>
+        <v>86.9878533534679</v>
       </c>
       <c r="AK11" s="72" t="n">
-        <v>85.59099960327148</v>
+        <v>85.59149971008301</v>
       </c>
       <c r="AL11" s="72" t="n">
-        <v>84.19416433056742</v>
+        <v>84.19514606669813</v>
       </c>
       <c r="AM11" s="76" t="n">
-        <v>0.3779385050137803</v>
+        <v>0.3812988473861946</v>
       </c>
       <c r="AN11" s="29" t="n">
-        <v>3.263977005009009</v>
+        <v>3.262832519852175</v>
       </c>
       <c r="AO11" s="77" t="n">
-        <v>1.318194764009776</v>
+        <v>1.318040122169786</v>
       </c>
       <c r="AP11" s="72" t="n">
         <v>90.13999938964844</v>
@@ -4443,22 +4443,22 @@
         <v>75.16000366210938</v>
       </c>
       <c r="AR11" s="29" t="n">
-        <v>-5.424893968004618</v>
+        <v>-5.413797744021709</v>
       </c>
       <c r="AS11" s="78" t="n">
-        <v>67.35647006454938</v>
+        <v>67.42324001837574</v>
       </c>
       <c r="AT11" s="26" t="n">
-        <v>0.001998097852452752</v>
+        <v>0.00211565939470959</v>
       </c>
       <c r="AU11" s="26" t="n">
-        <v>-0.0009375580609161105</v>
+        <v>-0.0008203409506870596</v>
       </c>
       <c r="AV11" s="26" t="n">
-        <v>0.03912724340139673</v>
+        <v>0.03924916119904243</v>
       </c>
       <c r="AW11" s="26" t="n">
-        <v>0.09745107704794687</v>
+        <v>0.09757983781250879</v>
       </c>
       <c r="AX11" s="79" t="inlineStr">
         <is>
@@ -4570,10 +4570,10 @@
         <v>115.8300018310547</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>5319546</v>
+        <v>5658526</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>1.066299352650941</v>
+        <v>1.130407198630101</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>49.40193762534471</v>
@@ -4676,7 +4676,7 @@
         </is>
       </c>
       <c r="C13" s="26" t="n">
-        <v>0.008717340089801739</v>
+        <v>0.008539397794954384</v>
       </c>
       <c r="D13" s="27" t="n">
         <v>6</v>
@@ -4745,10 +4745,10 @@
         </is>
       </c>
       <c r="R13" s="70" t="n">
-        <v>113.4000015258789</v>
+        <v>113.379997253418</v>
       </c>
       <c r="S13" s="71" t="n">
-        <v>0.9800033569335938</v>
+        <v>0.9599990844726562</v>
       </c>
       <c r="T13" s="72" t="n">
         <v>113.4150009155273</v>
@@ -4760,61 +4760,61 @@
         <v>112.8450012207031</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>3244198</v>
+        <v>3366972</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>0.8100592228515445</v>
+        <v>0.8394285695195491</v>
       </c>
       <c r="Y13" s="28" t="n">
-        <v>56.81104466027816</v>
+        <v>56.75377954276501</v>
       </c>
       <c r="Z13" s="28" t="n">
-        <v>77.97031712968646</v>
+        <v>77.47516198296228</v>
       </c>
       <c r="AA13" s="28" t="n">
         <v>13.49986566465467</v>
       </c>
       <c r="AB13" s="75" t="n">
-        <v>0.5163016908110194</v>
+        <v>0.5147059083924859</v>
       </c>
       <c r="AC13" s="75" t="n">
-        <v>0.4543890005497054</v>
+        <v>0.4540698440659988</v>
       </c>
       <c r="AD13" s="75" t="n">
-        <v>0.06191269026131396</v>
+        <v>0.0606360643264871</v>
       </c>
       <c r="AE13" s="72" t="n">
-        <v>112.2173063679453</v>
+        <v>112.2128609740651</v>
       </c>
       <c r="AF13" s="72" t="n">
-        <v>111.6617569070491</v>
+        <v>111.6599383368254</v>
       </c>
       <c r="AG13" s="72" t="n">
-        <v>110.4591996765137</v>
+        <v>110.4587995910644</v>
       </c>
       <c r="AH13" s="72" t="n">
-        <v>112.582799911499</v>
+        <v>112.5825998687744</v>
       </c>
       <c r="AI13" s="72" t="n">
-        <v>114.0189999771118</v>
+        <v>114.0188999557495</v>
       </c>
       <c r="AJ13" s="72" t="n">
-        <v>113.642670034062</v>
+        <v>113.6382058003006</v>
       </c>
       <c r="AK13" s="72" t="n">
-        <v>111.7744998931885</v>
+        <v>111.7734996795654</v>
       </c>
       <c r="AL13" s="72" t="n">
-        <v>109.906329752315</v>
+        <v>109.9087935588303</v>
       </c>
       <c r="AM13" s="76" t="n">
-        <v>0.9350518181203786</v>
+        <v>0.9307642786143717</v>
       </c>
       <c r="AN13" s="29" t="n">
-        <v>3.342748377597231</v>
+        <v>3.336580005244354</v>
       </c>
       <c r="AO13" s="77" t="n">
-        <v>1.511676335240576</v>
+        <v>1.511943048823355</v>
       </c>
       <c r="AP13" s="72" t="n">
         <v>120.4049987792969</v>
@@ -4823,22 +4823,22 @@
         <v>105.0299987792969</v>
       </c>
       <c r="AR13" s="29" t="n">
-        <v>-5.817862484478886</v>
+        <v>-5.834476638927411</v>
       </c>
       <c r="AS13" s="78" t="n">
-        <v>54.43904225419207</v>
+        <v>54.30893316501524</v>
       </c>
       <c r="AT13" s="26" t="n">
-        <v>0.01786193158923965</v>
+        <v>0.01768237614714829</v>
       </c>
       <c r="AU13" s="26" t="n">
-        <v>0.02281950677930222</v>
+        <v>0.02263907679855559</v>
       </c>
       <c r="AV13" s="26" t="n">
-        <v>0.002563883953341728</v>
+        <v>0.00238702715594985</v>
       </c>
       <c r="AW13" s="26" t="n">
-        <v>-0.03669724473350133</v>
+        <v>-0.03686717569046283</v>
       </c>
       <c r="AX13" s="79" t="inlineStr">
         <is>
@@ -4866,7 +4866,7 @@
         </is>
       </c>
       <c r="C14" s="33" t="n">
-        <v>-0.005854605643518473</v>
+        <v>-0.006232329108589174</v>
       </c>
       <c r="D14" s="34" t="n">
         <v>10</v>
@@ -4878,24 +4878,24 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G14" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I14" s="30" t="inlineStr">
+        <is>
           <t>Same</t>
         </is>
       </c>
-      <c r="G14" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H14" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I14" s="30" t="inlineStr">
-        <is>
-          <t>Same</t>
-        </is>
-      </c>
       <c r="J14" s="30" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4917,7 +4917,7 @@
         </is>
       </c>
       <c r="N14" s="80" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O14" s="30" t="inlineStr">
         <is>
@@ -4935,10 +4935,10 @@
         </is>
       </c>
       <c r="R14" s="81" t="n">
-        <v>52.63999938964844</v>
+        <v>52.61999893188477</v>
       </c>
       <c r="S14" s="82" t="n">
-        <v>-0.3100013732910156</v>
+        <v>-0.3300018310546875</v>
       </c>
       <c r="T14" s="83" t="n">
         <v>53.45000076293945</v>
@@ -4950,61 +4950,61 @@
         <v>52.33499908447266</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>13039854</v>
+        <v>14287443</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>1.200175312233383</v>
+        <v>1.307495394703732</v>
       </c>
       <c r="Y14" s="35" t="n">
-        <v>51.18485252513628</v>
+        <v>51.01920682289664</v>
       </c>
       <c r="Z14" s="35" t="n">
-        <v>36.47540535089762</v>
+        <v>35.65571399760174</v>
       </c>
       <c r="AA14" s="35" t="n">
         <v>14.79868881918597</v>
       </c>
       <c r="AB14" s="86" t="n">
-        <v>0.2819247713413375</v>
+        <v>0.2803292932291299</v>
       </c>
       <c r="AC14" s="86" t="n">
-        <v>0.3852990069094271</v>
+        <v>0.3849799112869856</v>
       </c>
       <c r="AD14" s="86" t="n">
-        <v>-0.1033742355680896</v>
+        <v>-0.1046506180578556</v>
       </c>
       <c r="AE14" s="83" t="n">
-        <v>52.81552252679378</v>
+        <v>52.81107798062408</v>
       </c>
       <c r="AF14" s="83" t="n">
-        <v>52.63827511159779</v>
+        <v>52.63645688816472</v>
       </c>
       <c r="AG14" s="83" t="n">
-        <v>51.81119987487793</v>
+        <v>51.81079986572266</v>
       </c>
       <c r="AH14" s="83" t="n">
-        <v>51.56830001831054</v>
+        <v>51.56810001373291</v>
       </c>
       <c r="AI14" s="83" t="n">
-        <v>50.02227499008179</v>
+        <v>50.02217498779297</v>
       </c>
       <c r="AJ14" s="83" t="n">
-        <v>53.90641538850587</v>
+        <v>53.90620090904133</v>
       </c>
       <c r="AK14" s="83" t="n">
-        <v>52.84000034332276</v>
+        <v>52.83900032043457</v>
       </c>
       <c r="AL14" s="83" t="n">
-        <v>51.77358529813964</v>
+        <v>51.77179973182781</v>
       </c>
       <c r="AM14" s="87" t="n">
-        <v>0.4062274324721398</v>
+        <v>0.3973944585076951</v>
       </c>
       <c r="AN14" s="36" t="n">
-        <v>4.036393028971179</v>
+        <v>4.03944276816319</v>
       </c>
       <c r="AO14" s="88" t="n">
-        <v>1.623349448464686</v>
+        <v>1.623966471131708</v>
       </c>
       <c r="AP14" s="83" t="n">
         <v>54.18999862670898</v>
@@ -5013,22 +5013,22 @@
         <v>42.03499984741211</v>
       </c>
       <c r="AR14" s="36" t="n">
-        <v>-2.860304994170249</v>
+        <v>-2.897213018290068</v>
       </c>
       <c r="AS14" s="89" t="n">
-        <v>87.24805106767597</v>
+        <v>87.08350594408667</v>
       </c>
       <c r="AT14" s="33" t="n">
-        <v>-0.01108397816384998</v>
+        <v>-0.0114597147397596</v>
       </c>
       <c r="AU14" s="33" t="n">
-        <v>0</v>
+        <v>-0.0003799479102503112</v>
       </c>
       <c r="AV14" s="33" t="n">
-        <v>0.01975979230665259</v>
+        <v>0.01937233670460836</v>
       </c>
       <c r="AW14" s="33" t="n">
-        <v>0.1607497499627784</v>
+        <v>0.1603087255209565</v>
       </c>
       <c r="AX14" s="90" t="inlineStr">
         <is>
@@ -5056,7 +5056,7 @@
         </is>
       </c>
       <c r="C15" s="26" t="n">
-        <v>0.01296290601799632</v>
+        <v>0.01290846970806347</v>
       </c>
       <c r="D15" s="27" t="n">
         <v>3</v>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G15" s="23" t="inlineStr">
@@ -5125,10 +5125,10 @@
         </is>
       </c>
       <c r="R15" s="70" t="n">
-        <v>185.9799957275391</v>
+        <v>185.9700012207031</v>
       </c>
       <c r="S15" s="71" t="n">
-        <v>2.379989624023438</v>
+        <v>2.3699951171875</v>
       </c>
       <c r="T15" s="72" t="n">
         <v>183.5200042724609</v>
@@ -5140,61 +5140,61 @@
         <v>182.5</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>5835122</v>
+        <v>6090009</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>0.9668648026996621</v>
+        <v>1.006972497100184</v>
       </c>
       <c r="Y15" s="28" t="n">
-        <v>53.30975797119432</v>
+        <v>53.29494491643694</v>
       </c>
       <c r="Z15" s="28" t="n">
-        <v>55.37503835351318</v>
+        <v>55.29774127310062</v>
       </c>
       <c r="AA15" s="28" t="n">
         <v>11.28058245136133</v>
       </c>
       <c r="AB15" s="75" t="n">
-        <v>0.6876754241711183</v>
+        <v>0.6868781415745104</v>
       </c>
       <c r="AC15" s="75" t="n">
-        <v>0.8479187452147254</v>
+        <v>0.847759288695404</v>
       </c>
       <c r="AD15" s="75" t="n">
-        <v>-0.1602433210436072</v>
+        <v>-0.1608811471208935</v>
       </c>
       <c r="AE15" s="72" t="n">
-        <v>184.879065831376</v>
+        <v>184.8768448298569</v>
       </c>
       <c r="AF15" s="72" t="n">
-        <v>184.3666050254255</v>
+        <v>184.3656964338949</v>
       </c>
       <c r="AG15" s="72" t="n">
-        <v>182.5532006835938</v>
+        <v>182.553000793457</v>
       </c>
       <c r="AH15" s="72" t="n">
-        <v>178.6247009277344</v>
+        <v>178.624600982666</v>
       </c>
       <c r="AI15" s="72" t="n">
-        <v>160.1278751373291</v>
+        <v>160.1278251647949</v>
       </c>
       <c r="AJ15" s="72" t="n">
-        <v>191.5917482899507</v>
+        <v>191.5911659134844</v>
       </c>
       <c r="AK15" s="72" t="n">
-        <v>185.7330009460449</v>
+        <v>185.7325012207031</v>
       </c>
       <c r="AL15" s="72" t="n">
-        <v>179.8742536021391</v>
+        <v>179.8738365279218</v>
       </c>
       <c r="AM15" s="76" t="n">
-        <v>0.5210791460183953</v>
+        <v>0.5202691238067136</v>
       </c>
       <c r="AN15" s="29" t="n">
-        <v>6.308784453019991</v>
+        <v>6.30871242703991</v>
       </c>
       <c r="AO15" s="77" t="n">
-        <v>2.017235271040187</v>
+        <v>2.017343682459092</v>
       </c>
       <c r="AP15" s="72" t="n">
         <v>198.7299957275391</v>
@@ -5203,22 +5203,22 @@
         <v>126.6800003051758</v>
       </c>
       <c r="AR15" s="29" t="n">
-        <v>-6.415740086604938</v>
+        <v>-6.420769275479699</v>
       </c>
       <c r="AS15" s="78" t="n">
-        <v>82.30395446209484</v>
+        <v>82.29008283479304</v>
       </c>
       <c r="AT15" s="26" t="n">
-        <v>-0.01394414333440253</v>
+        <v>-0.013997133667914</v>
       </c>
       <c r="AU15" s="26" t="n">
-        <v>0.000376483589107357</v>
+        <v>0.0003227236695815261</v>
       </c>
       <c r="AV15" s="26" t="n">
-        <v>-0.03722111357643598</v>
+        <v>-0.03727285301284267</v>
       </c>
       <c r="AW15" s="26" t="n">
-        <v>0.291796861503359</v>
+        <v>0.2917274407438175</v>
       </c>
       <c r="AX15" s="79" t="inlineStr">
         <is>
@@ -5330,10 +5330,10 @@
         <v>43.84000015258789</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>4143450</v>
+        <v>4414470</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>0.8075550724221049</v>
+        <v>0.8581103153064147</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>43.70604864099334</v>
@@ -5412,17 +5412,17 @@
       </c>
       <c r="AX16" s="90" t="inlineStr">
         <is>
+          <t>Sector Update: Financial Stocks Gain Late Afternoon</t>
+        </is>
+      </c>
+      <c r="AY16" s="90" t="inlineStr">
+        <is>
           <t>Sector Update: Financial Stocks Higher Thursday Afternoon</t>
         </is>
       </c>
-      <c r="AY16" s="90" t="inlineStr">
+      <c r="AZ16" s="90" t="inlineStr">
         <is>
           <t>Sector Update: Financial Stocks Higher Late Afternoon</t>
-        </is>
-      </c>
-      <c r="AZ16" s="90" t="inlineStr">
-        <is>
-          <t>Sector Update: Financial Stocks Rise Wednesday Afternoon</t>
         </is>
       </c>
     </row>
@@ -5436,7 +5436,7 @@
         </is>
       </c>
       <c r="C17" s="26" t="n">
-        <v>0.007968131407967594</v>
+        <v>0.008436855537846455</v>
       </c>
       <c r="D17" s="27" t="n">
         <v>7</v>
@@ -5505,10 +5505,10 @@
         </is>
       </c>
       <c r="R17" s="70" t="n">
-        <v>43.0099983215332</v>
+        <v>43.02999877929688</v>
       </c>
       <c r="S17" s="71" t="n">
-        <v>0.3400001525878906</v>
+        <v>0.3600006103515625</v>
       </c>
       <c r="T17" s="72" t="n">
         <v>42.81999969482422</v>
@@ -5520,61 +5520,61 @@
         <v>42.79000091552734</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>20601238</v>
+        <v>22875638</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>1.029162828498838</v>
+        <v>1.136328048216559</v>
       </c>
       <c r="Y17" s="28" t="n">
-        <v>43.00853421006479</v>
+        <v>43.26204319173591</v>
       </c>
       <c r="Z17" s="28" t="n">
-        <v>41.21854243063133</v>
+        <v>41.93540448083218</v>
       </c>
       <c r="AA17" s="28" t="n">
         <v>16.71578460388293</v>
       </c>
       <c r="AB17" s="75" t="n">
-        <v>-0.4935861129895756</v>
+        <v>-0.491990634877375</v>
       </c>
       <c r="AC17" s="75" t="n">
-        <v>-0.4643723743420835</v>
+        <v>-0.4640532787196434</v>
       </c>
       <c r="AD17" s="75" t="n">
-        <v>-0.02921373864749205</v>
+        <v>-0.02793735615773163</v>
       </c>
       <c r="AE17" s="72" t="n">
-        <v>42.9113476677261</v>
+        <v>42.9157922138958</v>
       </c>
       <c r="AF17" s="72" t="n">
-        <v>43.40497489175099</v>
+        <v>43.40679311518405</v>
       </c>
       <c r="AG17" s="72" t="n">
-        <v>44.49500007629395</v>
+        <v>44.49540008544922</v>
       </c>
       <c r="AH17" s="72" t="n">
-        <v>44.77259986877441</v>
+        <v>44.77279987335205</v>
       </c>
       <c r="AI17" s="72" t="n">
-        <v>44.6714249420166</v>
+        <v>44.67152494430542</v>
       </c>
       <c r="AJ17" s="72" t="n">
-        <v>44.55475261675537</v>
+        <v>44.5544930970511</v>
       </c>
       <c r="AK17" s="72" t="n">
-        <v>43.38700027465821</v>
+        <v>43.38800029754638</v>
       </c>
       <c r="AL17" s="72" t="n">
-        <v>42.21924793256104</v>
+        <v>42.22150749804167</v>
       </c>
       <c r="AM17" s="76" t="n">
-        <v>0.3385779503349379</v>
+        <v>0.3465479090820306</v>
       </c>
       <c r="AN17" s="29" t="n">
-        <v>5.382959571783238</v>
+        <v>5.377029554278317</v>
       </c>
       <c r="AO17" s="77" t="n">
-        <v>1.501804572681108</v>
+        <v>1.501106529925419</v>
       </c>
       <c r="AP17" s="72" t="n">
         <v>47.79999923706055</v>
@@ -5583,22 +5583,22 @@
         <v>41.15000152587891</v>
       </c>
       <c r="AR17" s="29" t="n">
-        <v>-10.02092257736593</v>
+        <v>-9.979080614849401</v>
       </c>
       <c r="AS17" s="78" t="n">
-        <v>27.96988625314569</v>
+        <v>28.27064512002534</v>
       </c>
       <c r="AT17" s="26" t="n">
-        <v>-0.003937053785110778</v>
+        <v>-0.003473865790152075</v>
       </c>
       <c r="AU17" s="26" t="n">
-        <v>-0.01488780412621638</v>
+        <v>-0.0144297084360292</v>
       </c>
       <c r="AV17" s="26" t="n">
-        <v>-0.02116523291401473</v>
+        <v>-0.02071005634622314</v>
       </c>
       <c r="AW17" s="26" t="n">
-        <v>0.00749589377180282</v>
+        <v>0.007964398302303222</v>
       </c>
       <c r="AX17" s="79" t="inlineStr">
         <is>
@@ -5645,7 +5645,7 @@
         </is>
       </c>
       <c r="C19" s="26" t="n">
-        <v>0.01044232781374466</v>
+        <v>0.01046841189654324</v>
       </c>
       <c r="D19" s="27" t="n">
         <v>2</v>
@@ -5714,10 +5714,10 @@
         </is>
       </c>
       <c r="R19" s="70" t="n">
-        <v>773.1500244140625</v>
+        <v>773.1699829101562</v>
       </c>
       <c r="S19" s="71" t="n">
-        <v>7.99005126953125</v>
+        <v>8.010009765625</v>
       </c>
       <c r="T19" s="72" t="n">
         <v>767.9000244140625</v>
@@ -5729,61 +5729,61 @@
         <v>767.4500122070312</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>37276512</v>
+        <v>42648446</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>1.021643195735175</v>
+        <v>1.160330888149106</v>
       </c>
       <c r="Y19" s="28" t="n">
-        <v>58.77649139395812</v>
+        <v>58.79115045203841</v>
       </c>
       <c r="Z19" s="28" t="n">
-        <v>79.01737203821565</v>
+        <v>79.13273874204428</v>
       </c>
       <c r="AA19" s="28" t="n">
         <v>13.44376294928172</v>
       </c>
       <c r="AB19" s="75" t="n">
-        <v>3.069369028978258</v>
+        <v>3.07096115972081</v>
       </c>
       <c r="AC19" s="75" t="n">
-        <v>3.90001341073205</v>
+        <v>3.90033183688056</v>
       </c>
       <c r="AD19" s="75" t="n">
-        <v>-0.8306443817537916</v>
+        <v>-0.8293706771597504</v>
       </c>
       <c r="AE19" s="72" t="n">
-        <v>767.7018123284879</v>
+        <v>767.7062475498421</v>
       </c>
       <c r="AF19" s="72" t="n">
-        <v>765.5851549077978</v>
+        <v>765.5869693165336</v>
       </c>
       <c r="AG19" s="72" t="n">
-        <v>756.1390014648438</v>
+        <v>756.1394006347656</v>
       </c>
       <c r="AH19" s="72" t="n">
-        <v>744.5563012695312</v>
+        <v>744.5565008544922</v>
       </c>
       <c r="AI19" s="72" t="n">
-        <v>711.6302005004883</v>
+        <v>711.6303002929687</v>
       </c>
       <c r="AJ19" s="72" t="n">
-        <v>778.0323789695482</v>
+        <v>778.0351647978197</v>
       </c>
       <c r="AK19" s="72" t="n">
-        <v>769.2054962158203</v>
+        <v>769.206494140625</v>
       </c>
       <c r="AL19" s="72" t="n">
-        <v>760.3786134620924</v>
+        <v>760.3778234834302</v>
       </c>
       <c r="AM19" s="76" t="n">
-        <v>0.7234383478457502</v>
+        <v>0.7244669058020271</v>
       </c>
       <c r="AN19" s="29" t="n">
-        <v>2.295064920142297</v>
+        <v>2.295526812227012</v>
       </c>
       <c r="AO19" s="77" t="n">
-        <v>0.8247771104614723</v>
+        <v>0.8247558197865869</v>
       </c>
       <c r="AP19" s="72" t="n">
         <v>779.3699951171875</v>
@@ -5792,22 +5792,22 @@
         <v>629.280029296875</v>
       </c>
       <c r="AR19" s="29" t="n">
-        <v>-0.7980767468716565</v>
+        <v>-0.7955158969263354</v>
       </c>
       <c r="AS19" s="78" t="n">
-        <v>95.85583841722534</v>
+        <v>95.86913610570484</v>
       </c>
       <c r="AT19" s="26" t="n">
-        <v>0.002658603155274664</v>
+        <v>0.002684486304964206</v>
       </c>
       <c r="AU19" s="26" t="n">
-        <v>0.004364887154453712</v>
+        <v>0.00439081435104427</v>
       </c>
       <c r="AV19" s="26" t="n">
-        <v>0.02121279767123352</v>
+        <v>0.02123915978853219</v>
       </c>
       <c r="AW19" s="26" t="n">
-        <v>0.1337840858022281</v>
+        <v>0.1338133538931976</v>
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
@@ -5917,10 +5917,10 @@
         <v>709.6937866210938</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>27984653</v>
+        <v>29342845</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.9136779999442776</v>
+        <v>0.9559025285381031</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>52.85437750437693</v>
@@ -6021,10 +6021,10 @@
         </is>
       </c>
       <c r="C21" s="26" t="n">
-        <v>0.003979398222152097</v>
+        <v>0.004013443884859136</v>
       </c>
       <c r="D21" s="27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E21" s="23" t="inlineStr">
         <is>
@@ -6090,10 +6090,10 @@
         </is>
       </c>
       <c r="R21" s="70" t="n">
-        <v>295.1799926757812</v>
+        <v>295.1900024414062</v>
       </c>
       <c r="S21" s="71" t="n">
-        <v>1.16998291015625</v>
+        <v>1.17999267578125</v>
       </c>
       <c r="T21" s="72" t="n">
         <v>295.7900085449219</v>
@@ -6105,61 +6105,61 @@
         <v>293.4299926757812</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>16038850</v>
+        <v>16613075</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>0.9484342100030616</v>
+        <v>0.9807251019376435</v>
       </c>
       <c r="Y21" s="28" t="n">
-        <v>46.65428964450938</v>
+        <v>46.67148684589938</v>
       </c>
       <c r="Z21" s="28" t="n">
-        <v>36.28131455239423</v>
+        <v>36.3510205122538</v>
       </c>
       <c r="AA21" s="28" t="n">
         <v>19.93049326643414</v>
       </c>
       <c r="AB21" s="75" t="n">
-        <v>-0.7170652868219349</v>
+        <v>-0.7162667869999382</v>
       </c>
       <c r="AC21" s="75" t="n">
-        <v>0.2743904745372794</v>
+        <v>0.2745501745016787</v>
       </c>
       <c r="AD21" s="75" t="n">
-        <v>-0.9914557613592143</v>
+        <v>-0.9908169615016169</v>
       </c>
       <c r="AE21" s="72" t="n">
-        <v>295.5545575878534</v>
+        <v>295.5567819802145</v>
       </c>
       <c r="AF21" s="72" t="n">
-        <v>297.1338999562503</v>
+        <v>297.1348099349435</v>
       </c>
       <c r="AG21" s="72" t="n">
-        <v>297.0718005371094</v>
+        <v>297.0720007324219</v>
       </c>
       <c r="AH21" s="72" t="n">
-        <v>290.2329010009765</v>
+        <v>290.2330010986328</v>
       </c>
       <c r="AI21" s="72" t="n">
-        <v>272.364450302124</v>
+        <v>272.3645003509521</v>
       </c>
       <c r="AJ21" s="72" t="n">
-        <v>306.4633595599753</v>
+        <v>306.462777686003</v>
       </c>
       <c r="AK21" s="72" t="n">
-        <v>299.1425003051758</v>
+        <v>299.143000793457</v>
       </c>
       <c r="AL21" s="72" t="n">
-        <v>291.8216410503762</v>
+        <v>291.823223900911</v>
       </c>
       <c r="AM21" s="76" t="n">
-        <v>0.2293686784924412</v>
+        <v>0.2299782213255524</v>
       </c>
       <c r="AN21" s="29" t="n">
-        <v>4.89456312448487</v>
+        <v>4.893831293482214</v>
       </c>
       <c r="AO21" s="77" t="n">
-        <v>1.134769820088047</v>
+        <v>1.134731340533037</v>
       </c>
       <c r="AP21" s="72" t="n">
         <v>305.1799926757812</v>
@@ -6168,22 +6168,22 @@
         <v>228.8999938964844</v>
       </c>
       <c r="AR21" s="29" t="n">
-        <v>-3.27675478078403</v>
+        <v>-3.273474826047396</v>
       </c>
       <c r="AS21" s="78" t="n">
-        <v>86.89040356577182</v>
+        <v>86.90352596454632</v>
       </c>
       <c r="AT21" s="26" t="n">
-        <v>-0.0154431303842949</v>
+        <v>-0.01540974335348699</v>
       </c>
       <c r="AU21" s="26" t="n">
-        <v>-0.01531172734466524</v>
+        <v>-0.01527833585788585</v>
       </c>
       <c r="AV21" s="26" t="n">
-        <v>0.01085573372193838</v>
+        <v>0.01089001256612265</v>
       </c>
       <c r="AW21" s="26" t="n">
-        <v>0.1991387239372933</v>
+        <v>0.1991793875929484</v>
       </c>
       <c r="AX21" s="79" t="inlineStr">
         <is>
@@ -6209,10 +6209,10 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>0.004043256336109913</v>
+        <v>0.003667131125943079</v>
       </c>
       <c r="D22" s="34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E22" s="30" t="inlineStr">
         <is>
@@ -6278,10 +6278,10 @@
         </is>
       </c>
       <c r="R22" s="81" t="n">
-        <v>106.7799987792969</v>
+        <v>106.7399978637695</v>
       </c>
       <c r="S22" s="82" t="n">
-        <v>0.4300003051757812</v>
+        <v>0.3899993896484375</v>
       </c>
       <c r="T22" s="83" t="n">
         <v>103</v>
@@ -6293,61 +6293,61 @@
         <v>98.62000274658203</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>53290604</v>
+        <v>54538100</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>0.9836683881425153</v>
+        <v>1.005537655968398</v>
       </c>
       <c r="Y22" s="35" t="n">
-        <v>39.33796822889906</v>
+        <v>39.31394302464612</v>
       </c>
       <c r="Z22" s="35" t="n">
-        <v>13.99656376230992</v>
+        <v>13.92795155190141</v>
       </c>
       <c r="AA22" s="35" t="n">
         <v>20.05925473325475</v>
       </c>
       <c r="AB22" s="86" t="n">
-        <v>-10.77548603426438</v>
+        <v>-10.77867699048879</v>
       </c>
       <c r="AC22" s="86" t="n">
-        <v>-10.45858757131133</v>
+        <v>-10.45922576255621</v>
       </c>
       <c r="AD22" s="86" t="n">
-        <v>-0.3168984629530485</v>
+        <v>-0.3194512279325821</v>
       </c>
       <c r="AE22" s="83" t="n">
-        <v>111.9179347600227</v>
+        <v>111.9090456676833</v>
       </c>
       <c r="AF22" s="83" t="n">
-        <v>122.1318498512239</v>
+        <v>122.1282134043578</v>
       </c>
       <c r="AG22" s="83" t="n">
-        <v>147.915599822998</v>
+        <v>147.9147998046875</v>
       </c>
       <c r="AH22" s="83" t="n">
-        <v>163.4701000976563</v>
+        <v>163.469700088501</v>
       </c>
       <c r="AI22" s="83" t="n">
-        <v>108.4174999713898</v>
+        <v>108.4172999668121</v>
       </c>
       <c r="AJ22" s="83" t="n">
-        <v>152.484279384695</v>
+        <v>152.4873396300005</v>
       </c>
       <c r="AK22" s="83" t="n">
-        <v>124.4775001525879</v>
+        <v>124.4755001068115</v>
       </c>
       <c r="AL22" s="83" t="n">
-        <v>96.4707209204808</v>
+        <v>96.46366058362254</v>
       </c>
       <c r="AM22" s="87" t="n">
-        <v>0.1840496862094995</v>
+        <v>0.1834284619480264</v>
       </c>
       <c r="AN22" s="36" t="n">
-        <v>44.99894229523508</v>
+        <v>45.00779591028312</v>
       </c>
       <c r="AO22" s="88" t="n">
-        <v>12.95409405606911</v>
+        <v>12.9589486151139</v>
       </c>
       <c r="AP22" s="83" t="n">
         <v>302</v>
@@ -6356,22 +6356,22 @@
         <v>23.97999954223633</v>
       </c>
       <c r="AR22" s="36" t="n">
-        <v>-64.64238451016659</v>
+        <v>-64.65562984643394</v>
       </c>
       <c r="AS22" s="89" t="n">
-        <v>29.78202974632373</v>
+        <v>29.76764196290474</v>
       </c>
       <c r="AT22" s="33" t="n">
-        <v>-0.1322227051519648</v>
+        <v>-0.1325477836934948</v>
       </c>
       <c r="AU22" s="33" t="n">
-        <v>-0.1914894157826267</v>
+        <v>-0.1917922923882829</v>
       </c>
       <c r="AV22" s="33" t="n">
-        <v>-0.593528763542102</v>
+        <v>-0.5936810319610918</v>
       </c>
       <c r="AW22" s="33" t="n">
-        <v>1.540566306937285</v>
+        <v>1.539614583961099</v>
       </c>
       <c r="AX22" s="90" t="inlineStr">
         <is>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
@@ -6502,10 +6502,10 @@
         <v>324.1099853515625</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>34667051</v>
+        <v>37197362</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.8828002339443918</v>
+        <v>0.9441929425958945</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>63.3841943924303</v>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
-          <t>How Apple's John Ternus inherited a 'reckoning' with China</t>
+          <t>What Happens To Qualcomm Stock If The New Revenue Earns Less?</t>
         </is>
       </c>
       <c r="AY24" s="79" t="inlineStr">
@@ -6690,10 +6690,10 @@
         <v>440.5</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>13795477</v>
+        <v>14826068</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>0.7750721329410792</v>
+        <v>0.8305693193246186</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>42.75037085775087</v>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>Could a $10,000 Investment in AMD Double by the End of 2028?</t>
+          <t>AMD (AMD) Stock May Be 24% Undervalued On Saudi AI Expansion</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
-          <t>ASUS Expands AI Infrastructure Ecosystem from Cloud to Edge</t>
+          <t>Why Is AMD (AMD) Becoming More Important In Secure AI Infrastructure?</t>
         </is>
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>Why Is Advanced Micro (AMD) Down 5.2% Since Last Earnings Report?</t>
+          <t>Cathie Wood Sold About $72.8 Million of AMD and Bought About $53 Million of Nvidia. What Changed?</t>
         </is>
       </c>
     </row>
@@ -6878,10 +6878,10 @@
         <v>256</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>25054524</v>
+        <v>26809147</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.7647190022275767</v>
+        <v>0.8160886640327858</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>49.89729833030852</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
-          <t>Amazon Signed a Multibillion-Dollar Deal With a 175-Year-Old Glassmaker. Is Fiber the Next AI Bottleneck?</t>
+          <t>Amazon vs. Microsoft: 1 Key Metric Identifies the Superior Artificial Intelligence (AI) Cloud Stock</t>
         </is>
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
+          <t>Top Analyst Reports for Amazon, AbbVie &amp; Alibaba</t>
+        </is>
+      </c>
+      <c r="AZ26" s="79" t="inlineStr">
+        <is>
           <t>Microsoft, Amazon and 8 More Stocks Set to Win in a $26 Trillion AI Market</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>This Is The Biggest Reason I Keep Accumulating Amazon Stock After Jumping 10% This Year</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>84.38999938964844</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>7962256</v>
+        <v>8200546</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>1.640607019091461</v>
+        <v>1.685568198964707</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>60.64394628659645</v>
@@ -7254,10 +7254,10 @@
         <v>225.4600067138672</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>3454439</v>
+        <v>3988455</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>0.9595712000722669</v>
+        <v>1.099752935378756</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>43.1821885698378</v>
@@ -7442,10 +7442,10 @@
         <v>61.06999969482422</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>7443437</v>
+        <v>7712346</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>0.721810448780269</v>
+        <v>0.7469134330044204</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>46.90028524397902</v>
@@ -7630,10 +7630,10 @@
         <v>342.3305053710938</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>59051560</v>
+        <v>60115767</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>2.625767961256873</v>
+        <v>2.666778961403967</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>37.51016967676528</v>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
-          <t>Broadcom's 2028 AI revenue outlook is what's really 'important'</t>
+          <t>Broadcom Shares Fall 5.6% Even as Revenue Surges 86%</t>
         </is>
       </c>
       <c r="AY30" s="79" t="inlineStr">
         <is>
-          <t>Broadcom Delivered Bullish AI Commentary on Fiscal 2027, 2028 Revenue Outlook, Demand Visibility, UBS Says</t>
+          <t>Why Broadcom (AVGO) Stock Is Nosediving</t>
         </is>
       </c>
       <c r="AZ30" s="79" t="inlineStr">
         <is>
-          <t>Kyndryl Holdings (KD) Expands Broadcom Alliance, Is The Stock Still Undervalued?</t>
+          <t>Broadcom Forecasts Steep Ramp In AI Revenue</t>
         </is>
       </c>
     </row>
@@ -7734,7 +7734,7 @@
         </is>
       </c>
       <c r="C31" s="33" t="n">
-        <v>0.04394065917242362</v>
+        <v>0.04399258781898019</v>
       </c>
       <c r="D31" s="34" t="n">
         <v>8</v>
@@ -7746,7 +7746,7 @@
       </c>
       <c r="F31" s="30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G31" s="30" t="inlineStr">
@@ -7785,7 +7785,7 @@
         </is>
       </c>
       <c r="N31" s="80" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O31" s="30" t="inlineStr">
         <is>
@@ -7803,10 +7803,10 @@
         </is>
       </c>
       <c r="R31" s="81" t="n">
-        <v>100.6149978637695</v>
+        <v>100.620002746582</v>
       </c>
       <c r="S31" s="82" t="n">
-        <v>4.235000610351562</v>
+        <v>4.240005493164062</v>
       </c>
       <c r="T31" s="83" t="n">
         <v>98.98999786376953</v>
@@ -7818,61 +7818,61 @@
         <v>98.72000122070312</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>2396396</v>
+        <v>3216302</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.8890672005926532</v>
+        <v>1.175377094891935</v>
       </c>
       <c r="Y31" s="35" t="n">
-        <v>53.85734515399562</v>
+        <v>53.86463558689864</v>
       </c>
       <c r="Z31" s="35" t="n">
-        <v>38.03173707449242</v>
+        <v>38.0601255236825</v>
       </c>
       <c r="AA31" s="35" t="n">
         <v>16.02560998343604</v>
       </c>
       <c r="AB31" s="86" t="n">
-        <v>1.306426685059975</v>
+        <v>1.306825934970945</v>
       </c>
       <c r="AC31" s="86" t="n">
-        <v>1.7065943601783</v>
+        <v>1.706674210160494</v>
       </c>
       <c r="AD31" s="86" t="n">
-        <v>-0.4001676751183247</v>
+        <v>-0.3998482751895489</v>
       </c>
       <c r="AE31" s="83" t="n">
-        <v>99.76640219555451</v>
+        <v>99.76751439173506</v>
       </c>
       <c r="AF31" s="83" t="n">
-        <v>98.79102937454574</v>
+        <v>98.79148436389234</v>
       </c>
       <c r="AG31" s="83" t="n">
-        <v>95.45110000610352</v>
+        <v>95.45120010375976</v>
       </c>
       <c r="AH31" s="83" t="n">
-        <v>104.0227497863769</v>
+        <v>104.0227998352051</v>
       </c>
       <c r="AI31" s="83" t="n">
-        <v>105.2803247451782</v>
+        <v>105.2803497695923</v>
       </c>
       <c r="AJ31" s="83" t="n">
-        <v>106.7384477434802</v>
+        <v>106.7388310101748</v>
       </c>
       <c r="AK31" s="83" t="n">
-        <v>99.67924995422364</v>
+        <v>99.67950019836425</v>
       </c>
       <c r="AL31" s="83" t="n">
-        <v>92.62005216496712</v>
+        <v>92.62016938655371</v>
       </c>
       <c r="AM31" s="87" t="n">
-        <v>0.5662786294903099</v>
+        <v>0.5666141432729205</v>
       </c>
       <c r="AN31" s="36" t="n">
-        <v>14.16382605707478</v>
+        <v>14.16405739949002</v>
       </c>
       <c r="AO31" s="88" t="n">
-        <v>4.113441840578714</v>
+        <v>4.113237236187875</v>
       </c>
       <c r="AP31" s="83" t="n">
         <v>135.2400054931641</v>
@@ -7881,22 +7881,22 @@
         <v>74.62999725341797</v>
       </c>
       <c r="AR31" s="36" t="n">
-        <v>-25.60263695873978</v>
+        <v>-25.59893621738426</v>
       </c>
       <c r="AS31" s="89" t="n">
-        <v>42.87245846851978</v>
+        <v>42.88071598729903</v>
       </c>
       <c r="AT31" s="33" t="n">
-        <v>-0.05374780277315894</v>
+        <v>-0.05370073343500115</v>
       </c>
       <c r="AU31" s="33" t="n">
-        <v>0.06730668766996084</v>
+        <v>0.06735977861077669</v>
       </c>
       <c r="AV31" s="33" t="n">
-        <v>-0.1175670862476914</v>
+        <v>-0.1175231914664263</v>
       </c>
       <c r="AW31" s="33" t="n">
-        <v>0.09973767857757854</v>
+        <v>0.09979238273026581</v>
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
@@ -8006,10 +8006,10 @@
         <v>79.04000091552734</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>16987141</v>
+        <v>18737553</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>0.6280517896294787</v>
+        <v>0.6905339040657145</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>46.47792492475057</v>
@@ -8110,7 +8110,7 @@
         </is>
       </c>
       <c r="C33" s="33" t="n">
-        <v>0.04823240480617752</v>
+        <v>0.04914669207938038</v>
       </c>
       <c r="D33" s="34" t="n">
         <v>5</v>
@@ -8179,10 +8179,10 @@
         </is>
       </c>
       <c r="R33" s="81" t="n">
-        <v>515.9400024414062</v>
+        <v>516.3900146484375</v>
       </c>
       <c r="S33" s="82" t="n">
-        <v>23.739990234375</v>
+        <v>24.19000244140625</v>
       </c>
       <c r="T33" s="83" t="n">
         <v>486.3099975585938</v>
@@ -8194,61 +8194,61 @@
         <v>478.306396484375</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>18803945</v>
+        <v>20266015</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>2.365965876403778</v>
+        <v>2.52668698948853</v>
       </c>
       <c r="Y33" s="35" t="n">
-        <v>62.47909653795556</v>
+        <v>62.5415624260926</v>
       </c>
       <c r="Z33" s="35" t="n">
-        <v>86.37154480750023</v>
+        <v>86.7848170515018</v>
       </c>
       <c r="AA33" s="35" t="n">
         <v>9.244106021666912</v>
       </c>
       <c r="AB33" s="86" t="n">
-        <v>12.02442571002194</v>
+        <v>12.06032411969966</v>
       </c>
       <c r="AC33" s="86" t="n">
-        <v>9.400957805664699</v>
+        <v>9.408137487600243</v>
       </c>
       <c r="AD33" s="86" t="n">
-        <v>2.623467904357245</v>
+        <v>2.652186632099415</v>
       </c>
       <c r="AE33" s="83" t="n">
-        <v>471.7156197715044</v>
+        <v>471.815622484178</v>
       </c>
       <c r="AF33" s="83" t="n">
-        <v>458.3412919665577</v>
+        <v>458.382202167197</v>
       </c>
       <c r="AG33" s="83" t="n">
-        <v>437.1495989990235</v>
+        <v>437.1585992431641</v>
       </c>
       <c r="AH33" s="83" t="n">
-        <v>367.0556986999512</v>
+        <v>367.0601988220215</v>
       </c>
       <c r="AI33" s="83" t="n">
-        <v>251.4406495666504</v>
+        <v>251.4428996276855</v>
       </c>
       <c r="AJ33" s="83" t="n">
-        <v>510.1528702752637</v>
+        <v>510.2766170482452</v>
       </c>
       <c r="AK33" s="83" t="n">
-        <v>462.5735000610351</v>
+        <v>462.5960006713867</v>
       </c>
       <c r="AL33" s="83" t="n">
-        <v>414.9941298468066</v>
+        <v>414.9153842945283</v>
       </c>
       <c r="AM33" s="87" t="n">
-        <v>1.060815560820642</v>
+        <v>1.064107787028939</v>
       </c>
       <c r="AN33" s="36" t="n">
-        <v>20.57159357721556</v>
+        <v>20.6143660159869</v>
       </c>
       <c r="AO33" s="88" t="n">
-        <v>6.329534985633925</v>
+        <v>6.324019061763271</v>
       </c>
       <c r="AP33" s="83" t="n">
         <v>530.780029296875</v>
@@ -8257,36 +8257,36 @@
         <v>110.2200012207031</v>
       </c>
       <c r="AR33" s="36" t="n">
-        <v>-2.795890206179641</v>
+        <v>-2.711107022526826</v>
       </c>
       <c r="AS33" s="89" t="n">
-        <v>96.4713653545836</v>
+        <v>96.57836844022866</v>
       </c>
       <c r="AT33" s="33" t="n">
-        <v>0.09249140679402212</v>
+        <v>0.09344429756970851</v>
       </c>
       <c r="AU33" s="33" t="n">
-        <v>0.1150637320721599</v>
+        <v>0.1160363108384426</v>
       </c>
       <c r="AV33" s="33" t="n">
-        <v>0.2224618347684779</v>
+        <v>0.2235280881035022</v>
       </c>
       <c r="AW33" s="33" t="n">
-        <v>3.09866550443857</v>
+        <v>3.10224043466458</v>
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
-          <t>Dell Is Now Up 20% in a Month: Take Profits, or Buy More?</t>
+          <t>AI Infrastructure Demand Remains Red-Hot: HPE, AVGO, DELL Deliver</t>
         </is>
       </c>
       <c r="AY33" s="90" t="inlineStr">
         <is>
-          <t>Could Dell Be the Next Magnificent Seven Stock?</t>
+          <t>Bank of America sees 41% upside in surging AI stock</t>
         </is>
       </c>
       <c r="AZ33" s="90" t="inlineStr">
         <is>
-          <t>Dell Earnings Surge: Is It the Next Big AI Stock to Buy in 2026?</t>
+          <t>CLS Stock Jumps 12% As Broadcom AI Call Sparks Switch Rally</t>
         </is>
       </c>
     </row>
@@ -8310,7 +8310,7 @@
       </c>
       <c r="F34" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Same</t>
         </is>
       </c>
       <c r="G34" s="23" t="inlineStr">
@@ -8382,10 +8382,10 @@
         <v>336.3800048828125</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>11640568</v>
+        <v>12835737</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.766810155053832</v>
+        <v>0.8422252133990685</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>46.87941335471027</v>
@@ -8474,7 +8474,7 @@
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>AI wants electricity now. The electric grid needs years to catch up</t>
+          <t>Tesla's 45 Cybercabs Face a $1.3 Trillion Reality Check</t>
         </is>
       </c>
     </row>
@@ -8570,10 +8570,10 @@
         <v>39.02999877929688</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>43775049</v>
+        <v>44874993</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>0.9599586729865889</v>
+        <v>0.9828943146758904</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>52.29302829294181</v>
@@ -8758,10 +8758,10 @@
         <v>87.72499847412109</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>74985819</v>
+        <v>79677381</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.7763475089877393</v>
+        <v>0.8229218722870226</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>45.47576951193744</v>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
+          <t>Intel (INTC) Outperforms Broader Market: What You Need to Know</t>
+        </is>
+      </c>
+      <c r="AY36" s="79" t="inlineStr">
+        <is>
+          <t>Nvidia’s $5 Billion Intel Bet Was Worth $30 Billion by June. Is the Partnership Still Mispriced?</t>
+        </is>
+      </c>
+      <c r="AZ36" s="79" t="inlineStr">
+        <is>
           <t>ASUS Expands AI Infrastructure Ecosystem from Cloud to Edge</t>
-        </is>
-      </c>
-      <c r="AY36" s="79" t="inlineStr">
-        <is>
-          <t>AMD is Quietly Eating Intel’s Lunch</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>Intel (INTC) Could Be 82% Below Fair Value After Kasm AI Partnership</t>
         </is>
       </c>
     </row>
@@ -8946,10 +8946,10 @@
         <v>500.7999877929688</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>22168345</v>
+        <v>24108434</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.9458652368457289</v>
+        <v>1.024403823153436</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>66.11056614319938</v>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
-          <t>Canva’s productivity push is starting to gain traction—and in Southeast Asia, it’s happening on phones</t>
+          <t>S&amp;P 500, Dow End Best Day In A Month On Calmer Yields As Rate Hike Bets Wane — SPCX, VSXY, NVDA, TSLA In Focus</t>
         </is>
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
-          <t>Microsoft's AI Shake-Up Changes What Investors See</t>
+          <t>Microsoft Finally Reveals Azure's $29.4 Billion Core</t>
         </is>
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>Microsoft, Amazon and 8 More Stocks Set to Win in a $26 Trillion AI Market</t>
+          <t>Amazon vs. Microsoft: 1 Key Metric Identifies the Superior Artificial Intelligence (AI) Cloud Stock</t>
         </is>
       </c>
     </row>
@@ -9134,10 +9134,10 @@
         <v>127.5875015258789</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>42445799</v>
+        <v>44800410</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>1.53015511708225</v>
+        <v>1.608212477241803</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>67.78995829466069</v>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Coinbase, Circle, MicroStrategy stocks surge on crypto rebound</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Saylor says Strategy’s Bitcoin-heavy reserve capital surpasses nearly all S&amp;P 500 financial firms</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>Strategy (MSTR) Looks Cheap As Bitcoin Buying Resumes With 4,603 More Coins</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>MicroStrategy Reserve Capital Beats All S&amp;P 500 Financials But Berkshire, MSTR Still Slips</t>
         </is>
       </c>
     </row>
@@ -9322,10 +9322,10 @@
         <v>918.880126953125</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>23723224</v>
+        <v>24105584</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.8579647504841599</v>
+        <v>0.8711906777793956</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>53.48729626756077</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>China Is Grabbing Memory Market Share. This Stock Could Be a Big Loser.</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
           <t>Micron, SanDisk Lag Tech Rally as China Grabs Memory Market Share</t>
         </is>
       </c>
-      <c r="AY39" s="90" t="inlineStr">
+      <c r="AZ39" s="90" t="inlineStr">
         <is>
           <t>Micron's 11% Drop Hasn't Shaken Wall Street's Bull Case</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>The Fed's September Decision Could Hit Micron Harder Than Its Own Earnings</t>
         </is>
       </c>
     </row>
@@ -9438,7 +9438,7 @@
       </c>
       <c r="F40" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Same</t>
         </is>
       </c>
       <c r="G40" s="23" t="inlineStr">
@@ -9510,10 +9510,10 @@
         <v>196.6300048828125</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>10438843</v>
+        <v>10639270</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>0.4692948440856147</v>
+        <v>0.4780899678316393</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>48.37077454734214</v>
@@ -9698,10 +9698,10 @@
         <v>81.62999725341797</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>23071599</v>
+        <v>23970646</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>0.8472874465772849</v>
+        <v>0.878853436103154</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>63.65191183967269</v>
@@ -9802,7 +9802,7 @@
         </is>
       </c>
       <c r="C42" s="26" t="n">
-        <v>-0.007621931717695318</v>
+        <v>-0.007113790014099619</v>
       </c>
       <c r="D42" s="27" t="n">
         <v>23</v>
@@ -9871,10 +9871,10 @@
         </is>
       </c>
       <c r="R42" s="70" t="n">
-        <v>9.765000343322754</v>
+        <v>9.770000457763672</v>
       </c>
       <c r="S42" s="71" t="n">
-        <v>-0.07499980926513672</v>
+        <v>-0.06999969482421875</v>
       </c>
       <c r="T42" s="72" t="n">
         <v>9.760000228881836</v>
@@ -9886,61 +9886,61 @@
         <v>9.539999961853027</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>71481044</v>
+        <v>81929446</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>1.054112456011614</v>
+        <v>1.198955589499316</v>
       </c>
       <c r="Y42" s="28" t="n">
-        <v>42.78947923002418</v>
+        <v>42.85202081378689</v>
       </c>
       <c r="Z42" s="28" t="n">
-        <v>14.15096603000415</v>
+        <v>14.46543860617213</v>
       </c>
       <c r="AA42" s="28" t="n">
         <v>13.09263785060373</v>
       </c>
       <c r="AB42" s="75" t="n">
-        <v>-0.1340415964857264</v>
+        <v>-0.1336427269576745</v>
       </c>
       <c r="AC42" s="75" t="n">
-        <v>-0.1435260559518347</v>
+        <v>-0.1434462820462243</v>
       </c>
       <c r="AD42" s="75" t="n">
-        <v>0.009484459466108264</v>
+        <v>0.009803555088549798</v>
       </c>
       <c r="AE42" s="72" t="n">
-        <v>10.03305777497242</v>
+        <v>10.03416891151484</v>
       </c>
       <c r="AF42" s="72" t="n">
-        <v>10.13315978604743</v>
+        <v>10.1336143419057</v>
       </c>
       <c r="AG42" s="72" t="n">
-        <v>10.60909997940063</v>
+        <v>10.60919998168945</v>
       </c>
       <c r="AH42" s="72" t="n">
-        <v>12.01465000152588</v>
+        <v>12.01470000267029</v>
       </c>
       <c r="AI42" s="72" t="n">
-        <v>9.589174997806548</v>
+        <v>9.589199998378753</v>
       </c>
       <c r="AJ42" s="72" t="n">
-        <v>10.99456497934714</v>
+        <v>10.99440967320634</v>
       </c>
       <c r="AK42" s="72" t="n">
-        <v>10.12125005722046</v>
+        <v>10.12150006294251</v>
       </c>
       <c r="AL42" s="72" t="n">
-        <v>9.247935135093774</v>
+        <v>9.248590452678668</v>
       </c>
       <c r="AM42" s="76" t="n">
-        <v>0.2960359402595739</v>
+        <v>0.2986620830806338</v>
       </c>
       <c r="AN42" s="29" t="n">
-        <v>17.25705653332151</v>
+        <v>17.24862134733943</v>
       </c>
       <c r="AO42" s="77" t="n">
-        <v>4.707074405059595</v>
+        <v>4.704665407147163</v>
       </c>
       <c r="AP42" s="72" t="n">
         <v>17.45000076293945</v>
@@ -9949,22 +9949,22 @@
         <v>4.480000019073486</v>
       </c>
       <c r="AR42" s="29" t="n">
-        <v>-44.04011509236268</v>
+        <v>-44.01146114266464</v>
       </c>
       <c r="AS42" s="78" t="n">
-        <v>40.74787988542526</v>
+        <v>40.7864312667217</v>
       </c>
       <c r="AT42" s="26" t="n">
-        <v>-0.07790366358621159</v>
+        <v>-0.0774315092548733</v>
       </c>
       <c r="AU42" s="26" t="n">
-        <v>0.01931110867327979</v>
+        <v>0.0198330412913108</v>
       </c>
       <c r="AV42" s="26" t="n">
-        <v>-0.4124548826573244</v>
+        <v>-0.4121540334281767</v>
       </c>
       <c r="AW42" s="26" t="n">
-        <v>0.5092736723309077</v>
+        <v>0.5100464875709481</v>
       </c>
       <c r="AX42" s="79" t="inlineStr">
         <is>
@@ -10074,10 +10074,10 @@
         <v>224.75</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>127001728</v>
+        <v>133890362</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.9996046625221428</v>
+        <v>1.050974552707904</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>59.20979550440254</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Stock Market Today: Dow Pops On Fed Official's Dovish Rates View; Nvidia Hovers In Buy Zone (Live Coverage)</t>
+          <t>Nvidia’s $12.93 Billion Hugging Face Deal Expands Jensen Huang's AI Platform Beyond Chips</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Sector Update: Tech Stocks Rise Late Afternoon</t>
+          <t>Nvidia’s $5 Billion Intel Bet Was Worth $30 Billion by June. Is the Partnership Still Mispriced?</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Better Small Modular Reactor Stock to Buy After the Sell-Off: Oklo vs. NuScale Power</t>
+          <t>Rosenblatt Doubles Down on Nvidia After Massive Deal</t>
         </is>
       </c>
     </row>
@@ -10262,10 +10262,10 @@
         <v>171.9375</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>36980824</v>
+        <v>38010148</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>1.03936596019443</v>
+        <v>1.066752623224575</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>60.53699266646308</v>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
-          <t>Sector Update: Tech Stocks Rise Late Afternoon</t>
+          <t>Palantir Technologies, Workiva, Elastic, RingCentral, and 8x8 Shares Skyrocket, What You Need To Know</t>
         </is>
       </c>
       <c r="AY44" s="79" t="inlineStr">
         <is>
-          <t>Michael Burry doubles down on his surprising AI bet</t>
+          <t>Palantir Stock Jumps on Expanded PwC AI Deal</t>
         </is>
       </c>
       <c r="AZ44" s="79" t="inlineStr">
         <is>
-          <t>The $1 Trillion Question Hanging Over Palantir Stock</t>
+          <t>Palantir Stock Defies Red Flag and Skyrockets 8% – Here’s Why</t>
         </is>
       </c>
     </row>
@@ -10450,10 +10450,10 @@
         <v>164.9049987792969</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>6516183</v>
+        <v>6987656</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.7135553191303785</v>
+        <v>0.7632138336630525</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>52.87989293804576</v>
@@ -10638,10 +10638,10 @@
         <v>62.36000061035156</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>18270422</v>
+        <v>18818827</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>1.040859834961954</v>
+        <v>1.070430141537631</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>36.14248318653912</v>
@@ -10826,10 +10826,10 @@
         <v>1511</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>8375587</v>
+        <v>8670816</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.6373043357432135</v>
+        <v>0.6590282924394725</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>52.58214372024118</v>
@@ -11014,10 +11014,10 @@
         <v>365.9100036621094</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>61561072</v>
+        <v>62838720</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>1.682983365551952</v>
+        <v>1.71491725396638</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>60.53898330136157</v>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
-          <t>Tesla Cybercab: Here's What To Expect From Thursday's Event</t>
+          <t>Dow Jones Futures: Stocks Jump On Fed's Waller; Tesla Cybercab Event Private, Jobs Report Looms</t>
         </is>
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>Tesla Is Now Up 18% in a Month: Take Profits, or Buy More?</t>
+          <t>Tesla Launching Cybercab Robotaxis. Here's What To Look For.</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Market Indexes Rally as Tesla and Goldman Sachs Take the Wheel</t>
+          <t>Tesla's 45 Cybercabs Face a $1.3 Trillion Reality Check</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 3 Sep 2026, 08:01 PM · Yahoo Finance data</t>
+          <t>Built 3 Sep 2026, 10:37 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 3 Sep 2026, 08:01 PM · Yahoo Finance data</t>
+          <t>Built 3 Sep 2026, 10:37 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 3 Sep 2026, 08:01 PM · Yahoo Finance data</t>
+          <t>Built 3 Sep 2026, 10:37 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 3 Sep 2026, 08:01 PM · Yahoo Finance data</t>
+          <t>Built 3 Sep 2026, 10:37 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -43355,22 +43355,22 @@
         </is>
       </c>
       <c r="D6" s="26" t="n">
-        <v>-0.006913919215374764</v>
+        <v>-0.007373206433021195</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>0.037885718310118</v>
+        <v>0.03740571194106179</v>
       </c>
       <c r="F6" s="26" t="n">
-        <v>0.1280736484832767</v>
+        <v>0.1275519315673546</v>
       </c>
       <c r="G6" s="26" t="n">
-        <v>0.100423869680851</v>
+        <v>0.09991494036735382</v>
       </c>
       <c r="H6" s="26" t="n">
-        <v>0.1446512547402579</v>
+        <v>0.1441218709334182</v>
       </c>
       <c r="I6" s="26" t="n">
-        <v>0.4459830835962213</v>
+        <v>0.4453143383987213</v>
       </c>
       <c r="J6" s="27" t="n">
         <v>7</v>
@@ -43393,22 +43393,22 @@
         </is>
       </c>
       <c r="D7" s="33" t="n">
-        <v>0.001965864954553087</v>
+        <v>0.00179241147189213</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>0.009966146618659355</v>
+        <v>0.009791308181914093</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>0.05561640728770745</v>
+        <v>0.05543366618982959</v>
       </c>
       <c r="G7" s="33" t="n">
-        <v>0.1394660126230156</v>
+        <v>0.1392687560545276</v>
       </c>
       <c r="H7" s="33" t="n">
-        <v>0.1259176737242489</v>
+        <v>0.1257227625515955</v>
       </c>
       <c r="I7" s="33" t="n">
-        <v>0.1194443790042614</v>
+        <v>0.1192505884441486</v>
       </c>
       <c r="J7" s="34" t="n">
         <v>7</v>
@@ -43431,22 +43431,22 @@
         </is>
       </c>
       <c r="D8" s="26" t="n">
-        <v>0.008717340089801739</v>
+        <v>0.008539397794954384</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>0.01786193158923965</v>
+        <v>0.01768237614714829</v>
       </c>
       <c r="F8" s="26" t="n">
-        <v>0.02281950677930222</v>
+        <v>0.02263907679855559</v>
       </c>
       <c r="G8" s="26" t="n">
-        <v>0.002563883953341728</v>
+        <v>0.00238702715594985</v>
       </c>
       <c r="H8" s="26" t="n">
-        <v>-0.0425531983420947</v>
+        <v>-0.0427220962823901</v>
       </c>
       <c r="I8" s="26" t="n">
-        <v>-0.03669724473350133</v>
+        <v>-0.03686717569046283</v>
       </c>
       <c r="J8" s="27" t="n">
         <v>7</v>
@@ -43469,22 +43469,22 @@
         </is>
       </c>
       <c r="D9" s="33" t="n">
-        <v>0.01543529989600545</v>
+        <v>0.01560876739959438</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>0.01157564195890104</v>
+        <v>0.01174845011449688</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>0.009482745466561138</v>
+        <v>0.009655196091224338</v>
       </c>
       <c r="G9" s="33" t="n">
-        <v>0.1218624406534616</v>
+        <v>0.1220540891779616</v>
       </c>
       <c r="H9" s="33" t="n">
-        <v>0.1428850236234978</v>
+        <v>0.1430802634501587</v>
       </c>
       <c r="I9" s="33" t="n">
-        <v>0.06901586174372687</v>
+        <v>0.06919848245117377</v>
       </c>
       <c r="J9" s="34" t="n">
         <v>8</v>
@@ -43507,22 +43507,22 @@
         </is>
       </c>
       <c r="D10" s="26" t="n">
-        <v>0.01296290601799632</v>
+        <v>0.01290846970806347</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>-0.01394414333440253</v>
+        <v>-0.013997133667914</v>
       </c>
       <c r="F10" s="26" t="n">
-        <v>0.000376483589107357</v>
+        <v>0.0003227236695815261</v>
       </c>
       <c r="G10" s="26" t="n">
-        <v>-0.03722111357643598</v>
+        <v>-0.03727285301284267</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>0.3267228238318394</v>
+        <v>0.3266515261619996</v>
       </c>
       <c r="I10" s="26" t="n">
-        <v>0.291796861503359</v>
+        <v>0.2917274407438175</v>
       </c>
       <c r="J10" s="27" t="n">
         <v>8</v>
@@ -43536,34 +43536,34 @@
     <row r="11">
       <c r="B11" s="31" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="C11" s="32" t="inlineStr">
         <is>
-          <t>State Street Consumer Staples Select Sector SPDR ETF</t>
+          <t>State Street Materials Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D11" s="33" t="n">
-        <v>-0.003273690907203086</v>
+        <v>-0.006232329108589174</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>0.001998097852452752</v>
+        <v>-0.0114597147397596</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>-0.0009375580609161105</v>
+        <v>-0.0003799479102503112</v>
       </c>
       <c r="G11" s="33" t="n">
-        <v>0.03912724340139673</v>
+        <v>0.01937233670460836</v>
       </c>
       <c r="H11" s="33" t="n">
-        <v>-0.001873359738308489</v>
+        <v>0.03521536565706906</v>
       </c>
       <c r="I11" s="33" t="n">
-        <v>0.09745107704794687</v>
+        <v>0.1603087255209565</v>
       </c>
       <c r="J11" s="34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K11" s="102" t="inlineStr">
         <is>
@@ -43574,72 +43574,72 @@
     <row r="12">
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>State Street Utilities Select Sector SPDR ETF</t>
+          <t>State Street Consumer Staples Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D12" s="26" t="n">
-        <v>0.007968131407967594</v>
+        <v>-0.003156747888692357</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>-0.003937053785110778</v>
+        <v>0.00211565939470959</v>
       </c>
       <c r="F12" s="26" t="n">
-        <v>-0.01488780412621638</v>
+        <v>-0.0008203409506870596</v>
       </c>
       <c r="G12" s="26" t="n">
-        <v>-0.02116523291401473</v>
+        <v>0.03924916119904243</v>
       </c>
       <c r="H12" s="26" t="n">
-        <v>-0.08294249632804895</v>
+        <v>-0.001756252422986937</v>
       </c>
       <c r="I12" s="26" t="n">
-        <v>0.00749589377180282</v>
+        <v>0.09757983781250879</v>
       </c>
       <c r="J12" s="27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" s="101" t="inlineStr">
         <is>
-          <t>Long-term down, short-term mixed</t>
+          <t>Long-term up, short-term mixed</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="31" t="inlineStr">
         <is>
-          <t>XLY</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="C13" s="32" t="inlineStr">
         <is>
-          <t>State Street Consumer Discretionary Select Sector SPDR ETF</t>
+          <t>State Street Utilities Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D13" s="33" t="n">
-        <v>0.01392998838254322</v>
+        <v>0.008436855537846455</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>0.005005193690040155</v>
+        <v>-0.003473865790152075</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>-0.01837491837821092</v>
+        <v>-0.0144297084360292</v>
       </c>
       <c r="G13" s="33" t="n">
-        <v>-0.00682247174811057</v>
+        <v>-0.02071005634622314</v>
       </c>
       <c r="H13" s="33" t="n">
-        <v>-0.000772234791321158</v>
+        <v>-0.08251604734909457</v>
       </c>
       <c r="I13" s="33" t="n">
-        <v>-0.02470483617088104</v>
+        <v>0.007964398302303222</v>
       </c>
       <c r="J13" s="34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K13" s="102" t="inlineStr">
         <is>
@@ -43650,69 +43650,69 @@
     <row r="14">
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>State Street Real Estate Select Sector SPDR ETF</t>
+          <t>State Street Consumer Discretionary Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D14" s="26" t="n">
-        <v>0.01189116083254094</v>
+        <v>0.01392998838254322</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>-0.009180471312425831</v>
+        <v>0.005005193690040155</v>
       </c>
       <c r="F14" s="26" t="n">
-        <v>-0.02101771563947363</v>
+        <v>-0.01837491837821092</v>
       </c>
       <c r="G14" s="26" t="n">
-        <v>-0.003378412628915695</v>
+        <v>-0.00682247174811057</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>0.0209967661330932</v>
+        <v>-0.000772234791321158</v>
       </c>
       <c r="I14" s="26" t="n">
-        <v>0.09665431656410628</v>
+        <v>-0.02470483617088104</v>
       </c>
       <c r="J14" s="27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K14" s="101" t="inlineStr">
         <is>
-          <t>Long-term up, short-term mixed</t>
+          <t>Long-term down, short-term mixed</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="31" t="inlineStr">
         <is>
-          <t>XLI</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="C15" s="32" t="inlineStr">
         <is>
-          <t>State Street Industrial Select Sector SPDR ETF</t>
+          <t>State Street Real Estate Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D15" s="33" t="n">
-        <v>0.01018633244166245</v>
+        <v>0.01189116083254094</v>
       </c>
       <c r="E15" s="33" t="n">
-        <v>-0.02382555756663962</v>
+        <v>-0.009180471312425831</v>
       </c>
       <c r="F15" s="33" t="n">
-        <v>-0.06337543563493342</v>
+        <v>-0.02101771563947363</v>
       </c>
       <c r="G15" s="33" t="n">
-        <v>-0.009196243995793107</v>
+        <v>-0.003378412628915695</v>
       </c>
       <c r="H15" s="33" t="n">
-        <v>0.01441355203259564</v>
+        <v>0.0209967661330932</v>
       </c>
       <c r="I15" s="33" t="n">
-        <v>0.1251933907957785</v>
+        <v>0.09665431656410628</v>
       </c>
       <c r="J15" s="34" t="n">
         <v>2</v>
@@ -43726,34 +43726,34 @@
     <row r="16">
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>XLI</t>
         </is>
       </c>
       <c r="C16" s="25" t="inlineStr">
         <is>
-          <t>State Street Materials Select Sector SPDR ETF</t>
+          <t>State Street Industrial Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D16" s="26" t="n">
-        <v>-0.005854605643518473</v>
+        <v>0.0103021113084425</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>-0.01108397816384998</v>
+        <v>-0.02371367685008763</v>
       </c>
       <c r="F16" s="26" t="n">
-        <v>0</v>
+        <v>-0.06326808778515758</v>
       </c>
       <c r="G16" s="26" t="n">
-        <v>0.01975979230665259</v>
+        <v>-0.009082686593175682</v>
       </c>
       <c r="H16" s="26" t="n">
-        <v>0.03560884307283119</v>
+        <v>0.01452981538691844</v>
       </c>
       <c r="I16" s="26" t="n">
-        <v>0.1607497499627784</v>
+        <v>0.1253223507821801</v>
       </c>
       <c r="J16" s="27" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K16" s="101" t="inlineStr">
         <is>
@@ -44168,7 +44168,7 @@
         </is>
       </c>
       <c r="E14" s="26" t="n">
-        <v>0.04823240480617752</v>
+        <v>0.04914669207938038</v>
       </c>
       <c r="F14" s="27" t="n">
         <v>8</v>
@@ -44196,7 +44196,7 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
-        <v>0.04823240480617752</v>
+        <v>0.04914669207938038</v>
       </c>
       <c r="F15" s="34" t="n">
         <v>8</v>
@@ -44220,11 +44220,11 @@
       </c>
       <c r="D16" s="104" t="inlineStr">
         <is>
-          <t>Volume 2.4x its 20-day average</t>
+          <t>Volume 2.5x its 20-day average</t>
         </is>
       </c>
       <c r="E16" s="26" t="n">
-        <v>0.04823240480617752</v>
+        <v>0.04914669207938038</v>
       </c>
       <c r="F16" s="27" t="n">
         <v>8</v>
@@ -44308,7 +44308,7 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
-        <v>0.01543529989600545</v>
+        <v>0.01560876739959438</v>
       </c>
       <c r="F19" s="34" t="n">
         <v>8</v>
@@ -44336,7 +44336,7 @@
         </is>
       </c>
       <c r="E20" s="26" t="n">
-        <v>0.01296290601799632</v>
+        <v>0.01290846970806347</v>
       </c>
       <c r="F20" s="27" t="n">
         <v>8</v>
@@ -44364,7 +44364,7 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
-        <v>0.01296290601799632</v>
+        <v>0.01290846970806347</v>
       </c>
       <c r="F21" s="34" t="n">
         <v>8</v>
@@ -44392,7 +44392,7 @@
         </is>
       </c>
       <c r="E22" s="26" t="n">
-        <v>0.01044232781374466</v>
+        <v>0.01046841189654324</v>
       </c>
       <c r="F22" s="27" t="n">
         <v>8</v>
@@ -44518,21 +44518,21 @@
     <row r="27">
       <c r="B27" s="31" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="C27" s="102" t="inlineStr">
         <is>
-          <t>Invesco QQQ Trust</t>
-        </is>
-      </c>
-      <c r="D27" s="107" t="inlineStr">
-        <is>
-          <t>8 EMA crossed above 21</t>
+          <t>Cameco Corporation</t>
+        </is>
+      </c>
+      <c r="D27" s="105" t="inlineStr">
+        <is>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E27" s="33" t="n">
-        <v>0.01188595227547085</v>
+        <v>0.04399258781898019</v>
       </c>
       <c r="F27" s="34" t="n">
         <v>7</v>
@@ -44546,21 +44546,21 @@
     <row r="28">
       <c r="B28" s="24" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="C28" s="101" t="inlineStr">
         <is>
-          <t>Invesco QQQ Trust</t>
+          <t>Cameco Corporation</t>
         </is>
       </c>
       <c r="D28" s="104" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Gapped up 2.7% at the open</t>
         </is>
       </c>
       <c r="E28" s="26" t="n">
-        <v>0.01188595227547085</v>
+        <v>0.04399258781898019</v>
       </c>
       <c r="F28" s="27" t="n">
         <v>7</v>
@@ -44574,21 +44574,21 @@
     <row r="29">
       <c r="B29" s="31" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="C29" s="102" t="inlineStr">
         <is>
-          <t>Invesco QQQ Trust</t>
+          <t>Cameco Corporation</t>
         </is>
       </c>
       <c r="D29" s="105" t="inlineStr">
         <is>
-          <t>Reclaimed the 50 DMA</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E29" s="33" t="n">
-        <v>0.01188595227547085</v>
+        <v>0.04399258781898019</v>
       </c>
       <c r="F29" s="34" t="n">
         <v>7</v>
@@ -44610,9 +44610,9 @@
           <t>Invesco QQQ Trust</t>
         </is>
       </c>
-      <c r="D30" s="104" t="inlineStr">
-        <is>
-          <t>Bands squeezing — a big move often follows</t>
+      <c r="D30" s="106" t="inlineStr">
+        <is>
+          <t>8 EMA crossed above 21</t>
         </is>
       </c>
       <c r="E30" s="26" t="n">
@@ -44630,21 +44630,21 @@
     <row r="31">
       <c r="B31" s="31" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="C31" s="102" t="inlineStr">
         <is>
-          <t>State Street Communication Services Select Sector SPDR ETF</t>
-        </is>
-      </c>
-      <c r="D31" s="107" t="inlineStr">
-        <is>
-          <t>MACD crossed up</t>
+          <t>Invesco QQQ Trust</t>
+        </is>
+      </c>
+      <c r="D31" s="105" t="inlineStr">
+        <is>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E31" s="33" t="n">
-        <v>0.008717340089801739</v>
+        <v>0.01188595227547085</v>
       </c>
       <c r="F31" s="34" t="n">
         <v>7</v>
@@ -44658,24 +44658,24 @@
     <row r="32">
       <c r="B32" s="24" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="C32" s="101" t="inlineStr">
         <is>
-          <t>Cameco Corporation</t>
+          <t>Invesco QQQ Trust</t>
         </is>
       </c>
       <c r="D32" s="104" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Reclaimed the 50 DMA</t>
         </is>
       </c>
       <c r="E32" s="26" t="n">
-        <v>0.04394065917242362</v>
+        <v>0.01188595227547085</v>
       </c>
       <c r="F32" s="27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G32" s="23" t="inlineStr">
         <is>
@@ -44686,24 +44686,24 @@
     <row r="33">
       <c r="B33" s="31" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="C33" s="102" t="inlineStr">
         <is>
-          <t>Cameco Corporation</t>
+          <t>Invesco QQQ Trust</t>
         </is>
       </c>
       <c r="D33" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 2.7% at the open</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E33" s="33" t="n">
-        <v>0.04394065917242362</v>
+        <v>0.01188595227547085</v>
       </c>
       <c r="F33" s="34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G33" s="30" t="inlineStr">
         <is>
@@ -44714,24 +44714,24 @@
     <row r="34">
       <c r="B34" s="24" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="C34" s="101" t="inlineStr">
         <is>
-          <t>Cameco Corporation</t>
-        </is>
-      </c>
-      <c r="D34" s="104" t="inlineStr">
-        <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>State Street Communication Services Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D34" s="106" t="inlineStr">
+        <is>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E34" s="26" t="n">
-        <v>0.04394065917242362</v>
+        <v>0.008539397794954384</v>
       </c>
       <c r="F34" s="27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G34" s="23" t="inlineStr">
         <is>
@@ -44798,24 +44798,24 @@
     <row r="37">
       <c r="B37" s="31" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="C37" s="102" t="inlineStr">
         <is>
-          <t>State Street Materials Select Sector SPDR ETF</t>
+          <t>Arm Holdings plc</t>
         </is>
       </c>
       <c r="D37" s="105" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped down 1.6% at the open</t>
         </is>
       </c>
       <c r="E37" s="33" t="n">
-        <v>-0.005854605643518473</v>
+        <v>0.03291320662288366</v>
       </c>
       <c r="F37" s="34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G37" s="30" t="inlineStr">
         <is>
@@ -44836,7 +44836,7 @@
       </c>
       <c r="D38" s="104" t="inlineStr">
         <is>
-          <t>Gapped down 1.6% at the open</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E38" s="26" t="n">
@@ -44854,21 +44854,21 @@
     <row r="39">
       <c r="B39" s="31" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="C39" s="102" t="inlineStr">
         <is>
-          <t>Arm Holdings plc</t>
+          <t>State Street Consumer Discretionary Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D39" s="105" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Reclaimed the 50 DMA</t>
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>0.03291320662288366</v>
+        <v>0.01392998838254322</v>
       </c>
       <c r="F39" s="34" t="n">
         <v>4</v>
@@ -44882,21 +44882,21 @@
     <row r="40">
       <c r="B40" s="24" t="inlineStr">
         <is>
-          <t>XLY</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="C40" s="101" t="inlineStr">
         <is>
-          <t>State Street Consumer Discretionary Select Sector SPDR ETF</t>
+          <t>State Street Materials Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D40" s="104" t="inlineStr">
         <is>
-          <t>Reclaimed the 50 DMA</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E40" s="26" t="n">
-        <v>0.01392998838254322</v>
+        <v>-0.006232329108589174</v>
       </c>
       <c r="F40" s="27" t="n">
         <v>4</v>
@@ -44980,7 +44980,7 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>-0.003273690907203086</v>
+        <v>-0.003156747888692357</v>
       </c>
       <c r="F43" s="34" t="n">
         <v>3</v>
@@ -45008,7 +45008,7 @@
         </is>
       </c>
       <c r="E44" s="26" t="n">
-        <v>-0.003273690907203086</v>
+        <v>-0.003156747888692357</v>
       </c>
       <c r="F44" s="27" t="n">
         <v>3</v>
@@ -45036,7 +45036,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>-0.003273690907203086</v>
+        <v>-0.003156747888692357</v>
       </c>
       <c r="F45" s="34" t="n">
         <v>3</v>
@@ -45092,7 +45092,7 @@
         </is>
       </c>
       <c r="E47" s="33" t="n">
-        <v>0.004043256336109913</v>
+        <v>0.003667131125943079</v>
       </c>
       <c r="F47" s="34" t="n">
         <v>2</v>
@@ -45116,7 +45116,7 @@
       </c>
       <c r="D48" s="104" t="inlineStr">
         <is>
-          <t>Volume 2.6x its 20-day average</t>
+          <t>Volume 2.7x its 20-day average</t>
         </is>
       </c>
       <c r="E48" s="26" t="n">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-03 23:15 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'08-31'!$5:$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'08-28'!$A$6:$AZ$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'08-28'!$5:$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 3 Sep 2026, 10:37 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 3 Sep 2026, 11:15 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1376,21 +1376,21 @@
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F8" s="8" t="n"/>
       <c r="G8" s="8" t="n"/>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>78%</t>
+          <t>79%</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="15" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="L8" s="10" t="n"/>
@@ -1404,7 +1404,7 @@
       <c r="P8" s="10" t="n"/>
       <c r="Q8" s="16" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>42</t>
         </is>
       </c>
       <c r="R8" s="12" t="n"/>
@@ -1413,14 +1413,14 @@
     <row r="9" ht="15" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>of 40 names</t>
+          <t>of 39 names</t>
         </is>
       </c>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>of 40 names</t>
+          <t>of 39 names</t>
         </is>
       </c>
       <c r="F9" s="8" t="n"/>
@@ -1441,7 +1441,7 @@
       <c r="M9" s="10" t="n"/>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>of 40 names</t>
+          <t>of 39 names</t>
         </is>
       </c>
       <c r="O9" s="10" t="n"/>
@@ -1957,11 +1957,11 @@
       </c>
       <c r="H29" s="24" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>ASTS</t>
         </is>
       </c>
       <c r="I29" s="26" t="n">
-        <v>-0.02744795458096083</v>
+        <v>-0.004326930307072097</v>
       </c>
       <c r="J29" s="27" t="n">
         <v>1</v>
@@ -1972,7 +1972,7 @@
         </is>
       </c>
       <c r="L29" s="28" t="n">
-        <v>37.51016967676528</v>
+        <v>46.90028524397902</v>
       </c>
     </row>
     <row r="30">
@@ -1997,22 +1997,22 @@
       </c>
       <c r="H30" s="31" t="inlineStr">
         <is>
-          <t>ASTS</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="I30" s="33" t="n">
-        <v>-0.004326930307072097</v>
+        <v>-0.001969093557282919</v>
       </c>
       <c r="J30" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K30" s="30" t="inlineStr">
         <is>
-          <t>Very Weak</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="L30" s="35" t="n">
-        <v>46.90028524397902</v>
+        <v>42.75037085775087</v>
       </c>
     </row>
     <row r="31">
@@ -2037,11 +2037,11 @@
       </c>
       <c r="H31" s="24" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>SOXL</t>
         </is>
       </c>
       <c r="I31" s="26" t="n">
-        <v>-0.001969093557282919</v>
+        <v>0.003667131125943079</v>
       </c>
       <c r="J31" s="27" t="n">
         <v>2</v>
@@ -2052,7 +2052,7 @@
         </is>
       </c>
       <c r="L31" s="28" t="n">
-        <v>42.75037085775087</v>
+        <v>39.31394302464612</v>
       </c>
     </row>
     <row r="32">
@@ -2077,11 +2077,11 @@
       </c>
       <c r="H32" s="31" t="inlineStr">
         <is>
-          <t>SOXL</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="I32" s="33" t="n">
-        <v>0.003667131125943079</v>
+        <v>0.004013443884859136</v>
       </c>
       <c r="J32" s="34" t="n">
         <v>2</v>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="L32" s="35" t="n">
-        <v>39.31394302464612</v>
+        <v>46.67148684589938</v>
       </c>
     </row>
     <row r="33">
@@ -2117,11 +2117,11 @@
       </c>
       <c r="H33" s="24" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="I33" s="26" t="n">
-        <v>0.004013443884859136</v>
+        <v>0.008436855537846455</v>
       </c>
       <c r="J33" s="27" t="n">
         <v>2</v>
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="L33" s="28" t="n">
-        <v>46.67148684589938</v>
+        <v>43.26204319173591</v>
       </c>
     </row>
     <row r="34">
@@ -2157,11 +2157,11 @@
       </c>
       <c r="H34" s="31" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>XLI</t>
         </is>
       </c>
       <c r="I34" s="33" t="n">
-        <v>0.008436855537846455</v>
+        <v>0.0103021113084425</v>
       </c>
       <c r="J34" s="34" t="n">
         <v>2</v>
@@ -2172,7 +2172,7 @@
         </is>
       </c>
       <c r="L34" s="35" t="n">
-        <v>43.26204319173591</v>
+        <v>36.50808171075061</v>
       </c>
     </row>
     <row r="35">
@@ -2197,11 +2197,11 @@
       </c>
       <c r="H35" s="24" t="inlineStr">
         <is>
-          <t>XLI</t>
+          <t>RKLB</t>
         </is>
       </c>
       <c r="I35" s="26" t="n">
-        <v>0.0103021113084425</v>
+        <v>0.0112520272003036</v>
       </c>
       <c r="J35" s="27" t="n">
         <v>2</v>
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="L35" s="28" t="n">
-        <v>36.50808171075061</v>
+        <v>36.14248318653912</v>
       </c>
     </row>
     <row r="36">
@@ -2237,11 +2237,11 @@
       </c>
       <c r="H36" s="31" t="inlineStr">
         <is>
-          <t>RKLB</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="I36" s="33" t="n">
-        <v>0.0112520272003036</v>
+        <v>0.01189116083254094</v>
       </c>
       <c r="J36" s="34" t="n">
         <v>2</v>
@@ -2252,7 +2252,7 @@
         </is>
       </c>
       <c r="L36" s="35" t="n">
-        <v>36.14248318653912</v>
+        <v>43.70604864099334</v>
       </c>
     </row>
     <row r="37">
@@ -2277,11 +2277,11 @@
       </c>
       <c r="H37" s="24" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="I37" s="26" t="n">
-        <v>0.01189116083254094</v>
+        <v>0.0320447286112655</v>
       </c>
       <c r="J37" s="27" t="n">
         <v>2</v>
@@ -2292,7 +2292,7 @@
         </is>
       </c>
       <c r="L37" s="28" t="n">
-        <v>43.70604864099334</v>
+        <v>48.37077454734214</v>
       </c>
     </row>
     <row r="38">
@@ -2317,11 +2317,11 @@
       </c>
       <c r="H38" s="31" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="I38" s="33" t="n">
-        <v>0.0320447286112655</v>
+        <v>0.04485354305856615</v>
       </c>
       <c r="J38" s="34" t="n">
         <v>2</v>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="L38" s="35" t="n">
-        <v>48.37077454734214</v>
+        <v>46.47792492475057</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
@@ -2421,22 +2421,22 @@
       </c>
       <c r="H43" s="24" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I43" s="26" t="n">
-        <v>-0.02744795458096083</v>
+        <v>-0.008178391002234719</v>
       </c>
       <c r="J43" s="27" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K43" s="23" t="inlineStr">
         <is>
-          <t>Very Weak</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="L43" s="28" t="n">
-        <v>37.51016967676528</v>
+        <v>52.87989293804576</v>
       </c>
     </row>
     <row r="44">
@@ -2461,14 +2461,14 @@
       </c>
       <c r="H44" s="31" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="I44" s="33" t="n">
-        <v>-0.008178391002234719</v>
+        <v>-0.007373206433021195</v>
       </c>
       <c r="J44" s="34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K44" s="30" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="L44" s="35" t="n">
-        <v>52.87989293804576</v>
+        <v>67.62030622942083</v>
       </c>
     </row>
     <row r="45">
@@ -2501,22 +2501,22 @@
       </c>
       <c r="H45" s="24" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="I45" s="26" t="n">
-        <v>-0.007373206433021195</v>
+        <v>-0.007113790014099619</v>
       </c>
       <c r="J45" s="27" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K45" s="23" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="L45" s="28" t="n">
-        <v>67.62030622942083</v>
+        <v>42.85202081378689</v>
       </c>
     </row>
     <row r="46">
@@ -2541,22 +2541,22 @@
       </c>
       <c r="H46" s="31" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="I46" s="33" t="n">
-        <v>-0.007113790014099619</v>
+        <v>-0.006232329108589174</v>
       </c>
       <c r="J46" s="34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K46" s="30" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="L46" s="35" t="n">
-        <v>42.85202081378689</v>
+        <v>51.01920682289664</v>
       </c>
     </row>
     <row r="47">
@@ -2581,22 +2581,22 @@
       </c>
       <c r="H47" s="24" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>ASTS</t>
         </is>
       </c>
       <c r="I47" s="26" t="n">
-        <v>-0.006232329108589174</v>
+        <v>-0.004326930307072097</v>
       </c>
       <c r="J47" s="27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K47" s="23" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Very Weak</t>
         </is>
       </c>
       <c r="L47" s="28" t="n">
-        <v>51.01920682289664</v>
+        <v>46.90028524397902</v>
       </c>
     </row>
     <row r="48">
@@ -2621,22 +2621,22 @@
       </c>
       <c r="H48" s="31" t="inlineStr">
         <is>
-          <t>ASTS</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="I48" s="33" t="n">
-        <v>-0.004326930307072097</v>
+        <v>-0.003156747888692357</v>
       </c>
       <c r="J48" s="34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K48" s="30" t="inlineStr">
         <is>
-          <t>Very Weak</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="L48" s="35" t="n">
-        <v>46.90028524397902</v>
+        <v>48.95291184688658</v>
       </c>
     </row>
     <row r="49">
@@ -2661,14 +2661,14 @@
       </c>
       <c r="H49" s="24" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="I49" s="26" t="n">
-        <v>-0.003156747888692357</v>
+        <v>-0.001969093557282919</v>
       </c>
       <c r="J49" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K49" s="23" t="inlineStr">
         <is>
@@ -2676,7 +2676,7 @@
         </is>
       </c>
       <c r="L49" s="28" t="n">
-        <v>48.95291184688658</v>
+        <v>42.75037085775087</v>
       </c>
     </row>
     <row r="50">
@@ -2701,22 +2701,22 @@
       </c>
       <c r="H50" s="31" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="I50" s="33" t="n">
-        <v>-0.001969093557282919</v>
+        <v>-0.0007253134963550734</v>
       </c>
       <c r="J50" s="34" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="K50" s="30" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="L50" s="35" t="n">
-        <v>42.75037085775087</v>
+        <v>63.65191183967269</v>
       </c>
     </row>
     <row r="51">
@@ -2741,11 +2741,11 @@
       </c>
       <c r="H51" s="24" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="I51" s="26" t="n">
-        <v>-0.0007253134963550734</v>
+        <v>0.001023539201315593</v>
       </c>
       <c r="J51" s="27" t="n">
         <v>7</v>
@@ -2756,7 +2756,7 @@
         </is>
       </c>
       <c r="L51" s="28" t="n">
-        <v>63.65191183967269</v>
+        <v>52.58214372024118</v>
       </c>
     </row>
     <row r="52">
@@ -2781,11 +2781,11 @@
       </c>
       <c r="H52" s="31" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="I52" s="33" t="n">
-        <v>0.001023539201315593</v>
+        <v>0.00179241147189213</v>
       </c>
       <c r="J52" s="34" t="n">
         <v>7</v>
@@ -2796,7 +2796,7 @@
         </is>
       </c>
       <c r="L52" s="35" t="n">
-        <v>52.58214372024118</v>
+        <v>61.24050752750126</v>
       </c>
     </row>
   </sheetData>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 3 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 3 Sep 2026, 11:15 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3132,22 +3132,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>31 of 40</t>
+          <t>31 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>9 of 40</t>
+          <t>8 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>5.3 / 9</t>
+          <t>5.4 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>21 of 40</t>
+          <t>21 of 39</t>
         </is>
       </c>
     </row>
@@ -6584,17 +6584,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
+          <t>Dan Ives Says M&amp;A Is the ‘Missing Piece’ for Apple in AI Arms Race — New CEO John Ternus Could Finally Shak...</t>
+        </is>
+      </c>
+      <c r="AY24" s="79" t="inlineStr">
+        <is>
           <t>What Happens To Qualcomm Stock If The New Revenue Earns Less?</t>
         </is>
       </c>
-      <c r="AY24" s="79" t="inlineStr">
+      <c r="AZ24" s="79" t="inlineStr">
         <is>
           <t>Apple (AAPL) Faces Mixed Outlook Ahead of Foldable iPhone Launch</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>Apple faces £2 bn lawsuit in UK over app privacy feature</t>
         </is>
       </c>
     </row>
@@ -6965,12 +6965,12 @@
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
+          <t>Amazon Signed a Multibillion-Dollar Deal With a 175-Year-Old Glassmaker. Is Fiber the Next AI Bottleneck?</t>
+        </is>
+      </c>
+      <c r="AZ26" s="79" t="inlineStr">
+        <is>
           <t>Top Analyst Reports for Amazon, AbbVie &amp; Alibaba</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Microsoft, Amazon and 8 More Stocks Set to Win in a $26 Trillion AI Market</t>
         </is>
       </c>
     </row>
@@ -7545,171 +7545,57 @@
           <t>AVGO</t>
         </is>
       </c>
-      <c r="C30" s="26" t="n">
-        <v>-0.02744795458096083</v>
-      </c>
-      <c r="D30" s="27" t="n">
-        <v>25</v>
-      </c>
-      <c r="E30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F30" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L30" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N30" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="O30" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-      <c r="P30" s="25" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C30" s="26" t="n"/>
+      <c r="D30" s="27" t="n"/>
+      <c r="E30" s="23" t="n"/>
+      <c r="F30" s="23" t="n"/>
+      <c r="G30" s="23" t="n"/>
+      <c r="H30" s="23" t="n"/>
+      <c r="I30" s="23" t="n"/>
+      <c r="J30" s="23" t="n"/>
+      <c r="K30" s="23" t="n"/>
+      <c r="L30" s="23" t="n"/>
+      <c r="M30" s="23" t="n"/>
+      <c r="N30" s="69" t="n"/>
+      <c r="O30" s="23" t="n"/>
+      <c r="P30" s="25" t="n"/>
       <c r="Q30" s="25" t="inlineStr">
         <is>
           <t>Broadcom Inc.</t>
         </is>
       </c>
-      <c r="R30" s="70" t="n">
-        <v>357.1600036621094</v>
-      </c>
-      <c r="S30" s="71" t="n">
-        <v>-10.07998657226562</v>
-      </c>
-      <c r="T30" s="72" t="n">
-        <v>351.614990234375</v>
-      </c>
-      <c r="U30" s="72" t="n">
-        <v>359.3999938964844</v>
-      </c>
-      <c r="V30" s="72" t="n">
-        <v>342.3305053710938</v>
-      </c>
-      <c r="W30" s="73" t="n">
-        <v>60115767</v>
-      </c>
-      <c r="X30" s="74" t="n">
-        <v>2.666778961403967</v>
-      </c>
-      <c r="Y30" s="28" t="n">
-        <v>37.51016967676528</v>
-      </c>
-      <c r="Z30" s="28" t="n">
-        <v>26.00321499704079</v>
-      </c>
-      <c r="AA30" s="28" t="n">
-        <v>22.72566419470456</v>
-      </c>
-      <c r="AB30" s="75" t="n">
-        <v>-8.502136860224084</v>
-      </c>
-      <c r="AC30" s="75" t="n">
-        <v>-7.068182913720201</v>
-      </c>
-      <c r="AD30" s="75" t="n">
-        <v>-1.433953946503883</v>
-      </c>
-      <c r="AE30" s="72" t="n">
-        <v>366.3384274771434</v>
-      </c>
-      <c r="AF30" s="72" t="n">
-        <v>375.7477269644173</v>
-      </c>
-      <c r="AG30" s="72" t="n">
-        <v>384.0817999267578</v>
-      </c>
-      <c r="AH30" s="72" t="n">
-        <v>398.3593008422852</v>
-      </c>
-      <c r="AI30" s="72" t="n">
-        <v>369.7574003601074</v>
-      </c>
-      <c r="AJ30" s="72" t="n">
-        <v>430.2575826074662</v>
-      </c>
-      <c r="AK30" s="72" t="n">
-        <v>381.8164993286133</v>
-      </c>
-      <c r="AL30" s="72" t="n">
-        <v>333.3754160497604</v>
-      </c>
-      <c r="AM30" s="76" t="n">
-        <v>0.2455001622840689</v>
-      </c>
-      <c r="AN30" s="29" t="n">
-        <v>25.37401257621489</v>
-      </c>
-      <c r="AO30" s="77" t="n">
-        <v>3.788657765020125</v>
-      </c>
-      <c r="AP30" s="72" t="n">
-        <v>495</v>
-      </c>
-      <c r="AQ30" s="72" t="n">
-        <v>289.9599914550781</v>
-      </c>
-      <c r="AR30" s="29" t="n">
-        <v>-27.84646390664457</v>
-      </c>
-      <c r="AS30" s="78" t="n">
-        <v>32.7740974475762</v>
-      </c>
-      <c r="AT30" s="26" t="n">
-        <v>-0.03870378573529543</v>
-      </c>
-      <c r="AU30" s="26" t="n">
-        <v>-0.1461222035372461</v>
-      </c>
-      <c r="AV30" s="26" t="n">
-        <v>-0.1474063628468687</v>
-      </c>
-      <c r="AW30" s="26" t="n">
-        <v>0.03195607443961102</v>
-      </c>
+      <c r="R30" s="70" t="n"/>
+      <c r="S30" s="71" t="n"/>
+      <c r="T30" s="72" t="n"/>
+      <c r="U30" s="72" t="n"/>
+      <c r="V30" s="72" t="n"/>
+      <c r="W30" s="73" t="n"/>
+      <c r="X30" s="74" t="n"/>
+      <c r="Y30" s="28" t="n"/>
+      <c r="Z30" s="28" t="n"/>
+      <c r="AA30" s="28" t="n"/>
+      <c r="AB30" s="75" t="n"/>
+      <c r="AC30" s="75" t="n"/>
+      <c r="AD30" s="75" t="n"/>
+      <c r="AE30" s="72" t="n"/>
+      <c r="AF30" s="72" t="n"/>
+      <c r="AG30" s="72" t="n"/>
+      <c r="AH30" s="72" t="n"/>
+      <c r="AI30" s="72" t="n"/>
+      <c r="AJ30" s="72" t="n"/>
+      <c r="AK30" s="72" t="n"/>
+      <c r="AL30" s="72" t="n"/>
+      <c r="AM30" s="76" t="n"/>
+      <c r="AN30" s="29" t="n"/>
+      <c r="AO30" s="77" t="n"/>
+      <c r="AP30" s="72" t="n"/>
+      <c r="AQ30" s="72" t="n"/>
+      <c r="AR30" s="29" t="n"/>
+      <c r="AS30" s="78" t="n"/>
+      <c r="AT30" s="26" t="n"/>
+      <c r="AU30" s="26" t="n"/>
+      <c r="AV30" s="26" t="n"/>
+      <c r="AW30" s="26" t="n"/>
       <c r="AX30" s="79" t="inlineStr">
         <is>
           <t>Broadcom Shares Fall 5.6% Even as Revenue Surges 86%</t>
@@ -11096,17 +10982,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>Musk Said Robots Will Outproduce All Humans, Then Promised Austin 30,000 Jobs</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
           <t>Dow Jones Futures: Stocks Jump On Fed's Waller; Tesla Cybercab Event Private, Jobs Report Looms</t>
         </is>
       </c>
-      <c r="AY48" s="79" t="inlineStr">
-        <is>
-          <t>Tesla Launching Cybercab Robotaxis. Here's What To Look For.</t>
-        </is>
-      </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Tesla's 45 Cybercabs Face a $1.3 Trillion Reality Check</t>
+          <t>Tesla is asking people if they want to buy and run Cybercab fleets</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11529,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 3 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 3 Sep 2026, 11:15 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -11668,22 +11554,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>30 of 40</t>
+          <t>30 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>10 of 40</t>
+          <t>9 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>4.0 / 9</t>
+          <t>4.1 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>13 of 40</t>
+          <t>13 of 39</t>
         </is>
       </c>
     </row>
@@ -15829,171 +15715,57 @@
           <t>AVGO</t>
         </is>
       </c>
-      <c r="C30" s="26" t="n">
-        <v>-0.006600309699600682</v>
-      </c>
-      <c r="D30" s="27" t="n">
-        <v>20</v>
-      </c>
-      <c r="E30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F30" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L30" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N30" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="O30" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-      <c r="P30" s="25" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C30" s="26" t="n"/>
+      <c r="D30" s="27" t="n"/>
+      <c r="E30" s="23" t="n"/>
+      <c r="F30" s="23" t="n"/>
+      <c r="G30" s="23" t="n"/>
+      <c r="H30" s="23" t="n"/>
+      <c r="I30" s="23" t="n"/>
+      <c r="J30" s="23" t="n"/>
+      <c r="K30" s="23" t="n"/>
+      <c r="L30" s="23" t="n"/>
+      <c r="M30" s="23" t="n"/>
+      <c r="N30" s="69" t="n"/>
+      <c r="O30" s="23" t="n"/>
+      <c r="P30" s="25" t="n"/>
       <c r="Q30" s="25" t="inlineStr">
         <is>
           <t>Broadcom Inc.</t>
         </is>
       </c>
-      <c r="R30" s="70" t="n">
-        <v>367.239990234375</v>
-      </c>
-      <c r="S30" s="71" t="n">
-        <v>-2.44000244140625</v>
-      </c>
-      <c r="T30" s="72" t="n">
-        <v>369.6799926757812</v>
-      </c>
-      <c r="U30" s="72" t="n">
-        <v>371.0899963378906</v>
-      </c>
-      <c r="V30" s="72" t="n">
-        <v>364.6499938964844</v>
-      </c>
-      <c r="W30" s="73" t="n">
-        <v>38874600</v>
-      </c>
-      <c r="X30" s="74" t="n">
-        <v>1.921436532630159</v>
-      </c>
-      <c r="Y30" s="28" t="n">
-        <v>42.128064745238</v>
-      </c>
-      <c r="Z30" s="28" t="n">
-        <v>27.51440103145891</v>
-      </c>
-      <c r="AA30" s="28" t="n">
-        <v>21.57471555558841</v>
-      </c>
-      <c r="AB30" s="75" t="n">
-        <v>-7.916960229685571</v>
-      </c>
-      <c r="AC30" s="75" t="n">
-        <v>-6.70969442709423</v>
-      </c>
-      <c r="AD30" s="75" t="n">
-        <v>-1.207265802591341</v>
-      </c>
-      <c r="AE30" s="72" t="n">
-        <v>368.9608342814388</v>
-      </c>
-      <c r="AF30" s="72" t="n">
-        <v>377.6064992946481</v>
-      </c>
-      <c r="AG30" s="72" t="n">
-        <v>384.58</v>
-      </c>
-      <c r="AH30" s="72" t="n">
-        <v>398.585200805664</v>
-      </c>
-      <c r="AI30" s="72" t="n">
-        <v>369.6839002990723</v>
-      </c>
-      <c r="AJ30" s="72" t="n">
-        <v>434.8378629372112</v>
-      </c>
-      <c r="AK30" s="72" t="n">
-        <v>384.9869995117188</v>
-      </c>
-      <c r="AL30" s="72" t="n">
-        <v>335.1361360862263</v>
-      </c>
-      <c r="AM30" s="76" t="n">
-        <v>0.3219989779728831</v>
-      </c>
-      <c r="AN30" s="29" t="n">
-        <v>25.89742692024332</v>
-      </c>
-      <c r="AO30" s="77" t="n">
-        <v>3.446341995677256</v>
-      </c>
-      <c r="AP30" s="72" t="n">
-        <v>495</v>
-      </c>
-      <c r="AQ30" s="72" t="n">
-        <v>289.9599914550781</v>
-      </c>
-      <c r="AR30" s="29" t="n">
-        <v>-25.81010298295454</v>
-      </c>
-      <c r="AS30" s="78" t="n">
-        <v>37.69020462285327</v>
-      </c>
-      <c r="AT30" s="26" t="n">
-        <v>0.03276243431048109</v>
-      </c>
-      <c r="AU30" s="26" t="n">
-        <v>-0.1217716017356836</v>
-      </c>
-      <c r="AV30" s="26" t="n">
-        <v>-0.2336874114404076</v>
-      </c>
-      <c r="AW30" s="26" t="n">
-        <v>0.06108056561124875</v>
-      </c>
+      <c r="R30" s="70" t="n"/>
+      <c r="S30" s="71" t="n"/>
+      <c r="T30" s="72" t="n"/>
+      <c r="U30" s="72" t="n"/>
+      <c r="V30" s="72" t="n"/>
+      <c r="W30" s="73" t="n"/>
+      <c r="X30" s="74" t="n"/>
+      <c r="Y30" s="28" t="n"/>
+      <c r="Z30" s="28" t="n"/>
+      <c r="AA30" s="28" t="n"/>
+      <c r="AB30" s="75" t="n"/>
+      <c r="AC30" s="75" t="n"/>
+      <c r="AD30" s="75" t="n"/>
+      <c r="AE30" s="72" t="n"/>
+      <c r="AF30" s="72" t="n"/>
+      <c r="AG30" s="72" t="n"/>
+      <c r="AH30" s="72" t="n"/>
+      <c r="AI30" s="72" t="n"/>
+      <c r="AJ30" s="72" t="n"/>
+      <c r="AK30" s="72" t="n"/>
+      <c r="AL30" s="72" t="n"/>
+      <c r="AM30" s="76" t="n"/>
+      <c r="AN30" s="29" t="n"/>
+      <c r="AO30" s="77" t="n"/>
+      <c r="AP30" s="72" t="n"/>
+      <c r="AQ30" s="72" t="n"/>
+      <c r="AR30" s="29" t="n"/>
+      <c r="AS30" s="78" t="n"/>
+      <c r="AT30" s="26" t="n"/>
+      <c r="AU30" s="26" t="n"/>
+      <c r="AV30" s="26" t="n"/>
+      <c r="AW30" s="26" t="n"/>
       <c r="AX30" s="25" t="n"/>
       <c r="AY30" s="25" t="n"/>
       <c r="AZ30" s="25" t="n"/>
@@ -16185,7 +15957,7 @@
         <v>-0.01124005114350968</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
@@ -17065,7 +16837,7 @@
         <v>-0.008382862523551915</v>
       </c>
       <c r="D37" s="34" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E37" s="30" t="inlineStr">
         <is>
@@ -17241,7 +17013,7 @@
         <v>-0.01353295042585745</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -17945,7 +17717,7 @@
         <v>-0.009063459196570256</v>
       </c>
       <c r="D42" s="27" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
@@ -18297,7 +18069,7 @@
         <v>-0.0581369028542128</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
@@ -19579,7 +19351,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 3 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 3 Sep 2026, 11:15 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19604,22 +19376,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>5 of 40</t>
+          <t>5 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>35 of 40</t>
+          <t>34 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>3.2 / 9</t>
+          <t>3.3 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>9 of 40</t>
+          <t>9 of 39</t>
         </is>
       </c>
     </row>
@@ -22889,7 +22661,7 @@
         <v>-0.02360217505168549</v>
       </c>
       <c r="D25" s="34" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E25" s="30" t="inlineStr">
         <is>
@@ -23065,7 +22837,7 @@
         <v>-0.01867032778937106</v>
       </c>
       <c r="D26" s="27" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
@@ -23241,7 +23013,7 @@
         <v>-0.02909895842760113</v>
       </c>
       <c r="D27" s="34" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E27" s="30" t="inlineStr">
         <is>
@@ -23417,7 +23189,7 @@
         <v>-0.02930840490496478</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
@@ -23593,7 +23365,7 @@
         <v>-0.05583755198412677</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E29" s="30" t="inlineStr">
         <is>
@@ -23765,171 +23537,57 @@
           <t>AVGO</t>
         </is>
       </c>
-      <c r="C30" s="26" t="n">
-        <v>-0.001782156042112182</v>
-      </c>
-      <c r="D30" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="E30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H30" s="23" t="inlineStr">
-        <is>
-          <t>Same</t>
-        </is>
-      </c>
-      <c r="I30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L30" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N30" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="O30" s="23" t="inlineStr">
-        <is>
-          <t>Weak</t>
-        </is>
-      </c>
-      <c r="P30" s="25" t="inlineStr">
-        <is>
-          <t>Long-term up, short-term mixed</t>
-        </is>
-      </c>
+      <c r="C30" s="26" t="n"/>
+      <c r="D30" s="27" t="n"/>
+      <c r="E30" s="23" t="n"/>
+      <c r="F30" s="23" t="n"/>
+      <c r="G30" s="23" t="n"/>
+      <c r="H30" s="23" t="n"/>
+      <c r="I30" s="23" t="n"/>
+      <c r="J30" s="23" t="n"/>
+      <c r="K30" s="23" t="n"/>
+      <c r="L30" s="23" t="n"/>
+      <c r="M30" s="23" t="n"/>
+      <c r="N30" s="69" t="n"/>
+      <c r="O30" s="23" t="n"/>
+      <c r="P30" s="25" t="n"/>
       <c r="Q30" s="25" t="inlineStr">
         <is>
           <t>Broadcom Inc.</t>
         </is>
       </c>
-      <c r="R30" s="70" t="n">
-        <v>369.6799926757812</v>
-      </c>
-      <c r="S30" s="71" t="n">
-        <v>-0.660003662109375</v>
-      </c>
-      <c r="T30" s="72" t="n">
-        <v>364.25</v>
-      </c>
-      <c r="U30" s="72" t="n">
-        <v>371.3999938964844</v>
-      </c>
-      <c r="V30" s="72" t="n">
-        <v>362</v>
-      </c>
-      <c r="W30" s="73" t="n">
-        <v>19288900</v>
-      </c>
-      <c r="X30" s="74" t="n">
-        <v>1.008183003229087</v>
-      </c>
-      <c r="Y30" s="28" t="n">
-        <v>43.32701006182213</v>
-      </c>
-      <c r="Z30" s="28" t="n">
-        <v>26.20891124506882</v>
-      </c>
-      <c r="AA30" s="28" t="n">
-        <v>21.64620451808354</v>
-      </c>
-      <c r="AB30" s="75" t="n">
-        <v>-8.081232177997094</v>
-      </c>
-      <c r="AC30" s="75" t="n">
-        <v>-6.407877976446394</v>
-      </c>
-      <c r="AD30" s="75" t="n">
-        <v>-1.6733542015507</v>
-      </c>
-      <c r="AE30" s="72" t="n">
-        <v>369.4525040091713</v>
-      </c>
-      <c r="AF30" s="72" t="n">
-        <v>378.6431502006754</v>
-      </c>
-      <c r="AG30" s="72" t="n">
-        <v>384.8382000732422</v>
-      </c>
-      <c r="AH30" s="72" t="n">
-        <v>398.62830078125</v>
-      </c>
-      <c r="AI30" s="72" t="n">
-        <v>369.547600402832</v>
-      </c>
-      <c r="AJ30" s="72" t="n">
-        <v>438.7029643273173</v>
-      </c>
-      <c r="AK30" s="72" t="n">
-        <v>387.5389999389648</v>
-      </c>
-      <c r="AL30" s="72" t="n">
-        <v>336.3750355506123</v>
-      </c>
-      <c r="AM30" s="76" t="n">
-        <v>0.3254727963647674</v>
-      </c>
-      <c r="AN30" s="29" t="n">
-        <v>26.4045499402179</v>
-      </c>
-      <c r="AO30" s="77" t="n">
-        <v>3.552944855814614</v>
-      </c>
-      <c r="AP30" s="72" t="n">
-        <v>495</v>
-      </c>
-      <c r="AQ30" s="72" t="n">
-        <v>287.1700134277344</v>
-      </c>
-      <c r="AR30" s="29" t="n">
-        <v>-25.31717319681187</v>
-      </c>
-      <c r="AS30" s="78" t="n">
-        <v>39.70070951207848</v>
-      </c>
-      <c r="AT30" s="26" t="n">
-        <v>0.03627292368569268</v>
-      </c>
-      <c r="AU30" s="26" t="n">
-        <v>-0.05749182285629051</v>
-      </c>
-      <c r="AV30" s="26" t="n">
-        <v>-0.2323442343723602</v>
-      </c>
-      <c r="AW30" s="26" t="n">
-        <v>0.06813055809427815</v>
-      </c>
+      <c r="R30" s="70" t="n"/>
+      <c r="S30" s="71" t="n"/>
+      <c r="T30" s="72" t="n"/>
+      <c r="U30" s="72" t="n"/>
+      <c r="V30" s="72" t="n"/>
+      <c r="W30" s="73" t="n"/>
+      <c r="X30" s="74" t="n"/>
+      <c r="Y30" s="28" t="n"/>
+      <c r="Z30" s="28" t="n"/>
+      <c r="AA30" s="28" t="n"/>
+      <c r="AB30" s="75" t="n"/>
+      <c r="AC30" s="75" t="n"/>
+      <c r="AD30" s="75" t="n"/>
+      <c r="AE30" s="72" t="n"/>
+      <c r="AF30" s="72" t="n"/>
+      <c r="AG30" s="72" t="n"/>
+      <c r="AH30" s="72" t="n"/>
+      <c r="AI30" s="72" t="n"/>
+      <c r="AJ30" s="72" t="n"/>
+      <c r="AK30" s="72" t="n"/>
+      <c r="AL30" s="72" t="n"/>
+      <c r="AM30" s="76" t="n"/>
+      <c r="AN30" s="29" t="n"/>
+      <c r="AO30" s="77" t="n"/>
+      <c r="AP30" s="72" t="n"/>
+      <c r="AQ30" s="72" t="n"/>
+      <c r="AR30" s="29" t="n"/>
+      <c r="AS30" s="78" t="n"/>
+      <c r="AT30" s="26" t="n"/>
+      <c r="AU30" s="26" t="n"/>
+      <c r="AV30" s="26" t="n"/>
+      <c r="AW30" s="26" t="n"/>
       <c r="AX30" s="25" t="n"/>
       <c r="AY30" s="25" t="n"/>
       <c r="AZ30" s="25" t="n"/>
@@ -23945,7 +23603,7 @@
         <v>-0.02531389171652176</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E31" s="30" t="inlineStr">
         <is>
@@ -24121,7 +23779,7 @@
         <v>-0.03581106063593686</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
@@ -24297,7 +23955,7 @@
         <v>-0.06800291463242925</v>
       </c>
       <c r="D33" s="34" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E33" s="30" t="inlineStr">
         <is>
@@ -24473,7 +24131,7 @@
         <v>-0.01007723337380684</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
@@ -24649,7 +24307,7 @@
         <v>-0.007948321980374096</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -24825,7 +24483,7 @@
         <v>-0.006032855576357687</v>
       </c>
       <c r="D36" s="27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
@@ -25001,7 +24659,7 @@
         <v>-0.01235983249351691</v>
       </c>
       <c r="D37" s="34" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E37" s="30" t="inlineStr">
         <is>
@@ -25177,7 +24835,7 @@
         <v>-0.06062889303421481</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -25353,7 +25011,7 @@
         <v>-0.02637862437031413</v>
       </c>
       <c r="D39" s="34" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E39" s="30" t="inlineStr">
         <is>
@@ -25529,7 +25187,7 @@
         <v>-0.03286164112737533</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
@@ -25705,7 +25363,7 @@
         <v>-0.002961202765295323</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -25881,7 +25539,7 @@
         <v>-0.02071006223241978</v>
       </c>
       <c r="D42" s="27" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
@@ -26057,7 +25715,7 @@
         <v>-0.0151281653970361</v>
       </c>
       <c r="D43" s="34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E43" s="30" t="inlineStr">
         <is>
@@ -26233,7 +25891,7 @@
         <v>-0.03466040639889967</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
@@ -26409,7 +26067,7 @@
         <v>-0.02270058196958502</v>
       </c>
       <c r="D45" s="34" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
@@ -26585,7 +26243,7 @@
         <v>-0.02158944450796974</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
@@ -26761,7 +26419,7 @@
         <v>-0.01903999296889936</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -26937,7 +26595,7 @@
         <v>-0.03223268236356913</v>
       </c>
       <c r="D48" s="27" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
@@ -27515,7 +27173,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 3 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 3 Sep 2026, 11:15 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27540,12 +27198,12 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>19 of 40</t>
+          <t>18 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>21 of 40</t>
+          <t>21 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
@@ -27555,7 +27213,7 @@
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>15 of 40</t>
+          <t>15 of 39</t>
         </is>
       </c>
     </row>
@@ -30649,7 +30307,7 @@
         <v>-0.008914626195478559</v>
       </c>
       <c r="D24" s="27" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
@@ -31001,7 +30659,7 @@
         <v>-0.02499719943397638</v>
       </c>
       <c r="D26" s="27" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
@@ -31701,171 +31359,57 @@
           <t>AVGO</t>
         </is>
       </c>
-      <c r="C30" s="26" t="n">
-        <v>0.004202900721427705</v>
-      </c>
-      <c r="D30" s="27" t="n">
-        <v>13</v>
-      </c>
-      <c r="E30" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F30" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H30" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L30" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N30" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="O30" s="23" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P30" s="25" t="inlineStr">
-        <is>
-          <t>Long-term up, short-term mixed</t>
-        </is>
-      </c>
+      <c r="C30" s="26" t="n"/>
+      <c r="D30" s="27" t="n"/>
+      <c r="E30" s="23" t="n"/>
+      <c r="F30" s="23" t="n"/>
+      <c r="G30" s="23" t="n"/>
+      <c r="H30" s="23" t="n"/>
+      <c r="I30" s="23" t="n"/>
+      <c r="J30" s="23" t="n"/>
+      <c r="K30" s="23" t="n"/>
+      <c r="L30" s="23" t="n"/>
+      <c r="M30" s="23" t="n"/>
+      <c r="N30" s="69" t="n"/>
+      <c r="O30" s="23" t="n"/>
+      <c r="P30" s="25" t="n"/>
       <c r="Q30" s="25" t="inlineStr">
         <is>
           <t>Broadcom Inc.</t>
         </is>
       </c>
-      <c r="R30" s="70" t="n">
-        <v>370.3399963378906</v>
-      </c>
-      <c r="S30" s="71" t="n">
-        <v>1.54998779296875</v>
-      </c>
-      <c r="T30" s="72" t="n">
-        <v>369.5199890136719</v>
-      </c>
-      <c r="U30" s="72" t="n">
-        <v>372.75</v>
-      </c>
-      <c r="V30" s="72" t="n">
-        <v>366.2999877929688</v>
-      </c>
-      <c r="W30" s="73" t="n">
-        <v>21948000</v>
-      </c>
-      <c r="X30" s="74" t="n">
-        <v>1.117168008620538</v>
-      </c>
-      <c r="Y30" s="28" t="n">
-        <v>43.63895186508395</v>
-      </c>
-      <c r="Z30" s="28" t="n">
-        <v>26.53060980059774</v>
-      </c>
-      <c r="AA30" s="28" t="n">
-        <v>21.72319263153983</v>
-      </c>
-      <c r="AB30" s="75" t="n">
-        <v>-8.421794336196172</v>
-      </c>
-      <c r="AC30" s="75" t="n">
-        <v>-5.989539426058719</v>
-      </c>
-      <c r="AD30" s="75" t="n">
-        <v>-2.432254910137453</v>
-      </c>
-      <c r="AE30" s="72" t="n">
-        <v>369.3875072472828</v>
-      </c>
-      <c r="AF30" s="72" t="n">
-        <v>379.5394659531648</v>
-      </c>
-      <c r="AG30" s="72" t="n">
-        <v>385.2872003173828</v>
-      </c>
-      <c r="AH30" s="72" t="n">
-        <v>398.4806008911133</v>
-      </c>
-      <c r="AI30" s="72" t="n">
-        <v>369.4753004455566</v>
-      </c>
-      <c r="AJ30" s="72" t="n">
-        <v>442.0973316242758</v>
-      </c>
-      <c r="AK30" s="72" t="n">
-        <v>389.9630004882812</v>
-      </c>
-      <c r="AL30" s="72" t="n">
-        <v>337.8286693522867</v>
-      </c>
-      <c r="AM30" s="76" t="n">
-        <v>0.3118034342935829</v>
-      </c>
-      <c r="AN30" s="29" t="n">
-        <v>26.73809108593175</v>
-      </c>
-      <c r="AO30" s="77" t="n">
-        <v>3.624182680102603</v>
-      </c>
-      <c r="AP30" s="72" t="n">
-        <v>495</v>
-      </c>
-      <c r="AQ30" s="72" t="n">
-        <v>287.1700134277344</v>
-      </c>
-      <c r="AR30" s="29" t="n">
-        <v>-25.18383912365846</v>
-      </c>
-      <c r="AS30" s="78" t="n">
-        <v>40.01827853712381</v>
-      </c>
-      <c r="AT30" s="26" t="n">
-        <v>0.03227780760690346</v>
-      </c>
-      <c r="AU30" s="26" t="n">
-        <v>-0.04865393161939546</v>
-      </c>
-      <c r="AV30" s="26" t="n">
-        <v>-0.1948605444810436</v>
-      </c>
-      <c r="AW30" s="26" t="n">
-        <v>0.0700375319471247</v>
-      </c>
+      <c r="R30" s="70" t="n"/>
+      <c r="S30" s="71" t="n"/>
+      <c r="T30" s="72" t="n"/>
+      <c r="U30" s="72" t="n"/>
+      <c r="V30" s="72" t="n"/>
+      <c r="W30" s="73" t="n"/>
+      <c r="X30" s="74" t="n"/>
+      <c r="Y30" s="28" t="n"/>
+      <c r="Z30" s="28" t="n"/>
+      <c r="AA30" s="28" t="n"/>
+      <c r="AB30" s="75" t="n"/>
+      <c r="AC30" s="75" t="n"/>
+      <c r="AD30" s="75" t="n"/>
+      <c r="AE30" s="72" t="n"/>
+      <c r="AF30" s="72" t="n"/>
+      <c r="AG30" s="72" t="n"/>
+      <c r="AH30" s="72" t="n"/>
+      <c r="AI30" s="72" t="n"/>
+      <c r="AJ30" s="72" t="n"/>
+      <c r="AK30" s="72" t="n"/>
+      <c r="AL30" s="72" t="n"/>
+      <c r="AM30" s="76" t="n"/>
+      <c r="AN30" s="29" t="n"/>
+      <c r="AO30" s="77" t="n"/>
+      <c r="AP30" s="72" t="n"/>
+      <c r="AQ30" s="72" t="n"/>
+      <c r="AR30" s="29" t="n"/>
+      <c r="AS30" s="78" t="n"/>
+      <c r="AT30" s="26" t="n"/>
+      <c r="AU30" s="26" t="n"/>
+      <c r="AV30" s="26" t="n"/>
+      <c r="AW30" s="26" t="n"/>
       <c r="AX30" s="25" t="n"/>
       <c r="AY30" s="25" t="n"/>
       <c r="AZ30" s="25" t="n"/>
@@ -31881,7 +31425,7 @@
         <v>-0.01249874985801214</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E31" s="30" t="inlineStr">
         <is>
@@ -32233,7 +31777,7 @@
         <v>-0.0005040778398927026</v>
       </c>
       <c r="D33" s="34" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E33" s="30" t="inlineStr">
         <is>
@@ -32409,7 +31953,7 @@
         <v>-0.02178605084672747</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
@@ -32761,7 +32305,7 @@
         <v>0.0004470874592776841</v>
       </c>
       <c r="D36" s="27" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
@@ -32937,7 +32481,7 @@
         <v>-0.01215122854742678</v>
       </c>
       <c r="D37" s="34" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E37" s="30" t="inlineStr">
         <is>
@@ -33465,7 +33009,7 @@
         <v>-0.01367236567406971</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
@@ -33641,7 +33185,7 @@
         <v>-0.008198704832808712</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -33817,7 +33361,7 @@
         <v>-0.00685599359086031</v>
       </c>
       <c r="D42" s="27" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
@@ -34169,7 +33713,7 @@
         <v>0.0004831799877809129</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
@@ -34521,7 +34065,7 @@
         <v>-0.007299289100143769</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
@@ -35451,7 +34995,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 3 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 3 Sep 2026, 11:15 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35476,22 +35020,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>12 of 40</t>
+          <t>12 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>28 of 40</t>
+          <t>27 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>4.2 / 9</t>
+          <t>4.4 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>16 of 40</t>
+          <t>16 of 39</t>
         </is>
       </c>
     </row>
@@ -38761,7 +38305,7 @@
         <v>-0.02326562725379</v>
       </c>
       <c r="D25" s="34" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E25" s="30" t="inlineStr">
         <is>
@@ -39113,7 +38657,7 @@
         <v>-0.03192951480000428</v>
       </c>
       <c r="D27" s="34" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E27" s="30" t="inlineStr">
         <is>
@@ -39289,7 +38833,7 @@
         <v>-0.06332041548914424</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
@@ -39465,7 +39009,7 @@
         <v>-0.05517577254916717</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E29" s="30" t="inlineStr">
         <is>
@@ -39637,171 +39181,57 @@
           <t>AVGO</t>
         </is>
       </c>
-      <c r="C30" s="26" t="n">
-        <v>-0.007401625495918829</v>
-      </c>
-      <c r="D30" s="27" t="n">
-        <v>10</v>
-      </c>
-      <c r="E30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H30" s="23" t="inlineStr">
-        <is>
-          <t>Same</t>
-        </is>
-      </c>
-      <c r="I30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L30" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M30" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N30" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-      <c r="P30" s="25" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C30" s="26" t="n"/>
+      <c r="D30" s="27" t="n"/>
+      <c r="E30" s="23" t="n"/>
+      <c r="F30" s="23" t="n"/>
+      <c r="G30" s="23" t="n"/>
+      <c r="H30" s="23" t="n"/>
+      <c r="I30" s="23" t="n"/>
+      <c r="J30" s="23" t="n"/>
+      <c r="K30" s="23" t="n"/>
+      <c r="L30" s="23" t="n"/>
+      <c r="M30" s="23" t="n"/>
+      <c r="N30" s="69" t="n"/>
+      <c r="O30" s="23" t="n"/>
+      <c r="P30" s="25" t="n"/>
       <c r="Q30" s="25" t="inlineStr">
         <is>
           <t>Broadcom Inc.</t>
         </is>
       </c>
-      <c r="R30" s="70" t="n">
-        <v>368.7900085449219</v>
-      </c>
-      <c r="S30" s="71" t="n">
-        <v>-2.75</v>
-      </c>
-      <c r="T30" s="72" t="n">
-        <v>373.6000061035156</v>
-      </c>
-      <c r="U30" s="72" t="n">
-        <v>376.5899963378906</v>
-      </c>
-      <c r="V30" s="72" t="n">
-        <v>365.3500061035156</v>
-      </c>
-      <c r="W30" s="73" t="n">
-        <v>16596100</v>
-      </c>
-      <c r="X30" s="74" t="n">
-        <v>0.8548319139445547</v>
-      </c>
-      <c r="Y30" s="28" t="n">
-        <v>42.73994319076292</v>
-      </c>
-      <c r="Z30" s="28" t="n">
-        <v>24.41982790794276</v>
-      </c>
-      <c r="AA30" s="28" t="n">
-        <v>22.09664002115975</v>
-      </c>
-      <c r="AB30" s="75" t="n">
-        <v>-8.801177037003981</v>
-      </c>
-      <c r="AC30" s="75" t="n">
-        <v>-5.381475698524355</v>
-      </c>
-      <c r="AD30" s="75" t="n">
-        <v>-3.419701338479626</v>
-      </c>
-      <c r="AE30" s="72" t="n">
-        <v>369.1153675071091</v>
-      </c>
-      <c r="AF30" s="72" t="n">
-        <v>380.4594129146923</v>
-      </c>
-      <c r="AG30" s="72" t="n">
-        <v>386.1074005126953</v>
-      </c>
-      <c r="AH30" s="72" t="n">
-        <v>398.2835009765625</v>
-      </c>
-      <c r="AI30" s="72" t="n">
-        <v>369.3834004211426</v>
-      </c>
-      <c r="AJ30" s="72" t="n">
-        <v>442.4112952823579</v>
-      </c>
-      <c r="AK30" s="72" t="n">
-        <v>391.0575012207031</v>
-      </c>
-      <c r="AL30" s="72" t="n">
-        <v>339.7037071590483</v>
-      </c>
-      <c r="AM30" s="76" t="n">
-        <v>0.2831952528274042</v>
-      </c>
-      <c r="AN30" s="29" t="n">
-        <v>26.26406290704136</v>
-      </c>
-      <c r="AO30" s="77" t="n">
-        <v>3.784833888275186</v>
-      </c>
-      <c r="AP30" s="72" t="n">
-        <v>495</v>
-      </c>
-      <c r="AQ30" s="72" t="n">
-        <v>287.1700134277344</v>
-      </c>
-      <c r="AR30" s="29" t="n">
-        <v>-25.49696797072285</v>
-      </c>
-      <c r="AS30" s="78" t="n">
-        <v>39.27248250521683</v>
-      </c>
-      <c r="AT30" s="26" t="n">
-        <v>0.0009227746685473992</v>
-      </c>
-      <c r="AU30" s="26" t="n">
-        <v>-0.04911816205869646</v>
-      </c>
-      <c r="AV30" s="26" t="n">
-        <v>-0.174541671075323</v>
-      </c>
-      <c r="AW30" s="26" t="n">
-        <v>0.06555909286699024</v>
-      </c>
+      <c r="R30" s="70" t="n"/>
+      <c r="S30" s="71" t="n"/>
+      <c r="T30" s="72" t="n"/>
+      <c r="U30" s="72" t="n"/>
+      <c r="V30" s="72" t="n"/>
+      <c r="W30" s="73" t="n"/>
+      <c r="X30" s="74" t="n"/>
+      <c r="Y30" s="28" t="n"/>
+      <c r="Z30" s="28" t="n"/>
+      <c r="AA30" s="28" t="n"/>
+      <c r="AB30" s="75" t="n"/>
+      <c r="AC30" s="75" t="n"/>
+      <c r="AD30" s="75" t="n"/>
+      <c r="AE30" s="72" t="n"/>
+      <c r="AF30" s="72" t="n"/>
+      <c r="AG30" s="72" t="n"/>
+      <c r="AH30" s="72" t="n"/>
+      <c r="AI30" s="72" t="n"/>
+      <c r="AJ30" s="72" t="n"/>
+      <c r="AK30" s="72" t="n"/>
+      <c r="AL30" s="72" t="n"/>
+      <c r="AM30" s="76" t="n"/>
+      <c r="AN30" s="29" t="n"/>
+      <c r="AO30" s="77" t="n"/>
+      <c r="AP30" s="72" t="n"/>
+      <c r="AQ30" s="72" t="n"/>
+      <c r="AR30" s="29" t="n"/>
+      <c r="AS30" s="78" t="n"/>
+      <c r="AT30" s="26" t="n"/>
+      <c r="AU30" s="26" t="n"/>
+      <c r="AV30" s="26" t="n"/>
+      <c r="AW30" s="26" t="n"/>
       <c r="AX30" s="25" t="n"/>
       <c r="AY30" s="25" t="n"/>
       <c r="AZ30" s="25" t="n"/>
@@ -39817,7 +39247,7 @@
         <v>-0.05943759603113641</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E31" s="30" t="inlineStr">
         <is>
@@ -39993,7 +39423,7 @@
         <v>-0.02960829037404245</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
@@ -40169,7 +39599,7 @@
         <v>-0.03392203277851213</v>
       </c>
       <c r="D33" s="34" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E33" s="30" t="inlineStr">
         <is>
@@ -40521,7 +39951,7 @@
         <v>-0.1253392097053883</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -40697,7 +40127,7 @@
         <v>-0.02845037703741871</v>
       </c>
       <c r="D36" s="27" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
@@ -41049,7 +40479,7 @@
         <v>-0.07343520222782773</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -41401,7 +40831,7 @@
         <v>-0.04256684013924827</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
@@ -41753,7 +41183,7 @@
         <v>-0.03588291869363736</v>
       </c>
       <c r="D42" s="27" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
@@ -41929,7 +41359,7 @@
         <v>-0.04574959589106331</v>
       </c>
       <c r="D43" s="34" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E43" s="30" t="inlineStr">
         <is>
@@ -42457,7 +41887,7 @@
         <v>-0.04649784460844808</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
@@ -42809,7 +42239,7 @@
         <v>-0.01707955694679375</v>
       </c>
       <c r="D48" s="27" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
@@ -43864,7 +43294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G49"/>
+  <dimension ref="B2:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -45103,68 +44533,12 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="24" t="inlineStr">
-        <is>
-          <t>AVGO</t>
-        </is>
-      </c>
-      <c r="C48" s="101" t="inlineStr">
-        <is>
-          <t>Broadcom Inc.</t>
-        </is>
-      </c>
-      <c r="D48" s="104" t="inlineStr">
-        <is>
-          <t>Volume 2.7x its 20-day average</t>
-        </is>
-      </c>
-      <c r="E48" s="26" t="n">
-        <v>-0.02744795458096083</v>
-      </c>
-      <c r="F48" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="31" t="inlineStr">
-        <is>
-          <t>AVGO</t>
-        </is>
-      </c>
-      <c r="C49" s="102" t="inlineStr">
-        <is>
-          <t>Broadcom Inc.</t>
-        </is>
-      </c>
-      <c r="D49" s="105" t="inlineStr">
-        <is>
-          <t>Gapped down 4.3% at the open</t>
-        </is>
-      </c>
-      <c r="E49" s="33" t="n">
-        <v>-0.02744795458096083</v>
-      </c>
-      <c r="F49" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" s="30" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="B5:G49"/>
+  <autoFilter ref="B5:G47"/>
   <mergeCells count="1">
     <mergeCell ref="B2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E49">
+  <conditionalFormatting sqref="E6:E47">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>

</xml_diff>

<commit_message>
Daily workbook: 2026-09-04 23:02 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 4 Sep 2026, 10:23 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 4 Sep 2026, 11:02 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 4 Sep 2026, 10:23 PM · Yahoo Finance data</t>
+          <t>Built 4 Sep 2026, 11:02 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
+          <t>S&amp;P 500, Dow End Lower As Blowout Jobs Report Fans Rate Hike Fears, While Chipmaker Strength Aids Nasdaq —T...</t>
+        </is>
+      </c>
+      <c r="AY19" s="79" t="inlineStr">
+        <is>
           <t>This Is the Most Expensive Market in Decades. Is It Really Safe to Invest Right Now?</t>
         </is>
       </c>
-      <c r="AY19" s="79" t="inlineStr">
+      <c r="AZ19" s="79" t="inlineStr">
         <is>
           <t>GoPro Zooms 34% Higher on Starman Optical Merger and Markiplier Stake; Coherent Climbs 7%, Lumentum Gains 3%</t>
-        </is>
-      </c>
-      <c r="AZ19" s="79" t="inlineStr">
-        <is>
-          <t>SanDisk Rises 8%, Micron Gains 5%: Is the NAND Pricing Cycle Still Accelerating?</t>
         </is>
       </c>
     </row>
@@ -6589,12 +6589,12 @@
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Flash Buy Signals; Apple, Inflation Reports Ahead</t>
+        </is>
+      </c>
+      <c r="AZ24" s="79" t="inlineStr">
+        <is>
           <t>Why Apple (AAPL) Dipped More Than Broader Market Today</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>Top Research Reports for Apple, Broadcom &amp; Shell</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Jim Cramer Says “Someone Must Know Something” About Broadcom Inc. (NASDAQ:AVGO)’s Post-Earnings Share Dip</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Top Research Reports for Apple, Broadcom &amp; Shell</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>5-star analyst resets Broadcom stock price target</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Is AVGO Stock Poised for a Rebound After Broadcom's Strong Q3 Results?</t>
         </is>
       </c>
     </row>
@@ -8276,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
+          <t>Jim Cramer Couldn’t Stop Gushing About This Computer Hardware AI Stock</t>
+        </is>
+      </c>
+      <c r="AY33" s="90" t="inlineStr">
+        <is>
           <t>DELL Stock Hits 52-Week High: Does it Have More Room to Run?</t>
         </is>
       </c>
-      <c r="AY33" s="90" t="inlineStr">
+      <c r="AZ33" s="90" t="inlineStr">
         <is>
           <t>Super Micro Surges 7% as Semiconductors Lead a Flat Tape; Hewlett Packard Enterprise Falls 3%, Dell Edges H...</t>
-        </is>
-      </c>
-      <c r="AZ33" s="90" t="inlineStr">
-        <is>
-          <t>Dell Afterglow Continues. These Other Stocks Top Buy Points.</t>
         </is>
       </c>
     </row>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Jim Cramer Flagged Another Risk For Adobe Inc. (NASDAQ:ADBE)</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>Jim Cramer flagged one stock quietly concentrating portfolios</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
+      <c r="AZ34" s="79" t="inlineStr">
         <is>
           <t>Why IBM, Microsoft Back Move for Quantum Policy Czar</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Google Turns Three Everyday Apps Into Paid Gemini Microphones</t>
         </is>
       </c>
     </row>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
+          <t>Coatue Opened Positions in Intel and Cerebras. Is the AI Chip Trade Broadening Beyond NVIDIA?</t>
+        </is>
+      </c>
+      <c r="AY36" s="79" t="inlineStr">
+        <is>
           <t>Mizuho Resets Intel Target For the Rest of 2026</t>
         </is>
       </c>
-      <c r="AY36" s="79" t="inlineStr">
+      <c r="AZ36" s="79" t="inlineStr">
         <is>
           <t>Lone Star JV Spends $1.2B On 2M SF R&amp;D Portfolio In Silicon Valley</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>Why Intel Stock Popped Today</t>
         </is>
       </c>
     </row>
@@ -9404,12 +9404,12 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Flash Buy Signals; Apple, Inflation Reports Ahead</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
           <t>David Tepper Sold 41% of His Micron Shares and It Is Still His Second-Biggest Holding</t>
-        </is>
-      </c>
-      <c r="AY39" s="90" t="inlineStr">
-        <is>
-          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Flash Buy Signals; Apple, Inflation Reports Ahead</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Jim Cramer Believes Nvidia Corp. (NASDAQ:NVDA) Buying Back Half A Trillion Worth In Stock Would Be Great</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
+          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Flash Buy Signals; Apple, Inflation Reports Ahead</t>
+        </is>
+      </c>
+      <c r="AZ43" s="90" t="inlineStr">
+        <is>
           <t>Elon Musk Committed SpaceX to Building "Exclusively on Nvidia." Here's What That Locks In for SpaceX's Comp...</t>
-        </is>
-      </c>
-      <c r="AY43" s="90" t="inlineStr">
-        <is>
-          <t>AI compute provider Nscale is looking for $3.5B in pre-IPO financing</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Flash Buy Signals; Apple, Inflation Reports Ahead</t>
         </is>
       </c>
     </row>
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Flash Buy Signals; Apple, Inflation Reports Ahead</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
           <t>Stock Market Today: Dow Sinks Amid Rate Fears; Sandisk, KLA Lead Nasdaq-100 As Utilities Gain</t>
         </is>
       </c>
-      <c r="AY47" s="90" t="inlineStr">
+      <c r="AZ47" s="90" t="inlineStr">
         <is>
           <t>Analyst Has Strong Take on Micron, SanDisk Stocks</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>Micron, SanDisk Lead Memory Chip Stocks Rally on Strong AI Demand</t>
         </is>
       </c>
     </row>
@@ -11101,12 +11101,12 @@
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
+          <t>Tesla Launched the Cybercab Thursday, 6 Weeks After Removing Volume Production of It From This Year's Plan</t>
+        </is>
+      </c>
+      <c r="AZ48" s="79" t="inlineStr">
+        <is>
           <t>From Launch Party to Federal Probe: What Went Wrong With Tesla's Cybercab in 24 Hours</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Tesla (TSLA) Falls More Steeply Than Broader Market: What Investors Need to Know</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 4 Sep 2026, 10:23 PM · Yahoo Finance data</t>
+          <t>Built 4 Sep 2026, 11:02 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 4 Sep 2026, 10:23 PM · Yahoo Finance data</t>
+          <t>Built 4 Sep 2026, 11:02 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 4 Sep 2026, 10:23 PM · Yahoo Finance data</t>
+          <t>Built 4 Sep 2026, 11:02 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 4 Sep 2026, 10:23 PM · Yahoo Finance data</t>
+          <t>Built 4 Sep 2026, 11:02 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-07 20:41 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'09-01'!$5:$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'08-31'!$A$6:$AZ$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'08-31'!$5:$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 4 Sep 2026, 11:02 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 7 Sep 2026, 08:41 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1404,7 +1404,7 @@
       <c r="P8" s="10" t="n"/>
       <c r="Q8" s="16" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>38</t>
         </is>
       </c>
       <c r="R8" s="12" t="n"/>
@@ -2018,14 +2018,14 @@
     <row r="31">
       <c r="B31" s="24" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C31" s="26" t="n">
-        <v>0.07482312178459227</v>
+        <v>0.00836070775935327</v>
       </c>
       <c r="D31" s="27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E31" s="23" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="F31" s="28" t="n">
-        <v>53.52927511621272</v>
+        <v>60.39157103041679</v>
       </c>
       <c r="H31" s="24" t="inlineStr">
         <is>
@@ -2058,11 +2058,11 @@
     <row r="32">
       <c r="B32" s="31" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="C32" s="33" t="n">
-        <v>0.04505296133202719</v>
+        <v>0.07482312178459227</v>
       </c>
       <c r="D32" s="34" t="n">
         <v>8</v>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="F32" s="35" t="n">
-        <v>51.7442898847969</v>
+        <v>53.52927511621272</v>
       </c>
       <c r="H32" s="31" t="inlineStr">
         <is>
@@ -2098,11 +2098,11 @@
     <row r="33">
       <c r="B33" s="24" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="C33" s="26" t="n">
-        <v>0.0150080361357805</v>
+        <v>0.04505296133202719</v>
       </c>
       <c r="D33" s="27" t="n">
         <v>8</v>
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="F33" s="28" t="n">
-        <v>63.66351534495513</v>
+        <v>51.7442898847969</v>
       </c>
       <c r="H33" s="24" t="inlineStr">
         <is>
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="I33" s="26" t="n">
-        <v>0.002057860185984861</v>
+        <v>0.002071873185092388</v>
       </c>
       <c r="J33" s="27" t="n">
         <v>1</v>
@@ -2132,17 +2132,17 @@
         </is>
       </c>
       <c r="L33" s="28" t="n">
-        <v>38.04345929080058</v>
+        <v>38.04705952649971</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="31" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="C34" s="33" t="n">
-        <v>0.00836070775935327</v>
+        <v>0.0150080361357805</v>
       </c>
       <c r="D34" s="34" t="n">
         <v>8</v>
@@ -2153,7 +2153,7 @@
         </is>
       </c>
       <c r="F34" s="35" t="n">
-        <v>60.39157103041679</v>
+        <v>63.66351534495513</v>
       </c>
       <c r="H34" s="31" t="inlineStr">
         <is>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 4 Sep 2026, 11:02 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 08:41 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3614,16 +3614,16 @@
         <v>174.3399963378906</v>
       </c>
       <c r="U7" s="72" t="n">
-        <v>175.7749938964844</v>
+        <v>175.7799987792969</v>
       </c>
       <c r="V7" s="72" t="n">
         <v>174.1000061035156</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>5807775</v>
+        <v>5841600</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>0.9194254555600739</v>
+        <v>0.9245327363500614</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>38.89644652840126</v>
@@ -3632,7 +3632,7 @@
         <v>26.14618481270283</v>
       </c>
       <c r="AA7" s="28" t="n">
-        <v>25.67048740529762</v>
+        <v>25.66774107790977</v>
       </c>
       <c r="AB7" s="75" t="n">
         <v>-2.150334477861264</v>
@@ -3674,7 +3674,7 @@
         <v>10.09407349005902</v>
       </c>
       <c r="AO7" s="77" t="n">
-        <v>1.399426741109238</v>
+        <v>1.399630707344618</v>
       </c>
       <c r="AP7" s="72" t="n">
         <v>188.1900024414062</v>
@@ -3804,16 +3804,16 @@
         <v>171.3899993896484</v>
       </c>
       <c r="U8" s="83" t="n">
-        <v>172.5325012207031</v>
+        <v>172.5299987792969</v>
       </c>
       <c r="V8" s="83" t="n">
-        <v>171.2350006103516</v>
+        <v>171.2400054931641</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>6068699</v>
+        <v>6083000</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.8220440424387842</v>
+        <v>0.823901402718211</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>55.49904605891764</v>
@@ -3822,7 +3822,7 @@
         <v>36.80977460079121</v>
       </c>
       <c r="AA8" s="35" t="n">
-        <v>27.21330025120935</v>
+        <v>27.21565887309683</v>
       </c>
       <c r="AB8" s="86" t="n">
         <v>2.171795734698321</v>
@@ -3864,7 +3864,7 @@
         <v>6.242793151423582</v>
       </c>
       <c r="AO8" s="88" t="n">
-        <v>1.523066162305396</v>
+        <v>1.52285765158167</v>
       </c>
       <c r="AP8" s="83" t="n">
         <v>176.6000061035156</v>
@@ -4000,10 +4000,10 @@
         <v>57.91999816894531</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>26249596</v>
+        <v>26345200</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>0.9465192594140487</v>
+        <v>0.9498028754888005</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>55.48490520235243</v>
@@ -4187,13 +4187,13 @@
         <v>64.33000183105469</v>
       </c>
       <c r="V10" s="83" t="n">
-        <v>63.375</v>
+        <v>63.38000106811523</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>26088239</v>
+        <v>26281800</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>1.015822317560993</v>
+        <v>1.022973683585705</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>63.1419828676078</v>
@@ -4202,7 +4202,7 @@
         <v>65.32064786499038</v>
       </c>
       <c r="AA10" s="35" t="n">
-        <v>27.79215071422096</v>
+        <v>27.79717980666603</v>
       </c>
       <c r="AB10" s="86" t="n">
         <v>1.431671632215661</v>
@@ -4244,7 +4244,7 @@
         <v>8.62123254027785</v>
       </c>
       <c r="AO10" s="88" t="n">
-        <v>1.830732073401575</v>
+        <v>1.830174441236882</v>
       </c>
       <c r="AP10" s="83" t="n">
         <v>65.51999664306641</v>
@@ -4374,16 +4374,16 @@
         <v>84.81999969482422</v>
       </c>
       <c r="U11" s="72" t="n">
-        <v>85.29000091552734</v>
+        <v>85.30000305175781</v>
       </c>
       <c r="V11" s="72" t="n">
         <v>84.54000091552734</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>9823945</v>
+        <v>9903700</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.11131011260251</v>
+        <v>1.11982704570523</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>45.23385101242543</v>
@@ -4434,7 +4434,7 @@
         <v>3.392922385647933</v>
       </c>
       <c r="AO11" s="77" t="n">
-        <v>1.29785730515503</v>
+        <v>1.298701994545795</v>
       </c>
       <c r="AP11" s="72" t="n">
         <v>90.13999938964844</v>
@@ -4570,10 +4570,10 @@
         <v>114.4599990844727</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>5071369</v>
+        <v>5120000</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>1.013169759045266</v>
+        <v>1.022388715384554</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>44.57163034145746</v>
@@ -4757,13 +4757,13 @@
         <v>113.2900009155273</v>
       </c>
       <c r="V13" s="72" t="n">
-        <v>111.879997253418</v>
+        <v>111.875</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>2683037</v>
+        <v>2689600</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>0.6729645801653736</v>
+        <v>0.674555203876385</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>51.76547604388368</v>
@@ -4772,7 +4772,7 @@
         <v>44.05936574062708</v>
       </c>
       <c r="AA13" s="28" t="n">
-        <v>13.60542362334407</v>
+        <v>13.60236670559791</v>
       </c>
       <c r="AB13" s="75" t="n">
         <v>0.4768781871747763</v>
@@ -4814,7 +4814,7 @@
         <v>3.312441843346797</v>
       </c>
       <c r="AO13" s="77" t="n">
-        <v>1.516502792182393</v>
+        <v>1.516821409228364</v>
       </c>
       <c r="AP13" s="72" t="n">
         <v>120.4049987792969</v>
@@ -4947,13 +4947,13 @@
         <v>52.66999816894531</v>
       </c>
       <c r="V14" s="83" t="n">
-        <v>51.97499847412109</v>
+        <v>51.97999954223633</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>10873762</v>
+        <v>10873800</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>1.00518864889215</v>
+        <v>1.00519198512429</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>49.4676143244987</v>
@@ -4962,7 +4962,7 @@
         <v>28.27864815807864</v>
       </c>
       <c r="AA14" s="35" t="n">
-        <v>14.67800803150836</v>
+        <v>14.68486547704828</v>
       </c>
       <c r="AB14" s="86" t="n">
         <v>0.2304403794357057</v>
@@ -5004,7 +5004,7 @@
         <v>4.093904564425986</v>
       </c>
       <c r="AO14" s="88" t="n">
-        <v>1.607810943237288</v>
+        <v>1.607129747279159</v>
       </c>
       <c r="AP14" s="83" t="n">
         <v>54.18999862670898</v>
@@ -5140,10 +5140,10 @@
         <v>186.4199981689453</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>5081462</v>
+        <v>5103800</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>0.8491878409696834</v>
+        <v>0.8527616843705749</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>55.29688065294555</v>
@@ -5222,12 +5222,12 @@
       </c>
       <c r="AX15" s="79" t="inlineStr">
         <is>
+          <t>Sector Update: Tech Stocks Rise Late Afternoon</t>
+        </is>
+      </c>
+      <c r="AY15" s="79" t="inlineStr">
+        <is>
           <t>Blowout jobs report raises worries of Fed rate hike: AlphaCheck</t>
-        </is>
-      </c>
-      <c r="AY15" s="79" t="inlineStr">
-        <is>
-          <t>Sector Update: Tech Stocks Rise Late Afternoon</t>
         </is>
       </c>
       <c r="AZ15" s="79" t="inlineStr">
@@ -5324,16 +5324,16 @@
         <v>44.04000091552734</v>
       </c>
       <c r="U16" s="83" t="n">
-        <v>44.27500152587891</v>
+        <v>44.27999877929688</v>
       </c>
       <c r="V16" s="83" t="n">
         <v>43.875</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>3761109</v>
+        <v>3829200</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>0.7318342943625612</v>
+        <v>0.7445901419391973</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>40.1911612158916</v>
@@ -5342,7 +5342,7 @@
         <v>19.21059922822713</v>
       </c>
       <c r="AA16" s="35" t="n">
-        <v>15.03752197299594</v>
+        <v>15.02292579591458</v>
       </c>
       <c r="AB16" s="86" t="n">
         <v>-0.2422262788982081</v>
@@ -5384,7 +5384,7 @@
         <v>4.440833217234127</v>
       </c>
       <c r="AO16" s="88" t="n">
-        <v>1.173863809120602</v>
+        <v>1.174676344222428</v>
       </c>
       <c r="AP16" s="83" t="n">
         <v>46.45500183105469</v>
@@ -5517,13 +5517,13 @@
         <v>43.22999954223633</v>
       </c>
       <c r="V17" s="72" t="n">
-        <v>42.7599983215332</v>
+        <v>42.75</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>18838974</v>
+        <v>18858100</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>0.935472252533345</v>
+        <v>0.9363775123613292</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>43.93351550138382</v>
@@ -5574,7 +5574,7 @@
         <v>5.392769992681686</v>
       </c>
       <c r="AO17" s="77" t="n">
-        <v>1.470195056267271</v>
+        <v>1.471852822733022</v>
       </c>
       <c r="AP17" s="72" t="n">
         <v>47.79999923706055</v>
@@ -5729,10 +5729,10 @@
         <v>769</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>32960393</v>
+        <v>34015600</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.908793946613346</v>
+        <v>0.9365260466110001</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>55.61138482356586</v>
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
-          <t>S&amp;P 500, Dow End Lower As Blowout Jobs Report Fans Rate Hike Fears, While Chipmaker Strength Aids Nasdaq —T...</t>
+          <t>IBB Just Beat the S&amp;P 500 by 22 Points in Three Months. Are You Late to the Party?</t>
         </is>
       </c>
       <c r="AY19" s="79" t="inlineStr">
         <is>
-          <t>This Is the Most Expensive Market in Decades. Is It Really Safe to Invest Right Now?</t>
+          <t>Microsoft Is Close to a New All-Time High. This Number Will Determine If It Keeps Climbing</t>
         </is>
       </c>
       <c r="AZ19" s="79" t="inlineStr">
         <is>
-          <t>GoPro Zooms 34% Higher on Starman Optical Merger and Markiplier Stake; Coherent Climbs 7%, Lumentum Gains 3%</t>
+          <t>Roblox Has Collapsed 47% This Year: Is It Time to Switch to Take-Two or GameStop?</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5908,7 @@
         <v>1.2900390625</v>
       </c>
       <c r="T20" s="83" t="n">
-        <v>719.3599853515625</v>
+        <v>719.3499755859375</v>
       </c>
       <c r="U20" s="83" t="n">
         <v>721.8599853515625</v>
@@ -5917,10 +5917,10 @@
         <v>716.5599975585938</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>32489892</v>
+        <v>32784600</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>1.05579885949037</v>
+        <v>1.06486585157502</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>53.61942940327157</v>
@@ -5999,17 +5999,17 @@
       </c>
       <c r="AX20" s="90" t="inlineStr">
         <is>
+          <t>This ETF Would Have Increased Your Investment by 6x Over the Past 10 Years -- and It's Still Soaring</t>
+        </is>
+      </c>
+      <c r="AY20" s="90" t="inlineStr">
+        <is>
+          <t>The VIX Is Playing Tricks: Why Stocks Are Volatile, But the Fear Gauge Is Sleeping</t>
+        </is>
+      </c>
+      <c r="AZ20" s="90" t="inlineStr">
+        <is>
           <t>Exchange-Traded Funds Mixed, US Equities Lower After Midday</t>
-        </is>
-      </c>
-      <c r="AY20" s="90" t="inlineStr">
-        <is>
-          <t>GoPro Zooms 34% Higher on Starman Optical Merger and Markiplier Stake; Coherent Climbs 7%, Lumentum Gains 3%</t>
-        </is>
-      </c>
-      <c r="AZ20" s="90" t="inlineStr">
-        <is>
-          <t>SCHG Owns More Apple Than Tesla, Meta and Palantir Combined. Is That Why Growth Investors Are Falling Behind?</t>
         </is>
       </c>
     </row>
@@ -6102,13 +6102,13 @@
         <v>296.1799926757812</v>
       </c>
       <c r="V21" s="72" t="n">
-        <v>293.5700073242188</v>
+        <v>293.5599975585938</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>13897211</v>
+        <v>13951100</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>0.8313961430271718</v>
+        <v>0.8344855204251892</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>48.14623240653629</v>
@@ -6159,7 +6159,7 @@
         <v>4.920574083904603</v>
       </c>
       <c r="AO21" s="77" t="n">
-        <v>1.113740340880568</v>
+        <v>1.113981881110743</v>
       </c>
       <c r="AP21" s="72" t="n">
         <v>305.1799926757812</v>
@@ -6187,17 +6187,17 @@
       </c>
       <c r="AX21" s="79" t="inlineStr">
         <is>
+          <t>3 ETFs That Could Move as Rate Expectations Shift</t>
+        </is>
+      </c>
+      <c r="AY21" s="79" t="inlineStr">
+        <is>
           <t>Forget IWM: The Small-Cap Fund That Screens Out Money-Losers Charges 84% Less, and It’s Winning by 2.5 Points</t>
         </is>
       </c>
-      <c r="AY21" s="79" t="inlineStr">
+      <c r="AZ21" s="79" t="inlineStr">
         <is>
           <t>Small Caps Pay Too: The 42% Friday Payer Riding the Russell’s Big Year</t>
-        </is>
-      </c>
-      <c r="AZ21" s="79" t="inlineStr">
-        <is>
-          <t>Small Caps Are Beating the S&amp;P for Once. This Fund Pays 14% While They Run</t>
         </is>
       </c>
     </row>
@@ -6287,16 +6287,16 @@
         <v>111.2200012207031</v>
       </c>
       <c r="U22" s="83" t="n">
-        <v>118.1750030517578</v>
+        <v>118.1800003051758</v>
       </c>
       <c r="V22" s="83" t="n">
-        <v>109.75</v>
+        <v>109.7300033569336</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>62998272</v>
+        <v>63251400</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>1.159165591762556</v>
+        <v>1.163552171650776</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>45.44506021968484</v>
@@ -6305,7 +6305,7 @@
         <v>47.87068862423708</v>
       </c>
       <c r="AA22" s="35" t="n">
-        <v>19.58635703872865</v>
+        <v>19.58597074313625</v>
       </c>
       <c r="AB22" s="86" t="n">
         <v>-9.817400463372863</v>
@@ -6347,7 +6347,7 @@
         <v>44.11439815483754</v>
       </c>
       <c r="AO22" s="88" t="n">
-        <v>11.64831211952354</v>
+        <v>11.6486164737838</v>
       </c>
       <c r="AP22" s="83" t="n">
         <v>302</v>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
@@ -6493,7 +6493,7 @@
         <v>-8.239990234375</v>
       </c>
       <c r="T24" s="72" t="n">
-        <v>328.3049926757812</v>
+        <v>328.3099975585938</v>
       </c>
       <c r="U24" s="72" t="n">
         <v>328.9299926757812</v>
@@ -6502,10 +6502,10 @@
         <v>317.8599853515625</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>38272821</v>
+        <v>39551800</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.9667505992467851</v>
+        <v>0.9974457220667698</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>53.88621122935447</v>
@@ -6584,17 +6584,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
-          <t>Apple's John Ternus needs to be his own type of CEO and 'not Tim Cook 2'</t>
+          <t>KeyBanc Delivers Stark Warning on Apple Stock Ahead of iPhone 18 Launch</t>
         </is>
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Flash Buy Signals; Apple, Inflation Reports Ahead</t>
+          <t>Apple’s new CEO faces a staggering $14 billion iPhone test</t>
         </is>
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Why Apple (AAPL) Dipped More Than Broader Market Today</t>
+          <t>Apple Faces Its Biggest iPhone Test in Years -- Morgan Stanley Sees $14B Foldable Opportunity</t>
         </is>
       </c>
     </row>
@@ -6690,10 +6690,10 @@
         <v>458</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>19364684</v>
+        <v>19651900</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>1.10719337981666</v>
+        <v>1.12269338094845</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>49.6732371841989</v>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>Intel Climbs 4%, AMD Rises 3%, NVIDIA Ticks Up as Chip Stocks Shrug Off Rising Rate Hike Odds</t>
+          <t>Wall Street Is Worried About AMD. Here’s Why Long-Term Investors Shouldn’t Be</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
-          <t>Cathie Wood Cuts AMD and Puts $53 Million Into Nvidia</t>
+          <t>AMD Is Behind The AI Chip Shift Nobody Is Talking About</t>
         </is>
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>ORCL Eyes Breakout as AMD and Intel Test Key Support</t>
+          <t>AMD’s Whole AI Story Has One Threat It Cannot Ignore: Broadcom</t>
         </is>
       </c>
     </row>
@@ -6869,7 +6869,7 @@
         <v>-0.389984130859375</v>
       </c>
       <c r="T26" s="72" t="n">
-        <v>259.2149963378906</v>
+        <v>259.0700073242188</v>
       </c>
       <c r="U26" s="72" t="n">
         <v>261.1199951171875</v>
@@ -6878,10 +6878,10 @@
         <v>255.2899932861328</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>29968655</v>
+        <v>30698000</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.9175878288958084</v>
+        <v>0.9388707890469152</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>49.54908461556442</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
-          <t>Amazon's $100 Billion Anthropic Contract Gets a 45% Cheaper Engine</t>
+          <t>Fatal Amazon Plane Crash Delays Hundreds of Miami Flights</t>
         </is>
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Cramer Says the Magnificent Seven Are Finally Cheap and Most Investors Will Miss It</t>
+          <t>Are Retail-Wholesale Stocks Lagging Amazon.com (AMZN) This Year?</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>DOJ expands beef price probe to eight retailers, including Walmart and Amazon, with inflation a key issue a...</t>
+          <t>Amazon.com, Inc. (AMZN) is Attracting Investor Attention: Here is What You Should Know</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>85.80000305175781</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>3440341</v>
+        <v>3450700</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>0.7343095758532827</v>
+        <v>0.7364391958008005</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>58.3459649207801</v>
@@ -7148,17 +7148,17 @@
       </c>
       <c r="AX27" s="90" t="inlineStr">
         <is>
-          <t>Cathie Wood buys $44.5 million of tumbling tech stock</t>
+          <t>Cathie Wood buys $3.5 million of surging tech stock</t>
         </is>
       </c>
       <c r="AY27" s="90" t="inlineStr">
         <is>
-          <t>Nvidia Blew Wall Street Away with Its Q2 Results. Cathie Wood Is Celebrating by Buying More Than 243,000 Sh...</t>
+          <t>Cathie Wood's 2 Biggest Positions Are Both Elon Musk Companies. Together They Are 16% of the Fund.</t>
         </is>
       </c>
       <c r="AZ27" s="90" t="inlineStr">
         <is>
-          <t>Cathie Wood's Ark Has Delivered Just a 13.8% Annualized Return Since 2014, Roughly Matching the S&amp;P 500. Sh...</t>
+          <t>Cathie Wood’s Ark Invest Buys HOOD Stock As Robinhood Sees Its Third-Best Week In Six Months</t>
         </is>
       </c>
     </row>
@@ -7245,7 +7245,7 @@
         <v>9.5</v>
       </c>
       <c r="T28" s="72" t="n">
-        <v>248.8390045166016</v>
+        <v>248.5899963378906</v>
       </c>
       <c r="U28" s="72" t="n">
         <v>255.6900024414062</v>
@@ -7254,10 +7254,10 @@
         <v>247.5099945068359</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>4120464</v>
+        <v>4126100</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>1.131635532891704</v>
+        <v>1.133095698405027</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>47.95177147980165</v>
@@ -7336,17 +7336,17 @@
       </c>
       <c r="AX28" s="79" t="inlineStr">
         <is>
+          <t>Arm Expands Into AI Accelerators With Samsung — But It’s Not the Data Center Goldmine Investors Hope For</t>
+        </is>
+      </c>
+      <c r="AY28" s="79" t="inlineStr">
+        <is>
+          <t>Rising CPU Demand Positions Arm Holdings (ARM) for Gains</t>
+        </is>
+      </c>
+      <c r="AZ28" s="79" t="inlineStr">
+        <is>
           <t>Can ARM's AGI CPU Push Unlock $15B in Revenues by FY'31?</t>
-        </is>
-      </c>
-      <c r="AY28" s="79" t="inlineStr">
-        <is>
-          <t>ARM vs. Sandisk: Comparing Steady Historical Revenue Generation Against Rapid Sequential Revenue Expansion</t>
-        </is>
-      </c>
-      <c r="AZ28" s="79" t="inlineStr">
-        <is>
-          <t>Why Arm Holdings Stock Fell on Tuesday</t>
         </is>
       </c>
     </row>
@@ -7433,19 +7433,19 @@
         <v>0.1800003051757812</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>63.43999862670898</v>
+        <v>63.40000152587891</v>
       </c>
       <c r="U29" s="83" t="n">
-        <v>65.75</v>
+        <v>65.76000213623047</v>
       </c>
       <c r="V29" s="83" t="n">
         <v>61.66999816894531</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>10104414</v>
+        <v>10216600</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>0.9991953859870389</v>
+        <v>1.009729041643935</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>47.16085559699919</v>
@@ -7454,7 +7454,7 @@
         <v>45.90278931238216</v>
       </c>
       <c r="AA29" s="35" t="n">
-        <v>13.53102658052938</v>
+        <v>13.53342673358475</v>
       </c>
       <c r="AB29" s="86" t="n">
         <v>-2.047894896957622</v>
@@ -7496,7 +7496,7 @@
         <v>31.50978950370434</v>
       </c>
       <c r="AO29" s="88" t="n">
-        <v>7.301854407621104</v>
+        <v>7.303000994503515</v>
       </c>
       <c r="AP29" s="83" t="n">
         <v>133.8600006103516</v>
@@ -7524,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
-          <t>AST SpaceMobile vs. Space Exploration Technologies: Which Telecom Stock Is a Better Buy in 2026?</t>
+          <t>AST SpaceMobile Director Adriana Cisneros Buys $619,235 Shares. What Does This Mean for Investors?</t>
         </is>
       </c>
       <c r="AY29" s="90" t="inlineStr">
         <is>
-          <t>SPCX Stock Blasts Past ASTS, RKLB, LUNR, PL — Here’s Everything Shaking Up Space Stocks This Week</t>
+          <t>The Real Satellite Race Isn’t About Rockets — It’s About Who Controls the Spectrum in Your Phone</t>
         </is>
       </c>
       <c r="AZ29" s="90" t="inlineStr">
         <is>
-          <t>ASTS Stock Is Surging on a New Analyst Target. Here’s How High It Can Soar.</t>
+          <t>Forget Starlink? Japan’s $1 Billion BlueBird Play Makes ASTS the National Satellite OS</t>
         </is>
       </c>
     </row>
@@ -7546,7 +7546,7 @@
         </is>
       </c>
       <c r="C30" s="26" t="n">
-        <v>0.002057860185984861</v>
+        <v>0.002071873185092388</v>
       </c>
       <c r="D30" s="27" t="n">
         <v>14</v>
@@ -7615,76 +7615,76 @@
         </is>
       </c>
       <c r="R30" s="70" t="n">
-        <v>357.8949890136719</v>
+        <v>357.8999938964844</v>
       </c>
       <c r="S30" s="71" t="n">
-        <v>0.7349853515625</v>
+        <v>0.739990234375</v>
       </c>
       <c r="T30" s="72" t="n">
-        <v>360.0050048828125</v>
+        <v>359.7000122070312</v>
       </c>
       <c r="U30" s="72" t="n">
-        <v>360.0450134277344</v>
+        <v>360.1600036621094</v>
       </c>
       <c r="V30" s="72" t="n">
         <v>353.7000122070312</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>32481307</v>
+        <v>32773600</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>1.385842174155349</v>
+        <v>1.397441730266662</v>
       </c>
       <c r="Y30" s="28" t="n">
-        <v>38.04345929080058</v>
+        <v>38.04705952649971</v>
       </c>
       <c r="Z30" s="28" t="n">
-        <v>35.82278036480611</v>
+        <v>35.83429907920521</v>
       </c>
       <c r="AA30" s="28" t="n">
-        <v>23.72914532271137</v>
+        <v>23.71759503882551</v>
       </c>
       <c r="AB30" s="75" t="n">
-        <v>-8.805086820661245</v>
+        <v>-8.804687570750275</v>
       </c>
       <c r="AC30" s="75" t="n">
-        <v>-7.415563695108411</v>
+        <v>-7.415483845126216</v>
       </c>
       <c r="AD30" s="75" t="n">
-        <v>-1.389523125552834</v>
+        <v>-1.389203725624059</v>
       </c>
       <c r="AE30" s="72" t="n">
-        <v>364.4621078185942</v>
+        <v>364.4632200147747</v>
       </c>
       <c r="AF30" s="72" t="n">
-        <v>374.1247507870768</v>
+        <v>374.1252057764234</v>
       </c>
       <c r="AG30" s="72" t="n">
-        <v>383.661499633789</v>
+        <v>383.6615997314453</v>
       </c>
       <c r="AH30" s="72" t="n">
-        <v>398.1304507446289</v>
+        <v>398.130500793457</v>
       </c>
       <c r="AI30" s="72" t="n">
-        <v>369.8336253356933</v>
+        <v>369.8336503601074</v>
       </c>
       <c r="AJ30" s="72" t="n">
-        <v>422.932819448747</v>
+        <v>422.9326113622287</v>
       </c>
       <c r="AK30" s="72" t="n">
-        <v>378.3232482910156</v>
+        <v>378.3234985351563</v>
       </c>
       <c r="AL30" s="72" t="n">
-        <v>333.7136771332842</v>
+        <v>333.7143857080838</v>
       </c>
       <c r="AM30" s="76" t="n">
-        <v>0.2710327767429874</v>
+        <v>0.2710837164836281</v>
       </c>
       <c r="AN30" s="29" t="n">
-        <v>23.58278078825152</v>
+        <v>23.58252289365901</v>
       </c>
       <c r="AO30" s="77" t="n">
-        <v>3.637457540758624</v>
+        <v>3.639701613912953</v>
       </c>
       <c r="AP30" s="72" t="n">
         <v>495</v>
@@ -7693,36 +7693,36 @@
         <v>289.9599914550781</v>
       </c>
       <c r="AR30" s="29" t="n">
-        <v>-27.69798201744003</v>
+        <v>-27.69697093000316</v>
       </c>
       <c r="AS30" s="78" t="n">
-        <v>33.13255692910781</v>
+        <v>33.13499785897706</v>
       </c>
       <c r="AT30" s="26" t="n">
-        <v>-0.02954261037124295</v>
+        <v>-0.02952903928011652</v>
       </c>
       <c r="AU30" s="26" t="n">
-        <v>-0.1490239846376646</v>
+        <v>-0.1490120844005451</v>
       </c>
       <c r="AV30" s="26" t="n">
-        <v>-0.07216192979509406</v>
+        <v>-0.07214895470197202</v>
       </c>
       <c r="AW30" s="26" t="n">
-        <v>0.03407969575888559</v>
+        <v>0.03409415655843562</v>
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
-          <t>Jim Cramer Says “Someone Must Know Something” About Broadcom Inc. (NASDAQ:AVGO)’s Post-Earnings Share Dip</t>
+          <t>Broadcom Inc. (AVGO)’s AI Opportunity Expands Across AI Infrastructure</t>
         </is>
       </c>
       <c r="AY30" s="79" t="inlineStr">
         <is>
-          <t>Top Research Reports for Apple, Broadcom &amp; Shell</t>
+          <t>Broadcom vs Marvell: One of These AI Chip Stocks Is a Clear Winner</t>
         </is>
       </c>
       <c r="AZ30" s="79" t="inlineStr">
         <is>
-          <t>5-star analyst resets Broadcom stock price target</t>
+          <t>Broadcom Inc. (AVGO) Is a Trending Stock: Facts to Know Before Betting on It</t>
         </is>
       </c>
     </row>
@@ -7815,13 +7815,13 @@
         <v>101.5400009155273</v>
       </c>
       <c r="V31" s="83" t="n">
-        <v>99.61000061035156</v>
+        <v>99.51999664306641</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>1550370</v>
+        <v>1554900</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.5842640228057313</v>
+        <v>0.5859211612159305</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>54.05207932909197</v>
@@ -7872,7 +7872,7 @@
         <v>14.00692232542185</v>
       </c>
       <c r="AO31" s="88" t="n">
-        <v>3.951729625582283</v>
+        <v>3.958111256456225</v>
       </c>
       <c r="AP31" s="83" t="n">
         <v>135.2400054931641</v>
@@ -7997,7 +7997,7 @@
         <v>4.800003051757812</v>
       </c>
       <c r="T32" s="72" t="n">
-        <v>85.98000335693359</v>
+        <v>85.72499847412109</v>
       </c>
       <c r="U32" s="72" t="n">
         <v>89.62999725341797</v>
@@ -8006,10 +8006,10 @@
         <v>84.90000152587891</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>20537770</v>
+        <v>20732400</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>0.7541887865692521</v>
+        <v>0.7610640227433788</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>52.00788852164074</v>
@@ -8088,17 +8088,17 @@
       </c>
       <c r="AX32" s="79" t="inlineStr">
         <is>
-          <t>BigBear.ai vs. CoreWeave: Evaluating the Better Artificial Intelligence Stock to Buy for 2026</t>
+          <t>CRWV Stock Takes a 13% Hit in 3 Months: Time to Buy, Hold or Bail Out?</t>
         </is>
       </c>
       <c r="AY32" s="79" t="inlineStr">
         <is>
-          <t>CoreWeave to Participate in the Goldman Sachs Communacopia + Technology Conference</t>
+          <t>Nebius Stock Up 254% in a Year: Should You Buy, Hold or Sell?</t>
         </is>
       </c>
       <c r="AZ32" s="79" t="inlineStr">
         <is>
-          <t>CoreWeave (CRWV) Could Be 21% Overvalued After The Rescale Cloud Deal</t>
+          <t>Nvidia’s $99 Billion Portfolio Is Turning Intel and CoreWeave Into an AI Stress Test</t>
         </is>
       </c>
     </row>
@@ -8188,25 +8188,25 @@
         <v>513.780029296875</v>
       </c>
       <c r="U33" s="83" t="n">
-        <v>534.9600219726562</v>
+        <v>534.989990234375</v>
       </c>
       <c r="V33" s="83" t="n">
-        <v>510.2699890136719</v>
+        <v>510.1499938964844</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>10960031</v>
+        <v>11108300</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>1.318663912567873</v>
+        <v>1.335311965072221</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>63.66351534495513</v>
       </c>
       <c r="Z33" s="35" t="n">
-        <v>90.43070078416703</v>
+        <v>90.40673923250029</v>
       </c>
       <c r="AA33" s="35" t="n">
-        <v>9.865862732315552</v>
+        <v>9.866654611304808</v>
       </c>
       <c r="AB33" s="86" t="n">
         <v>15.7781744109642</v>
@@ -8248,19 +8248,19 @@
         <v>23.36758426314429</v>
       </c>
       <c r="AO33" s="88" t="n">
-        <v>6.121899206618705</v>
+        <v>6.123942872361161</v>
       </c>
       <c r="AP33" s="83" t="n">
-        <v>534.9600219726562</v>
+        <v>534.989990234375</v>
       </c>
       <c r="AQ33" s="83" t="n">
         <v>110.2200012207031</v>
       </c>
       <c r="AR33" s="36" t="n">
-        <v>-2.022582413601703</v>
+        <v>-2.028070764685563</v>
       </c>
       <c r="AS33" s="89" t="n">
-        <v>97.45255761275729</v>
+        <v>97.44568216527456</v>
       </c>
       <c r="AT33" s="33" t="n">
         <v>0.1488252364269551</v>
@@ -8276,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
-          <t>Jim Cramer Couldn’t Stop Gushing About This Computer Hardware AI Stock</t>
+          <t>Dell &amp; 2 Momentum Stocks to Buy Now for Explosive Upside</t>
         </is>
       </c>
       <c r="AY33" s="90" t="inlineStr">
         <is>
-          <t>DELL Stock Hits 52-Week High: Does it Have More Room to Run?</t>
+          <t>Jim Cramer Explains Why “Buyers Flocked in” for Dell (DELL)</t>
         </is>
       </c>
       <c r="AZ33" s="90" t="inlineStr">
         <is>
-          <t>Super Micro Surges 7% as Semiconductors Lead a Flat Tape; Hewlett Packard Enterprise Falls 3%, Dell Edges H...</t>
+          <t>DELL Expands Consumer PC Reach: Can It Challenge HPQ &amp; AAPL?</t>
         </is>
       </c>
     </row>
@@ -8310,7 +8310,7 @@
       </c>
       <c r="F34" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Same</t>
         </is>
       </c>
       <c r="G34" s="23" t="inlineStr">
@@ -8373,7 +8373,7 @@
         <v>-3.769989013671875</v>
       </c>
       <c r="T34" s="72" t="n">
-        <v>339.2049865722656</v>
+        <v>339.1799926757812</v>
       </c>
       <c r="U34" s="72" t="n">
         <v>340.1799926757812</v>
@@ -8382,10 +8382,10 @@
         <v>333.75</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>12195409</v>
+        <v>12676800</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.806290417278123</v>
+        <v>0.836785615271892</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>43.96862904014093</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
-          <t>Jim Cramer Flagged Another Risk For Adobe Inc. (NASDAQ:ADBE)</t>
+          <t>Google-Backed Pixxel Raises $100 Million in India's Biggest Space-Tech Round</t>
         </is>
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
-          <t>Jim Cramer flagged one stock quietly concentrating portfolios</t>
+          <t>Alphabet May Be the Mag 7 Stock Investors Are Underestimating</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Why IBM, Microsoft Back Move for Quantum Policy Czar</t>
+          <t>Agentic Commerce Optimisation: Azoma on Which Platforms Help Brands Get Recommended by AI Shopping Agents</t>
         </is>
       </c>
     </row>
@@ -8561,7 +8561,7 @@
         <v>3.029998779296875</v>
       </c>
       <c r="T35" s="83" t="n">
-        <v>41.02000045776367</v>
+        <v>41.04999923706055</v>
       </c>
       <c r="U35" s="83" t="n">
         <v>44.74499893188477</v>
@@ -8570,10 +8570,10 @@
         <v>41</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>35805723</v>
+        <v>36132300</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>0.7812574030649195</v>
+        <v>0.7881023102382216</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>57.15950356150678</v>
@@ -8652,17 +8652,17 @@
       </c>
       <c r="AX35" s="90" t="inlineStr">
         <is>
-          <t>IREN Climbs 4% on $2.4B Blue Owl-Led GPU Financing; Cipher Digital Gains 2%</t>
+          <t>IREN Jumps 23% as Its AI Business Starts to Take Over the Story</t>
         </is>
       </c>
       <c r="AY35" s="90" t="inlineStr">
         <is>
-          <t>Blue Owl leads $2.4 billion IREN GPU financing at 9%</t>
+          <t>IREN’s AI Pricing Is Exploding — Why the Neocloud’s $2.6 Billion Contract Base Could Scale Dramatically</t>
         </is>
       </c>
       <c r="AZ35" s="90" t="inlineStr">
         <is>
-          <t>IREN obtains $2.4B private credit financing to buy Nvidia chips</t>
+          <t>APLD Slides 36% in 3 Months: Should Investors Exit or Hold the Stock?</t>
         </is>
       </c>
     </row>
@@ -8749,19 +8749,19 @@
         <v>4.1300048828125</v>
       </c>
       <c r="T36" s="72" t="n">
-        <v>92.36000061035156</v>
+        <v>92.44999694824219</v>
       </c>
       <c r="U36" s="72" t="n">
         <v>95.94000244140625</v>
       </c>
       <c r="V36" s="72" t="n">
-        <v>91.87010192871094</v>
+        <v>91.87000274658203</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>97018400</v>
+        <v>97428100</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.9915221009495907</v>
+        <v>0.995500796324208</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>51.7442898847969</v>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
-          <t>Coatue Opened Positions in Intel and Cerebras. Is the AI Chip Trade Broadening Beyond NVIDIA?</t>
+          <t>Prediction: Intel Stock Is Up Big in 2026. But the Best May Still Be Ahead</t>
         </is>
       </c>
       <c r="AY36" s="79" t="inlineStr">
         <is>
-          <t>Mizuho Resets Intel Target For the Rest of 2026</t>
+          <t>Nvidia just sent a strong signal to AMD and Intel investors</t>
         </is>
       </c>
       <c r="AZ36" s="79" t="inlineStr">
         <is>
-          <t>Lone Star JV Spends $1.2B On 2M SF R&amp;D Portfolio In Silicon Valley</t>
+          <t>AMD and Intel Soared as Nvidia Lagged: Has the AI Trade Changed?</t>
         </is>
       </c>
     </row>
@@ -8946,10 +8946,10 @@
         <v>499.3599853515625</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>17437000</v>
+        <v>18074400</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.7593015749291571</v>
+        <v>0.785966669993275</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>59.36327597001683</v>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
-          <t>Why IBM, Microsoft Back Move for Quantum Policy Czar</t>
+          <t>Nvidia, Microsoft at Center of $7 Trillion AI Boom</t>
         </is>
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
-          <t>Stifel Revamps Microsoft Target With a Catch</t>
+          <t>Microsoft Has a $1,000 Problem With Its Next Xbox</t>
         </is>
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>Microsoft Drops 1.6%, Opens Azure's $101.9 Billion Door</t>
+          <t>Microsoft Is Close to a New All-Time High. This Number Will Determine If It Keeps Climbing</t>
         </is>
       </c>
     </row>
@@ -9125,19 +9125,19 @@
         <v>-2.020004272460938</v>
       </c>
       <c r="T38" s="72" t="n">
-        <v>137.2200012207031</v>
+        <v>137.3500061035156</v>
       </c>
       <c r="U38" s="72" t="n">
         <v>144.3999938964844</v>
       </c>
       <c r="V38" s="72" t="n">
-        <v>137.0675048828125</v>
+        <v>137.0700073242188</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>26374686</v>
+        <v>27054700</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.9505035535867831</v>
+        <v>0.9738169729307915</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>66.19651579663915</v>
@@ -9188,7 +9188,7 @@
         <v>59.4034632349296</v>
       </c>
       <c r="AO38" s="77" t="n">
-        <v>6.064735586583529</v>
+        <v>6.064610414447036</v>
       </c>
       <c r="AP38" s="72" t="n">
         <v>365.2099914550781</v>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
-          <t>Bitmine Sinks 6%, Strategy Slips: Is the Crypto Treasury Trade Unwinding?</t>
+          <t>Strategy Is Down More Than 50% in 12 Months. One Analyst Thinks the Stock Is About to Triple</t>
         </is>
       </c>
       <c r="AY38" s="79" t="inlineStr">
         <is>
-          <t>Michael Saylor Says Strategy Now Has More Reserve Capital Than Every S&amp;P 500 Finance Giant Except Berkshire...</t>
+          <t>MicroStrategy Drops $250 Bitcoin Jordans. But You Can’t Buy With Crypto</t>
         </is>
       </c>
       <c r="AZ38" s="79" t="inlineStr">
         <is>
-          <t>Michael Saylor Says ‘We’re Back’ as Strategy Resumes Bitcoin Buying. What Comes Next for MSTR Stock.</t>
+          <t>Michael Saylor's Strategy Continues to Sell Bitcoin. That's Why I'm Doubling Down on Bitcoin Right Now.</t>
         </is>
       </c>
     </row>
@@ -9313,7 +9313,7 @@
         <v>58.4300537109375</v>
       </c>
       <c r="T39" s="83" t="n">
-        <v>971.0599975585938</v>
+        <v>971.3400268554688</v>
       </c>
       <c r="U39" s="83" t="n">
         <v>1017.77001953125</v>
@@ -9322,10 +9322,10 @@
         <v>969</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>34925945</v>
+        <v>35116600</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>1.261270266663148</v>
+        <v>1.267718917482713</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>60.14679067938084</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Flash Buy Signals; Apple, Inflation Reports Ahead</t>
+          <t>Is Micron Technology Stock Running Out of Steam?</t>
         </is>
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
-          <t>David Tepper Sold 41% of His Micron Shares and It Is Still His Second-Biggest Holding</t>
+          <t>Why Micron and SK Hynix Sit in the Most Valuable Spot in the Entire Compute Stack</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
         <is>
-          <t>Analyst Has Strong Take on Micron, SanDisk Stocks</t>
+          <t>Everyone Is Watching Nvidia. But This Memory Stock Could Be the Next AI Winner</t>
         </is>
       </c>
     </row>
@@ -9501,7 +9501,7 @@
         <v>15.75999450683594</v>
       </c>
       <c r="T40" s="72" t="n">
-        <v>209.8919982910156</v>
+        <v>210.1900024414062</v>
       </c>
       <c r="U40" s="72" t="n">
         <v>226.5800018310547</v>
@@ -9510,10 +9510,10 @@
         <v>209.4049987792969</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>14803876</v>
+        <v>14890300</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>0.677375245757632</v>
+        <v>0.6811950271477512</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>53.52927511621272</v>
@@ -9592,17 +9592,17 @@
       </c>
       <c r="AX40" s="79" t="inlineStr">
         <is>
+          <t>Nebius Stock Up 254% in a Year: Should You Buy, Hold or Sell?</t>
+        </is>
+      </c>
+      <c r="AY40" s="79" t="inlineStr">
+        <is>
           <t>Billionaire Stephen Mandel’s Top 2 AI Stock Picks</t>
         </is>
       </c>
-      <c r="AY40" s="79" t="inlineStr">
+      <c r="AZ40" s="79" t="inlineStr">
         <is>
           <t>CoreWeave vs. Nebius: Which AI Infrastructure Stock Is the Better Buy?</t>
-        </is>
-      </c>
-      <c r="AZ40" s="79" t="inlineStr">
-        <is>
-          <t>3 Founder Backed Growth Stocks To Watch In September 2026</t>
         </is>
       </c>
     </row>
@@ -9698,10 +9698,10 @@
         <v>78.23000335693359</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>39850506</v>
+        <v>40066200</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>1.421796834890664</v>
+        <v>1.428942594534659</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>49.16100735547449</v>
@@ -9780,17 +9780,17 @@
       </c>
       <c r="AX41" s="90" t="inlineStr">
         <is>
-          <t>Walt Disney vs. Netflix: Which Media Stock Is a Better Buy in 2026?</t>
+          <t>Is Netflix Stock More Likely to Hit $100 or $60 by the End of 2026?</t>
         </is>
       </c>
       <c r="AY41" s="90" t="inlineStr">
         <is>
-          <t>NFLX Stock Falls 4% As Netflix Hikes UK Subscription Prices — Region Accounts For About 20% Of EMEA Revenue</t>
+          <t>Investors Heavily Search Netflix, Inc. (NFLX): Here is What You Need to Know</t>
         </is>
       </c>
       <c r="AZ41" s="90" t="inlineStr">
         <is>
-          <t>Netflix subscription rises above £20 a month for first time</t>
+          <t>Netflix Has Momentum Despite Being Down in 2026. One Analyst’s Price Target Implies 70% Upside</t>
         </is>
       </c>
     </row>
@@ -9880,16 +9880,16 @@
         <v>10</v>
       </c>
       <c r="U42" s="72" t="n">
-        <v>10.10499954223633</v>
+        <v>10.10999965667725</v>
       </c>
       <c r="V42" s="72" t="n">
-        <v>9.932000160217285</v>
+        <v>9.930000305175781</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>45518995</v>
+        <v>45824000</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>0.6683527848122022</v>
+        <v>0.6726805300353824</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>47.17559913079245</v>
@@ -9898,7 +9898,7 @@
         <v>40.83332075012855</v>
       </c>
       <c r="AA42" s="28" t="n">
-        <v>12.55979865142888</v>
+        <v>12.54951106034842</v>
       </c>
       <c r="AB42" s="75" t="n">
         <v>-0.1271678064059536</v>
@@ -9940,7 +9940,7 @@
         <v>15.7948809207682</v>
       </c>
       <c r="AO42" s="77" t="n">
-        <v>4.493943217535415</v>
+        <v>4.497504045461661</v>
       </c>
       <c r="AP42" s="72" t="n">
         <v>17.45000076293945</v>
@@ -10041,7 +10041,7 @@
         </is>
       </c>
       <c r="N43" s="80" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O43" s="30" t="inlineStr">
         <is>
@@ -10065,7 +10065,7 @@
         <v>1.910003662109375</v>
       </c>
       <c r="T43" s="83" t="n">
-        <v>231.1419982910156</v>
+        <v>231.0899963378906</v>
       </c>
       <c r="U43" s="83" t="n">
         <v>234.7599945068359</v>
@@ -10074,10 +10074,10 @@
         <v>229.6300048828125</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>132204717</v>
+        <v>134946800</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>1.026731349422683</v>
+        <v>1.046912245494214</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>60.39157103041679</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Jim Cramer Believes Nvidia Corp. (NASDAQ:NVDA) Buying Back Half A Trillion Worth In Stock Would Be Great</t>
+          <t>Jim Cramer Discusses NVIDIA (NVDA) Acquiring Hugging Face</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Flash Buy Signals; Apple, Inflation Reports Ahead</t>
+          <t>Could This Vanguard Growth ETF Be a No-Brainer Buy for Long-Term Investors?</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Elon Musk Committed SpaceX to Building "Exclusively on Nvidia." Here's What That Locks In for SpaceX's Comp...</t>
+          <t>Nvidia, Microsoft at Center of $7 Trillion AI Boom</t>
         </is>
       </c>
     </row>
@@ -10253,7 +10253,7 @@
         <v>-8.199996948242188</v>
       </c>
       <c r="T44" s="72" t="n">
-        <v>180.0200042724609</v>
+        <v>180.0099945068359</v>
       </c>
       <c r="U44" s="72" t="n">
         <v>182.1900024414062</v>
@@ -10262,10 +10262,10 @@
         <v>173.6699981689453</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>27620762</v>
+        <v>27895300</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>0.8334926717933018</v>
+        <v>0.8414286729082638</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>54.156136979617</v>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
-          <t>Palantir (PLTR) Stock Fair Value Edges Higher After Strong Q2 And Raised Guidance</t>
+          <t>Cathie Wood Is Moving Money From Palantir Into Rocket Lab and Fintech</t>
         </is>
       </c>
       <c r="AY44" s="79" t="inlineStr">
         <is>
-          <t>Palantir just won the Army and lost Michael Burry</t>
+          <t>Cathie Wood Dumps $25 Million of Palantir Shares. Should PLTR Investors Worry?</t>
         </is>
       </c>
       <c r="AZ44" s="79" t="inlineStr">
         <is>
-          <t>SCHG Owns More Apple Than Tesla, Meta and Palantir Combined. Is That Why Growth Investors Are Falling Behind?</t>
+          <t>Palantir Surged 51% in August. The Rest of Tech Wasn't Even Close</t>
         </is>
       </c>
     </row>
@@ -10441,7 +10441,7 @@
         <v>0.1699981689453125</v>
       </c>
       <c r="T45" s="83" t="n">
-        <v>169.8200073242188</v>
+        <v>169.9799957275391</v>
       </c>
       <c r="U45" s="83" t="n">
         <v>170.6300048828125</v>
@@ -10450,10 +10450,10 @@
         <v>167.0399932861328</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>8495424</v>
+        <v>8531400</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.9341388349337777</v>
+        <v>0.9379091685639812</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>53.07748990482058</v>
@@ -10638,10 +10638,10 @@
         <v>63.20000076293945</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>14797841</v>
+        <v>14867600</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>0.864714088590396</v>
+        <v>0.8686134265378823</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>37.19328452182177</v>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
-          <t>Cathie Wood Just Bought 705,102 Shares of a Rocket Company 50 Times Smaller Than SpaceX</t>
+          <t>Cathie Wood Is Moving Money From Palantir Into Rocket Lab and Fintech</t>
         </is>
       </c>
       <c r="AY46" s="79" t="inlineStr">
         <is>
-          <t>SPCX Stock Blasts Past ASTS, RKLB, LUNR, PL — Here’s Everything Shaking Up Space Stocks This Week</t>
+          <t>The Real Satellite Race Isn’t About Rockets — It’s About Who Controls the Spectrum in Your Phone</t>
         </is>
       </c>
       <c r="AZ46" s="79" t="inlineStr">
         <is>
-          <t>Is Rocket Lab Stock a Millionaire Maker?</t>
+          <t>Cathie Wood Buys $45 Million of Rocket Lab Stock</t>
         </is>
       </c>
     </row>
@@ -10817,7 +10817,7 @@
         <v>185.010009765625</v>
       </c>
       <c r="T47" s="83" t="n">
-        <v>1585.589965820312</v>
+        <v>1586</v>
       </c>
       <c r="U47" s="83" t="n">
         <v>1740</v>
@@ -10826,10 +10826,10 @@
         <v>1581</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>16217211</v>
+        <v>16487100</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>1.221999037596914</v>
+        <v>1.24107374396338</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>61.24267366525383</v>
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Flash Buy Signals; Apple, Inflation Reports Ahead</t>
+          <t>Innovation Engine Drives SharkNinja’s (SN) Sustainable Advantage</t>
         </is>
       </c>
       <c r="AY47" s="90" t="inlineStr">
         <is>
-          <t>Stock Market Today: Dow Sinks Amid Rate Fears; Sandisk, KLA Lead Nasdaq-100 As Utilities Gain</t>
+          <t>Nike Exits S&amp;P 100 After Nearly 18 Years. Dell, SanDisk and 2 Tech Giants Take Its Place</t>
         </is>
       </c>
       <c r="AZ47" s="90" t="inlineStr">
         <is>
-          <t>Analyst Has Strong Take on Micron, SanDisk Stocks</t>
+          <t>Sandisk Jumps 12% as AI Storage Trade Keeps Running</t>
         </is>
       </c>
     </row>
@@ -11005,19 +11005,19 @@
         <v>-22.29000854492188</v>
       </c>
       <c r="T48" s="72" t="n">
-        <v>362.1799926757812</v>
+        <v>362.0700073242188</v>
       </c>
       <c r="U48" s="72" t="n">
         <v>364.6900024414062</v>
       </c>
       <c r="V48" s="72" t="n">
-        <v>351.3200988769531</v>
+        <v>351.3200073242188</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>64559388</v>
+        <v>64829000</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>1.701892134477516</v>
+        <v>1.708392439317929</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>50.92656358273328</v>
@@ -11026,7 +11026,7 @@
         <v>43.38621623071099</v>
       </c>
       <c r="AA48" s="28" t="n">
-        <v>22.80348946706436</v>
+        <v>22.80348165299782</v>
       </c>
       <c r="AB48" s="75" t="n">
         <v>3.659291261924011</v>
@@ -11068,7 +11068,7 @@
         <v>13.87044531288085</v>
       </c>
       <c r="AO48" s="77" t="n">
-        <v>4.312073231750098</v>
+        <v>4.312075078643816</v>
       </c>
       <c r="AP48" s="72" t="n">
         <v>498.8299865722656</v>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
-          <t>No steering wheel, no problem: Can Tesla speed by Cybercab probe?</t>
+          <t>Goldman Sachs Delivers Stark Message on Tesla Stock</t>
         </is>
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>Tesla Launched the Cybercab Thursday, 6 Weeks After Removing Volume Production of It From This Year's Plan</t>
+          <t>Cybercab Could Transform Tesla, But Regulatory Risks Loom</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>From Launch Party to Federal Probe: What Went Wrong With Tesla's Cybercab in 24 Hours</t>
+          <t>Is Tesla Stock Under $360 a Share an Obvious Buy in September?</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 4 Sep 2026, 11:02 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 08:41 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 4 Sep 2026, 11:02 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 08:41 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 4 Sep 2026, 11:02 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 08:41 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 4 Sep 2026, 11:02 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 08:41 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -43864,7 +43864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G45"/>
+  <dimension ref="B2:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -44238,21 +44238,21 @@
     <row r="17">
       <c r="B17" s="31" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="C17" s="102" t="inlineStr">
         <is>
-          <t>IREN Limited</t>
-        </is>
-      </c>
-      <c r="D17" s="105" t="inlineStr">
-        <is>
-          <t>Gapped down 1.5% at the open</t>
+          <t>Advanced Micro Devices, Inc.</t>
+        </is>
+      </c>
+      <c r="D17" s="106" t="inlineStr">
+        <is>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E17" s="33" t="n">
-        <v>0.07274906766604095</v>
+        <v>0.04693529351593129</v>
       </c>
       <c r="F17" s="34" t="n">
         <v>7</v>
@@ -44266,21 +44266,21 @@
     <row r="18">
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="C18" s="101" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices, Inc.</t>
-        </is>
-      </c>
-      <c r="D18" s="107" t="inlineStr">
-        <is>
-          <t>MACD crossed up</t>
+          <t>State Street Technology Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D18" s="104" t="inlineStr">
+        <is>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E18" s="26" t="n">
-        <v>0.04693529351593129</v>
+        <v>0.007044133731219926</v>
       </c>
       <c r="F18" s="27" t="n">
         <v>7</v>
@@ -44294,21 +44294,21 @@
     <row r="19">
       <c r="B19" s="31" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="C19" s="102" t="inlineStr">
         <is>
-          <t>State Street Technology Select Sector SPDR ETF</t>
+          <t>Strategy Inc</t>
         </is>
       </c>
       <c r="D19" s="105" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped down 5.2% at the open</t>
         </is>
       </c>
       <c r="E19" s="33" t="n">
-        <v>0.007044133731219926</v>
+        <v>-0.01394837847189589</v>
       </c>
       <c r="F19" s="34" t="n">
         <v>7</v>
@@ -44322,24 +44322,24 @@
     <row r="20">
       <c r="B20" s="24" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="C20" s="101" t="inlineStr">
         <is>
-          <t>Strategy Inc</t>
+          <t>CoreWeave, Inc.</t>
         </is>
       </c>
       <c r="D20" s="104" t="inlineStr">
         <is>
-          <t>Gapped down 5.2% at the open</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E20" s="26" t="n">
-        <v>-0.01394837847189589</v>
+        <v>0.05676446535410284</v>
       </c>
       <c r="F20" s="27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G20" s="23" t="inlineStr">
         <is>
@@ -44360,7 +44360,7 @@
       </c>
       <c r="D21" s="105" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Reclaimed the 50 DMA</t>
         </is>
       </c>
       <c r="E21" s="33" t="n">
@@ -44378,21 +44378,21 @@
     <row r="22">
       <c r="B22" s="24" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="C22" s="101" t="inlineStr">
         <is>
-          <t>CoreWeave, Inc.</t>
+          <t>Cameco Corporation</t>
         </is>
       </c>
       <c r="D22" s="104" t="inlineStr">
         <is>
-          <t>Reclaimed the 50 DMA</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E22" s="26" t="n">
-        <v>0.05676446535410284</v>
+        <v>0.00119255728395995</v>
       </c>
       <c r="F22" s="27" t="n">
         <v>6</v>
@@ -44406,21 +44406,21 @@
     <row r="23">
       <c r="B23" s="31" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="C23" s="102" t="inlineStr">
         <is>
-          <t>CoreWeave, Inc.</t>
+          <t>State Street SPDR S&amp;P 500 ETF Trust</t>
         </is>
       </c>
       <c r="D23" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 1.7% at the open</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E23" s="33" t="n">
-        <v>0.05676446535410284</v>
+        <v>-0.003854237146576178</v>
       </c>
       <c r="F23" s="34" t="n">
         <v>6</v>
@@ -44434,56 +44434,56 @@
     <row r="24">
       <c r="B24" s="24" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>SOXL</t>
         </is>
       </c>
       <c r="C24" s="101" t="inlineStr">
         <is>
-          <t>Cameco Corporation</t>
-        </is>
-      </c>
-      <c r="D24" s="104" t="inlineStr">
-        <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Direxion Daily Semiconductor Bull 3X Shares</t>
+        </is>
+      </c>
+      <c r="D24" s="107" t="inlineStr">
+        <is>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E24" s="26" t="n">
-        <v>0.00119255728395995</v>
+        <v>0.09874462363189629</v>
       </c>
       <c r="F24" s="27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="31" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SOXL</t>
         </is>
       </c>
       <c r="C25" s="102" t="inlineStr">
         <is>
-          <t>State Street SPDR S&amp;P 500 ETF Trust</t>
+          <t>Direxion Daily Semiconductor Bull 3X Shares</t>
         </is>
       </c>
       <c r="D25" s="105" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Reclaimed the 200 DMA</t>
         </is>
       </c>
       <c r="E25" s="33" t="n">
-        <v>-0.003854237146576178</v>
+        <v>0.09874462363189629</v>
       </c>
       <c r="F25" s="34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G25" s="30" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
@@ -44498,9 +44498,9 @@
           <t>Direxion Daily Semiconductor Bull 3X Shares</t>
         </is>
       </c>
-      <c r="D26" s="107" t="inlineStr">
-        <is>
-          <t>MACD crossed up</t>
+      <c r="D26" s="104" t="inlineStr">
+        <is>
+          <t>Gapped up 4.2% at the open</t>
         </is>
       </c>
       <c r="E26" s="26" t="n">
@@ -44518,21 +44518,21 @@
     <row r="27">
       <c r="B27" s="31" t="inlineStr">
         <is>
-          <t>SOXL</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="C27" s="102" t="inlineStr">
         <is>
-          <t>Direxion Daily Semiconductor Bull 3X Shares</t>
-        </is>
-      </c>
-      <c r="D27" s="105" t="inlineStr">
-        <is>
-          <t>Reclaimed the 200 DMA</t>
+          <t>Arm Holdings plc</t>
+        </is>
+      </c>
+      <c r="D27" s="106" t="inlineStr">
+        <is>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E27" s="33" t="n">
-        <v>0.09874462363189629</v>
+        <v>0.03916072444622976</v>
       </c>
       <c r="F27" s="34" t="n">
         <v>5</v>
@@ -44546,21 +44546,21 @@
     <row r="28">
       <c r="B28" s="24" t="inlineStr">
         <is>
-          <t>SOXL</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="C28" s="101" t="inlineStr">
         <is>
-          <t>Direxion Daily Semiconductor Bull 3X Shares</t>
+          <t>Arm Holdings plc</t>
         </is>
       </c>
       <c r="D28" s="104" t="inlineStr">
         <is>
-          <t>Gapped up 4.2% at the open</t>
+          <t>Gapped up 2.5% at the open</t>
         </is>
       </c>
       <c r="E28" s="26" t="n">
-        <v>0.09874462363189629</v>
+        <v>0.03916072444622976</v>
       </c>
       <c r="F28" s="27" t="n">
         <v>5</v>
@@ -44582,9 +44582,9 @@
           <t>Arm Holdings plc</t>
         </is>
       </c>
-      <c r="D29" s="106" t="inlineStr">
-        <is>
-          <t>MACD crossed up</t>
+      <c r="D29" s="105" t="inlineStr">
+        <is>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E29" s="33" t="n">
@@ -44602,21 +44602,21 @@
     <row r="30">
       <c r="B30" s="24" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="C30" s="101" t="inlineStr">
         <is>
-          <t>Arm Holdings plc</t>
+          <t>Tesla, Inc.</t>
         </is>
       </c>
       <c r="D30" s="104" t="inlineStr">
         <is>
-          <t>Gapped up 2.6% at the open</t>
+          <t>Lost the 50 DMA</t>
         </is>
       </c>
       <c r="E30" s="26" t="n">
-        <v>0.03916072444622976</v>
+        <v>-0.05922365978717725</v>
       </c>
       <c r="F30" s="27" t="n">
         <v>5</v>
@@ -44630,21 +44630,21 @@
     <row r="31">
       <c r="B31" s="31" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="C31" s="102" t="inlineStr">
         <is>
-          <t>Arm Holdings plc</t>
+          <t>Tesla, Inc.</t>
         </is>
       </c>
       <c r="D31" s="105" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped down 3.8% at the open</t>
         </is>
       </c>
       <c r="E31" s="33" t="n">
-        <v>0.03916072444622976</v>
+        <v>-0.05922365978717725</v>
       </c>
       <c r="F31" s="34" t="n">
         <v>5</v>
@@ -44658,24 +44658,24 @@
     <row r="32">
       <c r="B32" s="24" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="C32" s="101" t="inlineStr">
         <is>
-          <t>Tesla, Inc.</t>
+          <t>Palantir Technologies Inc.</t>
         </is>
       </c>
       <c r="D32" s="104" t="inlineStr">
         <is>
-          <t>Lost the 50 DMA</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E32" s="26" t="n">
-        <v>-0.05922365978717725</v>
+        <v>-0.04492410564335281</v>
       </c>
       <c r="F32" s="27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G32" s="23" t="inlineStr">
         <is>
@@ -44686,40 +44686,40 @@
     <row r="33">
       <c r="B33" s="31" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="C33" s="102" t="inlineStr">
         <is>
-          <t>Tesla, Inc.</t>
+          <t>Nokia Oyj</t>
         </is>
       </c>
       <c r="D33" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 3.8% at the open</t>
+          <t>Gapped up 2.4% at the open</t>
         </is>
       </c>
       <c r="E33" s="33" t="n">
-        <v>-0.05922365978717725</v>
+        <v>0.02661200235675665</v>
       </c>
       <c r="F33" s="34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G33" s="30" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Weak</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="24" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="C34" s="101" t="inlineStr">
         <is>
-          <t>Palantir Technologies Inc.</t>
+          <t>Nokia Oyj</t>
         </is>
       </c>
       <c r="D34" s="104" t="inlineStr">
@@ -44728,35 +44728,35 @@
         </is>
       </c>
       <c r="E34" s="26" t="n">
-        <v>-0.04492410564335281</v>
+        <v>0.02661200235675665</v>
       </c>
       <c r="F34" s="27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G34" s="23" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Weak</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="31" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>ASTS</t>
         </is>
       </c>
       <c r="C35" s="102" t="inlineStr">
         <is>
-          <t>Nokia Oyj</t>
+          <t>AST SpaceMobile, Inc.</t>
         </is>
       </c>
       <c r="D35" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 2.4% at the open</t>
+          <t>Gapped up 2.0% at the open</t>
         </is>
       </c>
       <c r="E35" s="33" t="n">
-        <v>0.02661200235675665</v>
+        <v>0.002897155996801626</v>
       </c>
       <c r="F35" s="34" t="n">
         <v>3</v>
@@ -44770,21 +44770,21 @@
     <row r="36">
       <c r="B36" s="24" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="C36" s="101" t="inlineStr">
         <is>
-          <t>Nokia Oyj</t>
-        </is>
-      </c>
-      <c r="D36" s="104" t="inlineStr">
-        <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>State Street Utilities Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D36" s="107" t="inlineStr">
+        <is>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E36" s="26" t="n">
-        <v>0.02661200235675665</v>
+        <v>0.001162050968541273</v>
       </c>
       <c r="F36" s="27" t="n">
         <v>3</v>
@@ -44798,24 +44798,24 @@
     <row r="37">
       <c r="B37" s="31" t="inlineStr">
         <is>
-          <t>ASTS</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="C37" s="102" t="inlineStr">
         <is>
-          <t>AST SpaceMobile, Inc.</t>
+          <t>State Street Materials Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D37" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 2.1% at the open</t>
+          <t>RSI dropped below 50</t>
         </is>
       </c>
       <c r="E37" s="33" t="n">
-        <v>0.002897155996801626</v>
+        <v>-0.003420758434616977</v>
       </c>
       <c r="F37" s="34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G37" s="30" t="inlineStr">
         <is>
@@ -44826,24 +44826,24 @@
     <row r="38">
       <c r="B38" s="24" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="C38" s="101" t="inlineStr">
         <is>
-          <t>State Street Utilities Select Sector SPDR ETF</t>
-        </is>
-      </c>
-      <c r="D38" s="107" t="inlineStr">
-        <is>
-          <t>MACD crossed up</t>
+          <t>State Street Materials Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D38" s="104" t="inlineStr">
+        <is>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E38" s="26" t="n">
-        <v>0.001162050968541273</v>
+        <v>-0.003420758434616977</v>
       </c>
       <c r="F38" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G38" s="23" t="inlineStr">
         <is>
@@ -44854,21 +44854,21 @@
     <row r="39">
       <c r="B39" s="31" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="C39" s="102" t="inlineStr">
         <is>
-          <t>State Street Materials Select Sector SPDR ETF</t>
+          <t>Netflix, Inc.</t>
         </is>
       </c>
       <c r="D39" s="105" t="inlineStr">
         <is>
-          <t>RSI dropped below 50</t>
+          <t>MACD crossed down</t>
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>-0.003420758434616977</v>
+        <v>-0.05346556510032285</v>
       </c>
       <c r="F39" s="34" t="n">
         <v>2</v>
@@ -44882,21 +44882,21 @@
     <row r="40">
       <c r="B40" s="24" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="C40" s="101" t="inlineStr">
         <is>
-          <t>State Street Materials Select Sector SPDR ETF</t>
+          <t>Netflix, Inc.</t>
         </is>
       </c>
       <c r="D40" s="104" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>RSI dropped below 50</t>
         </is>
       </c>
       <c r="E40" s="26" t="n">
-        <v>-0.003420758434616977</v>
+        <v>-0.05346556510032285</v>
       </c>
       <c r="F40" s="27" t="n">
         <v>2</v>
@@ -44910,68 +44910,68 @@
     <row r="41">
       <c r="B41" s="31" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="C41" s="102" t="inlineStr">
         <is>
-          <t>Netflix, Inc.</t>
+          <t>State Street Consumer Staples Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D41" s="105" t="inlineStr">
         <is>
-          <t>MACD crossed down</t>
+          <t>Lost the 50 DMA</t>
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>-0.05346556510032285</v>
+        <v>-0.007975607414239305</v>
       </c>
       <c r="F41" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G41" s="30" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Very Weak</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="24" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="C42" s="101" t="inlineStr">
         <is>
-          <t>Netflix, Inc.</t>
+          <t>Alphabet Inc.</t>
         </is>
       </c>
       <c r="D42" s="104" t="inlineStr">
         <is>
-          <t>RSI dropped below 50</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E42" s="26" t="n">
-        <v>-0.05346556510032285</v>
+        <v>-0.01111828820032235</v>
       </c>
       <c r="F42" s="27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G42" s="23" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Very Weak</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="31" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="C43" s="102" t="inlineStr">
         <is>
-          <t>State Street Consumer Staples Select Sector SPDR ETF</t>
+          <t>State Street Consumer Discretionary Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D43" s="105" t="inlineStr">
@@ -44980,79 +44980,23 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>-0.007975607414239305</v>
+        <v>-0.01330925154171614</v>
       </c>
       <c r="F43" s="34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43" s="30" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="24" t="inlineStr">
-        <is>
-          <t>GOOG</t>
-        </is>
-      </c>
-      <c r="C44" s="101" t="inlineStr">
-        <is>
-          <t>Alphabet Inc.</t>
-        </is>
-      </c>
-      <c r="D44" s="104" t="inlineStr">
-        <is>
-          <t>Bands squeezing — a big move often follows</t>
-        </is>
-      </c>
-      <c r="E44" s="26" t="n">
-        <v>-0.01111828820032235</v>
-      </c>
-      <c r="F44" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="31" t="inlineStr">
-        <is>
-          <t>XLY</t>
-        </is>
-      </c>
-      <c r="C45" s="102" t="inlineStr">
-        <is>
-          <t>State Street Consumer Discretionary Select Sector SPDR ETF</t>
-        </is>
-      </c>
-      <c r="D45" s="105" t="inlineStr">
-        <is>
-          <t>Lost the 50 DMA</t>
-        </is>
-      </c>
-      <c r="E45" s="33" t="n">
-        <v>-0.01330925154171614</v>
-      </c>
-      <c r="F45" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" s="30" t="inlineStr">
         <is>
           <t>Very Weak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B5:G45"/>
+  <autoFilter ref="B5:G43"/>
   <mergeCells count="1">
     <mergeCell ref="B2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E45">
+  <conditionalFormatting sqref="E6:E43">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>

</xml_diff>

<commit_message>
Daily workbook: 2026-09-07 22:52 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 7 Sep 2026, 08:41 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 7 Sep 2026, 10:51 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 7 Sep 2026, 08:41 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 10:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5999,17 +5999,17 @@
       </c>
       <c r="AX20" s="90" t="inlineStr">
         <is>
+          <t>QQQ Charged 0.20% for Years. The Fee Only Fell After Shareholders Approved a Structural Change</t>
+        </is>
+      </c>
+      <c r="AY20" s="90" t="inlineStr">
+        <is>
           <t>This ETF Would Have Increased Your Investment by 6x Over the Past 10 Years -- and It's Still Soaring</t>
         </is>
       </c>
-      <c r="AY20" s="90" t="inlineStr">
+      <c r="AZ20" s="90" t="inlineStr">
         <is>
           <t>The VIX Is Playing Tricks: Why Stocks Are Volatile, But the Fear Gauge Is Sleeping</t>
-        </is>
-      </c>
-      <c r="AZ20" s="90" t="inlineStr">
-        <is>
-          <t>Exchange-Traded Funds Mixed, US Equities Lower After Midday</t>
         </is>
       </c>
     </row>
@@ -6584,17 +6584,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
-          <t>KeyBanc Delivers Stark Warning on Apple Stock Ahead of iPhone 18 Launch</t>
+          <t>Apple's $54 Billion iPhone Engine Hits an AI Memory Squeeze</t>
         </is>
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
-          <t>Apple’s new CEO faces a staggering $14 billion iPhone test</t>
+          <t>Tim Cook Delivered a 2,720% Total Return Over 15 Years. Here's Whether John Ternus Can Do the Same for Appl...</t>
         </is>
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Apple Faces Its Biggest iPhone Test in Years -- Morgan Stanley Sees $14B Foldable Opportunity</t>
+          <t>Apple's $320 Stock Faces Huawei's 68% Foldable Fortress</t>
         </is>
       </c>
     </row>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
+          <t>AMD Stock Jumps After Unveiling $100,000-Plus AI Workstation for 2027</t>
+        </is>
+      </c>
+      <c r="AY25" s="90" t="inlineStr">
+        <is>
           <t>Wall Street Is Worried About AMD. Here’s Why Long-Term Investors Shouldn’t Be</t>
         </is>
       </c>
-      <c r="AY25" s="90" t="inlineStr">
+      <c r="AZ25" s="90" t="inlineStr">
         <is>
           <t>AMD Is Behind The AI Chip Shift Nobody Is Talking About</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>AMD’s Whole AI Story Has One Threat It Cannot Ignore: Broadcom</t>
         </is>
       </c>
     </row>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
-          <t>Fatal Amazon Plane Crash Delays Hundreds of Miami Flights</t>
+          <t>Scene of Fatal Amazon Plane Crash in Miami Is ‘Devastating’</t>
         </is>
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Are Retail-Wholesale Stocks Lagging Amazon.com (AMZN) This Year?</t>
+          <t>Amazon's 250-Flight Air Network Faces a Fatal Miami Investigation</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Amazon.com, Inc. (AMZN) is Attracting Investor Attention: Here is What You Should Know</t>
+          <t>Is Amazon Stock at $255 a Share an Obvious Buy Right Now?</t>
         </is>
       </c>
     </row>
@@ -7524,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
+          <t>Is AST SpaceMobile a Millionaire-Maker Over The Next Decade?</t>
+        </is>
+      </c>
+      <c r="AY29" s="90" t="inlineStr">
+        <is>
           <t>AST SpaceMobile Director Adriana Cisneros Buys $619,235 Shares. What Does This Mean for Investors?</t>
         </is>
       </c>
-      <c r="AY29" s="90" t="inlineStr">
+      <c r="AZ29" s="90" t="inlineStr">
         <is>
           <t>The Real Satellite Race Isn’t About Rockets — It’s About Who Controls the Spectrum in Your Phone</t>
-        </is>
-      </c>
-      <c r="AZ29" s="90" t="inlineStr">
-        <is>
-          <t>Forget Starlink? Japan’s $1 Billion BlueBird Play Makes ASTS the National Satellite OS</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Broadcom’s AI Forecast Suggests Hyperscalers Want More Than Just Nvidia GPUs</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Broadcom Inc. (AVGO)’s AI Opportunity Expands Across AI Infrastructure</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>Broadcom vs Marvell: One of These AI Chip Stocks Is a Clear Winner</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Broadcom Inc. (AVGO) Is a Trending Stock: Facts to Know Before Betting on It</t>
         </is>
       </c>
     </row>
@@ -7910,7 +7910,7 @@
       </c>
       <c r="AZ31" s="90" t="inlineStr">
         <is>
-          <t>Cameco (TSX:CCO) Tests Nuclear Growth Hopes On A Fair Value Gap</t>
+          <t>Jefferies Sees Cameco (CCJ) and BWXT as Winners in the Nuclear Boom</t>
         </is>
       </c>
     </row>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Google's AI Slashes Contrail Warming 40% in a Real-World Test</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>Google-Backed Pixxel Raises $100 Million in India's Biggest Space-Tech Round</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
+      <c r="AZ34" s="79" t="inlineStr">
         <is>
           <t>Alphabet May Be the Mag 7 Stock Investors Are Underestimating</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Agentic Commerce Optimisation: Azoma on Which Platforms Help Brands Get Recommended by AI Shopping Agents</t>
         </is>
       </c>
     </row>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
+          <t>5-star analyst resets Intel stock price target</t>
+        </is>
+      </c>
+      <c r="AY36" s="79" t="inlineStr">
+        <is>
           <t>Prediction: Intel Stock Is Up Big in 2026. But the Best May Still Be Ahead</t>
         </is>
       </c>
-      <c r="AY36" s="79" t="inlineStr">
+      <c r="AZ36" s="79" t="inlineStr">
         <is>
           <t>Nvidia just sent a strong signal to AMD and Intel investors</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>AMD and Intel Soared as Nvidia Lagged: Has the AI Trade Changed?</t>
         </is>
       </c>
     </row>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Micron's $50 Billion Guide Gets an 8.3% Signal From Seoul</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
+          <t>Micron, SanDisk get new aggressive price targets from top analyst</t>
+        </is>
+      </c>
+      <c r="AZ39" s="90" t="inlineStr">
+        <is>
           <t>Is Micron Technology Stock Running Out of Steam?</t>
-        </is>
-      </c>
-      <c r="AY39" s="90" t="inlineStr">
-        <is>
-          <t>Why Micron and SK Hynix Sit in the Most Valuable Spot in the Entire Compute Stack</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Everyone Is Watching Nvidia. But This Memory Stock Could Be the Next AI Winner</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Jim Cramer Discusses NVIDIA (NVDA) Acquiring Hugging Face</t>
+          <t>Palantir Stock Leads August Rally -- Nvidia, Salesforce and Super Micro Jump</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Could This Vanguard Growth ETF Be a No-Brainer Buy for Long-Term Investors?</t>
+          <t>Nvidia Insider Makes Stunning $410 Million Stock Move</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Nvidia, Microsoft at Center of $7 Trillion AI Boom</t>
+          <t>Tencent Slips 1% While Its AI-Chip Bet Attacks Nvidia's China Moat</t>
         </is>
       </c>
     </row>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Palantir Stock Leads August Rally -- Nvidia, Salesforce and Super Micro Jump</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
+          <t>Burry’s Palantir Warning Is Back. Accenture Shows What Investors Should Check</t>
+        </is>
+      </c>
+      <c r="AZ44" s="79" t="inlineStr">
+        <is>
           <t>Cathie Wood Is Moving Money From Palantir Into Rocket Lab and Fintech</t>
-        </is>
-      </c>
-      <c r="AY44" s="79" t="inlineStr">
-        <is>
-          <t>Cathie Wood Dumps $25 Million of Palantir Shares. Should PLTR Investors Worry?</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Palantir Surged 51% in August. The Rest of Tech Wasn't Even Close</t>
         </is>
       </c>
     </row>
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>Sandisk Soars Nearly 12% Before Joining the S&amp;P 100</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
+          <t>Micron, SanDisk get new aggressive price targets from top analyst</t>
+        </is>
+      </c>
+      <c r="AZ47" s="90" t="inlineStr">
+        <is>
           <t>Innovation Engine Drives SharkNinja’s (SN) Sustainable Advantage</t>
-        </is>
-      </c>
-      <c r="AY47" s="90" t="inlineStr">
-        <is>
-          <t>Nike Exits S&amp;P 100 After Nearly 18 Years. Dell, SanDisk and 2 Tech Giants Take Its Place</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>Sandisk Jumps 12% as AI Storage Trade Keeps Running</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 7 Sep 2026, 08:41 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 10:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 7 Sep 2026, 08:41 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 10:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 7 Sep 2026, 08:41 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 10:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 7 Sep 2026, 08:41 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 10:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-07 23:29 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 7 Sep 2026, 10:51 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 7 Sep 2026, 11:29 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 7 Sep 2026, 10:51 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 11:29 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 7 Sep 2026, 10:51 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 11:29 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 7 Sep 2026, 10:51 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 11:29 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 7 Sep 2026, 10:51 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 11:29 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 7 Sep 2026, 10:51 PM · Yahoo Finance data</t>
+          <t>Built 7 Sep 2026, 11:29 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-08 22:43 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'09-02'!$5:$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'09-01'!$A$6:$AZ$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'09-01'!$5:$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 8 Sep 2026, 08:02 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 8 Sep 2026, 10:43 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1390,7 +1390,7 @@
       <c r="J8" s="8" t="n"/>
       <c r="K8" s="15" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="L8" s="10" t="n"/>
@@ -1404,7 +1404,7 @@
       <c r="P8" s="10" t="n"/>
       <c r="Q8" s="16" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>58</t>
         </is>
       </c>
       <c r="R8" s="12" t="n"/>
@@ -1523,22 +1523,22 @@
         </is>
       </c>
       <c r="E14" s="26" t="n">
-        <v>0.01100533652705571</v>
+        <v>0.01108334548129264</v>
       </c>
       <c r="F14" s="27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G14" s="28" t="n">
-        <v>66.17874588140691</v>
+        <v>66.19848629337565</v>
       </c>
       <c r="H14" s="29" t="n">
-        <v>8.992534896549875</v>
+        <v>9.000761401287027</v>
       </c>
       <c r="I14" s="26" t="n">
-        <v>0.01258599619603817</v>
+        <v>0.01266412711363518</v>
       </c>
       <c r="J14" s="26" t="n">
-        <v>0.1263478154721467</v>
+        <v>0.1264347242272419</v>
       </c>
     </row>
     <row r="15">
@@ -1559,7 +1559,7 @@
         <v>0.008588647078887623</v>
       </c>
       <c r="F15" s="34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G15" s="35" t="n">
         <v>48.76529694830028</v>
@@ -1622,22 +1622,22 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
-        <v>-0.0007967185788519959</v>
+        <v>-0.0006828768287838738</v>
       </c>
       <c r="F17" s="34" t="n">
         <v>2</v>
       </c>
       <c r="G17" s="35" t="n">
-        <v>39.81401726539807</v>
+        <v>39.86747270631402</v>
       </c>
       <c r="H17" s="36" t="n">
-        <v>-2.066650765349909</v>
+        <v>-2.055711540290439</v>
       </c>
       <c r="I17" s="33" t="n">
-        <v>-0.004874181582700698</v>
+        <v>-0.004760804388276862</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v>-0.0241218118166906</v>
+        <v>-0.02401062755332628</v>
       </c>
     </row>
     <row r="18">
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="E18" s="26" t="n">
-        <v>-0.004373809418090291</v>
+        <v>-0.004552371166540725</v>
       </c>
       <c r="F18" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G18" s="28" t="n">
-        <v>50.0460883623922</v>
+        <v>49.97831737646933</v>
       </c>
       <c r="H18" s="29" t="n">
-        <v>0.7633600223907022</v>
+        <v>0.7456526247258566</v>
       </c>
       <c r="I18" s="26" t="n">
-        <v>0.0007177627104955064</v>
+        <v>0.0005382878080617548</v>
       </c>
       <c r="J18" s="26" t="n">
-        <v>0.002606749802492869</v>
+        <v>0.002426936117450929</v>
       </c>
     </row>
     <row r="19">
@@ -1721,22 +1721,22 @@
         </is>
       </c>
       <c r="E20" s="26" t="n">
-        <v>-0.006739178085651609</v>
+        <v>-0.006621011774235575</v>
       </c>
       <c r="F20" s="27" t="n">
         <v>2</v>
       </c>
       <c r="G20" s="28" t="n">
-        <v>42.33075771069067</v>
+        <v>42.37844791946197</v>
       </c>
       <c r="H20" s="29" t="n">
-        <v>-1.185861127811172</v>
+        <v>-1.174337755058386</v>
       </c>
       <c r="I20" s="26" t="n">
-        <v>-0.01141446437262328</v>
+        <v>-0.01129685427093907</v>
       </c>
       <c r="J20" s="26" t="n">
-        <v>-0.01304042028354058</v>
+        <v>-0.01292300361867404</v>
       </c>
     </row>
     <row r="21">
@@ -1754,22 +1754,22 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
-        <v>-0.007745252725428697</v>
+        <v>-0.008006315977894363</v>
       </c>
       <c r="F21" s="34" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="35" t="n">
-        <v>42.03041121598466</v>
+        <v>41.94979478135864</v>
       </c>
       <c r="H21" s="36" t="n">
-        <v>-1.911194394984128</v>
+        <v>-1.936495511209113</v>
       </c>
       <c r="I21" s="33" t="n">
-        <v>-0.02204305494080361</v>
+        <v>-0.02230035642668704</v>
       </c>
       <c r="J21" s="33" t="n">
-        <v>-0.04872354361377162</v>
+        <v>-0.04897382543543116</v>
       </c>
     </row>
     <row r="22">
@@ -1787,22 +1787,22 @@
         </is>
       </c>
       <c r="E22" s="26" t="n">
-        <v>-0.009343971712462262</v>
+        <v>-0.009534706580738517</v>
       </c>
       <c r="F22" s="27" t="n">
         <v>3</v>
       </c>
       <c r="G22" s="28" t="n">
-        <v>45.41830871370646</v>
+        <v>45.3425445112604</v>
       </c>
       <c r="H22" s="29" t="n">
-        <v>0.2319146171392283</v>
+        <v>0.2130033586920765</v>
       </c>
       <c r="I22" s="26" t="n">
-        <v>-0.01404437052678953</v>
+        <v>-0.0142342004089524</v>
       </c>
       <c r="J22" s="26" t="n">
-        <v>-0.0172152825748153</v>
+        <v>-0.0174045019489163</v>
       </c>
     </row>
     <row r="23">
@@ -1820,22 +1820,22 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
-        <v>-0.01368327349095233</v>
+        <v>-0.0137693503970896</v>
       </c>
       <c r="F23" s="34" t="n">
         <v>3</v>
       </c>
       <c r="G23" s="35" t="n">
-        <v>48.05141437193593</v>
+        <v>48.01095166648066</v>
       </c>
       <c r="H23" s="36" t="n">
-        <v>0.6532232619636202</v>
+        <v>0.6446159632309101</v>
       </c>
       <c r="I23" s="33" t="n">
-        <v>-0.007017826818954909</v>
+        <v>-0.00710448542568809</v>
       </c>
       <c r="J23" s="33" t="n">
-        <v>-0.005121496124307234</v>
+        <v>-0.005208320225830065</v>
       </c>
     </row>
     <row r="24">
@@ -1853,22 +1853,22 @@
         </is>
       </c>
       <c r="E24" s="26" t="n">
-        <v>-0.02502183355201748</v>
+        <v>-0.02519680456298767</v>
       </c>
       <c r="F24" s="27" t="n">
         <v>3</v>
       </c>
       <c r="G24" s="28" t="n">
-        <v>44.78249044535038</v>
+        <v>44.72210407835785</v>
       </c>
       <c r="H24" s="29" t="n">
-        <v>0.7811225631442209</v>
+        <v>0.7634007231370532</v>
       </c>
       <c r="I24" s="26" t="n">
-        <v>-0.0198193371472255</v>
+        <v>-0.01999524180582679</v>
       </c>
       <c r="J24" s="26" t="n">
-        <v>0.008932949370805243</v>
+        <v>0.008751884784717445</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -2001,7 +2001,7 @@
         </is>
       </c>
       <c r="I30" s="33" t="n">
-        <v>-0.007745252725428697</v>
+        <v>-0.008006315977894363</v>
       </c>
       <c r="J30" s="34" t="n">
         <v>1</v>
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="L30" s="35" t="n">
-        <v>42.03041121598466</v>
+        <v>41.94979478135864</v>
       </c>
     </row>
     <row r="31">
@@ -2041,7 +2041,7 @@
         </is>
       </c>
       <c r="I31" s="26" t="n">
-        <v>-0.006739178085651609</v>
+        <v>-0.006621011774235575</v>
       </c>
       <c r="J31" s="27" t="n">
         <v>2</v>
@@ -2052,7 +2052,7 @@
         </is>
       </c>
       <c r="L31" s="28" t="n">
-        <v>42.33075771069067</v>
+        <v>42.37844791946197</v>
       </c>
     </row>
     <row r="32">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="C32" s="33" t="n">
-        <v>0.06281157838618334</v>
+        <v>0.06181454656683427</v>
       </c>
       <c r="D32" s="34" t="n">
         <v>9</v>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="F32" s="35" t="n">
-        <v>55.88489331573219</v>
+        <v>55.76913742500214</v>
       </c>
       <c r="H32" s="31" t="inlineStr">
         <is>
@@ -2157,11 +2157,11 @@
       </c>
       <c r="H34" s="31" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="I34" s="33" t="n">
-        <v>-0.004459333403163956</v>
+        <v>-0.004552371166540725</v>
       </c>
       <c r="J34" s="34" t="n">
         <v>2</v>
@@ -2172,7 +2172,7 @@
         </is>
       </c>
       <c r="L34" s="35" t="n">
-        <v>45.94367785704903</v>
+        <v>49.97831737646933</v>
       </c>
     </row>
     <row r="35">
@@ -2197,11 +2197,11 @@
       </c>
       <c r="H35" s="24" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="I35" s="26" t="n">
-        <v>-0.0007967185788519959</v>
+        <v>-0.004526861571173213</v>
       </c>
       <c r="J35" s="27" t="n">
         <v>2</v>
@@ -2212,17 +2212,17 @@
         </is>
       </c>
       <c r="L35" s="28" t="n">
-        <v>39.81401726539807</v>
+        <v>45.91187219850499</v>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="31" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="C36" s="33" t="n">
-        <v>0.003150343559036095</v>
+        <v>0.01108334548129264</v>
       </c>
       <c r="D36" s="34" t="n">
         <v>9</v>
@@ -2233,15 +2233,15 @@
         </is>
       </c>
       <c r="F36" s="35" t="n">
-        <v>56.207320537553</v>
+        <v>66.19848629337565</v>
       </c>
       <c r="H36" s="31" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="I36" s="33" t="n">
-        <v>0.0297848668452132</v>
+        <v>-0.0006828768287838738</v>
       </c>
       <c r="J36" s="34" t="n">
         <v>2</v>
@@ -2252,20 +2252,20 @@
         </is>
       </c>
       <c r="L36" s="35" t="n">
-        <v>45.33346661314823</v>
+        <v>39.86747270631402</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="24" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="C37" s="26" t="n">
-        <v>0.03744695378055884</v>
+        <v>0.003150343559036095</v>
       </c>
       <c r="D37" s="27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E37" s="23" t="inlineStr">
         <is>
@@ -2273,18 +2273,18 @@
         </is>
       </c>
       <c r="F37" s="28" t="n">
-        <v>52.24195279097528</v>
+        <v>56.207320537553</v>
       </c>
       <c r="H37" s="24" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="I37" s="26" t="n">
-        <v>-0.02502183355201748</v>
+        <v>0.0297848668452132</v>
       </c>
       <c r="J37" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
@@ -2292,17 +2292,17 @@
         </is>
       </c>
       <c r="L37" s="28" t="n">
-        <v>44.78249044535038</v>
+        <v>45.33346661314823</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="31" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="C38" s="33" t="n">
-        <v>0.01783869829554785</v>
+        <v>0.03744695378055884</v>
       </c>
       <c r="D38" s="34" t="n">
         <v>8</v>
@@ -2313,15 +2313,15 @@
         </is>
       </c>
       <c r="F38" s="35" t="n">
-        <v>65.0245878859218</v>
+        <v>52.24195279097528</v>
       </c>
       <c r="H38" s="31" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="I38" s="33" t="n">
-        <v>-0.02311706956328952</v>
+        <v>-0.02519680456298767</v>
       </c>
       <c r="J38" s="34" t="n">
         <v>3</v>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="L38" s="35" t="n">
-        <v>51.29456085708777</v>
+        <v>44.72210407835785</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="I44" s="33" t="n">
-        <v>-0.02502183355201748</v>
+        <v>-0.02519680456298767</v>
       </c>
       <c r="J44" s="34" t="n">
         <v>3</v>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="L44" s="35" t="n">
-        <v>44.78249044535038</v>
+        <v>44.72210407835785</v>
       </c>
     </row>
     <row r="45">
@@ -2526,7 +2526,7 @@
         </is>
       </c>
       <c r="C46" s="33" t="n">
-        <v>0.06281157838618334</v>
+        <v>0.06181454656683427</v>
       </c>
       <c r="D46" s="34" t="n">
         <v>9</v>
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="F46" s="35" t="n">
-        <v>55.88489331573219</v>
+        <v>55.76913742500214</v>
       </c>
       <c r="H46" s="31" t="inlineStr">
         <is>
@@ -2646,7 +2646,7 @@
         </is>
       </c>
       <c r="C49" s="26" t="n">
-        <v>0.05192704664625403</v>
+        <v>0.05107433429498753</v>
       </c>
       <c r="D49" s="27" t="n">
         <v>6</v>
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="F49" s="28" t="n">
-        <v>48.67183074907373</v>
+        <v>48.62192842970096</v>
       </c>
       <c r="H49" s="24" t="inlineStr">
         <is>
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="I49" s="26" t="n">
-        <v>-0.01368327349095233</v>
+        <v>-0.0137693503970896</v>
       </c>
       <c r="J49" s="27" t="n">
         <v>3</v>
@@ -2676,7 +2676,7 @@
         </is>
       </c>
       <c r="L49" s="28" t="n">
-        <v>48.05141437193593</v>
+        <v>48.01095166648066</v>
       </c>
     </row>
     <row r="50">
@@ -2748,7 +2748,7 @@
         <v>-0.01150690386138653</v>
       </c>
       <c r="J51" s="27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K51" s="23" t="inlineStr">
         <is>
@@ -2785,7 +2785,7 @@
         </is>
       </c>
       <c r="I52" s="33" t="n">
-        <v>-0.009343971712462262</v>
+        <v>-0.009534706580738517</v>
       </c>
       <c r="J52" s="34" t="n">
         <v>3</v>
@@ -2796,7 +2796,7 @@
         </is>
       </c>
       <c r="L52" s="35" t="n">
-        <v>45.41830871370646</v>
+        <v>45.3425445112604</v>
       </c>
     </row>
   </sheetData>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Sep 2026, 08:02 PM · Yahoo Finance data</t>
+          <t>Built 8 Sep 2026, 10:43 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3142,12 +3142,12 @@
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>5.4 / 9</t>
+          <t>5.5 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>21 of 40</t>
+          <t>22 of 40</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3548,7 @@
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G7" s="23" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>174.2700042724609</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>5949174</v>
+        <v>6185829</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>0.923215127336724</v>
+        <v>0.9581806777989758</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>37.09729108830635</v>
@@ -3726,7 +3726,7 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>-0.02502183355201748</v>
+        <v>-0.02519680456298767</v>
       </c>
       <c r="D8" s="34" t="n">
         <v>11</v>
@@ -3795,10 +3795,10 @@
         </is>
       </c>
       <c r="R8" s="81" t="n">
-        <v>167.1600036621094</v>
+        <v>167.1300048828125</v>
       </c>
       <c r="S8" s="82" t="n">
-        <v>-4.289993286132812</v>
+        <v>-4.319992065429688</v>
       </c>
       <c r="T8" s="83" t="n">
         <v>168.2899932861328</v>
@@ -3810,61 +3810,61 @@
         <v>166.9349975585938</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>10415966</v>
+        <v>10776391</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>1.378836899887444</v>
+        <v>1.423153888164355</v>
       </c>
       <c r="Y8" s="35" t="n">
-        <v>44.78249044535038</v>
+        <v>44.72210407835785</v>
       </c>
       <c r="Z8" s="35" t="n">
-        <v>2.328048676520273</v>
+        <v>2.017663236533914</v>
       </c>
       <c r="AA8" s="35" t="n">
         <v>25.49629080616576</v>
       </c>
       <c r="AB8" s="86" t="n">
-        <v>1.639045903626254</v>
+        <v>1.636652838611127</v>
       </c>
       <c r="AC8" s="86" t="n">
-        <v>2.416443405132549</v>
+        <v>2.415964792129524</v>
       </c>
       <c r="AD8" s="86" t="n">
-        <v>-0.7773975015062953</v>
+        <v>-0.779311953518397</v>
       </c>
       <c r="AE8" s="83" t="n">
-        <v>171.0317713413937</v>
+        <v>171.0251049459944</v>
       </c>
       <c r="AF8" s="83" t="n">
-        <v>170.1947375429226</v>
+        <v>170.1920103811683</v>
       </c>
       <c r="AG8" s="83" t="n">
-        <v>165.8643994140625</v>
+        <v>165.8637994384766</v>
       </c>
       <c r="AH8" s="83" t="n">
-        <v>157.1923999023437</v>
+        <v>157.1920999145508</v>
       </c>
       <c r="AI8" s="83" t="n">
-        <v>155.4477499389648</v>
+        <v>155.4475999450684</v>
       </c>
       <c r="AJ8" s="83" t="n">
-        <v>176.7599479193007</v>
+        <v>176.7629124122553</v>
       </c>
       <c r="AK8" s="83" t="n">
-        <v>171.2484977722168</v>
+        <v>171.246997833252</v>
       </c>
       <c r="AL8" s="83" t="n">
-        <v>165.7370476251329</v>
+        <v>165.7310832542486</v>
       </c>
       <c r="AM8" s="87" t="n">
-        <v>0.1290908925057894</v>
+        <v>0.1268077676446398</v>
       </c>
       <c r="AN8" s="36" t="n">
-        <v>6.436786563132175</v>
+        <v>6.442056968933639</v>
       </c>
       <c r="AO8" s="88" t="n">
-        <v>1.643301999378363</v>
+        <v>1.643596961698456</v>
       </c>
       <c r="AP8" s="83" t="n">
         <v>176.6000061035156</v>
@@ -3873,22 +3873,22 @@
         <v>133.7299957275391</v>
       </c>
       <c r="AR8" s="36" t="n">
-        <v>-5.345414561238981</v>
+        <v>-5.362401411895878</v>
       </c>
       <c r="AS8" s="89" t="n">
-        <v>77.97993898621442</v>
+        <v>77.90996284430594</v>
       </c>
       <c r="AT8" s="33" t="n">
-        <v>-0.0198193371472255</v>
+        <v>-0.01999524180582679</v>
       </c>
       <c r="AU8" s="33" t="n">
-        <v>0.008932949370805243</v>
+        <v>0.008751884784717445</v>
       </c>
       <c r="AV8" s="33" t="n">
-        <v>0.09505411297601873</v>
+        <v>0.09485759295966534</v>
       </c>
       <c r="AW8" s="33" t="n">
-        <v>0.07984496360907012</v>
+        <v>0.0796511730489573</v>
       </c>
       <c r="AX8" s="90" t="inlineStr">
         <is>
@@ -3916,7 +3916,7 @@
         </is>
       </c>
       <c r="C9" s="26" t="n">
-        <v>-0.01368327349095233</v>
+        <v>-0.0137693503970896</v>
       </c>
       <c r="D9" s="27" t="n">
         <v>10</v>
@@ -3985,10 +3985,10 @@
         </is>
       </c>
       <c r="R9" s="70" t="n">
-        <v>57.30500030517578</v>
+        <v>57.29999923706055</v>
       </c>
       <c r="S9" s="71" t="n">
-        <v>-0.7949981689453125</v>
+        <v>-0.7999992370605469</v>
       </c>
       <c r="T9" s="72" t="n">
         <v>57.70500183105469</v>
@@ -4000,61 +4000,61 @@
         <v>57.2599983215332</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>35700282</v>
+        <v>38063059</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>1.265114208027167</v>
+        <v>1.343220765722555</v>
       </c>
       <c r="Y9" s="28" t="n">
-        <v>48.05141437193593</v>
+        <v>48.01095166648066</v>
       </c>
       <c r="Z9" s="28" t="n">
-        <v>23.37282714441463</v>
+        <v>23.07690571369884</v>
       </c>
       <c r="AA9" s="28" t="n">
         <v>18.46505946477791</v>
       </c>
       <c r="AB9" s="75" t="n">
-        <v>0.2584065141210914</v>
+        <v>0.2580075685164616</v>
       </c>
       <c r="AC9" s="75" t="n">
-        <v>0.3678833062969867</v>
+        <v>0.3678035171760607</v>
       </c>
       <c r="AD9" s="75" t="n">
-        <v>-0.1094767921758953</v>
+        <v>-0.1097959486595992</v>
       </c>
       <c r="AE9" s="72" t="n">
-        <v>57.80986284406844</v>
+        <v>57.80875149559839</v>
       </c>
       <c r="AF9" s="72" t="n">
-        <v>57.67835174851741</v>
+        <v>57.67789710596148</v>
       </c>
       <c r="AG9" s="72" t="n">
-        <v>56.93310005187988</v>
+        <v>56.93300003051758</v>
       </c>
       <c r="AH9" s="72" t="n">
-        <v>54.54054996490478</v>
+        <v>54.54049995422363</v>
       </c>
       <c r="AI9" s="72" t="n">
-        <v>53.51737503051758</v>
+        <v>53.517350025177</v>
       </c>
       <c r="AJ9" s="72" t="n">
-        <v>58.65700297946822</v>
+        <v>58.6574080107208</v>
       </c>
       <c r="AK9" s="72" t="n">
-        <v>57.83874988555908</v>
+        <v>57.83849983215332</v>
       </c>
       <c r="AL9" s="72" t="n">
-        <v>57.02049679164994</v>
+        <v>57.01959165358583</v>
       </c>
       <c r="AM9" s="76" t="n">
-        <v>0.1738481135260042</v>
+        <v>0.1712081957498762</v>
       </c>
       <c r="AN9" s="29" t="n">
-        <v>2.82942869798588</v>
+        <v>2.831706150553508</v>
       </c>
       <c r="AO9" s="77" t="n">
-        <v>1.174982680027602</v>
+        <v>1.175085230961202</v>
       </c>
       <c r="AP9" s="72" t="n">
         <v>58.59999847412109</v>
@@ -4063,22 +4063,22 @@
         <v>47.66999816894531</v>
       </c>
       <c r="AR9" s="29" t="n">
-        <v>-2.209894543797997</v>
+        <v>-2.218428789950655</v>
       </c>
       <c r="AS9" s="78" t="n">
-        <v>88.15189265518977</v>
+        <v>88.10613722997842</v>
       </c>
       <c r="AT9" s="26" t="n">
-        <v>-0.007017826818954909</v>
+        <v>-0.00710448542568809</v>
       </c>
       <c r="AU9" s="26" t="n">
-        <v>-0.005121496124307234</v>
+        <v>-0.005208320225830065</v>
       </c>
       <c r="AV9" s="26" t="n">
-        <v>0.1026553580750613</v>
+        <v>0.1025591281732379</v>
       </c>
       <c r="AW9" s="26" t="n">
-        <v>0.0462844591240601</v>
+        <v>0.04619314877033642</v>
       </c>
       <c r="AX9" s="79" t="inlineStr">
         <is>
@@ -4106,7 +4106,7 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>0.01100533652705571</v>
+        <v>0.01108334548129264</v>
       </c>
       <c r="D10" s="34" t="n">
         <v>1</v>
@@ -4118,14 +4118,14 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G10" s="30" t="inlineStr">
+        <is>
           <t>Same</t>
         </is>
       </c>
-      <c r="G10" s="30" t="inlineStr">
-        <is>
-          <t>Same</t>
-        </is>
-      </c>
       <c r="H10" s="30" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4157,7 +4157,7 @@
         </is>
       </c>
       <c r="N10" s="80" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O10" s="30" t="inlineStr">
         <is>
@@ -4175,10 +4175,10 @@
         </is>
       </c>
       <c r="R10" s="81" t="n">
-        <v>64.76499938964844</v>
+        <v>64.76999664306641</v>
       </c>
       <c r="S10" s="82" t="n">
-        <v>0.7050018310546875</v>
+        <v>0.7099990844726562</v>
       </c>
       <c r="T10" s="83" t="n">
         <v>64.83000183105469</v>
@@ -4190,61 +4190,61 @@
         <v>64.31199645996094</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>26177295</v>
+        <v>27876575</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>1.033999515277455</v>
+        <v>1.097437765384704</v>
       </c>
       <c r="Y10" s="35" t="n">
-        <v>66.17874588140691</v>
+        <v>66.19848629337565</v>
       </c>
       <c r="Z10" s="35" t="n">
-        <v>82.06655340355647</v>
+        <v>82.18525314305131</v>
       </c>
       <c r="AA10" s="35" t="n">
         <v>27.84150329734461</v>
       </c>
       <c r="AB10" s="86" t="n">
-        <v>1.425053564059759</v>
+        <v>1.425452205358056</v>
       </c>
       <c r="AC10" s="86" t="n">
-        <v>1.424654896439632</v>
+        <v>1.424734624699291</v>
       </c>
       <c r="AD10" s="86" t="n">
-        <v>0.0003986676201273021</v>
+        <v>0.0007175806587649269</v>
       </c>
       <c r="AE10" s="83" t="n">
-        <v>64.11422698418846</v>
+        <v>64.11533748494801</v>
       </c>
       <c r="AF10" s="83" t="n">
-        <v>62.76978139535805</v>
+        <v>62.77023569112333</v>
       </c>
       <c r="AG10" s="83" t="n">
-        <v>59.42150024414062</v>
+        <v>59.42160018920899</v>
       </c>
       <c r="AH10" s="83" t="n">
-        <v>58.30155010223389</v>
+        <v>58.30160007476807</v>
       </c>
       <c r="AI10" s="83" t="n">
-        <v>54.92702491760254</v>
+        <v>54.92704990386963</v>
       </c>
       <c r="AJ10" s="83" t="n">
-        <v>65.63080728586772</v>
+        <v>65.63171549782244</v>
       </c>
       <c r="AK10" s="83" t="n">
-        <v>63.10025005340576</v>
+        <v>63.10049991607666</v>
       </c>
       <c r="AL10" s="83" t="n">
-        <v>60.56969282094381</v>
+        <v>60.56928433433087</v>
       </c>
       <c r="AM10" s="87" t="n">
-        <v>0.828929398412194</v>
+        <v>0.8297816154083356</v>
       </c>
       <c r="AN10" s="36" t="n">
-        <v>8.020751836387918</v>
+        <v>8.0228067451519</v>
       </c>
       <c r="AO10" s="88" t="n">
-        <v>1.811089167517567</v>
+        <v>1.810949435048805</v>
       </c>
       <c r="AP10" s="83" t="n">
         <v>65.51999664306641</v>
@@ -4253,36 +4253,36 @@
         <v>42.34999847412109</v>
       </c>
       <c r="AR10" s="36" t="n">
-        <v>-1.152315769384071</v>
+        <v>-1.14468870333706</v>
       </c>
       <c r="AS10" s="89" t="n">
-        <v>96.74148764314583</v>
+        <v>96.76305541963649</v>
       </c>
       <c r="AT10" s="33" t="n">
-        <v>0.01258599619603817</v>
+        <v>0.01266412711363518</v>
       </c>
       <c r="AU10" s="33" t="n">
-        <v>0.1263478154721467</v>
+        <v>0.1264347242272419</v>
       </c>
       <c r="AV10" s="33" t="n">
-        <v>0.1103205444298097</v>
+        <v>0.1104062165241195</v>
       </c>
       <c r="AW10" s="33" t="n">
-        <v>0.4485573857267353</v>
+        <v>0.4486691561029441</v>
       </c>
       <c r="AX10" s="90" t="inlineStr">
         <is>
+          <t>Sector Update: Energy Stocks Gain Late Afternoon</t>
+        </is>
+      </c>
+      <c r="AY10" s="90" t="inlineStr">
+        <is>
           <t>Sector Update: Energy</t>
         </is>
       </c>
-      <c r="AY10" s="90" t="inlineStr">
+      <c r="AZ10" s="90" t="inlineStr">
         <is>
           <t>Blowout jobs report raises worries of Fed rate hike: AlphaCheck</t>
-        </is>
-      </c>
-      <c r="AZ10" s="90" t="inlineStr">
-        <is>
-          <t>Bond yields still high as investors weigh rate hike risk: AlphaCheck</t>
         </is>
       </c>
     </row>
@@ -4296,7 +4296,7 @@
         </is>
       </c>
       <c r="C11" s="26" t="n">
-        <v>-0.006739178085651609</v>
+        <v>-0.006621011774235575</v>
       </c>
       <c r="D11" s="27" t="n">
         <v>7</v>
@@ -4365,10 +4365,10 @@
         </is>
       </c>
       <c r="R11" s="70" t="n">
-        <v>84.01000213623047</v>
+        <v>84.01999664306641</v>
       </c>
       <c r="S11" s="71" t="n">
-        <v>-0.5699996948242188</v>
+        <v>-0.5600051879882812</v>
       </c>
       <c r="T11" s="72" t="n">
         <v>84.27999877929688</v>
@@ -4380,61 +4380,61 @@
         <v>83.80999755859375</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>12346694</v>
+        <v>13529156</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.354485166758239</v>
+        <v>1.474641698026466</v>
       </c>
       <c r="Y11" s="28" t="n">
-        <v>42.33075771069067</v>
+        <v>42.37844791946197</v>
       </c>
       <c r="Z11" s="28" t="n">
-        <v>5.464600478608533</v>
+        <v>5.73767416264352</v>
       </c>
       <c r="AA11" s="28" t="n">
         <v>12.87555988659817</v>
       </c>
       <c r="AB11" s="75" t="n">
-        <v>-0.1007477601409761</v>
+        <v>-0.09995047754436825</v>
       </c>
       <c r="AC11" s="75" t="n">
-        <v>0.11973289205469</v>
+        <v>0.1198923485740115</v>
       </c>
       <c r="AD11" s="75" t="n">
-        <v>-0.220480652195666</v>
+        <v>-0.2198428261183798</v>
       </c>
       <c r="AE11" s="72" t="n">
-        <v>84.99988485064777</v>
+        <v>85.00210585216688</v>
       </c>
       <c r="AF11" s="72" t="n">
-        <v>85.29253610625362</v>
+        <v>85.29344469778415</v>
       </c>
       <c r="AG11" s="72" t="n">
-        <v>85.0181999206543</v>
+        <v>85.01839981079101</v>
       </c>
       <c r="AH11" s="72" t="n">
-        <v>84.41630012512206</v>
+        <v>84.41640007019043</v>
       </c>
       <c r="AI11" s="72" t="n">
-        <v>83.36030025482178</v>
+        <v>83.36035022735595</v>
       </c>
       <c r="AJ11" s="72" t="n">
-        <v>87.1005302755715</v>
+        <v>87.09913133087643</v>
       </c>
       <c r="AK11" s="72" t="n">
-        <v>85.51749992370605</v>
+        <v>85.51799964904785</v>
       </c>
       <c r="AL11" s="72" t="n">
-        <v>83.93446957184061</v>
+        <v>83.93686796721927</v>
       </c>
       <c r="AM11" s="76" t="n">
-        <v>0.02385695394306634</v>
+        <v>0.02628771430061936</v>
       </c>
       <c r="AN11" s="29" t="n">
-        <v>3.702237210577338</v>
+        <v>3.697775177897732</v>
       </c>
       <c r="AO11" s="77" t="n">
-        <v>1.279588493694595</v>
+        <v>1.279436281644388</v>
       </c>
       <c r="AP11" s="72" t="n">
         <v>90.13999938964844</v>
@@ -4443,22 +4443,22 @@
         <v>75.16000366210938</v>
       </c>
       <c r="AR11" s="29" t="n">
-        <v>-6.800529504021635</v>
+        <v>-6.789441743977697</v>
       </c>
       <c r="AS11" s="78" t="n">
-        <v>59.07877835940468</v>
+        <v>59.14549738267893</v>
       </c>
       <c r="AT11" s="26" t="n">
-        <v>-0.01141446437262328</v>
+        <v>-0.01129685427093907</v>
       </c>
       <c r="AU11" s="26" t="n">
-        <v>-0.01304042028354058</v>
+        <v>-0.01292300361867404</v>
       </c>
       <c r="AV11" s="26" t="n">
-        <v>0.01131578722594861</v>
+        <v>0.0114361015015314</v>
       </c>
       <c r="AW11" s="26" t="n">
-        <v>0.08148817979127787</v>
+        <v>0.08161684234015376</v>
       </c>
       <c r="AX11" s="79" t="inlineStr">
         <is>
@@ -4486,7 +4486,7 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>-0.007745252725428697</v>
+        <v>-0.008006315977894363</v>
       </c>
       <c r="D12" s="34" t="n">
         <v>8</v>
@@ -4555,10 +4555,10 @@
         </is>
       </c>
       <c r="R12" s="81" t="n">
-        <v>114.0199966430664</v>
+        <v>113.9899978637695</v>
       </c>
       <c r="S12" s="82" t="n">
-        <v>-0.8900070190429688</v>
+        <v>-0.9200057983398438</v>
       </c>
       <c r="T12" s="83" t="n">
         <v>114.4700012207031</v>
@@ -4570,61 +4570,61 @@
         <v>113.75</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>6525252</v>
+        <v>7811077</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>1.276748061804977</v>
+        <v>1.50934927929379</v>
       </c>
       <c r="Y12" s="35" t="n">
-        <v>42.03041121598466</v>
+        <v>41.94979478135864</v>
       </c>
       <c r="Z12" s="35" t="n">
-        <v>5.084684881435419</v>
+        <v>4.519735859032862</v>
       </c>
       <c r="AA12" s="35" t="n">
         <v>11.84696289897842</v>
       </c>
       <c r="AB12" s="86" t="n">
-        <v>-0.4180060848270131</v>
+        <v>-0.4203991498421402</v>
       </c>
       <c r="AC12" s="86" t="n">
-        <v>-0.01328083163369766</v>
+        <v>-0.01375944463672309</v>
       </c>
       <c r="AD12" s="86" t="n">
-        <v>-0.4047252531933154</v>
+        <v>-0.4066397052054171</v>
       </c>
       <c r="AE12" s="83" t="n">
-        <v>115.5151183888538</v>
+        <v>115.5084519934544</v>
       </c>
       <c r="AF12" s="83" t="n">
-        <v>116.2643500443745</v>
+        <v>116.2616228826202</v>
       </c>
       <c r="AG12" s="83" t="n">
-        <v>116.2415995788574</v>
+        <v>116.2409996032715</v>
       </c>
       <c r="AH12" s="83" t="n">
-        <v>116.9485998535156</v>
+        <v>116.9482998657227</v>
       </c>
       <c r="AI12" s="83" t="n">
-        <v>116.9775249099731</v>
+        <v>116.9773749160767</v>
       </c>
       <c r="AJ12" s="83" t="n">
-        <v>119.7805320092117</v>
+        <v>119.785077054902</v>
       </c>
       <c r="AK12" s="83" t="n">
-        <v>116.9054988861084</v>
+        <v>116.9039989471435</v>
       </c>
       <c r="AL12" s="83" t="n">
-        <v>114.0304657630052</v>
+        <v>114.0229208393851</v>
       </c>
       <c r="AM12" s="87" t="n">
-        <v>-0.001820695534708708</v>
+        <v>-0.005713655510921202</v>
       </c>
       <c r="AN12" s="36" t="n">
-        <v>4.918559264528974</v>
+        <v>4.928964164965954</v>
       </c>
       <c r="AO12" s="88" t="n">
-        <v>1.424836852364758</v>
+        <v>1.425211827073672</v>
       </c>
       <c r="AP12" s="83" t="n">
         <v>125.0100021362305</v>
@@ -4633,22 +4633,22 @@
         <v>105.1900024414062</v>
       </c>
       <c r="AR12" s="36" t="n">
-        <v>-8.791300940214075</v>
+        <v>-8.815298043473208</v>
       </c>
       <c r="AS12" s="89" t="n">
-        <v>44.55093005862162</v>
+        <v>44.39957395489419</v>
       </c>
       <c r="AT12" s="33" t="n">
-        <v>-0.02204305494080361</v>
+        <v>-0.02230035642668704</v>
       </c>
       <c r="AU12" s="33" t="n">
-        <v>-0.04872354361377162</v>
+        <v>-0.04897382543543116</v>
       </c>
       <c r="AV12" s="33" t="n">
-        <v>-0.01187280313570171</v>
+        <v>-0.01213278042537624</v>
       </c>
       <c r="AW12" s="33" t="n">
-        <v>-0.04513865550406393</v>
+        <v>-0.0453898805135009</v>
       </c>
       <c r="AX12" s="90" t="inlineStr">
         <is>
@@ -4676,7 +4676,7 @@
         </is>
       </c>
       <c r="C13" s="26" t="n">
-        <v>-0.004373809418090291</v>
+        <v>-0.004552371166540725</v>
       </c>
       <c r="D13" s="27" t="n">
         <v>5</v>
@@ -4727,7 +4727,7 @@
         </is>
       </c>
       <c r="N13" s="69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O13" s="23" t="inlineStr">
         <is>
@@ -4745,10 +4745,10 @@
         </is>
       </c>
       <c r="R13" s="70" t="n">
-        <v>111.5400009155273</v>
+        <v>111.5199966430664</v>
       </c>
       <c r="S13" s="71" t="n">
-        <v>-0.4899978637695312</v>
+        <v>-0.5100021362304688</v>
       </c>
       <c r="T13" s="72" t="n">
         <v>111.5899963378906</v>
@@ -4760,61 +4760,61 @@
         <v>110.9649963378906</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>4982154</v>
+        <v>5655285</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>1.238270563796091</v>
+        <v>1.393911231801117</v>
       </c>
       <c r="Y13" s="28" t="n">
-        <v>50.0460883623922</v>
+        <v>49.97831737646933</v>
       </c>
       <c r="Z13" s="28" t="n">
-        <v>31.93070849487565</v>
+        <v>31.43555334815148</v>
       </c>
       <c r="AA13" s="28" t="n">
         <v>13.13904941230394</v>
       </c>
       <c r="AB13" s="75" t="n">
-        <v>0.4027184257243022</v>
+        <v>0.4011226433057686</v>
       </c>
       <c r="AC13" s="75" t="n">
-        <v>0.4474488952950639</v>
+        <v>0.4471297388113572</v>
       </c>
       <c r="AD13" s="75" t="n">
-        <v>-0.04473046957076171</v>
+        <v>-0.04600709550558857</v>
       </c>
       <c r="AE13" s="72" t="n">
-        <v>112.0317307051708</v>
+        <v>112.0272853112906</v>
       </c>
       <c r="AF13" s="72" t="n">
-        <v>111.6796184425315</v>
+        <v>111.6777998723077</v>
       </c>
       <c r="AG13" s="72" t="n">
-        <v>110.6949995422363</v>
+        <v>110.6945994567871</v>
       </c>
       <c r="AH13" s="72" t="n">
-        <v>112.4790998840332</v>
+        <v>112.4788998413086</v>
       </c>
       <c r="AI13" s="72" t="n">
-        <v>114.0217999649048</v>
+        <v>114.0216999435425</v>
       </c>
       <c r="AJ13" s="72" t="n">
-        <v>113.6536239281415</v>
+        <v>113.6532003749035</v>
       </c>
       <c r="AK13" s="72" t="n">
-        <v>111.7979995727539</v>
+        <v>111.7969993591309</v>
       </c>
       <c r="AL13" s="72" t="n">
-        <v>109.9423752173663</v>
+        <v>109.9407983433583</v>
       </c>
       <c r="AM13" s="76" t="n">
-        <v>0.4304819813133256</v>
+        <v>0.4253845047732718</v>
       </c>
       <c r="AN13" s="29" t="n">
-        <v>3.319602072450357</v>
+        <v>3.320663392422275</v>
       </c>
       <c r="AO13" s="77" t="n">
-        <v>1.482865681273606</v>
+        <v>1.483131675265752</v>
       </c>
       <c r="AP13" s="72" t="n">
         <v>120.4049987792969</v>
@@ -4823,22 +4823,22 @@
         <v>105.0299987792969</v>
       </c>
       <c r="AR13" s="29" t="n">
-        <v>-7.36264935313784</v>
+        <v>-7.379263507586376</v>
       </c>
       <c r="AS13" s="78" t="n">
-        <v>42.34147730881605</v>
+        <v>42.21136821963923</v>
       </c>
       <c r="AT13" s="26" t="n">
-        <v>0.0007177627104955064</v>
+        <v>0.0005382878080617548</v>
       </c>
       <c r="AU13" s="26" t="n">
-        <v>0.002606749802492869</v>
+        <v>0.002426936117450929</v>
       </c>
       <c r="AV13" s="26" t="n">
-        <v>0.004050810986328424</v>
+        <v>0.003870738314437405</v>
       </c>
       <c r="AW13" s="26" t="n">
-        <v>-0.05249745362803238</v>
+        <v>-0.05266738458499387</v>
       </c>
       <c r="AX13" s="79" t="inlineStr">
         <is>
@@ -4866,7 +4866,7 @@
         </is>
       </c>
       <c r="C14" s="33" t="n">
-        <v>-0.009343971712462262</v>
+        <v>-0.009534706580738517</v>
       </c>
       <c r="D14" s="34" t="n">
         <v>9</v>
@@ -4935,10 +4935,10 @@
         </is>
       </c>
       <c r="R14" s="81" t="n">
-        <v>51.95000076293945</v>
+        <v>51.93999862670898</v>
       </c>
       <c r="S14" s="82" t="n">
-        <v>-0.4899978637695312</v>
+        <v>-0.5</v>
       </c>
       <c r="T14" s="83" t="n">
         <v>52.36000061035156</v>
@@ -4950,61 +4950,61 @@
         <v>51.93500137329102</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>11452863</v>
+        <v>11931041</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>1.061074331944015</v>
+        <v>1.102933032370742</v>
       </c>
       <c r="Y14" s="35" t="n">
-        <v>45.41830871370646</v>
+        <v>45.3425445112604</v>
       </c>
       <c r="Z14" s="35" t="n">
-        <v>0.6651622136436071</v>
+        <v>0.2216079602932668</v>
       </c>
       <c r="AA14" s="35" t="n">
         <v>14.50877910679219</v>
       </c>
       <c r="AB14" s="86" t="n">
-        <v>0.1496393737477248</v>
+        <v>0.1488414825384581</v>
       </c>
       <c r="AC14" s="86" t="n">
-        <v>0.3131854786829287</v>
+        <v>0.3130259004410754</v>
       </c>
       <c r="AD14" s="86" t="n">
-        <v>-0.1635461049352038</v>
+        <v>-0.1641844179026173</v>
       </c>
       <c r="AE14" s="83" t="n">
-        <v>52.55559031552365</v>
+        <v>52.55336761858355</v>
       </c>
       <c r="AF14" s="83" t="n">
-        <v>52.5578155659165</v>
+        <v>52.55690628080464</v>
       </c>
       <c r="AG14" s="83" t="n">
-        <v>51.82979988098145</v>
+        <v>51.82959983825683</v>
       </c>
       <c r="AH14" s="83" t="n">
-        <v>51.57810001373291</v>
+        <v>51.57799999237061</v>
       </c>
       <c r="AI14" s="83" t="n">
-        <v>50.11670000076294</v>
+        <v>50.11664999008179</v>
       </c>
       <c r="AJ14" s="83" t="n">
-        <v>53.88709838608983</v>
+        <v>53.88803275778218</v>
       </c>
       <c r="AK14" s="83" t="n">
-        <v>52.75650024414062</v>
+        <v>52.7560001373291</v>
       </c>
       <c r="AL14" s="83" t="n">
-        <v>51.62590210219142</v>
+        <v>51.62396751687603</v>
       </c>
       <c r="AM14" s="87" t="n">
-        <v>0.1433306179812365</v>
+        <v>0.1395856904311072</v>
       </c>
       <c r="AN14" s="36" t="n">
-        <v>4.286099861503896</v>
+        <v>4.291578654584431</v>
       </c>
       <c r="AO14" s="88" t="n">
-        <v>1.595094859565964</v>
+        <v>1.595402028539928</v>
       </c>
       <c r="AP14" s="83" t="n">
         <v>54.18999862670898</v>
@@ -5013,22 +5013,22 @@
         <v>42.03499984741211</v>
       </c>
       <c r="AR14" s="36" t="n">
-        <v>-4.133600148617623</v>
+        <v>-4.15205768042044</v>
       </c>
       <c r="AS14" s="89" t="n">
-        <v>81.57138553082515</v>
+        <v>81.48909727714383</v>
       </c>
       <c r="AT14" s="33" t="n">
-        <v>-0.01404437052678953</v>
+        <v>-0.0142342004089524</v>
       </c>
       <c r="AU14" s="33" t="n">
-        <v>-0.0172152825748153</v>
+        <v>-0.0174045019489163</v>
       </c>
       <c r="AV14" s="33" t="n">
-        <v>0.03983189981853474</v>
+        <v>0.03963169692794688</v>
       </c>
       <c r="AW14" s="33" t="n">
-        <v>0.1455347852455748</v>
+        <v>0.1453142309662583</v>
       </c>
       <c r="AX14" s="90" t="inlineStr">
         <is>
@@ -5140,10 +5140,10 @@
         <v>187.0200042724609</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>7886687</v>
+        <v>8376789</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>1.302504012642008</v>
+        <v>1.377869119351926</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>56.207320537553</v>
@@ -5246,7 +5246,7 @@
         </is>
       </c>
       <c r="C16" s="33" t="n">
-        <v>-0.0007967185788519959</v>
+        <v>-0.0006828768287838738</v>
       </c>
       <c r="D16" s="34" t="n">
         <v>4</v>
@@ -5315,10 +5315,10 @@
         </is>
       </c>
       <c r="R16" s="81" t="n">
-        <v>43.89500045776367</v>
+        <v>43.90000152587891</v>
       </c>
       <c r="S16" s="82" t="n">
-        <v>-0.03499984741210938</v>
+        <v>-0.029998779296875</v>
       </c>
       <c r="T16" s="83" t="n">
         <v>43.66500091552734</v>
@@ -5330,61 +5330,61 @@
         <v>43.66120147705078</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>4716707</v>
+        <v>4811042</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>0.9223504831401624</v>
+        <v>0.9399307075299359</v>
       </c>
       <c r="Y16" s="35" t="n">
-        <v>39.81401726539807</v>
+        <v>39.86747270631402</v>
       </c>
       <c r="Z16" s="35" t="n">
-        <v>17.36850347538719</v>
+        <v>17.63171737532977</v>
       </c>
       <c r="AA16" s="35" t="n">
         <v>16.09873250539317</v>
       </c>
       <c r="AB16" s="86" t="n">
-        <v>-0.264953969438757</v>
+        <v>-0.2645550238341272</v>
       </c>
       <c r="AC16" s="86" t="n">
-        <v>-0.152846591403284</v>
+        <v>-0.1527668022823581</v>
       </c>
       <c r="AD16" s="86" t="n">
-        <v>-0.112107378035473</v>
+        <v>-0.1117882215517692</v>
       </c>
       <c r="AE16" s="83" t="n">
-        <v>44.17683746697216</v>
+        <v>44.17794881544221</v>
       </c>
       <c r="AF16" s="83" t="n">
-        <v>44.52978563175613</v>
+        <v>44.53024027431206</v>
       </c>
       <c r="AG16" s="83" t="n">
-        <v>44.82130020141602</v>
+        <v>44.82140022277832</v>
       </c>
       <c r="AH16" s="83" t="n">
-        <v>44.54565021514892</v>
+        <v>44.54570022583007</v>
       </c>
       <c r="AI16" s="83" t="n">
-        <v>43.0836750793457</v>
+        <v>43.08370008468628</v>
       </c>
       <c r="AJ16" s="83" t="n">
-        <v>45.662080349638</v>
+        <v>45.66163291099435</v>
       </c>
       <c r="AK16" s="83" t="n">
-        <v>44.62225074768067</v>
+        <v>44.62250080108642</v>
       </c>
       <c r="AL16" s="83" t="n">
-        <v>43.58242114572334</v>
+        <v>43.5833686911785</v>
       </c>
       <c r="AM16" s="87" t="n">
-        <v>0.1503031417128099</v>
+        <v>0.1523544656552202</v>
       </c>
       <c r="AN16" s="36" t="n">
-        <v>4.660587866072071</v>
+        <v>4.657435559428015</v>
       </c>
       <c r="AO16" s="88" t="n">
-        <v>1.189080427172075</v>
+        <v>1.188944967673121</v>
       </c>
       <c r="AP16" s="83" t="n">
         <v>46.45500183105469</v>
@@ -5393,22 +5393,22 @@
         <v>39.72499847412109</v>
       </c>
       <c r="AR16" s="36" t="n">
-        <v>-5.510712027525266</v>
+        <v>-5.499946624623298</v>
       </c>
       <c r="AS16" s="89" t="n">
-        <v>61.96136558158517</v>
+        <v>62.03567562052567</v>
       </c>
       <c r="AT16" s="33" t="n">
-        <v>-0.004874181582700698</v>
+        <v>-0.004760804388276862</v>
       </c>
       <c r="AU16" s="33" t="n">
-        <v>-0.0241218118166906</v>
+        <v>-0.02401062755332628</v>
       </c>
       <c r="AV16" s="33" t="n">
-        <v>-0.003066053265408653</v>
+        <v>-0.00295247006636512</v>
       </c>
       <c r="AW16" s="33" t="n">
-        <v>0.08785631022802143</v>
+        <v>0.08798025244126451</v>
       </c>
       <c r="AX16" s="90" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G17" s="23" t="inlineStr">
@@ -5487,11 +5487,11 @@
         </is>
       </c>
       <c r="N17" s="69" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O17" s="23" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="P17" s="25" t="inlineStr">
@@ -5520,10 +5520,10 @@
         <v>43.03499984741211</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>16898692</v>
+        <v>19693441</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>0.8572600883809205</v>
+        <v>0.9920038487658337</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>48.76529694830028</v>
@@ -5645,7 +5645,7 @@
         </is>
       </c>
       <c r="C19" s="26" t="n">
-        <v>-0.005440219203215357</v>
+        <v>-0.005492125910932955</v>
       </c>
       <c r="D19" s="27" t="n">
         <v>4</v>
@@ -5657,24 +5657,24 @@
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G19" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I19" s="23" t="inlineStr">
+        <is>
           <t>Same</t>
         </is>
       </c>
-      <c r="G19" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H19" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I19" s="23" t="inlineStr">
-        <is>
-          <t>Same</t>
-        </is>
-      </c>
       <c r="J19" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5696,11 +5696,11 @@
         </is>
       </c>
       <c r="N19" s="69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O19" s="23" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P19" s="25" t="inlineStr">
@@ -5714,10 +5714,10 @@
         </is>
       </c>
       <c r="R19" s="70" t="n">
-        <v>766</v>
+        <v>765.9600219726562</v>
       </c>
       <c r="S19" s="71" t="n">
-        <v>-4.19000244140625</v>
+        <v>-4.22998046875</v>
       </c>
       <c r="T19" s="72" t="n">
         <v>769.0700073242188</v>
@@ -5729,61 +5729,61 @@
         <v>765.1500244140625</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>33180231</v>
+        <v>43496831</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.9212233075687043</v>
+        <v>1.190604301859171</v>
       </c>
       <c r="Y19" s="28" t="n">
-        <v>51.40173051184327</v>
+        <v>51.36463221333177</v>
       </c>
       <c r="Z19" s="28" t="n">
-        <v>41.21375798144255</v>
+        <v>40.96105248943845</v>
       </c>
       <c r="AA19" s="28" t="n">
         <v>13.08669418896927</v>
       </c>
       <c r="AB19" s="75" t="n">
-        <v>2.700022622934398</v>
+        <v>2.69683349254808</v>
       </c>
       <c r="AC19" s="75" t="n">
-        <v>3.527417499015546</v>
+        <v>3.526779672938283</v>
       </c>
       <c r="AD19" s="75" t="n">
-        <v>-0.827394876081148</v>
+        <v>-0.8299461803902024</v>
       </c>
       <c r="AE19" s="72" t="n">
-        <v>767.7563723965673</v>
+        <v>767.7474883904908</v>
       </c>
       <c r="AF19" s="72" t="n">
-        <v>766.0049335212183</v>
+        <v>766.0012991550961</v>
       </c>
       <c r="AG19" s="72" t="n">
-        <v>757.5974011230469</v>
+        <v>757.5966015625</v>
       </c>
       <c r="AH19" s="72" t="n">
-        <v>745.9744006347656</v>
+        <v>745.9740008544921</v>
       </c>
       <c r="AI19" s="72" t="n">
-        <v>712.6825003051758</v>
+        <v>712.6823004150391</v>
       </c>
       <c r="AJ19" s="72" t="n">
-        <v>777.2434484569314</v>
+        <v>777.2439956536774</v>
       </c>
       <c r="AK19" s="72" t="n">
-        <v>768.7014923095703</v>
+        <v>768.6994934082031</v>
       </c>
       <c r="AL19" s="72" t="n">
-        <v>760.1595361622092</v>
+        <v>760.1549911627288</v>
       </c>
       <c r="AM19" s="76" t="n">
-        <v>0.3418692239244939</v>
+        <v>0.3396939132997553</v>
       </c>
       <c r="AN19" s="29" t="n">
-        <v>2.222437768839697</v>
+        <v>2.22310599102656</v>
       </c>
       <c r="AO19" s="77" t="n">
-        <v>0.8009022879495987</v>
+        <v>0.8009440897312178</v>
       </c>
       <c r="AP19" s="72" t="n">
         <v>779.3699951171875</v>
@@ -5792,22 +5792,22 @@
         <v>629.280029296875</v>
       </c>
       <c r="AR19" s="29" t="n">
-        <v>-1.715487534925841</v>
+        <v>-1.720617066161867</v>
       </c>
       <c r="AS19" s="78" t="n">
-        <v>91.09201268444951</v>
+        <v>91.06537664177654</v>
       </c>
       <c r="AT19" s="26" t="n">
-        <v>-0.001368864884529697</v>
+        <v>-0.00142098407881952</v>
       </c>
       <c r="AU19" s="26" t="n">
-        <v>-0.009388833864336976</v>
+        <v>-0.009440534491343189</v>
       </c>
       <c r="AV19" s="26" t="n">
-        <v>0.03622741586838174</v>
+        <v>0.03617333450027993</v>
       </c>
       <c r="AW19" s="26" t="n">
-        <v>0.1232989488459109</v>
+        <v>0.1232403231591064</v>
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
@@ -5816,12 +5816,12 @@
       </c>
       <c r="AY19" s="79" t="inlineStr">
         <is>
-          <t>5 Leveraged ETF Areas of Last Week</t>
+          <t>QQQ vs QQQM: Same Index, Same Stocks, Different Fee – and the Math Says One Leaves You Thousands Richer</t>
         </is>
       </c>
       <c r="AZ19" s="79" t="inlineStr">
         <is>
-          <t>Amgen Falls 10% as Novartis Trial Failure Clouds a Cholesterol Drug Class; NVS Stock Drops 14%</t>
+          <t>XYLD vs GPIX vs ISPY: We Compared 3 Ways to Sell Covered Calls on the S&amp;P 500, and the Highest Yield Is Not...</t>
         </is>
       </c>
     </row>
@@ -5917,10 +5917,10 @@
         <v>715.5700073242188</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>26307263</v>
+        <v>27628455</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.8543886996114936</v>
+        <v>0.8953764660533405</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>53.18709936797907</v>
@@ -5999,17 +5999,17 @@
       </c>
       <c r="AX20" s="90" t="inlineStr">
         <is>
+          <t>QQQ vs QQQM: Same Index, Same Stocks, Different Fee – and the Math Says One Leaves You Thousands Richer</t>
+        </is>
+      </c>
+      <c r="AY20" s="90" t="inlineStr">
+        <is>
           <t>Exchange-Traded Funds Mixed, US Equities Fall After Midday</t>
         </is>
       </c>
-      <c r="AY20" s="90" t="inlineStr">
+      <c r="AZ20" s="90" t="inlineStr">
         <is>
           <t>QQQ Charged 0.20% for Years. The Fee Only Fell After Shareholders Approved a Structural Change</t>
-        </is>
-      </c>
-      <c r="AZ20" s="90" t="inlineStr">
-        <is>
-          <t>This ETF Would Have Increased Your Investment by 6x Over the Past 10 Years -- and It's Still Soaring</t>
         </is>
       </c>
     </row>
@@ -6021,7 +6021,7 @@
         </is>
       </c>
       <c r="C21" s="26" t="n">
-        <v>-0.004459333403163956</v>
+        <v>-0.004526861571173213</v>
       </c>
       <c r="D21" s="27" t="n">
         <v>3</v>
@@ -6090,10 +6090,10 @@
         </is>
       </c>
       <c r="R21" s="70" t="n">
-        <v>294.6900024414062</v>
+        <v>294.6700134277344</v>
       </c>
       <c r="S21" s="71" t="n">
-        <v>-1.32000732421875</v>
+        <v>-1.339996337890625</v>
       </c>
       <c r="T21" s="72" t="n">
         <v>295.3399963378906</v>
@@ -6105,61 +6105,61 @@
         <v>294.260009765625</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>16255655</v>
+        <v>17205591</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>0.972248943536787</v>
+        <v>1.026149448371472</v>
       </c>
       <c r="Y21" s="28" t="n">
-        <v>45.94367785704903</v>
+        <v>45.91187219850499</v>
       </c>
       <c r="Z21" s="28" t="n">
-        <v>35.11905032220562</v>
+        <v>34.97032256892567</v>
       </c>
       <c r="AA21" s="28" t="n">
         <v>20.40181804023351</v>
       </c>
       <c r="AB21" s="75" t="n">
-        <v>-0.7766837930649331</v>
+        <v>-0.7782783582580919</v>
       </c>
       <c r="AC21" s="75" t="n">
-        <v>-0.09091189393194882</v>
+        <v>-0.09123080697058059</v>
       </c>
       <c r="AD21" s="75" t="n">
-        <v>-0.6857718991329842</v>
+        <v>-0.6870475512875113</v>
       </c>
       <c r="AE21" s="72" t="n">
-        <v>295.4424999715379</v>
+        <v>295.4380579684997</v>
       </c>
       <c r="AF21" s="72" t="n">
-        <v>296.819596016579</v>
+        <v>296.8177788335179</v>
       </c>
       <c r="AG21" s="72" t="n">
-        <v>296.911201171875</v>
+        <v>296.9108013916016</v>
       </c>
       <c r="AH21" s="72" t="n">
-        <v>290.7589010620117</v>
+        <v>290.758701171875</v>
       </c>
       <c r="AI21" s="72" t="n">
-        <v>272.9868504333496</v>
+        <v>272.9867504882812</v>
       </c>
       <c r="AJ21" s="72" t="n">
-        <v>306.1524612384081</v>
+        <v>306.1535370427105</v>
       </c>
       <c r="AK21" s="72" t="n">
-        <v>298.6010009765625</v>
+        <v>298.6000015258789</v>
       </c>
       <c r="AL21" s="72" t="n">
-        <v>291.0495407147169</v>
+        <v>291.0464660090473</v>
       </c>
       <c r="AM21" s="76" t="n">
-        <v>0.241043559818695</v>
+        <v>0.2398577070705955</v>
       </c>
       <c r="AN21" s="29" t="n">
-        <v>5.057893467971538</v>
+        <v>5.059300387295496</v>
       </c>
       <c r="AO21" s="77" t="n">
-        <v>1.083401409175358</v>
+        <v>1.083474901979489</v>
       </c>
       <c r="AP21" s="72" t="n">
         <v>305.1799926757812</v>
@@ -6168,22 +6168,22 @@
         <v>228.8999938964844</v>
       </c>
       <c r="AR21" s="29" t="n">
-        <v>-3.437312565086603</v>
+        <v>-3.443862474697845</v>
       </c>
       <c r="AS21" s="78" t="n">
-        <v>86.24804614283491</v>
+        <v>86.22184135259926</v>
       </c>
       <c r="AT21" s="26" t="n">
-        <v>0.00258568293322603</v>
+        <v>0.002517676897197063</v>
       </c>
       <c r="AU21" s="26" t="n">
-        <v>-0.02278152000532707</v>
+        <v>-0.02284780536755593</v>
       </c>
       <c r="AV21" s="26" t="n">
-        <v>0.03723915960486868</v>
+        <v>0.03716880300107972</v>
       </c>
       <c r="AW21" s="26" t="n">
-        <v>0.197148188403147</v>
+        <v>0.1970669850663964</v>
       </c>
       <c r="AX21" s="79" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>0.05192704664625403</v>
+        <v>0.05107433429498753</v>
       </c>
       <c r="D22" s="34" t="n">
         <v>1</v>
@@ -6278,10 +6278,10 @@
         </is>
       </c>
       <c r="R22" s="81" t="n">
-        <v>123.370002746582</v>
+        <v>123.2699966430664</v>
       </c>
       <c r="S22" s="82" t="n">
-        <v>6.090003967285156</v>
+        <v>5.989997863769531</v>
       </c>
       <c r="T22" s="83" t="n">
         <v>125.120002746582</v>
@@ -6293,61 +6293,61 @@
         <v>121.5999984741211</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>50614561</v>
+        <v>51964601</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>0.930653151956731</v>
+        <v>0.9542919908418375</v>
       </c>
       <c r="Y22" s="35" t="n">
-        <v>48.67183074907373</v>
+        <v>48.62192842970096</v>
       </c>
       <c r="Z22" s="35" t="n">
-        <v>70.47265963670442</v>
+        <v>70.1879042389408</v>
       </c>
       <c r="AA22" s="35" t="n">
         <v>18.43662711393569</v>
       </c>
       <c r="AB22" s="86" t="n">
-        <v>-8.466572093303455</v>
+        <v>-8.474549788170805</v>
       </c>
       <c r="AC22" s="86" t="n">
-        <v>-9.958002980836323</v>
+        <v>-9.959598519809793</v>
       </c>
       <c r="AD22" s="86" t="n">
-        <v>1.491430887532868</v>
+        <v>1.485048731638988</v>
       </c>
       <c r="AE22" s="83" t="n">
-        <v>115.3842379020385</v>
+        <v>115.3620143234794</v>
       </c>
       <c r="AF22" s="83" t="n">
-        <v>121.8404244499269</v>
+        <v>121.8313329859709</v>
       </c>
       <c r="AG22" s="83" t="n">
-        <v>143.3635997009277</v>
+        <v>143.3615995788574</v>
       </c>
       <c r="AH22" s="83" t="n">
-        <v>164.1635001373291</v>
+        <v>164.162500076294</v>
       </c>
       <c r="AI22" s="83" t="n">
-        <v>109.264599981308</v>
+        <v>109.2640999507904</v>
       </c>
       <c r="AJ22" s="83" t="n">
-        <v>150.0256692158687</v>
+        <v>150.0204269432186</v>
       </c>
       <c r="AK22" s="83" t="n">
-        <v>122.9955001831055</v>
+        <v>122.9904998779297</v>
       </c>
       <c r="AL22" s="83" t="n">
-        <v>95.96533115034225</v>
+        <v>95.96057281264075</v>
       </c>
       <c r="AM22" s="87" t="n">
-        <v>0.5069274920741826</v>
+        <v>0.5051701353921823</v>
       </c>
       <c r="AN22" s="36" t="n">
-        <v>43.95310233711469</v>
+        <v>43.9544958222247</v>
       </c>
       <c r="AO22" s="88" t="n">
-        <v>10.875870442058</v>
+        <v>10.88469378475996</v>
       </c>
       <c r="AP22" s="83" t="n">
         <v>302</v>
@@ -6356,22 +6356,22 @@
         <v>26.56999969482422</v>
       </c>
       <c r="AR22" s="36" t="n">
-        <v>-59.1490057130523</v>
+        <v>-59.18212031686543</v>
       </c>
       <c r="AS22" s="89" t="n">
-        <v>35.14504699724201</v>
+        <v>35.10873791565872</v>
       </c>
       <c r="AT22" s="33" t="n">
-        <v>0.09380265755098671</v>
+        <v>0.09291600002191625</v>
       </c>
       <c r="AU22" s="33" t="n">
-        <v>-0.1203564866553866</v>
+        <v>-0.1210695426519329</v>
       </c>
       <c r="AV22" s="33" t="n">
-        <v>-0.4165247761914398</v>
+        <v>-0.4169977524606457</v>
       </c>
       <c r="AW22" s="33" t="n">
-        <v>1.935284471322697</v>
+        <v>1.932905073120933</v>
       </c>
       <c r="AX22" s="90" t="inlineStr">
         <is>
@@ -6502,10 +6502,10 @@
         <v>314.9200134277344</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>31822388</v>
+        <v>35028027</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.8158837852712565</v>
+        <v>0.894396665511635</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>50.1995004401049</v>
@@ -6589,12 +6589,12 @@
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
-          <t>How Apple's stock is performing ahead of a pivotal product launch</t>
+          <t>Apple Is Set to Reveal New iPhones Wednesday—Here’s What You Need to Know</t>
         </is>
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Apple to Unveil First Foldable Phone</t>
+          <t>Apple event expected to debut foldable iPhone and new CEO John Ternus</t>
         </is>
       </c>
     </row>
@@ -6690,10 +6690,10 @@
         <v>486.5705871582031</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>26808296</v>
+        <v>27979240</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>1.50087064428304</v>
+        <v>1.561308671128961</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>57.03501141183438</v>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>F-Secure and AMD Silo AI Demonstrate Unique Approach to Helping Secure Digital Journeys in Agentic AI Era</t>
+          <t>Dow Jones Futures: Dow Skids But AMD, HPE Are New Buys; Apple iPhone Event Due</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices Sees AI Boom Fueling MI450, Helios and Server CPU Growth</t>
+          <t>AMD Just Put a $70 Billion Number on Its AI Ambitions</t>
         </is>
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>AI-Optimized Processors Fuel Advanced Micro Devices (AMD) Stock Growth</t>
+          <t>Why AMD Stock Popped Today?</t>
         </is>
       </c>
     </row>
@@ -6878,10 +6878,10 @@
         <v>254.75</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>26723936</v>
+        <v>28792611</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.8287435702599156</v>
+        <v>0.8900409310757634</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>48.12096671477681</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
-          <t>Qualcomm and Amazon ink deal for custom data center chips</t>
+          <t>AMD Jumps 6.7% While Amazon Opens a $60 Billion AI-Chip Door</t>
         </is>
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Qualcomm Stock Rises 6% on Multi-Generation Amazon Silicon Deal</t>
+          <t>Spotting Winners: Amazon (NASDAQ:AMZN) And Online Retail Stocks In Q2</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>The Market Marked AMZN Stock Down. The Numbers Push Back</t>
+          <t>DAL Stock Drops: Jefferies Sees Possible Snag To In-Cabin Experience Owing To SPCX-VSAT Spectrum Fight</t>
         </is>
       </c>
     </row>
@@ -6982,7 +6982,7 @@
         </is>
       </c>
       <c r="C27" s="33" t="n">
-        <v>-0.001159805992870688</v>
+        <v>-0.001623746087524025</v>
       </c>
       <c r="D27" s="34" t="n">
         <v>17</v>
@@ -6994,12 +6994,12 @@
       </c>
       <c r="F27" s="30" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G27" s="30" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H27" s="30" t="inlineStr">
@@ -7051,10 +7051,10 @@
         </is>
       </c>
       <c r="R27" s="81" t="n">
-        <v>86.12000274658203</v>
+        <v>86.08000183105469</v>
       </c>
       <c r="S27" s="82" t="n">
-        <v>-0.09999847412109375</v>
+        <v>-0.1399993896484375</v>
       </c>
       <c r="T27" s="83" t="n">
         <v>86.15000152587891</v>
@@ -7066,61 +7066,61 @@
         <v>85.20999908447266</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>3495437</v>
+        <v>3752324</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>0.7502544777912034</v>
+        <v>0.8031779813299504</v>
       </c>
       <c r="Y27" s="35" t="n">
-        <v>58.08830973887118</v>
+        <v>57.98587981166301</v>
       </c>
       <c r="Z27" s="35" t="n">
-        <v>76.57536479986958</v>
+        <v>76.02740728199275</v>
       </c>
       <c r="AA27" s="35" t="n">
         <v>25.45153673228566</v>
       </c>
       <c r="AB27" s="86" t="n">
-        <v>2.012868107416338</v>
+        <v>2.009677151191951</v>
       </c>
       <c r="AC27" s="86" t="n">
-        <v>2.021930047903917</v>
+        <v>2.021291856659039</v>
       </c>
       <c r="AD27" s="86" t="n">
-        <v>-0.009061940487578468</v>
+        <v>-0.01161470546708765</v>
       </c>
       <c r="AE27" s="83" t="n">
-        <v>85.39998872695128</v>
+        <v>85.39109963461188</v>
       </c>
       <c r="AF27" s="83" t="n">
-        <v>83.47866146236734</v>
+        <v>83.47502501550122</v>
       </c>
       <c r="AG27" s="83" t="n">
-        <v>79.91199966430663</v>
+        <v>79.91119964599609</v>
       </c>
       <c r="AH27" s="83" t="n">
-        <v>78.68219993591309</v>
+        <v>78.68179992675782</v>
       </c>
       <c r="AI27" s="83" t="n">
-        <v>76.97935010910034</v>
+        <v>76.9791501045227</v>
       </c>
       <c r="AJ27" s="83" t="n">
-        <v>88.5677000647153</v>
+        <v>88.56196773119783</v>
       </c>
       <c r="AK27" s="83" t="n">
-        <v>83.94549942016602</v>
+        <v>83.94349937438965</v>
       </c>
       <c r="AL27" s="83" t="n">
-        <v>79.32329877561673</v>
+        <v>79.32503101758147</v>
       </c>
       <c r="AM27" s="87" t="n">
-        <v>0.7352238136806429</v>
+        <v>0.7312998911766473</v>
       </c>
       <c r="AN27" s="36" t="n">
-        <v>11.0123846459335</v>
+        <v>11.00375464741998</v>
       </c>
       <c r="AO27" s="88" t="n">
-        <v>2.701031624354151</v>
+        <v>2.702286779274508</v>
       </c>
       <c r="AP27" s="83" t="n">
         <v>92.65000152587891</v>
@@ -7129,22 +7129,22 @@
         <v>62.94499969482422</v>
       </c>
       <c r="AR27" s="36" t="n">
-        <v>-7.048028787644345</v>
+        <v>-7.091203007685964</v>
       </c>
       <c r="AS27" s="89" t="n">
-        <v>78.0171742912664</v>
+        <v>77.88251375242905</v>
       </c>
       <c r="AT27" s="33" t="n">
-        <v>0.006427521955350457</v>
+        <v>0.005960057707716793</v>
       </c>
       <c r="AU27" s="33" t="n">
-        <v>0.08422513427801559</v>
+        <v>0.08372153468877142</v>
       </c>
       <c r="AV27" s="33" t="n">
-        <v>0.1349499982052622</v>
+        <v>0.1344228379920938</v>
       </c>
       <c r="AW27" s="33" t="n">
-        <v>0.1196048465501784</v>
+        <v>0.1190848138346356</v>
       </c>
       <c r="AX27" s="90" t="inlineStr">
         <is>
@@ -7254,10 +7254,10 @@
         <v>254.6399993896484</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>4946625</v>
+        <v>5095872</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>1.326304041451819</v>
+        <v>1.363592284656718</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>52.24195279097528</v>
@@ -7442,10 +7442,10 @@
         <v>63.15000152587891</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>11761743</v>
+        <v>12009781</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>1.181540009923967</v>
+        <v>1.204955773479053</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>52.47674092186459</v>
@@ -7630,10 +7630,10 @@
         <v>362.739990234375</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>26562775</v>
+        <v>29871614</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>1.102738743969184</v>
+        <v>1.231644128817539</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>45.33346661314823</v>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Broadcom CEO Sees AI Value Flowing to Frontier Models and Custom Chips</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
+          <t>Intel Leads Chip Stocks Rally as Qualcomm, AMD and Broadcom Stocks Jump</t>
+        </is>
+      </c>
+      <c r="AZ30" s="79" t="inlineStr">
+        <is>
           <t>Why Broadcom Stock Rallied Tuesday Morning</t>
-        </is>
-      </c>
-      <c r="AY30" s="79" t="inlineStr">
-        <is>
-          <t>Jim Cramer picks Nvidia and Broadcom as OpenAI GPT-6 Astra winners</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Amazon Just Handed Qualcomm a Slice of AWS’s AI Buildout</t>
         </is>
       </c>
     </row>
@@ -7734,7 +7734,7 @@
         </is>
       </c>
       <c r="C31" s="33" t="n">
-        <v>0.01211039553875048</v>
+        <v>0.0122096821820159</v>
       </c>
       <c r="D31" s="34" t="n">
         <v>14</v>
@@ -7803,10 +7803,10 @@
         </is>
       </c>
       <c r="R31" s="81" t="n">
-        <v>101.9599990844727</v>
+        <v>101.9700012207031</v>
       </c>
       <c r="S31" s="82" t="n">
-        <v>1.220001220703125</v>
+        <v>1.230003356933594</v>
       </c>
       <c r="T31" s="83" t="n">
         <v>102.495002746582</v>
@@ -7818,61 +7818,61 @@
         <v>101.5500030517578</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>1929177</v>
+        <v>2186442</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.7278364563826674</v>
+        <v>0.820913025928136</v>
       </c>
       <c r="Y31" s="35" t="n">
-        <v>56.00903873570904</v>
+        <v>56.02439410574521</v>
       </c>
       <c r="Z31" s="35" t="n">
-        <v>45.06880453003986</v>
+        <v>45.12615622058046</v>
       </c>
       <c r="AA31" s="35" t="n">
         <v>15.37669590983723</v>
       </c>
       <c r="AB31" s="86" t="n">
-        <v>1.363456883782675</v>
+        <v>1.364254774991949</v>
       </c>
       <c r="AC31" s="86" t="n">
-        <v>1.571725691618105</v>
+        <v>1.57188526985996</v>
       </c>
       <c r="AD31" s="86" t="n">
-        <v>-0.2082688078354304</v>
+        <v>-0.2076304948680112</v>
       </c>
       <c r="AE31" s="83" t="n">
-        <v>100.4228167754111</v>
+        <v>100.4250394723512</v>
       </c>
       <c r="AF31" s="83" t="n">
-        <v>99.24056533021594</v>
+        <v>99.2414746153278</v>
       </c>
       <c r="AG31" s="83" t="n">
-        <v>95.34380004882813</v>
+        <v>95.34400009155273</v>
       </c>
       <c r="AH31" s="83" t="n">
-        <v>103.698099822998</v>
+        <v>103.6981998443603</v>
       </c>
       <c r="AI31" s="83" t="n">
-        <v>105.4621997451782</v>
+        <v>105.4622497558594</v>
       </c>
       <c r="AJ31" s="83" t="n">
-        <v>107.0284530879407</v>
+        <v>107.0294958891796</v>
       </c>
       <c r="AK31" s="83" t="n">
-        <v>100.0795001983643</v>
+        <v>100.0800003051758</v>
       </c>
       <c r="AL31" s="83" t="n">
-        <v>93.13054730878778</v>
+        <v>93.13050472117202</v>
       </c>
       <c r="AM31" s="87" t="n">
-        <v>0.6353080756187865</v>
+        <v>0.6359811581057558</v>
       </c>
       <c r="AN31" s="36" t="n">
-        <v>13.88686569338013</v>
+        <v>13.88788082096832</v>
       </c>
       <c r="AO31" s="88" t="n">
-        <v>3.866797668803516</v>
+        <v>3.866418378457375</v>
       </c>
       <c r="AP31" s="83" t="n">
         <v>135.2400054931641</v>
@@ -7881,22 +7881,22 @@
         <v>74.98999786376953</v>
       </c>
       <c r="AR31" s="36" t="n">
-        <v>-24.60810785043454</v>
+        <v>-24.6007120090975</v>
       </c>
       <c r="AS31" s="89" t="n">
-        <v>44.76348183488878</v>
+        <v>44.78008288877079</v>
       </c>
       <c r="AT31" s="33" t="n">
-        <v>0.03240175049640115</v>
+        <v>0.03250302769378988</v>
       </c>
       <c r="AU31" s="33" t="n">
-        <v>0.04692473275967557</v>
+        <v>0.04702743464172876</v>
       </c>
       <c r="AV31" s="33" t="n">
-        <v>-0.03300458342522761</v>
+        <v>-0.03290972249959334</v>
       </c>
       <c r="AW31" s="33" t="n">
-        <v>0.114438752488476</v>
+        <v>0.114548077403374</v>
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
@@ -8006,10 +8006,10 @@
         <v>92.87999725341797</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>50102585</v>
+        <v>50881908</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>1.745629794349376</v>
+        <v>1.770378765848993</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>61.38093875257105</v>
@@ -8088,17 +8088,17 @@
       </c>
       <c r="AX32" s="79" t="inlineStr">
         <is>
+          <t>Why CoreWeave Stock Soared 12% Today</t>
+        </is>
+      </c>
+      <c r="AY32" s="79" t="inlineStr">
+        <is>
           <t>Billionaire David Tepper Just Bought These 2 Artificial Intelligence (AI) Stocks That Wall Street Thinks Co...</t>
         </is>
       </c>
-      <c r="AY32" s="79" t="inlineStr">
+      <c r="AZ32" s="79" t="inlineStr">
         <is>
           <t>CRWV Stock Takes a 13% Hit in 3 Months: Time to Buy, Hold or Bail Out?</t>
-        </is>
-      </c>
-      <c r="AZ32" s="79" t="inlineStr">
-        <is>
-          <t>Nebius Stock Up 254% in a Year: Should You Buy, Hold or Sell?</t>
         </is>
       </c>
     </row>
@@ -8110,7 +8110,7 @@
         </is>
       </c>
       <c r="C33" s="33" t="n">
-        <v>0.01783869829554785</v>
+        <v>0.01858280223254472</v>
       </c>
       <c r="D33" s="34" t="n">
         <v>13</v>
@@ -8179,10 +8179,10 @@
         </is>
       </c>
       <c r="R33" s="81" t="n">
-        <v>533.489990234375</v>
+        <v>533.8800048828125</v>
       </c>
       <c r="S33" s="82" t="n">
-        <v>9.3499755859375</v>
+        <v>9.739990234375</v>
       </c>
       <c r="T33" s="83" t="n">
         <v>521.1500244140625</v>
@@ -8194,61 +8194,61 @@
         <v>515.5601196289062</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>6260404</v>
+        <v>6589879</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.7468358570978624</v>
+        <v>0.784598704237046</v>
       </c>
       <c r="Y33" s="35" t="n">
-        <v>65.0245878859218</v>
+        <v>65.07915030378641</v>
       </c>
       <c r="Z33" s="35" t="n">
-        <v>95.76572344090685</v>
+        <v>96.10040124674029</v>
       </c>
       <c r="AA33" s="35" t="n">
         <v>10.54085024096999</v>
       </c>
       <c r="AB33" s="86" t="n">
-        <v>19.25707882367112</v>
+        <v>19.28819110331858</v>
       </c>
       <c r="AC33" s="86" t="n">
-        <v>12.39713166255265</v>
+        <v>12.40335411848215</v>
       </c>
       <c r="AD33" s="86" t="n">
-        <v>6.85994716111847</v>
+        <v>6.884836984836436</v>
       </c>
       <c r="AE33" s="83" t="n">
-        <v>494.564759642242</v>
+        <v>494.651429564117</v>
       </c>
       <c r="AF33" s="83" t="n">
-        <v>470.6447128577041</v>
+        <v>470.6801687348348</v>
       </c>
       <c r="AG33" s="83" t="n">
-        <v>442.1323992919922</v>
+        <v>442.140199584961</v>
       </c>
       <c r="AH33" s="83" t="n">
-        <v>374.0185989379883</v>
+        <v>374.0224990844727</v>
       </c>
       <c r="AI33" s="83" t="n">
-        <v>255.5051996231079</v>
+        <v>255.5071496963501</v>
       </c>
       <c r="AJ33" s="83" t="n">
-        <v>531.5637648284028</v>
+        <v>531.6638865410406</v>
       </c>
       <c r="AK33" s="83" t="n">
-        <v>469.8950012207031</v>
+        <v>469.914501953125</v>
       </c>
       <c r="AL33" s="83" t="n">
-        <v>408.2262376130034</v>
+        <v>408.1651173652094</v>
       </c>
       <c r="AM33" s="87" t="n">
-        <v>1.015617512767288</v>
+        <v>1.017944456908852</v>
       </c>
       <c r="AN33" s="36" t="n">
-        <v>26.24789088945201</v>
+        <v>26.28111468416662</v>
       </c>
       <c r="AO33" s="88" t="n">
-        <v>5.892983959488309</v>
+        <v>5.88867896577027</v>
       </c>
       <c r="AP33" s="83" t="n">
         <v>538.4243774414062</v>
@@ -8257,36 +8257,36 @@
         <v>110.2200012207031</v>
       </c>
       <c r="AR33" s="36" t="n">
-        <v>-0.9164494428130165</v>
+        <v>-0.8440131518911986</v>
       </c>
       <c r="AS33" s="89" t="n">
-        <v>98.84765605373262</v>
+        <v>98.93873747888753</v>
       </c>
       <c r="AT33" s="33" t="n">
-        <v>0.169908508167556</v>
+        <v>0.1707637846748369</v>
       </c>
       <c r="AU33" s="33" t="n">
-        <v>0.1756837233638675</v>
+        <v>0.1765432219157335</v>
       </c>
       <c r="AV33" s="33" t="n">
-        <v>0.3311625242881535</v>
+        <v>0.3321356875966073</v>
       </c>
       <c r="AW33" s="33" t="n">
-        <v>3.238083904310614</v>
+        <v>3.241182209497675</v>
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
+          <t>Is Dell Making Money Where You Think It Is?</t>
+        </is>
+      </c>
+      <c r="AY33" s="90" t="inlineStr">
+        <is>
           <t>Snowflake Expands in Cloud Analytics: Can It Challenge DELL &amp; ORCL?</t>
         </is>
       </c>
-      <c r="AY33" s="90" t="inlineStr">
+      <c r="AZ33" s="90" t="inlineStr">
         <is>
           <t>The Enterprise AI Fight Has a New Challenger and It Is Not Who You Would Expect</t>
-        </is>
-      </c>
-      <c r="AZ33" s="90" t="inlineStr">
-        <is>
-          <t>Why Did DELL, VOD, ZETA Stocks Surge To 52-Week Highs Last Week?</t>
         </is>
       </c>
     </row>
@@ -8310,7 +8310,7 @@
       </c>
       <c r="F34" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G34" s="23" t="inlineStr">
@@ -8382,10 +8382,10 @@
         <v>330.3900146484375</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>12912913</v>
+        <v>13853543</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.8520242027310269</v>
+        <v>0.9112613000926292</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>44.03811679114303</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
-          <t>Google Cloud Boss Makes Bold Claim About AI Chip Business</t>
+          <t>Google Warns EU Regulations Will Result In Lower Search Quality</t>
         </is>
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
-          <t>Will Direct TPU Sales Re-Rate Google Stock?</t>
+          <t>Bank of America Spots Reassuring Signal for Google Stock</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Google degrades E.U. search results to comply with DMA rules</t>
+          <t>Google, Blackstone Venture Faces Delays at Data-Center Sites</t>
         </is>
       </c>
     </row>
@@ -8570,10 +8570,10 @@
         <v>46.0099983215332</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>49654576</v>
+        <v>50573887</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>1.064175032340439</v>
+        <v>1.082810610039409</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>60.3906396358092</v>
@@ -8758,10 +8758,10 @@
         <v>100.3499984741211</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>135748800</v>
+        <v>139493818</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>1.362964390922728</v>
+        <v>1.397937442200805</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>61.6991840431096</v>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
-          <t>Why Broadcom Stock Rallied Tuesday Morning</t>
+          <t>Stock Market Today, Sept. 8: Stocks Slide Amid Surging Oil Prices, Persistent Geopolotical Tenisons</t>
         </is>
       </c>
       <c r="AY36" s="79" t="inlineStr">
         <is>
-          <t>Update: Market Chatter: Intel May Raise PC CPU Prices Another 10% in October; Shares Rise in Afternoon Trading</t>
+          <t>Intel Leads Chip Stocks Rally as Qualcomm, AMD and Broadcom Stocks Jump</t>
         </is>
       </c>
       <c r="AZ36" s="79" t="inlineStr">
         <is>
-          <t>Intel Stock Jumps on Major Analyst Upgrade</t>
+          <t>AMD, Amgen, Novartis, Qualcomn, Corning, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
     </row>
@@ -8874,7 +8874,7 @@
       </c>
       <c r="F37" s="30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G37" s="30" t="inlineStr">
@@ -8913,7 +8913,7 @@
         </is>
       </c>
       <c r="N37" s="80" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O37" s="30" t="inlineStr">
         <is>
@@ -8946,10 +8946,10 @@
         <v>490.1499938964844</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>15678467</v>
+        <v>18684730</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.7056011512252309</v>
+        <v>0.835246190975353</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>55.96867258696406</v>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
-          <t>Alphabet Stock Is Pulling Back From Its High. Here’s Why I’d Buy the Dip.</t>
+          <t>Microsoft's OpenAI Partnership Draws Fresh Legal Fire</t>
         </is>
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
-          <t>Network to Code Appoints Chris Millerick as Chief Revenue Officer to Scale Commercial Software Growth</t>
+          <t>Goldman's New AI Office Adds Just 1% to Its Engineering Army</t>
         </is>
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>AI Could Nearly Triple America's Data Center Footprint by 2030</t>
+          <t>Prop Industry Leader The5ers Brings Single Stock Futures via CME Feed</t>
         </is>
       </c>
     </row>
@@ -9134,10 +9134,10 @@
         <v>135.3800048828125</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>17715754</v>
+        <v>19289134</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.6329339733410267</v>
+        <v>0.6872149063484077</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>61.36705890882406</v>
@@ -9221,12 +9221,12 @@
       </c>
       <c r="AY38" s="79" t="inlineStr">
         <is>
+          <t>Strategy doubles STRC buyback to $2 billion as Bitcoin treasury grows</t>
+        </is>
+      </c>
+      <c r="AZ38" s="79" t="inlineStr">
+        <is>
           <t>Strategy CEO says 'never sell' was just a marketing slogan</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>Strategy's Return to Bitcoin Buying Lasted Exactly One Week</t>
         </is>
       </c>
     </row>
@@ -9322,10 +9322,10 @@
         <v>997.6400146484375</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>25252605</v>
+        <v>26367138</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.9158679708864907</v>
+        <v>0.9543612726384941</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>57.66197475179354</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
-          <t>Thinking of Buying Micron Stock Now? Here's 1 Green Flag and 1 Red Flag.</t>
+          <t>Micron (MU) Falls More Steeply Than Broader Market: What Investors Need to Know</t>
         </is>
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
-          <t>SK Hynix Jumps 7% as AI Diverts Memory From Phones; Micron Holds Steady, Apple Slips</t>
+          <t>Micron and Sandisk Soar as Goldman Sees New Memory Stock Rally</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
         <is>
-          <t>Micron Technology (MU) Rose on Elevated Demand for High-Bandwidth Memory</t>
+          <t>Goldman Says the Worst May Be Over for Micron and SanDisk</t>
         </is>
       </c>
     </row>
@@ -9510,10 +9510,10 @@
         <v>234.3249969482422</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>25750274</v>
+        <v>26604516</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>1.152738990388753</v>
+        <v>1.188707189744639</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>58.48647113982799</v>
@@ -9698,10 +9698,10 @@
         <v>75.91999816894531</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>32107555</v>
+        <v>33754561</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>1.134685407529787</v>
+        <v>1.189429264580592</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>45.43138140489266</v>
@@ -9802,7 +9802,7 @@
         </is>
       </c>
       <c r="C42" s="26" t="n">
-        <v>0.06281157838618334</v>
+        <v>0.06181454656683427</v>
       </c>
       <c r="D42" s="27" t="n">
         <v>4</v>
@@ -9871,10 +9871,10 @@
         </is>
       </c>
       <c r="R42" s="70" t="n">
-        <v>10.65999984741211</v>
+        <v>10.64999961853027</v>
       </c>
       <c r="S42" s="71" t="n">
-        <v>0.630000114440918</v>
+        <v>0.619999885559082</v>
       </c>
       <c r="T42" s="72" t="n">
         <v>10.46000003814697</v>
@@ -9886,61 +9886,61 @@
         <v>10.32999992370605</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>108781432</v>
+        <v>112224091</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>1.52289036766127</v>
+        <v>1.5673091469557</v>
       </c>
       <c r="Y42" s="28" t="n">
-        <v>55.88489331573219</v>
+        <v>55.76913742500214</v>
       </c>
       <c r="Z42" s="28" t="n">
-        <v>84.84849579516226</v>
+        <v>84.09090252290264</v>
       </c>
       <c r="AA42" s="28" t="n">
         <v>12.62105813084566</v>
       </c>
       <c r="AB42" s="75" t="n">
-        <v>-0.0703892377971389</v>
+        <v>-0.07118697685324094</v>
       </c>
       <c r="AC42" s="75" t="n">
-        <v>-0.126230317093964</v>
+        <v>-0.1263898649051844</v>
       </c>
       <c r="AD42" s="75" t="n">
-        <v>0.05584107929682505</v>
+        <v>0.05520288805194343</v>
       </c>
       <c r="AE42" s="72" t="n">
-        <v>10.17252185406472</v>
+        <v>10.17029958097986</v>
       </c>
       <c r="AF42" s="72" t="n">
-        <v>10.17290437885797</v>
+        <v>10.17199526714144</v>
       </c>
       <c r="AG42" s="72" t="n">
-        <v>10.48319997787476</v>
+        <v>10.48299997329712</v>
       </c>
       <c r="AH42" s="72" t="n">
-        <v>12.01819999694824</v>
+        <v>12.01809999465942</v>
       </c>
       <c r="AI42" s="72" t="n">
-        <v>9.626149997711181</v>
+        <v>9.626099996566772</v>
       </c>
       <c r="AJ42" s="72" t="n">
-        <v>10.9102128486372</v>
+        <v>10.90846297148201</v>
       </c>
       <c r="AK42" s="72" t="n">
-        <v>10.23150005340576</v>
+        <v>10.23100004196167</v>
       </c>
       <c r="AL42" s="72" t="n">
-        <v>9.552787258174327</v>
+        <v>9.553537112441333</v>
       </c>
       <c r="AM42" s="76" t="n">
-        <v>0.8156709266547955</v>
+        <v>0.8092417004021665</v>
       </c>
       <c r="AN42" s="29" t="n">
-        <v>13.26712196039157</v>
+        <v>13.24333743997212</v>
       </c>
       <c r="AO42" s="77" t="n">
-        <v>4.485590584481948</v>
+        <v>4.489802503178826</v>
       </c>
       <c r="AP42" s="72" t="n">
         <v>17.45000076293945</v>
@@ -9949,22 +9949,22 @@
         <v>4.480000019073486</v>
       </c>
       <c r="AR42" s="29" t="n">
-        <v>-38.91117833042185</v>
+        <v>-38.9684862298179</v>
       </c>
       <c r="AS42" s="78" t="n">
-        <v>47.64841537315557</v>
+        <v>47.57131261056271</v>
       </c>
       <c r="AT42" s="26" t="n">
-        <v>0.05128200063935684</v>
+        <v>0.05029578480668961</v>
       </c>
       <c r="AU42" s="26" t="n">
-        <v>0.1388889143609602</v>
+        <v>0.1378205138002078</v>
       </c>
       <c r="AV42" s="26" t="n">
-        <v>-0.2693625952072866</v>
+        <v>-0.2700480118472626</v>
       </c>
       <c r="AW42" s="26" t="n">
-        <v>0.6476043575105503</v>
+        <v>0.6460587270304696</v>
       </c>
       <c r="AX42" s="79" t="inlineStr">
         <is>
@@ -10074,10 +10074,10 @@
         <v>224.8500061035156</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>112572117</v>
+        <v>118984635</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.874440973657972</v>
+        <v>0.9219561243039245</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>56.14514785469748</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>6 Massive Reasons Standard Lithium Stock Popped 33% in August</t>
+          <t>Dow Jones Futures: Dow Skids But AMD, HPE Are New Buys; Apple iPhone Event Due</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>James Altucher: Elon Musk's Next Move Could Eclipse Everything He's Ever Built, and It May Be His Last</t>
+          <t>Prop Industry Leader The5ers Brings Single Stock Futures via CME Feed</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>1 No-Brainer ETF I'm Loading Up on in 2026 and Beyond</t>
+          <t>Nvidia Falls as Its Firmus Bet Lands OpenAI</t>
         </is>
       </c>
     </row>
@@ -10262,10 +10262,10 @@
         <v>170.0200042724609</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>21993292</v>
+        <v>24436325</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>0.7008287526950384</v>
+        <v>0.7756581915090189</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>51.29456085708777</v>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Palantir Technologies Inc. (PLTR) Falls More Steeply Than Broader Market: What Investors Need to Know</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>Sector Update: Tech Stocks Rise Late Afternoon</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>Palantir Wants to Kill the 'Pay-Per-Token' AI Economy</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Sector Update: Tech Stocks Gain Tuesday Afternoon</t>
         </is>
       </c>
     </row>
@@ -10450,10 +10450,10 @@
         <v>172.0352020263672</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>25046873</v>
+        <v>25627305</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>2.533689519128793</v>
+        <v>2.584816399101715</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>58.91644929504607</v>
@@ -10532,17 +10532,17 @@
       </c>
       <c r="AX45" s="90" t="inlineStr">
         <is>
-          <t>How They Run: Qualcomm CEO Cristiano Amon</t>
+          <t>Qualcomm and Amazon ink deal for custom data center chips</t>
         </is>
       </c>
       <c r="AY45" s="90" t="inlineStr">
         <is>
-          <t>Qualcomm and Amazon ink deal for custom data center chips</t>
+          <t>AMD Jumps 6.7% While Amazon Opens a $60 Billion AI-Chip Door</t>
         </is>
       </c>
       <c r="AZ45" s="90" t="inlineStr">
         <is>
-          <t>Qualcomm Stock Rises 6% on Multi-Generation Amazon Silicon Deal</t>
+          <t>Stock Market Today: Dow Dives, Qualcomm Clears Key Level On Amazon Deal; Fertilizer Leader Rises (Live Cove...</t>
         </is>
       </c>
     </row>
@@ -10638,10 +10638,10 @@
         <v>64.15000152587891</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>22391532</v>
+        <v>23996422</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>1.35416532106073</v>
+        <v>1.444215065552374</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>40.93796259622257</v>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Rocket Lab Introduces New Solar Cell — Can RKLB Tackle Supply Chain Constraints In The Space Power Industry?</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
+          <t>Rocket Lab Introduces High-Efficiency Solar Cell to Reduce Reliance on Supply-Constrained Critical Minerals</t>
+        </is>
+      </c>
+      <c r="AZ46" s="79" t="inlineStr">
+        <is>
           <t>SpaceX Rises 4% as Pivotal Research Launches Coverage at $220, Intuitive Machines Climbs 5%, Rocket Lab Gai...</t>
-        </is>
-      </c>
-      <c r="AY46" s="79" t="inlineStr">
-        <is>
-          <t>How Far Could RKLB Stock Fall In The Next Shock?</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>Grounded and Falling: Why One Wall Street Pro Says Rocket Lab Will More Than Double Soon</t>
         </is>
       </c>
     </row>
@@ -10826,10 +10826,10 @@
         <v>1733.780029296875</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>10879063</v>
+        <v>11080819</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.8189011189700732</v>
+        <v>0.8334550485156649</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>61.1120814610072</v>
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
-          <t>SanDisk Stock Has Soared More Than 500% in 2026. Can the Rally Possibly Continue?</t>
+          <t>Micron and Sandisk Soar as Goldman Sees New Memory Stock Rally</t>
         </is>
       </c>
       <c r="AY47" s="90" t="inlineStr">
         <is>
-          <t>SanDisk Up Over 40% Past Month: Can the Rally Last?</t>
+          <t>Goldman Says the Worst May Be Over for Micron and SanDisk</t>
         </is>
       </c>
       <c r="AZ47" s="90" t="inlineStr">
         <is>
-          <t>Goldman Spots Breakout Signal for Micron, SanDisk Stocks</t>
+          <t>Sandisk Jumps Nearly 3.5% as S&amp;P 100 Promotion Extends Its AI Run</t>
         </is>
       </c>
     </row>
@@ -11014,10 +11014,10 @@
         <v>355.7999877929688</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>49716440</v>
+        <v>50850639</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>1.268826722362927</v>
+        <v>1.295897356861204</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>55.7109935010271</v>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>Tesla Cybercab Could Beat Waymo on Cost by Up to 30 Cents A Mile, Goldman Says</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
+          <t>Uber Stock Falls As Wall Street Sizes Up Tesla's Cybercab Rollout</t>
+        </is>
+      </c>
+      <c r="AZ48" s="79" t="inlineStr">
+        <is>
           <t>Uber Falls 4% on Tesla Cybercab Threat as Slovenia Clears Full Self-Driving; TSLA Stock Rises 4%</t>
-        </is>
-      </c>
-      <c r="AY48" s="79" t="inlineStr">
-        <is>
-          <t>Tesla Stock Rises. Musk's Robotaxi Bet Gets a New Vehicle</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Tesla Jumps as Slovenia Opens Europe's Sixth FSD Door</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Sep 2026, 08:02 PM · Yahoo Finance data</t>
+          <t>Built 8 Sep 2026, 10:43 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Sep 2026, 08:02 PM · Yahoo Finance data</t>
+          <t>Built 8 Sep 2026, 10:43 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Sep 2026, 08:02 PM · Yahoo Finance data</t>
+          <t>Built 8 Sep 2026, 10:43 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Sep 2026, 08:02 PM · Yahoo Finance data</t>
+          <t>Built 8 Sep 2026, 10:43 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -43355,25 +43355,25 @@
         </is>
       </c>
       <c r="D6" s="26" t="n">
-        <v>0.01100533652705571</v>
+        <v>0.01108334548129264</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>0.01258599619603817</v>
+        <v>0.01266412711363518</v>
       </c>
       <c r="F6" s="26" t="n">
-        <v>0.1263478154721467</v>
+        <v>0.1264347242272419</v>
       </c>
       <c r="G6" s="26" t="n">
-        <v>0.1103205444298097</v>
+        <v>0.1104062165241195</v>
       </c>
       <c r="H6" s="26" t="n">
-        <v>0.1499467283484432</v>
+        <v>0.1500354579905785</v>
       </c>
       <c r="I6" s="26" t="n">
-        <v>0.4485573857267353</v>
+        <v>0.4486691561029441</v>
       </c>
       <c r="J6" s="27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K6" s="101" t="inlineStr">
         <is>
@@ -43393,22 +43393,22 @@
         </is>
       </c>
       <c r="D7" s="33" t="n">
-        <v>-0.02502183355201748</v>
+        <v>-0.02519680456298767</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>-0.0198193371472255</v>
+        <v>-0.01999524180582679</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>0.008932949370805243</v>
+        <v>0.008751884784717445</v>
       </c>
       <c r="G7" s="33" t="n">
-        <v>0.09505411297601873</v>
+        <v>0.09485759295966534</v>
       </c>
       <c r="H7" s="33" t="n">
-        <v>0.08362511094671254</v>
+        <v>0.08343064199581729</v>
       </c>
       <c r="I7" s="33" t="n">
-        <v>0.07984496360907012</v>
+        <v>0.0796511730489573</v>
       </c>
       <c r="J7" s="34" t="n">
         <v>3</v>
@@ -43431,25 +43431,25 @@
         </is>
       </c>
       <c r="D8" s="26" t="n">
-        <v>-0.004373809418090291</v>
+        <v>-0.004552371166540725</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>0.0007177627104955064</v>
+        <v>0.0005382878080617548</v>
       </c>
       <c r="F8" s="26" t="n">
-        <v>0.002606749802492869</v>
+        <v>0.002426936117450929</v>
       </c>
       <c r="G8" s="26" t="n">
-        <v>0.004050810986328424</v>
+        <v>0.003870738314437405</v>
       </c>
       <c r="H8" s="26" t="n">
-        <v>-0.05120786634982655</v>
+        <v>-0.05137802858933294</v>
       </c>
       <c r="I8" s="26" t="n">
-        <v>-0.05249745362803238</v>
+        <v>-0.05266738458499387</v>
       </c>
       <c r="J8" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K8" s="101" t="inlineStr">
         <is>
@@ -43525,7 +43525,7 @@
         <v>0.0178028147266085</v>
       </c>
       <c r="J10" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K10" s="101" t="inlineStr">
         <is>
@@ -43545,22 +43545,22 @@
         </is>
       </c>
       <c r="D11" s="33" t="n">
-        <v>-0.01368327349095233</v>
+        <v>-0.0137693503970896</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>-0.007017826818954909</v>
+        <v>-0.00710448542568809</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>-0.005121496124307234</v>
+        <v>-0.005208320225830065</v>
       </c>
       <c r="G11" s="33" t="n">
-        <v>0.1026553580750613</v>
+        <v>0.1025591281732379</v>
       </c>
       <c r="H11" s="33" t="n">
-        <v>0.1385853014179184</v>
+        <v>0.1384859358718564</v>
       </c>
       <c r="I11" s="33" t="n">
-        <v>0.0462844591240601</v>
+        <v>0.04619314877033642</v>
       </c>
       <c r="J11" s="34" t="n">
         <v>3</v>
@@ -43583,22 +43583,22 @@
         </is>
       </c>
       <c r="D12" s="26" t="n">
-        <v>-0.006739178085651609</v>
+        <v>-0.006621011774235575</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>-0.01141446437262328</v>
+        <v>-0.01129685427093907</v>
       </c>
       <c r="F12" s="26" t="n">
-        <v>-0.01304042028354058</v>
+        <v>-0.01292300361867404</v>
       </c>
       <c r="G12" s="26" t="n">
-        <v>0.01131578722594861</v>
+        <v>0.0114361015015314</v>
       </c>
       <c r="H12" s="26" t="n">
-        <v>-0.02279863971899831</v>
+        <v>-0.02268238397055089</v>
       </c>
       <c r="I12" s="26" t="n">
-        <v>0.08148817979127787</v>
+        <v>0.08161684234015376</v>
       </c>
       <c r="J12" s="27" t="n">
         <v>2</v>
@@ -43621,22 +43621,22 @@
         </is>
       </c>
       <c r="D13" s="33" t="n">
-        <v>-0.009343971712462262</v>
+        <v>-0.009534706580738517</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>-0.01404437052678953</v>
+        <v>-0.0142342004089524</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>-0.0172152825748153</v>
+        <v>-0.0174045019489163</v>
       </c>
       <c r="G13" s="33" t="n">
-        <v>0.03983189981853474</v>
+        <v>0.03963169692794688</v>
       </c>
       <c r="H13" s="33" t="n">
-        <v>0.03920782193766015</v>
+        <v>0.03900773920322043</v>
       </c>
       <c r="I13" s="33" t="n">
-        <v>0.1455347852455748</v>
+        <v>0.1453142309662583</v>
       </c>
       <c r="J13" s="34" t="n">
         <v>3</v>
@@ -43659,22 +43659,22 @@
         </is>
       </c>
       <c r="D14" s="26" t="n">
-        <v>-0.0007967185788519959</v>
+        <v>-0.0006828768287838738</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>-0.004874181582700698</v>
+        <v>-0.004760804388276862</v>
       </c>
       <c r="F14" s="26" t="n">
-        <v>-0.0241218118166906</v>
+        <v>-0.02401062755332628</v>
       </c>
       <c r="G14" s="26" t="n">
-        <v>-0.003066053265408653</v>
+        <v>-0.00295247006636512</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>0.02128899314268673</v>
+        <v>0.02140535117359632</v>
       </c>
       <c r="I14" s="26" t="n">
-        <v>0.08785631022802143</v>
+        <v>0.08798025244126451</v>
       </c>
       <c r="J14" s="27" t="n">
         <v>2</v>
@@ -43697,22 +43697,22 @@
         </is>
       </c>
       <c r="D15" s="33" t="n">
-        <v>-0.007745252725428697</v>
+        <v>-0.008006315977894363</v>
       </c>
       <c r="E15" s="33" t="n">
-        <v>-0.02204305494080361</v>
+        <v>-0.02230035642668704</v>
       </c>
       <c r="F15" s="33" t="n">
-        <v>-0.04872354361377162</v>
+        <v>-0.04897382543543116</v>
       </c>
       <c r="G15" s="33" t="n">
-        <v>-0.01187280313570171</v>
+        <v>-0.01213278042537624</v>
       </c>
       <c r="H15" s="33" t="n">
-        <v>-0.00497425353905645</v>
+        <v>-0.005236045844280168</v>
       </c>
       <c r="I15" s="33" t="n">
-        <v>-0.04513865550406393</v>
+        <v>-0.0453898805135009</v>
       </c>
       <c r="J15" s="34" t="n">
         <v>1</v>
@@ -43864,7 +43864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G61"/>
+  <dimension ref="B2:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -43996,7 +43996,7 @@
       </c>
       <c r="D8" s="106" t="inlineStr">
         <is>
-          <t>Reclaimed the 200 DMA</t>
+          <t>Volume 1.8x its 20-day average</t>
         </is>
       </c>
       <c r="E8" s="26" t="n">
@@ -44024,7 +44024,7 @@
       </c>
       <c r="D9" s="107" t="inlineStr">
         <is>
-          <t>Gapped up 4.0% at the open</t>
+          <t>Reclaimed the 200 DMA</t>
         </is>
       </c>
       <c r="E9" s="33" t="n">
@@ -44042,21 +44042,21 @@
     <row r="10">
       <c r="B10" s="24" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="C10" s="101" t="inlineStr">
         <is>
-          <t>Intel Corporation</t>
-        </is>
-      </c>
-      <c r="D10" s="104" t="inlineStr">
-        <is>
-          <t>8 EMA crossed above 21</t>
+          <t>CoreWeave, Inc.</t>
+        </is>
+      </c>
+      <c r="D10" s="106" t="inlineStr">
+        <is>
+          <t>Gapped up 4.0% at the open</t>
         </is>
       </c>
       <c r="E10" s="26" t="n">
-        <v>0.09050102184507414</v>
+        <v>0.1171665303177076</v>
       </c>
       <c r="F10" s="27" t="n">
         <v>9</v>
@@ -44078,9 +44078,9 @@
           <t>Intel Corporation</t>
         </is>
       </c>
-      <c r="D11" s="107" t="inlineStr">
-        <is>
-          <t>Reclaimed the 50 DMA</t>
+      <c r="D11" s="105" t="inlineStr">
+        <is>
+          <t>8 EMA crossed above 21</t>
         </is>
       </c>
       <c r="E11" s="33" t="n">
@@ -44108,7 +44108,7 @@
       </c>
       <c r="D12" s="106" t="inlineStr">
         <is>
-          <t>Gapped up 5.3% at the open</t>
+          <t>Reclaimed the 50 DMA</t>
         </is>
       </c>
       <c r="E12" s="26" t="n">
@@ -44126,21 +44126,21 @@
     <row r="13">
       <c r="B13" s="31" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="C13" s="102" t="inlineStr">
         <is>
-          <t>Nebius Group N.V.</t>
-        </is>
-      </c>
-      <c r="D13" s="105" t="inlineStr">
-        <is>
-          <t>MACD crossed up</t>
+          <t>Intel Corporation</t>
+        </is>
+      </c>
+      <c r="D13" s="107" t="inlineStr">
+        <is>
+          <t>Gapped up 5.3% at the open</t>
         </is>
       </c>
       <c r="E13" s="33" t="n">
-        <v>0.07725608701937992</v>
+        <v>0.09050102184507414</v>
       </c>
       <c r="F13" s="34" t="n">
         <v>9</v>
@@ -44164,7 +44164,7 @@
       </c>
       <c r="D14" s="104" t="inlineStr">
         <is>
-          <t>8 EMA crossed above 21</t>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E14" s="26" t="n">
@@ -44190,9 +44190,9 @@
           <t>Nebius Group N.V.</t>
         </is>
       </c>
-      <c r="D15" s="107" t="inlineStr">
-        <is>
-          <t>Gapped up 3.7% at the open</t>
+      <c r="D15" s="105" t="inlineStr">
+        <is>
+          <t>8 EMA crossed above 21</t>
         </is>
       </c>
       <c r="E15" s="33" t="n">
@@ -44210,21 +44210,21 @@
     <row r="16">
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="C16" s="101" t="inlineStr">
         <is>
-          <t>Nokia Oyj</t>
+          <t>Nebius Group N.V.</t>
         </is>
       </c>
       <c r="D16" s="106" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Gapped up 3.7% at the open</t>
         </is>
       </c>
       <c r="E16" s="26" t="n">
-        <v>0.06281157838618334</v>
+        <v>0.07725608701937992</v>
       </c>
       <c r="F16" s="27" t="n">
         <v>9</v>
@@ -44248,11 +44248,11 @@
       </c>
       <c r="D17" s="107" t="inlineStr">
         <is>
-          <t>Reclaimed the 50 DMA</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E17" s="33" t="n">
-        <v>0.06281157838618334</v>
+        <v>0.06181454656683427</v>
       </c>
       <c r="F17" s="34" t="n">
         <v>9</v>
@@ -44276,11 +44276,11 @@
       </c>
       <c r="D18" s="106" t="inlineStr">
         <is>
-          <t>Gapped up 4.3% at the open</t>
+          <t>Reclaimed the 50 DMA</t>
         </is>
       </c>
       <c r="E18" s="26" t="n">
-        <v>0.06281157838618334</v>
+        <v>0.06181454656683427</v>
       </c>
       <c r="F18" s="27" t="n">
         <v>9</v>
@@ -44304,11 +44304,11 @@
       </c>
       <c r="D19" s="107" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped up 4.3% at the open</t>
         </is>
       </c>
       <c r="E19" s="33" t="n">
-        <v>0.06281157838618334</v>
+        <v>0.06181454656683427</v>
       </c>
       <c r="F19" s="34" t="n">
         <v>9</v>
@@ -44322,21 +44322,21 @@
     <row r="20">
       <c r="B20" s="24" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="C20" s="101" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices, Inc.</t>
+          <t>Nokia Oyj</t>
         </is>
       </c>
       <c r="D20" s="106" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E20" s="26" t="n">
-        <v>0.05898608052877963</v>
+        <v>0.06181454656683427</v>
       </c>
       <c r="F20" s="27" t="n">
         <v>9</v>
@@ -44360,7 +44360,7 @@
       </c>
       <c r="D21" s="107" t="inlineStr">
         <is>
-          <t>Reclaimed the 50 DMA</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E21" s="33" t="n">
@@ -44388,7 +44388,7 @@
       </c>
       <c r="D22" s="106" t="inlineStr">
         <is>
-          <t>Gapped up 2.4% at the open</t>
+          <t>Reclaimed the 50 DMA</t>
         </is>
       </c>
       <c r="E22" s="26" t="n">
@@ -44406,21 +44406,21 @@
     <row r="23">
       <c r="B23" s="31" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="C23" s="102" t="inlineStr">
         <is>
-          <t>IREN Limited</t>
+          <t>Advanced Micro Devices, Inc.</t>
         </is>
       </c>
       <c r="D23" s="107" t="inlineStr">
         <is>
-          <t>Reclaimed the 200 DMA</t>
+          <t>Gapped up 2.4% at the open</t>
         </is>
       </c>
       <c r="E23" s="33" t="n">
-        <v>0.05035810171512822</v>
+        <v>0.05898608052877963</v>
       </c>
       <c r="F23" s="34" t="n">
         <v>9</v>
@@ -44444,7 +44444,7 @@
       </c>
       <c r="D24" s="106" t="inlineStr">
         <is>
-          <t>Gapped up 3.5% at the open</t>
+          <t>Reclaimed the 200 DMA</t>
         </is>
       </c>
       <c r="E24" s="26" t="n">
@@ -44462,21 +44462,21 @@
     <row r="25">
       <c r="B25" s="31" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="C25" s="102" t="inlineStr">
         <is>
-          <t>QUALCOMM Incorporated</t>
-        </is>
-      </c>
-      <c r="D25" s="105" t="inlineStr">
-        <is>
-          <t>Closed above upper band</t>
+          <t>IREN Limited</t>
+        </is>
+      </c>
+      <c r="D25" s="107" t="inlineStr">
+        <is>
+          <t>Gapped up 3.5% at the open</t>
         </is>
       </c>
       <c r="E25" s="33" t="n">
-        <v>0.03170552726421061</v>
+        <v>0.05035810171512822</v>
       </c>
       <c r="F25" s="34" t="n">
         <v>9</v>
@@ -44498,9 +44498,9 @@
           <t>QUALCOMM Incorporated</t>
         </is>
       </c>
-      <c r="D26" s="106" t="inlineStr">
-        <is>
-          <t>Volume 2.5x its 20-day average</t>
+      <c r="D26" s="104" t="inlineStr">
+        <is>
+          <t>Closed above upper band</t>
         </is>
       </c>
       <c r="E26" s="26" t="n">
@@ -44528,7 +44528,7 @@
       </c>
       <c r="D27" s="107" t="inlineStr">
         <is>
-          <t>Reclaimed the 50 DMA</t>
+          <t>Volume 2.6x its 20-day average</t>
         </is>
       </c>
       <c r="E27" s="33" t="n">
@@ -44556,7 +44556,7 @@
       </c>
       <c r="D28" s="106" t="inlineStr">
         <is>
-          <t>Gapped up 6.9% at the open</t>
+          <t>Reclaimed the 50 DMA</t>
         </is>
       </c>
       <c r="E28" s="26" t="n">
@@ -44574,21 +44574,21 @@
     <row r="29">
       <c r="B29" s="31" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="C29" s="102" t="inlineStr">
         <is>
-          <t>State Street Technology Select Sector SPDR ETF</t>
-        </is>
-      </c>
-      <c r="D29" s="105" t="inlineStr">
-        <is>
-          <t>MACD crossed up</t>
+          <t>QUALCOMM Incorporated</t>
+        </is>
+      </c>
+      <c r="D29" s="107" t="inlineStr">
+        <is>
+          <t>Gapped up 6.9% at the open</t>
         </is>
       </c>
       <c r="E29" s="33" t="n">
-        <v>0.003150343559036095</v>
+        <v>0.03170552726421061</v>
       </c>
       <c r="F29" s="34" t="n">
         <v>9</v>
@@ -44602,24 +44602,24 @@
     <row r="30">
       <c r="B30" s="24" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="C30" s="101" t="inlineStr">
         <is>
-          <t>Arm Holdings plc</t>
+          <t>State Street Energy Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D30" s="106" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E30" s="26" t="n">
-        <v>0.03744695378055884</v>
+        <v>0.01108334548129264</v>
       </c>
       <c r="F30" s="27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G30" s="23" t="inlineStr">
         <is>
@@ -44630,24 +44630,24 @@
     <row r="31">
       <c r="B31" s="31" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="C31" s="102" t="inlineStr">
         <is>
-          <t>Arm Holdings plc</t>
-        </is>
-      </c>
-      <c r="D31" s="107" t="inlineStr">
-        <is>
-          <t>Gapped up 3.7% at the open</t>
+          <t>State Street Technology Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D31" s="105" t="inlineStr">
+        <is>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E31" s="33" t="n">
-        <v>0.03744695378055884</v>
+        <v>0.003150343559036095</v>
       </c>
       <c r="F31" s="34" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G31" s="30" t="inlineStr">
         <is>
@@ -44668,7 +44668,7 @@
       </c>
       <c r="D32" s="106" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E32" s="26" t="n">
@@ -44686,21 +44686,21 @@
     <row r="33">
       <c r="B33" s="31" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="C33" s="102" t="inlineStr">
         <is>
-          <t>Dell Technologies Inc.</t>
-        </is>
-      </c>
-      <c r="D33" s="105" t="inlineStr">
-        <is>
-          <t>Closed above upper band</t>
+          <t>Arm Holdings plc</t>
+        </is>
+      </c>
+      <c r="D33" s="107" t="inlineStr">
+        <is>
+          <t>Gapped up 3.7% at the open</t>
         </is>
       </c>
       <c r="E33" s="33" t="n">
-        <v>0.01783869829554785</v>
+        <v>0.03744695378055884</v>
       </c>
       <c r="F33" s="34" t="n">
         <v>8</v>
@@ -44714,12 +44714,12 @@
     <row r="34">
       <c r="B34" s="24" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="C34" s="101" t="inlineStr">
         <is>
-          <t>State Street Energy Select Sector SPDR ETF</t>
+          <t>Arm Holdings plc</t>
         </is>
       </c>
       <c r="D34" s="106" t="inlineStr">
@@ -44728,7 +44728,7 @@
         </is>
       </c>
       <c r="E34" s="26" t="n">
-        <v>0.01100533652705571</v>
+        <v>0.03744695378055884</v>
       </c>
       <c r="F34" s="27" t="n">
         <v>8</v>
@@ -44742,28 +44742,28 @@
     <row r="35">
       <c r="B35" s="31" t="inlineStr">
         <is>
-          <t>ASTS</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="C35" s="102" t="inlineStr">
         <is>
-          <t>AST SpaceMobile, Inc.</t>
+          <t>Dell Technologies Inc.</t>
         </is>
       </c>
       <c r="D35" s="105" t="inlineStr">
         <is>
-          <t>MACD crossed up</t>
+          <t>Closed above upper band</t>
         </is>
       </c>
       <c r="E35" s="33" t="n">
-        <v>0.06114590417781884</v>
+        <v>0.01858280223254472</v>
       </c>
       <c r="F35" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G35" s="30" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Very Strong</t>
         </is>
       </c>
     </row>
@@ -44778,9 +44778,9 @@
           <t>AST SpaceMobile, Inc.</t>
         </is>
       </c>
-      <c r="D36" s="106" t="inlineStr">
-        <is>
-          <t>RSI crossed back above 50</t>
+      <c r="D36" s="104" t="inlineStr">
+        <is>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E36" s="26" t="n">
@@ -44808,7 +44808,7 @@
       </c>
       <c r="D37" s="107" t="inlineStr">
         <is>
-          <t>Gapped up 1.6% at the open</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E37" s="33" t="n">
@@ -44826,21 +44826,21 @@
     <row r="38">
       <c r="B38" s="24" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>ASTS</t>
         </is>
       </c>
       <c r="C38" s="101" t="inlineStr">
         <is>
-          <t>Tesla, Inc.</t>
+          <t>AST SpaceMobile, Inc.</t>
         </is>
       </c>
       <c r="D38" s="106" t="inlineStr">
         <is>
-          <t>Reclaimed the 50 DMA</t>
+          <t>Gapped up 1.6% at the open</t>
         </is>
       </c>
       <c r="E38" s="26" t="n">
-        <v>0.03976507462663403</v>
+        <v>0.06114590417781884</v>
       </c>
       <c r="F38" s="27" t="n">
         <v>7</v>
@@ -44854,21 +44854,21 @@
     <row r="39">
       <c r="B39" s="31" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="C39" s="102" t="inlineStr">
         <is>
-          <t>Cameco Corporation</t>
+          <t>Tesla, Inc.</t>
         </is>
       </c>
       <c r="D39" s="107" t="inlineStr">
         <is>
-          <t>Gapped up 1.7% at the open</t>
+          <t>Reclaimed the 50 DMA</t>
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>0.01211039553875048</v>
+        <v>0.03976507462663403</v>
       </c>
       <c r="F39" s="34" t="n">
         <v>7</v>
@@ -44892,11 +44892,11 @@
       </c>
       <c r="D40" s="106" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped up 1.7% at the open</t>
         </is>
       </c>
       <c r="E40" s="26" t="n">
-        <v>0.01211039553875048</v>
+        <v>0.0122096821820159</v>
       </c>
       <c r="F40" s="27" t="n">
         <v>7</v>
@@ -44910,21 +44910,21 @@
     <row r="41">
       <c r="B41" s="31" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="C41" s="102" t="inlineStr">
         <is>
-          <t>Sandisk Corporation</t>
+          <t>Cameco Corporation</t>
         </is>
       </c>
       <c r="D41" s="107" t="inlineStr">
         <is>
-          <t>Gapped up 1.7% at the open</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>-0.001155178026221226</v>
+        <v>0.0122096821820159</v>
       </c>
       <c r="F41" s="34" t="n">
         <v>7</v>
@@ -44948,7 +44948,7 @@
       </c>
       <c r="D42" s="106" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped up 1.7% at the open</t>
         </is>
       </c>
       <c r="E42" s="26" t="n">
@@ -44966,21 +44966,21 @@
     <row r="43">
       <c r="B43" s="31" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="C43" s="102" t="inlineStr">
         <is>
-          <t>ARK Innovation ETF</t>
+          <t>Sandisk Corporation</t>
         </is>
       </c>
       <c r="D43" s="107" t="inlineStr">
         <is>
-          <t>MACD crossed down</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>-0.001159805992870688</v>
+        <v>-0.001155178026221226</v>
       </c>
       <c r="F43" s="34" t="n">
         <v>7</v>
@@ -44994,21 +44994,21 @@
     <row r="44">
       <c r="B44" s="24" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>ARKK</t>
         </is>
       </c>
       <c r="C44" s="101" t="inlineStr">
         <is>
-          <t>Micron Technology, Inc.</t>
+          <t>ARK Innovation ETF</t>
         </is>
       </c>
       <c r="D44" s="106" t="inlineStr">
         <is>
-          <t>Gapped up 2.0% at the open</t>
+          <t>MACD crossed down</t>
         </is>
       </c>
       <c r="E44" s="26" t="n">
-        <v>-0.01606352281495027</v>
+        <v>-0.001623746087524025</v>
       </c>
       <c r="F44" s="27" t="n">
         <v>7</v>
@@ -45032,7 +45032,7 @@
       </c>
       <c r="D45" s="107" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped up 2.0% at the open</t>
         </is>
       </c>
       <c r="E45" s="33" t="n">
@@ -45050,24 +45050,24 @@
     <row r="46">
       <c r="B46" s="24" t="inlineStr">
         <is>
-          <t>SOXL</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="C46" s="101" t="inlineStr">
         <is>
-          <t>Direxion Daily Semiconductor Bull 3X Shares</t>
+          <t>Micron Technology, Inc.</t>
         </is>
       </c>
       <c r="D46" s="106" t="inlineStr">
         <is>
-          <t>Gapped up 6.7% at the open</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E46" s="26" t="n">
-        <v>0.05192704664625403</v>
+        <v>-0.01606352281495027</v>
       </c>
       <c r="F46" s="27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
@@ -45078,21 +45078,21 @@
     <row r="47">
       <c r="B47" s="31" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SOXL</t>
         </is>
       </c>
       <c r="C47" s="102" t="inlineStr">
         <is>
-          <t>Invesco QQQ Trust</t>
+          <t>Direxion Daily Semiconductor Bull 3X Shares</t>
         </is>
       </c>
       <c r="D47" s="107" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped up 6.7% at the open</t>
         </is>
       </c>
       <c r="E47" s="33" t="n">
-        <v>-0.0008345896889334625</v>
+        <v>0.05107433429498753</v>
       </c>
       <c r="F47" s="34" t="n">
         <v>6</v>
@@ -45106,21 +45106,21 @@
     <row r="48">
       <c r="B48" s="24" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="C48" s="101" t="inlineStr">
         <is>
-          <t>Strategy Inc</t>
+          <t>Invesco QQQ Trust</t>
         </is>
       </c>
       <c r="D48" s="106" t="inlineStr">
         <is>
-          <t>Lost the 200 DMA</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E48" s="26" t="n">
-        <v>-0.04397758154823495</v>
+        <v>-0.0008345896889334625</v>
       </c>
       <c r="F48" s="27" t="n">
         <v>6</v>
@@ -45144,7 +45144,7 @@
       </c>
       <c r="D49" s="107" t="inlineStr">
         <is>
-          <t>Gapped down 3.6% at the open</t>
+          <t>Lost the 200 DMA</t>
         </is>
       </c>
       <c r="E49" s="33" t="n">
@@ -45162,40 +45162,40 @@
     <row r="50">
       <c r="B50" s="24" t="inlineStr">
         <is>
-          <t>RKLB</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="C50" s="101" t="inlineStr">
         <is>
-          <t>Rocket Lab Corporation</t>
+          <t>Strategy Inc</t>
         </is>
       </c>
       <c r="D50" s="106" t="inlineStr">
         <is>
-          <t>Gapped up 1.6% at the open</t>
+          <t>Gapped down 3.6% at the open</t>
         </is>
       </c>
       <c r="E50" s="26" t="n">
-        <v>0.02505447489619406</v>
+        <v>-0.04397758154823495</v>
       </c>
       <c r="F50" s="27" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G50" s="23" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Strong</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="31" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="C51" s="102" t="inlineStr">
         <is>
-          <t>Alphabet Inc.</t>
+          <t>State Street SPDR S&amp;P 500 ETF Trust</t>
         </is>
       </c>
       <c r="D51" s="107" t="inlineStr">
@@ -45204,35 +45204,35 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>0.0002087838857429691</v>
+        <v>-0.005492125910932955</v>
       </c>
       <c r="F51" s="34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G51" s="30" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="24" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>RKLB</t>
         </is>
       </c>
       <c r="C52" s="101" t="inlineStr">
         <is>
-          <t>State Street Communication Services Select Sector SPDR ETF</t>
+          <t>Rocket Lab Corporation</t>
         </is>
       </c>
       <c r="D52" s="106" t="inlineStr">
         <is>
-          <t>MACD crossed down</t>
+          <t>Gapped up 1.6% at the open</t>
         </is>
       </c>
       <c r="E52" s="26" t="n">
-        <v>-0.004373809418090291</v>
+        <v>0.02505447489619406</v>
       </c>
       <c r="F52" s="27" t="n">
         <v>3</v>
@@ -45246,12 +45246,12 @@
     <row r="53">
       <c r="B53" s="31" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="C53" s="102" t="inlineStr">
         <is>
-          <t>State Street SPDR S&amp;P 500 ETF Trust</t>
+          <t>Alphabet Inc.</t>
         </is>
       </c>
       <c r="D53" s="107" t="inlineStr">
@@ -45260,7 +45260,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>-0.005440219203215357</v>
+        <v>0.0002087838857429691</v>
       </c>
       <c r="F53" s="34" t="n">
         <v>3</v>
@@ -45288,7 +45288,7 @@
         </is>
       </c>
       <c r="E54" s="26" t="n">
-        <v>-0.009343971712462262</v>
+        <v>-0.009534706580738517</v>
       </c>
       <c r="F54" s="27" t="n">
         <v>3</v>
@@ -45316,7 +45316,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>-0.01368327349095233</v>
+        <v>-0.0137693503970896</v>
       </c>
       <c r="F55" s="34" t="n">
         <v>3</v>
@@ -45372,7 +45372,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>-0.02502183355201748</v>
+        <v>-0.02519680456298767</v>
       </c>
       <c r="F57" s="34" t="n">
         <v>3</v>
@@ -45400,7 +45400,7 @@
         </is>
       </c>
       <c r="E58" s="26" t="n">
-        <v>-0.02502183355201748</v>
+        <v>-0.02519680456298767</v>
       </c>
       <c r="F58" s="27" t="n">
         <v>3</v>
@@ -45442,21 +45442,21 @@
     <row r="60">
       <c r="B60" s="24" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="C60" s="101" t="inlineStr">
         <is>
-          <t>Amazon.com, Inc.</t>
+          <t>State Street Communication Services Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D60" s="106" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>MACD crossed down</t>
         </is>
       </c>
       <c r="E60" s="26" t="n">
-        <v>-0.005957249184734059</v>
+        <v>-0.004552371166540725</v>
       </c>
       <c r="F60" s="27" t="n">
         <v>2</v>
@@ -45470,37 +45470,93 @@
     <row r="61">
       <c r="B61" s="31" t="inlineStr">
         <is>
+          <t>XLC</t>
+        </is>
+      </c>
+      <c r="C61" s="102" t="inlineStr">
+        <is>
+          <t>State Street Communication Services Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D61" s="107" t="inlineStr">
+        <is>
+          <t>RSI dropped below 50</t>
+        </is>
+      </c>
+      <c r="E61" s="33" t="n">
+        <v>-0.004552371166540725</v>
+      </c>
+      <c r="F61" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="G61" s="30" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="24" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C62" s="101" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="D62" s="106" t="inlineStr">
+        <is>
+          <t>Bands squeezing — a big move often follows</t>
+        </is>
+      </c>
+      <c r="E62" s="26" t="n">
+        <v>-0.005957249184734059</v>
+      </c>
+      <c r="F62" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G62" s="23" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="31" t="inlineStr">
+        <is>
           <t>XLY</t>
         </is>
       </c>
-      <c r="C61" s="102" t="inlineStr">
+      <c r="C63" s="102" t="inlineStr">
         <is>
           <t>State Street Consumer Discretionary Select Sector SPDR ETF</t>
         </is>
       </c>
-      <c r="D61" s="107" t="inlineStr">
+      <c r="D63" s="107" t="inlineStr">
         <is>
           <t>Closed below lower band</t>
         </is>
       </c>
-      <c r="E61" s="33" t="n">
-        <v>-0.007745252725428697</v>
-      </c>
-      <c r="F61" s="34" t="n">
+      <c r="E63" s="33" t="n">
+        <v>-0.008006315977894363</v>
+      </c>
+      <c r="F63" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G61" s="30" t="inlineStr">
+      <c r="G63" s="30" t="inlineStr">
         <is>
           <t>Very Weak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B5:G61"/>
+  <autoFilter ref="B5:G63"/>
   <mergeCells count="1">
     <mergeCell ref="B2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E61">
+  <conditionalFormatting sqref="E6:E63">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>

</xml_diff>

<commit_message>
Daily workbook: 2026-09-08 23:22 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 8 Sep 2026, 10:43 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 8 Sep 2026, 11:22 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Sep 2026, 10:43 PM · Yahoo Finance data</t>
+          <t>Built 8 Sep 2026, 11:22 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
+          <t>S&amp;P 500, Dow End Lower As Middle East Tensions Spur Oil Rally Ahead Of Key Inflation Data — META, QCOM, BE,...</t>
+        </is>
+      </c>
+      <c r="AY19" s="79" t="inlineStr">
+        <is>
           <t>Wall Street Keeps Asking How Much Meta Will Spend. The Better Question Is at What Price to Buy</t>
         </is>
       </c>
-      <c r="AY19" s="79" t="inlineStr">
+      <c r="AZ19" s="79" t="inlineStr">
         <is>
           <t>QQQ vs QQQM: Same Index, Same Stocks, Different Fee – and the Math Says One Leaves You Thousands Richer</t>
-        </is>
-      </c>
-      <c r="AZ19" s="79" t="inlineStr">
-        <is>
-          <t>XYLD vs GPIX vs ISPY: We Compared 3 Ways to Sell Covered Calls on the S&amp;P 500, and the Highest Yield Is Not...</t>
         </is>
       </c>
     </row>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>Jim Cramer Says Amazon and Alphabet Are Cheap. Their Cash Flows Complicate the Case</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
           <t>AMD Jumps 6.7% While Amazon Opens a $60 Billion AI-Chip Door</t>
         </is>
       </c>
-      <c r="AY26" s="79" t="inlineStr">
+      <c r="AZ26" s="79" t="inlineStr">
         <is>
           <t>Spotting Winners: Amazon (NASDAQ:AMZN) And Online Retail Stocks In Q2</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>DAL Stock Drops: Jefferies Sees Possible Snag To In-Cabin Experience Owing To SPCX-VSAT Spectrum Fight</t>
         </is>
       </c>
     </row>
@@ -8276,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
+          <t>Dell (DELL) Q2 2027 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AY33" s="90" t="inlineStr">
+        <is>
           <t>Is Dell Making Money Where You Think It Is?</t>
         </is>
       </c>
-      <c r="AY33" s="90" t="inlineStr">
+      <c r="AZ33" s="90" t="inlineStr">
         <is>
           <t>Snowflake Expands in Cloud Analytics: Can It Challenge DELL &amp; ORCL?</t>
-        </is>
-      </c>
-      <c r="AZ33" s="90" t="inlineStr">
-        <is>
-          <t>The Enterprise AI Fight Has a New Challenger and It Is Not Who You Would Expect</t>
         </is>
       </c>
     </row>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Jim Cramer Says Amazon and Alphabet Are Cheap. Their Cash Flows Complicate the Case</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
+          <t>Druckenmiller Exited Micron and Bought Alphabet. The AI Risks Moved With Him</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>Google Warns EU Regulations Will Result In Lower Search Quality</t>
-        </is>
-      </c>
-      <c r="AY34" s="79" t="inlineStr">
-        <is>
-          <t>Bank of America Spots Reassuring Signal for Google Stock</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Google, Blackstone Venture Faces Delays at Data-Center Sites</t>
         </is>
       </c>
     </row>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>Microsoft’s ‘Useful Yield’ Test Raises the Stakes for NVIDIA’s AI Economics</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
           <t>Microsoft's OpenAI Partnership Draws Fresh Legal Fire</t>
         </is>
       </c>
-      <c r="AY37" s="90" t="inlineStr">
+      <c r="AZ37" s="90" t="inlineStr">
         <is>
           <t>Goldman's New AI Office Adds Just 1% to Its Engineering Army</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Prop Industry Leader The5ers Brings Single Stock Futures via CME Feed</t>
         </is>
       </c>
     </row>
@@ -9221,12 +9221,12 @@
       </c>
       <c r="AY38" s="79" t="inlineStr">
         <is>
+          <t>Strategy just dropped $250 'Bitcoin' Jordans with one big catch</t>
+        </is>
+      </c>
+      <c r="AZ38" s="79" t="inlineStr">
+        <is>
           <t>Strategy doubles STRC buyback to $2 billion as Bitcoin treasury grows</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>Strategy CEO says 'never sell' was just a marketing slogan</t>
         </is>
       </c>
     </row>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Druckenmiller Exited Micron and Bought Alphabet. The AI Risks Moved With Him</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
           <t>Micron (MU) Falls More Steeply Than Broader Market: What Investors Need to Know</t>
         </is>
       </c>
-      <c r="AY39" s="90" t="inlineStr">
+      <c r="AZ39" s="90" t="inlineStr">
         <is>
           <t>Micron and Sandisk Soar as Goldman Sees New Memory Stock Rally</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Goldman Says the Worst May Be Over for Micron and SanDisk</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Why Okta Stock Soared 22% in August and Why There's More Upside Ahead</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Dow Jones Futures: Dow Skids But AMD, HPE Are New Buys; Apple iPhone Event Due</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>Prop Industry Leader The5ers Brings Single Stock Futures via CME Feed</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Nvidia Falls as Its Firmus Bet Lands OpenAI</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Sep 2026, 10:43 PM · Yahoo Finance data</t>
+          <t>Built 8 Sep 2026, 11:22 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Sep 2026, 10:43 PM · Yahoo Finance data</t>
+          <t>Built 8 Sep 2026, 11:22 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Sep 2026, 10:43 PM · Yahoo Finance data</t>
+          <t>Built 8 Sep 2026, 11:22 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Sep 2026, 10:43 PM · Yahoo Finance data</t>
+          <t>Built 8 Sep 2026, 11:22 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-09 23:12 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 9 Sep 2026, 10:35 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 9 Sep 2026, 11:12 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 9 Sep 2026, 10:35 PM · Yahoo Finance data</t>
+          <t>Built 9 Sep 2026, 11:12 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6589,12 +6589,12 @@
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Oil Prices, Yields Hit Stocks, Apple Unfolds iPhone. Inflation Data Due.</t>
+          <t>S&amp;P 500, Dow, Nasdaq End Lower As Oil Crosses $101, Yields Pop Following Bessent’s Expanded Buyback Plan — ...</t>
         </is>
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>S&amp;P 500, Dow, Nasdaq End Lower As Oil Crosses $101, Yields Pop Following Bessent’s Expanded Buyback Plan — ...</t>
+          <t>Apple Finds Advantages Across Fintech In Search Results</t>
         </is>
       </c>
     </row>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Oil Prices, Yields Hit Stocks, Apple Unfolds iPhone. Inflation Data Due.</t>
+          <t>Could Advanced Micro Devices (AMD)’s Partnership With Cisco Systems (CSCO) Unlock a Massive Middle East AI ...</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
-          <t>Could Advanced Micro Devices (AMD)’s Partnership With Cisco Systems (CSCO) Unlock a Massive Middle East AI ...</t>
+          <t>AMD, IBD Stock Of The Day, Runs Past Early Buy Point As Chipmaker Returns To Favor</t>
         </is>
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>AMD, IBD Stock Of The Day, Runs Past Early Buy Point As Chipmaker Returns To Favor</t>
+          <t>HostColor Stocks AMD Ryzen 9 9950X Dedicated Servers in Tokyo</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Broadcom Forecasts $230 Billion in AI Semiconductor Revenue in 2028. The Stock Could Reach $900 Per Share a...</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Broadcom (AVGO) Q3 2026 Earnings Call Transcript</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>What Investors Need To Understand About Broadcom, Credo and Snowflake Earnings</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Broadcom Stock Jumps -- AI Revenue Set to Double Again</t>
         </is>
       </c>
     </row>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>HIVE joins Google, Microsoft, and Amazon in new Canada data center pledge</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>Do Amazon and Alphabet's Combined $420 Billion in Capital Expenditures Make Sense?</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
+      <c r="AZ34" s="79" t="inlineStr">
         <is>
           <t>Google Commits €13B to Finland AI Infrastructure, Securing Its First Non-US Nuclear Deal</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Should You Buy Alphabet Stock For The Chips It Now Sells?</t>
         </is>
       </c>
     </row>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>HIVE joins Google, Microsoft, and Amazon in new Canada data center pledge</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
           <t>Can Microsoft Stock Keep Earning Like This?</t>
         </is>
       </c>
-      <c r="AY37" s="90" t="inlineStr">
+      <c r="AZ37" s="90" t="inlineStr">
         <is>
           <t>Microsoft CFO Touts AI Stack, Azure Efficiency and Agent Growth at Goldman Conference</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>ARPA-H Selects UpDoc to Lead Development of Autonomous Clinical AI System, in an Initiative Joined by Micro...</t>
         </is>
       </c>
     </row>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Strive Added 1,375 Bitcoin While Strategy Added None. Their Preferred Shares Explain Why.</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Strategy Put $176.3 Million Into Its Own Preferred Stock Instead of Bitcoin, With Its Last BTC Purchase Alr...</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
-        <is>
-          <t>Investors Heavily Search Strategy Inc (MSTR): Here is What You Need to Know</t>
-        </is>
-      </c>
       <c r="AZ38" s="79" t="inlineStr">
         <is>
-          <t>Strategy Launches $250 Bitcoin Air Jordans but Won’t Let You Pay in BTC</t>
+          <t>MicroStrategy Says It Has the One Thing JPMorgan Lacks</t>
         </is>
       </c>
     </row>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Jim Cramer Compares Palantir (PLTR) to an NFL Wide Receiver</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>Meet the AI Software Stock That’s Crushing Palantir (Hint: It’s Significantly Cheaper)</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>Palantir's CEO says a new partner will power data sovereignty</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Palantir Changed The Number It Wants You To Judge It By</t>
         </is>
       </c>
     </row>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>Goldman Sachs sends stark message to Tesla investors</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
           <t>Could Tesla’s (TSLA) Cybercab Unlock a New Growth Driver?</t>
         </is>
       </c>
-      <c r="AY48" s="79" t="inlineStr">
+      <c r="AZ48" s="79" t="inlineStr">
         <is>
           <t>45 Tesla Cybercabs Are Now Roaming Austin. Here's What That Means for the Robotaxi Business Wall Street Has...</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Entrepreneurs could hold the key to Tesla's Cybercab plans</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 9 Sep 2026, 10:35 PM · Yahoo Finance data</t>
+          <t>Built 9 Sep 2026, 11:12 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 9 Sep 2026, 10:35 PM · Yahoo Finance data</t>
+          <t>Built 9 Sep 2026, 11:12 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 9 Sep 2026, 10:35 PM · Yahoo Finance data</t>
+          <t>Built 9 Sep 2026, 11:12 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 9 Sep 2026, 10:35 PM · Yahoo Finance data</t>
+          <t>Built 9 Sep 2026, 11:12 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-10 23:08 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1299,7 +1299,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 10 Sep 2026, 10:37 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 10 Sep 2026, 11:08 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3104,7 +3104,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 10 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 10 Sep 2026, 11:08 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5813,12 +5813,12 @@
       </c>
       <c r="AY19" s="79" t="inlineStr">
         <is>
+          <t>S&amp;P 500, Dow, Nasdaq End Lower As Surging Oil Raises Odds For A September Rate Hike — ORCL, ADBE, M, NVDA, ...</t>
+        </is>
+      </c>
+      <c r="AZ19" s="79" t="inlineStr">
+        <is>
           <t>Oracle Jumped 36% in a Day After Last September’s Earnings, but Traders Are Betting Against It Tonight</t>
-        </is>
-      </c>
-      <c r="AZ19" s="79" t="inlineStr">
-        <is>
-          <t>Nuclear Stocks Slide as Piper Sandler Splits the Sector: Oklo, NuScale Power and X-Energy All Drop 5%</t>
         </is>
       </c>
     </row>
@@ -9025,17 +9025,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>Remain Bullish on AI Beneficiaries Like Bloom Energy</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
           <t>Nvidia stock edges higher on Microsoft data center expansion report</t>
         </is>
       </c>
-      <c r="AY37" s="90" t="inlineStr">
+      <c r="AZ37" s="90" t="inlineStr">
         <is>
           <t>Sector Update: Tech Stocks Fall Late Afternoon</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Microsoft's New School AI Rules Sacrifice Data to Preserve Access</t>
         </is>
       </c>
     </row>
@@ -10153,17 +10153,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Nvidia Returned $26 Billion to Shareholders Last Quarter Alone. Here's What That Buys You as an Investor.</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Jensen Huang explains why Nvidia will grow an astounding 70% next year</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>Jensen Huang just answered Michael Burry's Nvidia bear case</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Nvidia stock edges higher on Microsoft data center expansion report</t>
         </is>
       </c>
     </row>
@@ -11640,7 +11640,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 10 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 10 Sep 2026, 11:08 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19576,7 +19576,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 10 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 10 Sep 2026, 11:08 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27512,7 +27512,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 10 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 10 Sep 2026, 11:08 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35448,7 +35448,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 10 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 10 Sep 2026, 11:08 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-11 23:14 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 11 Sep 2026, 10:37 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 11 Sep 2026, 11:14 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 11 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 11 Sep 2026, 11:14 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>Palantir Co-Founder Peter Thiel's Hedge Fund Just Made a Big Bet on This AI Stock</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
           <t>Amazon Gains as S&amp;P Flags Its $100 Billion Debt Spree</t>
         </is>
       </c>
-      <c r="AY26" s="79" t="inlineStr">
+      <c r="AZ26" s="79" t="inlineStr">
         <is>
           <t>‘The Largest IPO Ever, Surpassing SpaceX’: Anthropic Is Up Next</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>OpenAI Rethinks Its Next Big Move</t>
         </is>
       </c>
     </row>
@@ -8088,17 +8088,17 @@
       </c>
       <c r="AX32" s="79" t="inlineStr">
         <is>
+          <t>Oracle Just Showed a Less Painful Way to Finance AI Clouds. That’s Awkward for CoreWeave</t>
+        </is>
+      </c>
+      <c r="AY32" s="79" t="inlineStr">
+        <is>
           <t>Oracle's AI Cloud Growth Lifts CoreWeave, Nebius and IREN</t>
         </is>
       </c>
-      <c r="AY32" s="79" t="inlineStr">
+      <c r="AZ32" s="79" t="inlineStr">
         <is>
           <t>CoreWeave Is My Top IPO Pick Right Now: Over 75% of Its Revenue Is Locked In Through Contracts</t>
-        </is>
-      </c>
-      <c r="AZ32" s="79" t="inlineStr">
-        <is>
-          <t>AMD, BE, CRWV In Focus: Situational Awareness Has Been Reportedly Buying Options Tied To These Stocks</t>
         </is>
       </c>
     </row>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>AI’s HBM Shortage Strengthens Micron’s Hand—and Pressures Nvidia’s GPU Economics</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
           <t>Applied Materials vs. Micron Technology: Which Technology Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
-      <c r="AY39" s="90" t="inlineStr">
+      <c r="AZ39" s="90" t="inlineStr">
         <is>
           <t>Micron Takes Unexpected Step as Tensions Rise</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Micron Stays Flat as 68-Month Bonuses Fail to End Strike Risk</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 11 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 11 Sep 2026, 11:14 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 11 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 11 Sep 2026, 11:14 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 11 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 11 Sep 2026, 11:14 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 11 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 11 Sep 2026, 11:14 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>